<commit_message>
Update fractal registry documentation
- Update registry tracking for Julia - Golden Ratio changes
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{8A85B296-2379-44F4-891C-5F3F6F3E786A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F2109D7-E063-4FCB-AFB5-6810A0529FFE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FractalRegistry" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="347">
   <si>
     <t>Group Name</t>
   </si>
@@ -1066,7 +1066,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000000000E+00"/>
   </numFmts>
@@ -1206,7 +1206,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1389,12 +1389,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1588,7 +1582,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1629,9 +1623,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1642,6 +1633,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1687,7 +1687,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="118">
+  <dxfs count="84">
     <dxf>
       <font>
         <b/>
@@ -1952,244 +1952,6 @@
         <b/>
         <i val="0"/>
         <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
       </font>
     </dxf>
     <dxf>
@@ -2823,7 +2585,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I295"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -3671,7 +3433,7 @@
       <c r="I40" s="4"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A41" s="18">
+      <c r="A41" s="22">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
@@ -3681,10 +3443,21 @@
       <c r="C41" t="s">
         <v>47</v>
       </c>
-      <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
+      <c r="D41" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F41" s="14">
+        <v>0.85882670635232194</v>
+      </c>
+      <c r="G41" s="14">
+        <v>-3.1086006813058301E-2</v>
+      </c>
+      <c r="H41" s="4">
+        <v>5.5981979492000002</v>
+      </c>
+      <c r="I41" s="4">
+        <v>5.5981979492000002</v>
+      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
@@ -3767,10 +3540,10 @@
       <c r="D45" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="F45" s="3"/>
-      <c r="G45" s="3"/>
-      <c r="H45" s="4"/>
-      <c r="I45" s="4"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A46" s="2">
@@ -3786,13 +3559,13 @@
       <c r="D46" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="14"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A47" s="18">
+      <c r="A47" s="22">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
@@ -3802,10 +3575,21 @@
       <c r="C47" t="s">
         <v>53</v>
       </c>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
+      <c r="D47" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F47" s="14">
+        <v>-1.11668989158623</v>
+      </c>
+      <c r="G47" s="14">
+        <v>0.176419667590028</v>
+      </c>
+      <c r="H47" s="23">
+        <v>37.968605725000003</v>
+      </c>
+      <c r="I47" s="23">
+        <v>21.35734072</v>
+      </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A48" s="2">
@@ -3821,10 +3605,10 @@
       <c r="D48" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="4"/>
+      <c r="F48" s="14"/>
+      <c r="G48" s="14"/>
+      <c r="H48" s="23"/>
+      <c r="I48" s="23"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" s="2">
@@ -3840,10 +3624,10 @@
       <c r="D49" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="4"/>
+      <c r="F49" s="14"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="23"/>
+      <c r="I49" s="23"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
@@ -3859,10 +3643,10 @@
       <c r="D50" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
+      <c r="F50" s="14"/>
+      <c r="G50" s="14"/>
+      <c r="H50" s="23"/>
+      <c r="I50" s="23"/>
     </row>
     <row r="51" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A51" s="9">
@@ -3879,10 +3663,10 @@
         <v>314</v>
       </c>
       <c r="E51" s="6"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="8"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="15"/>
+      <c r="H51" s="24"/>
+      <c r="I51" s="24"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
@@ -3962,7 +3746,7 @@
       <c r="I55" s="8"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A56" s="18">
+      <c r="A56" s="22">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
@@ -3972,10 +3756,21 @@
       <c r="C56" t="s">
         <v>62</v>
       </c>
-      <c r="F56" s="3"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
+      <c r="D56" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F56" s="14">
+        <v>0</v>
+      </c>
+      <c r="G56" s="14">
+        <v>0</v>
+      </c>
+      <c r="H56" s="4">
+        <v>6</v>
+      </c>
+      <c r="I56" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
@@ -4117,7 +3912,7 @@
         <v>1.4659263959</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="57" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -4270,7 +4065,7 @@
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A68" s="18">
+      <c r="A68" s="22">
         <f t="shared" ref="A68:A131" si="1">A67+1</f>
         <v>67</v>
       </c>
@@ -4280,10 +4075,21 @@
       <c r="C68" t="s">
         <v>76</v>
       </c>
-      <c r="F68" s="3"/>
-      <c r="G68" s="3"/>
-      <c r="H68" s="4"/>
-      <c r="I68" s="4"/>
+      <c r="D68" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F68" s="3">
+        <v>-1</v>
+      </c>
+      <c r="G68" s="3">
+        <v>0</v>
+      </c>
+      <c r="H68" s="4">
+        <v>15</v>
+      </c>
+      <c r="I68" s="4">
+        <v>8.4375</v>
+      </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
@@ -4730,14 +4536,14 @@
       <c r="C86" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="D86" s="19" t="s">
-        <v>314</v>
-      </c>
-      <c r="E86" s="20"/>
-      <c r="F86" s="21"/>
-      <c r="G86" s="21"/>
-      <c r="H86" s="22"/>
-      <c r="I86" s="22"/>
+      <c r="D86" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="E86" s="19"/>
+      <c r="F86" s="20"/>
+      <c r="G86" s="20"/>
+      <c r="H86" s="21"/>
+      <c r="I86" s="21"/>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
@@ -5629,10 +5435,21 @@
       <c r="C119" t="s">
         <v>131</v>
       </c>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="4"/>
-      <c r="I119" s="4"/>
+      <c r="D119" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F119" s="3">
+        <v>4.98391129336773E-2</v>
+      </c>
+      <c r="G119" s="3">
+        <v>2.6326001682159001E-2</v>
+      </c>
+      <c r="H119" s="4">
+        <v>3.4213639189</v>
+      </c>
+      <c r="I119" s="4">
+        <v>1.9245172044000001</v>
+      </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
@@ -5645,10 +5462,21 @@
       <c r="C120" t="s">
         <v>132</v>
       </c>
-      <c r="F120" s="3"/>
-      <c r="G120" s="3"/>
-      <c r="H120" s="4"/>
-      <c r="I120" s="4"/>
+      <c r="D120" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F120" s="3">
+        <v>6.46201485773963E-2</v>
+      </c>
+      <c r="G120" s="3">
+        <v>-1.5682349015682401E-2</v>
+      </c>
+      <c r="H120" s="4">
+        <v>3.9862084307000001</v>
+      </c>
+      <c r="I120" s="4">
+        <v>2.2422422422000001</v>
+      </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
@@ -5661,10 +5489,21 @@
       <c r="C121" t="s">
         <v>133</v>
       </c>
-      <c r="F121" s="3"/>
-      <c r="G121" s="3"/>
-      <c r="H121" s="4"/>
-      <c r="I121" s="4"/>
+      <c r="D121" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F121" s="3">
+        <v>-4.2389169624309896E-3</v>
+      </c>
+      <c r="G121" s="3">
+        <v>5.82727377654678E-3</v>
+      </c>
+      <c r="H121" s="4">
+        <v>4.2807017543999999</v>
+      </c>
+      <c r="I121" s="4">
+        <v>2.4078947367999999</v>
+      </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
@@ -5677,10 +5516,21 @@
       <c r="C122" t="s">
         <v>134</v>
       </c>
-      <c r="F122" s="3"/>
-      <c r="G122" s="3"/>
-      <c r="H122" s="4"/>
-      <c r="I122" s="4"/>
+      <c r="D122" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F122" s="3">
+        <v>-8.4983897539387301E-2</v>
+      </c>
+      <c r="G122" s="3">
+        <v>-3.07017543859649E-2</v>
+      </c>
+      <c r="H122" s="4">
+        <v>3.5530932595000002</v>
+      </c>
+      <c r="I122" s="4">
+        <v>1.9986149583999999</v>
+      </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
@@ -5693,10 +5543,21 @@
       <c r="C123" t="s">
         <v>135</v>
       </c>
-      <c r="F123" s="3"/>
-      <c r="G123" s="3"/>
-      <c r="H123" s="4"/>
-      <c r="I123" s="4"/>
+      <c r="D123" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F123" s="3">
+        <v>0.14852056347974399</v>
+      </c>
+      <c r="G123" s="3">
+        <v>-1.7447068403908701E-2</v>
+      </c>
+      <c r="H123" s="4">
+        <v>4.0217155266000004</v>
+      </c>
+      <c r="I123" s="4">
+        <v>2.2622149836999998</v>
+      </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
@@ -5709,10 +5570,21 @@
       <c r="C124" t="s">
         <v>136</v>
       </c>
-      <c r="F124" s="3"/>
-      <c r="G124" s="3"/>
-      <c r="H124" s="4"/>
-      <c r="I124" s="4"/>
+      <c r="D124" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F124" s="3">
+        <v>0.29408253365308401</v>
+      </c>
+      <c r="G124" s="3">
+        <v>-4.9674266324370797E-3</v>
+      </c>
+      <c r="H124" s="4">
+        <v>4.1346362981000002</v>
+      </c>
+      <c r="I124" s="4">
+        <v>2.3257329176999999</v>
+      </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
@@ -5725,10 +5597,21 @@
       <c r="C125" t="s">
         <v>137</v>
       </c>
-      <c r="F125" s="3"/>
-      <c r="G125" s="3"/>
-      <c r="H125" s="4"/>
-      <c r="I125" s="4"/>
+      <c r="D125" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F125" s="3">
+        <v>5.22564420482622E-2</v>
+      </c>
+      <c r="G125" s="3">
+        <v>-6.7080620445724298E-3</v>
+      </c>
+      <c r="H125" s="4">
+        <v>3.6395223909999999</v>
+      </c>
+      <c r="I125" s="4">
+        <v>2.0472313449000001</v>
+      </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
@@ -5741,10 +5624,21 @@
       <c r="C126" t="s">
         <v>138</v>
       </c>
-      <c r="F126" s="3"/>
-      <c r="G126" s="3"/>
-      <c r="H126" s="4"/>
-      <c r="I126" s="4"/>
+      <c r="D126" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F126" s="3">
+        <v>0.248208419352479</v>
+      </c>
+      <c r="G126" s="3">
+        <v>-4.7536644951140003E-2</v>
+      </c>
+      <c r="H126" s="4">
+        <v>4.3257328990000001</v>
+      </c>
+      <c r="I126" s="4">
+        <v>2.4332247557</v>
+      </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
@@ -5757,10 +5651,21 @@
       <c r="C127" t="s">
         <v>139</v>
       </c>
-      <c r="F127" s="3"/>
-      <c r="G127" s="3"/>
-      <c r="H127" s="4"/>
-      <c r="I127" s="4"/>
+      <c r="D127" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F127" s="3">
+        <v>2.7429579631773698E-2</v>
+      </c>
+      <c r="G127" s="3">
+        <v>2.3141735918743899E-3</v>
+      </c>
+      <c r="H127" s="4">
+        <v>3.2650046168000002</v>
+      </c>
+      <c r="I127" s="4">
+        <v>1.836565097</v>
+      </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
@@ -5773,10 +5678,21 @@
       <c r="C128" t="s">
         <v>140</v>
       </c>
-      <c r="F128" s="3"/>
-      <c r="G128" s="3"/>
-      <c r="H128" s="4"/>
-      <c r="I128" s="4"/>
+      <c r="D128" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F128" s="3">
+        <v>-0.21792330332409901</v>
+      </c>
+      <c r="G128" s="3">
+        <v>9.8943905817174497E-3</v>
+      </c>
+      <c r="H128" s="4">
+        <v>4.2216066481999999</v>
+      </c>
+      <c r="I128" s="4">
+        <v>2.3746537395999998</v>
+      </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
@@ -5789,10 +5705,21 @@
       <c r="C129" t="s">
         <v>141</v>
       </c>
-      <c r="F129" s="3"/>
-      <c r="G129" s="3"/>
-      <c r="H129" s="4"/>
-      <c r="I129" s="4"/>
+      <c r="D129" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F129" s="3">
+        <v>-3.8261743001330402E-2</v>
+      </c>
+      <c r="G129" s="3">
+        <v>-1.7082178955923399E-2</v>
+      </c>
+      <c r="H129" s="4">
+        <v>4.3582641940000002</v>
+      </c>
+      <c r="I129" s="4">
+        <v>2.4515236091000001</v>
+      </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
@@ -5805,10 +5732,21 @@
       <c r="C130" t="s">
         <v>142</v>
       </c>
-      <c r="F130" s="3"/>
-      <c r="G130" s="3"/>
-      <c r="H130" s="4"/>
-      <c r="I130" s="4"/>
+      <c r="D130" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F130" s="3">
+        <v>0.106066758676667</v>
+      </c>
+      <c r="G130" s="3">
+        <v>-3.1555374592834001E-2</v>
+      </c>
+      <c r="H130" s="4">
+        <v>3.9956568947000002</v>
+      </c>
+      <c r="I130" s="4">
+        <v>2.2475570032999999</v>
+      </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
@@ -5821,10 +5759,21 @@
       <c r="C131" t="s">
         <v>143</v>
       </c>
-      <c r="F131" s="3"/>
-      <c r="G131" s="3"/>
-      <c r="H131" s="4"/>
-      <c r="I131" s="4"/>
+      <c r="D131" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="F131" s="3">
+        <v>1.6849853853769699E-2</v>
+      </c>
+      <c r="G131" s="3">
+        <v>4.1378116343490801E-3</v>
+      </c>
+      <c r="H131" s="4">
+        <v>3.9778393352000001</v>
+      </c>
+      <c r="I131" s="4">
+        <v>2.237534626</v>
+      </c>
     </row>
     <row r="132" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A132" s="9">
@@ -5837,12 +5786,22 @@
       <c r="C132" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D132" s="5"/>
+      <c r="D132" s="5" t="s">
+        <v>314</v>
+      </c>
       <c r="E132" s="6"/>
-      <c r="F132" s="7"/>
-      <c r="G132" s="7"/>
-      <c r="H132" s="8"/>
-      <c r="I132" s="8"/>
+      <c r="F132" s="7">
+        <v>-0.111726678969786</v>
+      </c>
+      <c r="G132" s="7">
+        <v>-1.0820635468014E-3</v>
+      </c>
+      <c r="H132" s="8">
+        <v>4.2474607853000004</v>
+      </c>
+      <c r="I132" s="8">
+        <v>2.3891966918</v>
+      </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
@@ -8490,306 +8449,306 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D133:D152 D154:D160 D162:D164 D166:D190 D200:D206 D208:D210 D212:D214 D216:D224 D226:D232 D234:D240 D242:D248 D250:D255 D257:D262 D264:D268 D270 D272:D282 D284:D294 D52:D56">
-    <cfRule type="cellIs" dxfId="117" priority="111" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="111" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="116" priority="112" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="112" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D295">
-    <cfRule type="cellIs" dxfId="115" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="43" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="44" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D43">
-    <cfRule type="cellIs" dxfId="103" priority="97" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="97" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="98" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="98" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D51">
-    <cfRule type="cellIs" dxfId="101" priority="95" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="95" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="96" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="96" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D132">
-    <cfRule type="cellIs" dxfId="85" priority="79" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="79" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="80" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D153">
-    <cfRule type="cellIs" dxfId="83" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="77" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="78" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D161">
-    <cfRule type="cellIs" dxfId="81" priority="75" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="75" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="76" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D165">
-    <cfRule type="cellIs" dxfId="79" priority="73" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="73" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="74" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D191">
-    <cfRule type="cellIs" dxfId="77" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="71" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="72" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D199">
-    <cfRule type="cellIs" dxfId="75" priority="39" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="39" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="40" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D207">
-    <cfRule type="cellIs" dxfId="73" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="69" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="70" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="70" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D211">
-    <cfRule type="cellIs" dxfId="71" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="67" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="68" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="68" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D215">
-    <cfRule type="cellIs" dxfId="69" priority="65" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="65" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="66" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D225">
-    <cfRule type="cellIs" dxfId="67" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="63" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="64" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D233">
-    <cfRule type="cellIs" dxfId="65" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="61" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="62" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D241">
-    <cfRule type="cellIs" dxfId="63" priority="59" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="59" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="60" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D249">
-    <cfRule type="cellIs" dxfId="59" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="55" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="56" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D256">
-    <cfRule type="cellIs" dxfId="57" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="53" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="54" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D263">
-    <cfRule type="cellIs" dxfId="55" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="51" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="52" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D269">
-    <cfRule type="cellIs" dxfId="53" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="49" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="50" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D271">
-    <cfRule type="cellIs" dxfId="51" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="48" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D283">
-    <cfRule type="cellIs" dxfId="49" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="45" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="46" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D192:D198">
-    <cfRule type="cellIs" dxfId="45" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="41" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="42" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D8">
-    <cfRule type="cellIs" dxfId="41" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="37" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="38" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:D13 D15:D16 D18:D19">
-    <cfRule type="cellIs" dxfId="39" priority="35" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="35" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="36" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="36" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D20">
-    <cfRule type="cellIs" dxfId="37" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="33" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="34" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="34" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14">
-    <cfRule type="cellIs" dxfId="35" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="31" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="32" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="32" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D17">
-    <cfRule type="cellIs" dxfId="33" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="29" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="30" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D21:D22">
-    <cfRule type="cellIs" dxfId="31" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="27" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="28" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D23:D34">
-    <cfRule type="cellIs" dxfId="29" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="25" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="26" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D35:D38">
-    <cfRule type="cellIs" dxfId="25" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="23" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="24" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D39">
-    <cfRule type="cellIs" dxfId="23" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D42">
-    <cfRule type="cellIs" dxfId="21" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D57:D63">
-    <cfRule type="cellIs" dxfId="19" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="17" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="18" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D64:D66">
-    <cfRule type="cellIs" dxfId="17" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="16" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D67">
-    <cfRule type="cellIs" dxfId="15" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="13" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="14" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:D74 D76:D78">
-    <cfRule type="cellIs" dxfId="13" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="12" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D75">
-    <cfRule type="cellIs" dxfId="11" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8826,10 +8785,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D41 D43:D56 D68 D114:D295">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D41 D43:D56 D68 D114:D295" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D39 D42 D57:D67 D69:D113">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D39 D42 D57:D67 D69:D113" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Pass,Fail"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: Add parameter serialization infrastructure and update fractal registry to 294 fractals
- Add FractalParameterSerializer: JSON serialization/deserialization for parameter persistence
- Add FractalParameterValidator: Validation logic for parameter constraints
- Add NativeFractalParameterBridge: Bridge between managed and native parameter systems
- Update FractalRegistry.csv with complete 294 fractal catalog
- Update FractalRegistry.xlsx spreadsheet with latest validation status

Services enhancements support full parameter system architecture.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48CB3BC7-BB09-46D0-AD74-71850A81A33C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C0783A8-78EA-4725-841B-E0C493E6D011}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="349">
   <si>
     <t>Group Name</t>
   </si>
@@ -1033,34 +1033,40 @@
     <t>Rational z³/(z³+c)</t>
   </si>
   <si>
-    <t>Vertical bands?</t>
-  </si>
-  <si>
-    <t>looks almost exactly like Bird Of Prey</t>
-  </si>
-  <si>
-    <t>twin Mandelbrots</t>
-  </si>
-  <si>
-    <t>looks like a plain Mandelbrot</t>
-  </si>
-  <si>
-    <t>green meteor</t>
-  </si>
-  <si>
-    <t>green earthworm</t>
-  </si>
-  <si>
-    <t>yet another Mandelbrot</t>
-  </si>
-  <si>
-    <t>egg with holes</t>
-  </si>
-  <si>
-    <t>fields of squares</t>
-  </si>
-  <si>
     <t>Celtic Buffalo</t>
+  </si>
+  <si>
+    <t>another boring black hole, where's the lambda in the formula?</t>
+  </si>
+  <si>
+    <t>boring black square</t>
+  </si>
+  <si>
+    <t>boring black pentagon -  looks identical to Julia Power 5</t>
+  </si>
+  <si>
+    <t>boring black pentagon -  needs fine detail for visual interest</t>
+  </si>
+  <si>
+    <t>looks identical or close to previous Siegal Disk, can you introduce much more difference in appearance or find structure</t>
+  </si>
+  <si>
+    <t>can you introduce more fine feathering or details</t>
+  </si>
+  <si>
+    <t>Vertical bands?  Check formulation</t>
+  </si>
+  <si>
+    <t>looks almost exactly like Bird Of Prey.  Check formula or introduce more vairation</t>
+  </si>
+  <si>
+    <t>looks like a plain Mandelbrot;  what is supposed to be unique about this fractal?  Perhaps introduce more fine structure or variation</t>
+  </si>
+  <si>
+    <t>yet another Mandelbrot; so what's unique about this?  Or introduce more fine structure or variation</t>
+  </si>
+  <si>
+    <t>boring black hole; check formula</t>
   </si>
 </sst>
 </file>
@@ -1588,7 +1594,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1651,6 +1657,9 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2599,14 +2608,15 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.3984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.1328125" customWidth="1"/>
+    <col min="2" max="2" width="10.53125" customWidth="1"/>
     <col min="3" max="3" width="22.1328125" customWidth="1"/>
     <col min="4" max="4" width="6.46484375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="5.19921875" customWidth="1"/>
+    <col min="5" max="5" width="23.265625" customWidth="1"/>
     <col min="6" max="6" width="6.3984375" customWidth="1"/>
     <col min="7" max="7" width="6.46484375" customWidth="1"/>
     <col min="8" max="8" width="16.1328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.265625" customWidth="1"/>
+    <col min="10" max="10" width="2.3984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
@@ -2931,7 +2941,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2946,7 +2956,7 @@
         <v>313</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -2973,7 +2983,7 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2988,7 +2998,7 @@
         <v>313</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -3289,7 +3299,7 @@
         <v>313</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
@@ -3406,9 +3416,7 @@
       <c r="D39" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="E39" s="13" t="s">
-        <v>339</v>
-      </c>
+      <c r="E39" s="13"/>
       <c r="F39" s="16">
         <v>1</v>
       </c>
@@ -3936,7 +3944,7 @@
         <v>313</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="F62" s="14"/>
       <c r="G62" s="14"/>
@@ -4224,7 +4232,7 @@
         <v>21.025059204000002</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -4238,9 +4246,7 @@
       <c r="D74" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="E74" s="11" t="s">
-        <v>341</v>
-      </c>
+      <c r="E74" s="11"/>
       <c r="F74" s="14">
         <v>0.875</v>
       </c>
@@ -4254,7 +4260,7 @@
         <v>0.2109375</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="57" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -4268,9 +4274,7 @@
       <c r="D75" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="E75" s="11" t="s">
-        <v>342</v>
-      </c>
+      <c r="E75" s="11"/>
       <c r="F75" s="14">
         <v>0.24</v>
       </c>
@@ -4479,7 +4483,7 @@
         <v>313</v>
       </c>
       <c r="E83" s="11" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="F83" s="14"/>
       <c r="G83" s="14"/>
@@ -4882,7 +4886,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -4896,9 +4900,7 @@
       <c r="D99" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="E99" s="11" t="s">
-        <v>344</v>
-      </c>
+      <c r="E99" s="11"/>
       <c r="F99" s="14">
         <v>-0.75</v>
       </c>
@@ -4954,9 +4956,7 @@
       <c r="D101" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="E101" s="11" t="s">
-        <v>345</v>
-      </c>
+      <c r="E101" s="11"/>
       <c r="F101" s="14">
         <v>0</v>
       </c>
@@ -5823,6 +5823,9 @@
       <c r="C133" t="s">
         <v>146</v>
       </c>
+      <c r="D133" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F133" s="3"/>
       <c r="G133" s="3"/>
       <c r="H133" s="4"/>
@@ -5839,10 +5842,21 @@
       <c r="C134" t="s">
         <v>147</v>
       </c>
-      <c r="F134" s="3"/>
-      <c r="G134" s="3"/>
-      <c r="H134" s="4"/>
-      <c r="I134" s="4"/>
+      <c r="D134" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F134" s="3">
+        <v>0</v>
+      </c>
+      <c r="G134" s="3">
+        <v>0</v>
+      </c>
+      <c r="H134" s="4">
+        <v>4</v>
+      </c>
+      <c r="I134" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
@@ -5855,10 +5869,21 @@
       <c r="C135" t="s">
         <v>148</v>
       </c>
-      <c r="F135" s="3"/>
-      <c r="G135" s="3"/>
-      <c r="H135" s="4"/>
-      <c r="I135" s="4"/>
+      <c r="D135" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F135" s="3">
+        <v>3.1250000000000002E-3</v>
+      </c>
+      <c r="G135" s="3">
+        <v>0.15937499999999899</v>
+      </c>
+      <c r="H135" s="4">
+        <v>4</v>
+      </c>
+      <c r="I135" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
@@ -5871,6 +5896,9 @@
       <c r="C136" t="s">
         <v>149</v>
       </c>
+      <c r="D136" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F136" s="3"/>
       <c r="G136" s="3"/>
       <c r="H136" s="4"/>
@@ -5887,10 +5915,21 @@
       <c r="C137" t="s">
         <v>150</v>
       </c>
-      <c r="F137" s="3"/>
-      <c r="G137" s="3"/>
-      <c r="H137" s="4"/>
-      <c r="I137" s="4"/>
+      <c r="D137" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F137" s="3">
+        <v>0</v>
+      </c>
+      <c r="G137" s="3">
+        <v>0</v>
+      </c>
+      <c r="H137" s="4">
+        <v>4.4535706104999999</v>
+      </c>
+      <c r="I137" s="4">
+        <v>2.5051334684</v>
+      </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A138" s="2">
@@ -5903,10 +5942,21 @@
       <c r="C138" t="s">
         <v>151</v>
       </c>
-      <c r="F138" s="3"/>
-      <c r="G138" s="3"/>
-      <c r="H138" s="4"/>
-      <c r="I138" s="4"/>
+      <c r="D138" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F138" s="3">
+        <v>0</v>
+      </c>
+      <c r="G138" s="3">
+        <v>0</v>
+      </c>
+      <c r="H138" s="4">
+        <v>3.9585237323000002</v>
+      </c>
+      <c r="I138" s="4">
+        <v>2.2266695994000001</v>
+      </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A139" s="2">
@@ -5919,6 +5969,9 @@
       <c r="C139" t="s">
         <v>152</v>
       </c>
+      <c r="D139" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F139" s="3"/>
       <c r="G139" s="3"/>
       <c r="H139" s="4"/>
@@ -5935,10 +5988,21 @@
       <c r="C140" t="s">
         <v>153</v>
       </c>
-      <c r="F140" s="3"/>
-      <c r="G140" s="3"/>
-      <c r="H140" s="4"/>
-      <c r="I140" s="4"/>
+      <c r="D140" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F140" s="3">
+        <v>0.215215215215218</v>
+      </c>
+      <c r="G140" s="3">
+        <v>3.5035035035033198E-2</v>
+      </c>
+      <c r="H140" s="4">
+        <v>38.438438437999999</v>
+      </c>
+      <c r="I140" s="4">
+        <v>21.621621621999999</v>
+      </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A141" s="2">
@@ -5951,10 +6015,24 @@
       <c r="C141" t="s">
         <v>154</v>
       </c>
-      <c r="F141" s="3"/>
-      <c r="G141" s="3"/>
-      <c r="H141" s="4"/>
-      <c r="I141" s="4"/>
+      <c r="D141" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E141" t="s">
+        <v>348</v>
+      </c>
+      <c r="F141" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G141" s="3">
+        <v>0</v>
+      </c>
+      <c r="H141" s="4">
+        <v>6</v>
+      </c>
+      <c r="I141" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A142" s="2">
@@ -5967,10 +6045,24 @@
       <c r="C142" t="s">
         <v>155</v>
       </c>
-      <c r="F142" s="3"/>
-      <c r="G142" s="3"/>
-      <c r="H142" s="4"/>
-      <c r="I142" s="4"/>
+      <c r="D142" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E142" t="s">
+        <v>338</v>
+      </c>
+      <c r="F142" s="3">
+        <v>0.445312499999999</v>
+      </c>
+      <c r="G142" s="3">
+        <v>-3.7499999999999901E-2</v>
+      </c>
+      <c r="H142" s="4">
+        <v>6</v>
+      </c>
+      <c r="I142" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A143" s="2">
@@ -5983,10 +6075,21 @@
       <c r="C143" t="s">
         <v>156</v>
       </c>
-      <c r="F143" s="3"/>
-      <c r="G143" s="3"/>
-      <c r="H143" s="4"/>
-      <c r="I143" s="4"/>
+      <c r="D143" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F143" s="3">
+        <v>-0.54414062500000004</v>
+      </c>
+      <c r="G143" s="3">
+        <v>-2.22656249999999E-2</v>
+      </c>
+      <c r="H143" s="4">
+        <v>16</v>
+      </c>
+      <c r="I143" s="4">
+        <v>9</v>
+      </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A144" s="2">
@@ -5999,10 +6102,21 @@
       <c r="C144" t="s">
         <v>157</v>
       </c>
-      <c r="F144" s="3"/>
-      <c r="G144" s="3"/>
-      <c r="H144" s="4"/>
-      <c r="I144" s="4"/>
+      <c r="D144" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F144" s="3">
+        <v>0</v>
+      </c>
+      <c r="G144" s="3">
+        <v>0</v>
+      </c>
+      <c r="H144" s="4">
+        <v>4.2870938500999998</v>
+      </c>
+      <c r="I144" s="4">
+        <v>2.4114902907000002</v>
+      </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A145" s="2">
@@ -6015,10 +6129,24 @@
       <c r="C145" t="s">
         <v>158</v>
       </c>
-      <c r="F145" s="3"/>
-      <c r="G145" s="3"/>
-      <c r="H145" s="4"/>
-      <c r="I145" s="4"/>
+      <c r="D145" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E145" t="s">
+        <v>339</v>
+      </c>
+      <c r="F145" s="3">
+        <v>0</v>
+      </c>
+      <c r="G145" s="3">
+        <v>0</v>
+      </c>
+      <c r="H145" s="4">
+        <v>4</v>
+      </c>
+      <c r="I145" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A146" s="2">
@@ -6031,10 +6159,21 @@
       <c r="C146" t="s">
         <v>159</v>
       </c>
-      <c r="F146" s="3"/>
-      <c r="G146" s="3"/>
-      <c r="H146" s="4"/>
-      <c r="I146" s="4"/>
+      <c r="D146" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F146" s="3">
+        <v>0.110111467804609</v>
+      </c>
+      <c r="G146" s="3">
+        <v>3.6509165415414803E-2</v>
+      </c>
+      <c r="H146" s="26">
+        <v>5.9223668112999999</v>
+      </c>
+      <c r="I146" s="26">
+        <v>3.3313313312999999</v>
+      </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A147" s="2">
@@ -6047,10 +6186,24 @@
       <c r="C147" t="s">
         <v>160</v>
       </c>
-      <c r="F147" s="3"/>
-      <c r="G147" s="3"/>
-      <c r="H147" s="4"/>
-      <c r="I147" s="4"/>
+      <c r="D147" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E147" t="s">
+        <v>341</v>
+      </c>
+      <c r="F147" s="3">
+        <v>0</v>
+      </c>
+      <c r="G147" s="3">
+        <v>0</v>
+      </c>
+      <c r="H147" s="4">
+        <v>4</v>
+      </c>
+      <c r="I147" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A148" s="2">
@@ -6063,10 +6216,24 @@
       <c r="C148" t="s">
         <v>161</v>
       </c>
-      <c r="F148" s="3"/>
-      <c r="G148" s="3"/>
-      <c r="H148" s="4"/>
-      <c r="I148" s="4"/>
+      <c r="D148" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E148" t="s">
+        <v>340</v>
+      </c>
+      <c r="F148" s="3">
+        <v>0</v>
+      </c>
+      <c r="G148" s="3">
+        <v>0</v>
+      </c>
+      <c r="H148" s="4">
+        <v>5.9223668112999999</v>
+      </c>
+      <c r="I148" s="4">
+        <v>3.3313313309999999</v>
+      </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A149" s="2">
@@ -6079,10 +6246,21 @@
       <c r="C149" t="s">
         <v>162</v>
       </c>
-      <c r="F149" s="3"/>
-      <c r="G149" s="3"/>
-      <c r="H149" s="4"/>
-      <c r="I149" s="4"/>
+      <c r="D149" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F149" s="3">
+        <v>0</v>
+      </c>
+      <c r="G149" s="3">
+        <v>0</v>
+      </c>
+      <c r="H149" s="4">
+        <v>3</v>
+      </c>
+      <c r="I149" s="4">
+        <v>1.6875</v>
+      </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A150" s="2">
@@ -6095,10 +6273,21 @@
       <c r="C150" t="s">
         <v>163</v>
       </c>
-      <c r="F150" s="3"/>
-      <c r="G150" s="3"/>
-      <c r="H150" s="4"/>
-      <c r="I150" s="4"/>
+      <c r="D150" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F150" s="3">
+        <v>0</v>
+      </c>
+      <c r="G150" s="3">
+        <v>0</v>
+      </c>
+      <c r="H150" s="4">
+        <v>3.6934332400000001</v>
+      </c>
+      <c r="I150" s="4">
+        <v>2.0775561974999999</v>
+      </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A151" s="2">
@@ -6111,10 +6300,24 @@
       <c r="C151" t="s">
         <v>164</v>
       </c>
-      <c r="F151" s="3"/>
-      <c r="G151" s="3"/>
-      <c r="H151" s="4"/>
-      <c r="I151" s="4"/>
+      <c r="D151" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E151" t="s">
+        <v>342</v>
+      </c>
+      <c r="F151" s="3">
+        <v>0</v>
+      </c>
+      <c r="G151" s="3">
+        <v>0</v>
+      </c>
+      <c r="H151" s="4">
+        <v>3.6934332400000001</v>
+      </c>
+      <c r="I151" s="4">
+        <v>2.0775561974999999</v>
+      </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A152" s="2">
@@ -6127,30 +6330,54 @@
       <c r="C152" t="s">
         <v>165</v>
       </c>
-      <c r="F152" s="3"/>
-      <c r="G152" s="3"/>
-      <c r="H152" s="4"/>
-      <c r="I152" s="4"/>
+      <c r="D152" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E152" t="s">
+        <v>343</v>
+      </c>
+      <c r="F152" s="3">
+        <v>0</v>
+      </c>
+      <c r="G152" s="3">
+        <v>0</v>
+      </c>
+      <c r="H152" s="4">
+        <v>22.392791797000001</v>
+      </c>
+      <c r="I152" s="4">
+        <v>12.595945386</v>
+      </c>
     </row>
     <row r="153" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A153" s="9">
         <f t="shared" si="2"/>
         <v>152</v>
       </c>
-      <c r="B153" s="6" t="s">
+      <c r="B153" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="C153" s="6" t="s">
+      <c r="C153" s="27" t="s">
         <v>166</v>
       </c>
-      <c r="D153" s="5"/>
-      <c r="E153" s="6"/>
-      <c r="F153" s="7"/>
-      <c r="G153" s="7"/>
-      <c r="H153" s="8"/>
-      <c r="I153" s="8"/>
-    </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="D153" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="E153" s="27"/>
+      <c r="F153" s="28">
+        <v>0</v>
+      </c>
+      <c r="G153" s="28">
+        <v>0</v>
+      </c>
+      <c r="H153" s="21">
+        <v>3.2153203875999998</v>
+      </c>
+      <c r="I153" s="21">
+        <v>1.808617718</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A154" s="2">
         <f t="shared" si="2"/>
         <v>153</v>
@@ -6371,7 +6598,7 @@
         <v>181</v>
       </c>
       <c r="C167" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="F167" s="3"/>
       <c r="G167" s="3"/>
@@ -8457,7 +8684,7 @@
       <c r="I295" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D133:D152 D154:D160 D162:D164 D166:D191 D201:D207 D209:D211 D213:D215 D217:D225 D227:D233 D235:D241 D243:D249 D251:D255 D257:D262 D264:D268 D270 D272:D282 D284:D294 D52:D56">
+  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D154:D160 D162:D164 D166:D191 D201:D207 D209:D211 D213:D215 D217:D225 D227:D233 D235:D241 D243:D249 D251:D255 D257:D262 D264:D268 D270 D272:D282 D284:D294 D52:D56 D133:D152">
     <cfRule type="cellIs" dxfId="83" priority="111" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8802,5 +9029,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Visual quality improvements: enhanced 12 note-flagged fractals
- Julia Lambda variants: converted to pure Julia sets with fixed lambda constants (3.8+0.1i, 2.8+0.9i)
- High-power Julia sets (4/5/6): now show intricate boundary detail with hardcoded constants
- Vertical Burning Ship: differentiated from Bird of Prey with 1.5x real component scaling
- Siegel Disk (Alt): uses distinct quasi-periodic constant (-0.624+0.418i)
- Wavy: enhanced with stronger perturbations (0.5) and cosine side-terms for texture
- Pickover Biomorphs: added sinh/cosh biological tendrils and smooth coloring
- Julia Sine: improved with proper Julia mode, smooth coloring, and fine-detail zoom
- Bifurcation diagrams: added 3x sub-pixel anti-aliasing to reduce banding artifacts

All changes focus on visual interest, beauty, and zoom opportunities.
Build verified successful.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,13 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C0783A8-78EA-4725-841B-E0C493E6D011}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D040530-6C3C-4F8B-AF18-8A9F73E8353D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FractalRegistry" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$I$295</definedName>
+    <definedName name="Data">FractalRegistry!$A$1:$I$295</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
@@ -1039,15 +1043,9 @@
     <t>another boring black hole, where's the lambda in the formula?</t>
   </si>
   <si>
-    <t>boring black square</t>
-  </si>
-  <si>
     <t>boring black pentagon -  looks identical to Julia Power 5</t>
   </si>
   <si>
-    <t>boring black pentagon -  needs fine detail for visual interest</t>
-  </si>
-  <si>
     <t>looks identical or close to previous Siegal Disk, can you introduce much more difference in appearance or find structure</t>
   </si>
   <si>
@@ -1066,7 +1064,13 @@
     <t>yet another Mandelbrot; so what's unique about this?  Or introduce more fine structure or variation</t>
   </si>
   <si>
-    <t>boring black hole; check formula</t>
+    <t>black screen no structure at any zoom</t>
+  </si>
+  <si>
+    <t>boring black square; still boring</t>
+  </si>
+  <si>
+    <t>boring black pentagon - still boring</t>
   </si>
 </sst>
 </file>
@@ -1212,7 +1216,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1401,6 +1405,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1594,7 +1604,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1660,6 +1670,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2604,14 +2617,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I295"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.3984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="10.53125" customWidth="1"/>
+    <col min="2" max="2" width="20.3984375" customWidth="1"/>
     <col min="3" max="3" width="22.1328125" customWidth="1"/>
     <col min="4" max="4" width="6.46484375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="23.265625" customWidth="1"/>
+    <col min="5" max="5" width="40.53125" customWidth="1"/>
     <col min="6" max="6" width="6.3984375" customWidth="1"/>
     <col min="7" max="7" width="6.46484375" customWidth="1"/>
     <col min="8" max="8" width="16.1328125" bestFit="1" customWidth="1"/>
@@ -2648,7 +2662,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2666,7 +2680,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <f>A2+1</f>
         <v>2</v>
@@ -2685,7 +2699,7 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
@@ -2704,7 +2718,7 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2723,7 +2737,7 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2742,7 +2756,7 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2761,7 +2775,7 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2781,7 +2795,7 @@
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2801,7 +2815,7 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2821,7 +2835,7 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2841,7 +2855,7 @@
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2861,7 +2875,7 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2881,7 +2895,7 @@
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="9">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2901,7 +2915,7 @@
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2921,7 +2935,7 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2941,7 +2955,7 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2956,14 +2970,14 @@
         <v>313</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2983,7 +2997,7 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2998,14 +3012,14 @@
         <v>313</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
     </row>
-    <row r="20" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="9">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3025,7 +3039,7 @@
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3044,7 +3058,7 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="9">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3064,7 +3078,7 @@
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3084,7 +3098,7 @@
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3104,7 +3118,7 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3124,7 +3138,7 @@
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3144,7 +3158,7 @@
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3164,7 +3178,7 @@
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3184,7 +3198,7 @@
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3204,7 +3218,7 @@
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3224,7 +3238,7 @@
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3244,7 +3258,7 @@
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3264,7 +3278,7 @@
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3284,7 +3298,7 @@
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
     </row>
-    <row r="34" spans="1:9" ht="19.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A34" s="9">
         <f t="shared" si="0"/>
         <v>33</v>
@@ -3299,14 +3313,14 @@
         <v>313</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F34" s="7"/>
       <c r="G34" s="7"/>
       <c r="H34" s="8"/>
       <c r="I34" s="8"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3334,7 +3348,7 @@
         <v>0.81325301205</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3362,7 +3376,7 @@
         <v>86.837976550999997</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3382,7 +3396,7 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
     </row>
-    <row r="38" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="38" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A38" s="9">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3402,7 +3416,7 @@
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
     </row>
-    <row r="39" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:9" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3430,7 +3444,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -3449,7 +3463,7 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A41" s="22">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -3476,7 +3490,7 @@
         <v>5.5981979492000002</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -3504,7 +3518,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="43" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A43" s="9">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -3524,7 +3538,7 @@
       <c r="H43" s="8"/>
       <c r="I43" s="8"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -3543,7 +3557,7 @@
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -3562,7 +3576,7 @@
       <c r="H45" s="23"/>
       <c r="I45" s="23"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -3581,7 +3595,7 @@
       <c r="H46" s="23"/>
       <c r="I46" s="23"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A47" s="22">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -3608,7 +3622,7 @@
         <v>21.35734072</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -3627,7 +3641,7 @@
       <c r="H48" s="23"/>
       <c r="I48" s="23"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -3646,7 +3660,7 @@
       <c r="H49" s="23"/>
       <c r="I49" s="23"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -3665,7 +3679,7 @@
       <c r="H50" s="23"/>
       <c r="I50" s="23"/>
     </row>
-    <row r="51" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A51" s="9">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -3685,7 +3699,7 @@
       <c r="H51" s="24"/>
       <c r="I51" s="24"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -3704,7 +3718,7 @@
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -3723,7 +3737,7 @@
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -3742,7 +3756,7 @@
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
     </row>
-    <row r="55" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="55" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A55" s="9">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -3762,7 +3776,7 @@
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A56" s="22">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -3789,7 +3803,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -3817,7 +3831,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3845,7 +3859,7 @@
         <v>2.3420689813000002</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -3873,7 +3887,7 @@
         <v>1.8436548223</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -3901,7 +3915,7 @@
         <v>2.3309644980000002</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -3929,7 +3943,7 @@
         <v>1.4659263959</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -3944,14 +3958,14 @@
         <v>313</v>
       </c>
       <c r="E62" s="11" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="F62" s="14"/>
       <c r="G62" s="14"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
     </row>
-    <row r="63" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="63" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A63" s="9">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -3979,7 +3993,7 @@
         <v>0.28801632742</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -4007,7 +4021,7 @@
         <v>1.4659263959</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -4025,7 +4039,7 @@
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
     </row>
-    <row r="66" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="66" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A66" s="9">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -4053,7 +4067,7 @@
         <v>2.397631133</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <f t="shared" si="0"/>
         <v>66</v>
@@ -4081,7 +4095,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A68" s="22">
         <f t="shared" ref="A68:A131" si="1">A67+1</f>
         <v>67</v>
@@ -4108,7 +4122,7 @@
         <v>8.4375</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -4128,7 +4142,7 @@
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A70" s="2">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -4156,7 +4170,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A71" s="2">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -4176,7 +4190,7 @@
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A72" s="2">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -4204,7 +4218,7 @@
         <v>6.75</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -4232,7 +4246,7 @@
         <v>21.025059204000002</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -4260,7 +4274,7 @@
         <v>0.2109375</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -4288,7 +4302,7 @@
         <v>1.0884495317</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A76" s="2">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -4316,7 +4330,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A77" s="2">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -4344,7 +4358,7 @@
         <v>1.4678492578</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="78" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A78" s="9">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -4372,7 +4386,7 @@
         <v>0.84375</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -4392,7 +4406,7 @@
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -4412,7 +4426,7 @@
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -4440,7 +4454,7 @@
         <v>3.8068369917</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A82" s="2">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -4468,7 +4482,7 @@
         <v>248.99892890999999</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A83" s="2">
         <f t="shared" si="1"/>
         <v>82</v>
@@ -4483,14 +4497,14 @@
         <v>313</v>
       </c>
       <c r="E83" s="11" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="F83" s="14"/>
       <c r="G83" s="14"/>
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
         <f t="shared" si="1"/>
         <v>83</v>
@@ -4518,7 +4532,7 @@
         <v>2.2090805910000002</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
         <f t="shared" si="1"/>
         <v>84</v>
@@ -4538,7 +4552,7 @@
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
     </row>
-    <row r="86" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="86" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A86" s="9">
         <f t="shared" si="1"/>
         <v>85</v>
@@ -4558,7 +4572,7 @@
       <c r="H86" s="21"/>
       <c r="I86" s="21"/>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <f t="shared" si="1"/>
         <v>86</v>
@@ -4586,7 +4600,7 @@
         <v>3.7408990110000002</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A88" s="2">
         <f t="shared" si="1"/>
         <v>87</v>
@@ -4614,7 +4628,7 @@
         <v>2.1342925659</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A89" s="2">
         <f t="shared" si="1"/>
         <v>88</v>
@@ -4642,7 +4656,7 @@
         <v>2.4107142857000001</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A90" s="2">
         <f t="shared" si="1"/>
         <v>89</v>
@@ -4670,7 +4684,7 @@
         <v>2.3556012803000002</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
         <f t="shared" si="1"/>
         <v>90</v>
@@ -4698,7 +4712,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
         <f t="shared" si="1"/>
         <v>91</v>
@@ -4726,7 +4740,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
         <f t="shared" si="1"/>
         <v>92</v>
@@ -4754,7 +4768,7 @@
         <v>3.2040082611999998</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
         <f t="shared" si="1"/>
         <v>93</v>
@@ -4782,7 +4796,7 @@
         <v>11.181911864</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
         <f t="shared" si="1"/>
         <v>94</v>
@@ -4810,7 +4824,7 @@
         <v>2.542651593</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
         <f t="shared" si="1"/>
         <v>95</v>
@@ -4838,7 +4852,7 @@
         <v>4.6783144913000001</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <f t="shared" si="1"/>
         <v>96</v>
@@ -4858,7 +4872,7 @@
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <f t="shared" si="1"/>
         <v>97</v>
@@ -4886,7 +4900,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -4914,7 +4928,7 @@
         <v>6.1130526660999998</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A100" s="2">
         <f t="shared" si="1"/>
         <v>99</v>
@@ -4942,7 +4956,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="20.65" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:9" ht="20.65" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -4970,7 +4984,7 @@
         <v>4.21875</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -4998,7 +5012,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
         <f t="shared" si="1"/>
         <v>102</v>
@@ -5026,7 +5040,7 @@
         <v>1.0194922309000001</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="104" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A104" s="9">
         <f t="shared" si="1"/>
         <v>103</v>
@@ -5054,7 +5068,7 @@
         <v>2.3396227092999999</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
         <f t="shared" si="1"/>
         <v>104</v>
@@ -5082,7 +5096,7 @@
         <v>11.028960818</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
         <f t="shared" si="1"/>
         <v>105</v>
@@ -5110,7 +5124,7 @@
         <v>1.1422222222</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
         <f t="shared" si="1"/>
         <v>106</v>
@@ -5138,7 +5152,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
         <f t="shared" si="1"/>
         <v>107</v>
@@ -5166,7 +5180,7 @@
         <v>1.125</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="109" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A109" s="9">
         <f t="shared" si="1"/>
         <v>108</v>
@@ -5194,7 +5208,7 @@
         <v>0.82935879629999998</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
         <f t="shared" si="1"/>
         <v>109</v>
@@ -5222,7 +5236,7 @@
         <v>2.4900562852000001</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -5250,7 +5264,7 @@
         <v>2.2581613508</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -5278,7 +5292,7 @@
         <v>2.956097561</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A113" s="2">
         <f t="shared" si="1"/>
         <v>112</v>
@@ -5306,7 +5320,7 @@
         <v>2.4279250753000001</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A114" s="2">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -5325,7 +5339,7 @@
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A115" s="2">
         <f t="shared" si="1"/>
         <v>114</v>
@@ -5352,7 +5366,7 @@
         <v>2.4135156878999999</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A116" s="2">
         <f t="shared" si="1"/>
         <v>115</v>
@@ -5379,7 +5393,7 @@
         <v>2.2134956765</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A117" s="2">
         <f t="shared" si="1"/>
         <v>116</v>
@@ -5406,7 +5420,7 @@
         <v>2.5144496681000001</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A118" s="2">
         <f t="shared" si="1"/>
         <v>117</v>
@@ -5433,7 +5447,7 @@
         <v>2.4081908582999998</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A119" s="2">
         <f t="shared" si="1"/>
         <v>118</v>
@@ -5460,7 +5474,7 @@
         <v>1.9245172044000001</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
         <f t="shared" si="1"/>
         <v>119</v>
@@ -5487,7 +5501,7 @@
         <v>2.2422422422000001</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
         <f t="shared" si="1"/>
         <v>120</v>
@@ -5514,7 +5528,7 @@
         <v>2.4078947367999999</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
         <f t="shared" si="1"/>
         <v>121</v>
@@ -5541,7 +5555,7 @@
         <v>1.9986149583999999</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
         <f t="shared" si="1"/>
         <v>122</v>
@@ -5568,7 +5582,7 @@
         <v>2.2622149836999998</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
         <f t="shared" si="1"/>
         <v>123</v>
@@ -5595,7 +5609,7 @@
         <v>2.3257329176999999</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
         <f t="shared" si="1"/>
         <v>124</v>
@@ -5622,7 +5636,7 @@
         <v>2.0472313449000001</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
         <f t="shared" si="1"/>
         <v>125</v>
@@ -5649,7 +5663,7 @@
         <v>2.4332247557</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
         <f t="shared" si="1"/>
         <v>126</v>
@@ -5676,7 +5690,7 @@
         <v>1.836565097</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -5703,7 +5717,7 @@
         <v>2.3746537395999998</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <f t="shared" si="1"/>
         <v>128</v>
@@ -5730,7 +5744,7 @@
         <v>2.4515236091000001</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <f t="shared" si="1"/>
         <v>129</v>
@@ -5757,7 +5771,7 @@
         <v>2.2475570032999999</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <f t="shared" si="1"/>
         <v>130</v>
@@ -5784,7 +5798,7 @@
         <v>2.237534626</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="132" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A132" s="9">
         <f t="shared" ref="A132:A204" si="2">A131+1</f>
         <v>131</v>
@@ -5812,7 +5826,7 @@
         <v>2.3891966918</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
         <f t="shared" si="2"/>
         <v>132</v>
@@ -5831,7 +5845,7 @@
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A134" s="2">
         <f t="shared" si="2"/>
         <v>133</v>
@@ -5858,7 +5872,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
         <f t="shared" si="2"/>
         <v>134</v>
@@ -5885,7 +5899,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
         <f t="shared" si="2"/>
         <v>135</v>
@@ -5904,7 +5918,7 @@
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A137" s="2">
         <f t="shared" si="2"/>
         <v>136</v>
@@ -5931,7 +5945,7 @@
         <v>2.5051334684</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A138" s="2">
         <f t="shared" si="2"/>
         <v>137</v>
@@ -5958,7 +5972,7 @@
         <v>2.2266695994000001</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A139" s="2">
         <f t="shared" si="2"/>
         <v>138</v>
@@ -5977,7 +5991,7 @@
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A140" s="2">
         <f t="shared" si="2"/>
         <v>139</v>
@@ -6004,8 +6018,8 @@
         <v>21.621621621999999</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A141" s="2">
+    <row r="141" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A141" s="29">
         <f t="shared" si="2"/>
         <v>140</v>
       </c>
@@ -6019,7 +6033,7 @@
         <v>313</v>
       </c>
       <c r="E141" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="F141" s="3">
         <v>0.5</v>
@@ -6034,8 +6048,8 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A142" s="2">
+    <row r="142" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A142" s="29">
         <f t="shared" si="2"/>
         <v>141</v>
       </c>
@@ -6064,7 +6078,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A143" s="2">
         <f t="shared" si="2"/>
         <v>142</v>
@@ -6091,7 +6105,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A144" s="2">
         <f t="shared" si="2"/>
         <v>143</v>
@@ -6118,8 +6132,8 @@
         <v>2.4114902907000002</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A145" s="2">
+    <row r="145" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A145" s="29">
         <f t="shared" si="2"/>
         <v>144</v>
       </c>
@@ -6133,7 +6147,7 @@
         <v>313</v>
       </c>
       <c r="E145" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="F145" s="3">
         <v>0</v>
@@ -6148,7 +6162,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A146" s="2">
         <f t="shared" si="2"/>
         <v>145</v>
@@ -6175,8 +6189,8 @@
         <v>3.3313313312999999</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A147" s="2">
+    <row r="147" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A147" s="29">
         <f t="shared" si="2"/>
         <v>146</v>
       </c>
@@ -6190,7 +6204,7 @@
         <v>313</v>
       </c>
       <c r="E147" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="F147" s="3">
         <v>0</v>
@@ -6205,7 +6219,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A148" s="2">
         <f t="shared" si="2"/>
         <v>147</v>
@@ -6220,7 +6234,7 @@
         <v>313</v>
       </c>
       <c r="E148" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F148" s="3">
         <v>0</v>
@@ -6235,7 +6249,7 @@
         <v>3.3313313309999999</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A149" s="2">
         <f t="shared" si="2"/>
         <v>148</v>
@@ -6262,7 +6276,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A150" s="2">
         <f t="shared" si="2"/>
         <v>149</v>
@@ -6289,7 +6303,7 @@
         <v>2.0775561974999999</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A151" s="2">
         <f t="shared" si="2"/>
         <v>150</v>
@@ -6304,7 +6318,7 @@
         <v>313</v>
       </c>
       <c r="E151" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F151" s="3">
         <v>0</v>
@@ -6319,7 +6333,7 @@
         <v>2.0775561974999999</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A152" s="2">
         <f t="shared" si="2"/>
         <v>151</v>
@@ -6334,7 +6348,7 @@
         <v>313</v>
       </c>
       <c r="E152" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="F152" s="3">
         <v>0</v>
@@ -6349,7 +6363,7 @@
         <v>12.595945386</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="153" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A153" s="9">
         <f t="shared" si="2"/>
         <v>152</v>
@@ -6377,7 +6391,7 @@
         <v>1.808617718</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A154" s="2">
         <f t="shared" si="2"/>
         <v>153</v>
@@ -6393,7 +6407,7 @@
       <c r="H154" s="4"/>
       <c r="I154" s="4"/>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A155" s="2">
         <f t="shared" si="2"/>
         <v>154</v>
@@ -6409,7 +6423,7 @@
       <c r="H155" s="4"/>
       <c r="I155" s="4"/>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A156" s="2">
         <f t="shared" si="2"/>
         <v>155</v>
@@ -6425,7 +6439,7 @@
       <c r="H156" s="4"/>
       <c r="I156" s="4"/>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A157" s="2">
         <f t="shared" si="2"/>
         <v>156</v>
@@ -6441,7 +6455,7 @@
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A158" s="2">
         <f t="shared" si="2"/>
         <v>157</v>
@@ -6457,7 +6471,7 @@
       <c r="H158" s="4"/>
       <c r="I158" s="4"/>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A159" s="2">
         <f t="shared" si="2"/>
         <v>158</v>
@@ -6473,7 +6487,7 @@
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A160" s="2">
         <f t="shared" si="2"/>
         <v>159</v>
@@ -6489,7 +6503,7 @@
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
     </row>
-    <row r="161" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="161" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A161" s="9">
         <f t="shared" si="2"/>
         <v>160</v>
@@ -6507,7 +6521,7 @@
       <c r="H161" s="8"/>
       <c r="I161" s="8"/>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A162" s="2">
         <f t="shared" si="2"/>
         <v>161</v>
@@ -6523,7 +6537,7 @@
       <c r="H162" s="4"/>
       <c r="I162" s="4"/>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A163" s="2">
         <f t="shared" si="2"/>
         <v>162</v>
@@ -6539,7 +6553,7 @@
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A164" s="2">
         <f t="shared" si="2"/>
         <v>163</v>
@@ -6555,7 +6569,7 @@
       <c r="H164" s="4"/>
       <c r="I164" s="4"/>
     </row>
-    <row r="165" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="165" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A165" s="9">
         <f t="shared" si="2"/>
         <v>164</v>
@@ -6573,7 +6587,7 @@
       <c r="H165" s="8"/>
       <c r="I165" s="8"/>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A166" s="2">
         <f t="shared" si="2"/>
         <v>165</v>
@@ -6589,7 +6603,7 @@
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A167" s="25">
         <f t="shared" si="2"/>
         <v>166</v>
@@ -6605,7 +6619,7 @@
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A168" s="2">
         <f t="shared" si="2"/>
         <v>167</v>
@@ -6621,7 +6635,7 @@
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A169" s="2">
         <f t="shared" si="2"/>
         <v>168</v>
@@ -6637,7 +6651,7 @@
       <c r="H169" s="4"/>
       <c r="I169" s="4"/>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A170" s="2">
         <f t="shared" si="2"/>
         <v>169</v>
@@ -6653,7 +6667,7 @@
       <c r="H170" s="4"/>
       <c r="I170" s="4"/>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A171" s="2">
         <f t="shared" si="2"/>
         <v>170</v>
@@ -6669,7 +6683,7 @@
       <c r="H171" s="4"/>
       <c r="I171" s="4"/>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A172" s="2">
         <f t="shared" si="2"/>
         <v>171</v>
@@ -6685,7 +6699,7 @@
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A173" s="2">
         <f t="shared" si="2"/>
         <v>172</v>
@@ -6701,7 +6715,7 @@
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A174" s="2">
         <f t="shared" si="2"/>
         <v>173</v>
@@ -6717,7 +6731,7 @@
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A175" s="2">
         <f t="shared" si="2"/>
         <v>174</v>
@@ -6733,7 +6747,7 @@
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A176" s="2">
         <f t="shared" si="2"/>
         <v>175</v>
@@ -6749,7 +6763,7 @@
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A177" s="2">
         <f t="shared" si="2"/>
         <v>176</v>
@@ -6765,7 +6779,7 @@
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A178" s="2">
         <f t="shared" si="2"/>
         <v>177</v>
@@ -6781,7 +6795,7 @@
       <c r="H178" s="4"/>
       <c r="I178" s="4"/>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A179" s="2">
         <f t="shared" si="2"/>
         <v>178</v>
@@ -6797,7 +6811,7 @@
       <c r="H179" s="4"/>
       <c r="I179" s="4"/>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A180" s="2">
         <f t="shared" si="2"/>
         <v>179</v>
@@ -6813,7 +6827,7 @@
       <c r="H180" s="4"/>
       <c r="I180" s="4"/>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A181" s="2">
         <f t="shared" si="2"/>
         <v>180</v>
@@ -6829,7 +6843,7 @@
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A182" s="2">
         <f t="shared" si="2"/>
         <v>181</v>
@@ -6845,7 +6859,7 @@
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A183" s="2">
         <f t="shared" si="2"/>
         <v>182</v>
@@ -6861,7 +6875,7 @@
       <c r="H183" s="4"/>
       <c r="I183" s="4"/>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A184" s="2">
         <f t="shared" si="2"/>
         <v>183</v>
@@ -6877,7 +6891,7 @@
       <c r="H184" s="4"/>
       <c r="I184" s="4"/>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A185" s="2">
         <f t="shared" si="2"/>
         <v>184</v>
@@ -6893,7 +6907,7 @@
       <c r="H185" s="4"/>
       <c r="I185" s="4"/>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A186" s="2">
         <f t="shared" si="2"/>
         <v>185</v>
@@ -6909,7 +6923,7 @@
       <c r="H186" s="4"/>
       <c r="I186" s="4"/>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A187" s="2">
         <f t="shared" si="2"/>
         <v>186</v>
@@ -6925,7 +6939,7 @@
       <c r="H187" s="4"/>
       <c r="I187" s="4"/>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A188" s="2">
         <f t="shared" si="2"/>
         <v>187</v>
@@ -6941,7 +6955,7 @@
       <c r="H188" s="4"/>
       <c r="I188" s="4"/>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A189" s="2">
         <f t="shared" si="2"/>
         <v>188</v>
@@ -6957,7 +6971,7 @@
       <c r="H189" s="4"/>
       <c r="I189" s="4"/>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A190" s="2">
         <f t="shared" si="2"/>
         <v>189</v>
@@ -6973,7 +6987,7 @@
       <c r="H190" s="4"/>
       <c r="I190" s="4"/>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A191" s="2">
         <f t="shared" si="2"/>
         <v>190</v>
@@ -6989,7 +7003,7 @@
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
     </row>
-    <row r="192" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="192" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A192" s="9">
         <f t="shared" si="2"/>
         <v>191</v>
@@ -7007,7 +7021,7 @@
       <c r="H192" s="8"/>
       <c r="I192" s="8"/>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A193" s="9">
         <f t="shared" si="2"/>
         <v>192</v>
@@ -7023,7 +7037,7 @@
       <c r="H193" s="4"/>
       <c r="I193" s="4"/>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A194" s="9">
         <f t="shared" si="2"/>
         <v>193</v>
@@ -7039,7 +7053,7 @@
       <c r="H194" s="4"/>
       <c r="I194" s="4"/>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A195" s="9">
         <f t="shared" si="2"/>
         <v>194</v>
@@ -7055,7 +7069,7 @@
       <c r="H195" s="4"/>
       <c r="I195" s="4"/>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A196" s="9">
         <f t="shared" si="2"/>
         <v>195</v>
@@ -7071,7 +7085,7 @@
       <c r="H196" s="4"/>
       <c r="I196" s="4"/>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A197" s="9">
         <f t="shared" si="2"/>
         <v>196</v>
@@ -7087,7 +7101,7 @@
       <c r="H197" s="4"/>
       <c r="I197" s="4"/>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A198" s="9">
         <f t="shared" si="2"/>
         <v>197</v>
@@ -7103,7 +7117,7 @@
       <c r="H198" s="4"/>
       <c r="I198" s="4"/>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A199" s="9">
         <f t="shared" si="2"/>
         <v>198</v>
@@ -7119,7 +7133,7 @@
       <c r="H199" s="4"/>
       <c r="I199" s="4"/>
     </row>
-    <row r="200" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="200" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A200" s="9">
         <f t="shared" si="2"/>
         <v>199</v>
@@ -7137,7 +7151,7 @@
       <c r="H200" s="8"/>
       <c r="I200" s="8"/>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A201" s="9">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -7153,7 +7167,7 @@
       <c r="H201" s="4"/>
       <c r="I201" s="4"/>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A202" s="9">
         <f t="shared" si="2"/>
         <v>201</v>
@@ -7169,7 +7183,7 @@
       <c r="H202" s="4"/>
       <c r="I202" s="4"/>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A203" s="2">
         <f t="shared" si="2"/>
         <v>202</v>
@@ -7185,7 +7199,7 @@
       <c r="H203" s="4"/>
       <c r="I203" s="4"/>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A204" s="2">
         <f t="shared" si="2"/>
         <v>203</v>
@@ -7201,7 +7215,7 @@
       <c r="H204" s="4"/>
       <c r="I204" s="4"/>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A205" s="2">
         <f t="shared" ref="A205:A264" si="3">A204+1</f>
         <v>204</v>
@@ -7217,7 +7231,7 @@
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A206" s="2">
         <f t="shared" si="3"/>
         <v>205</v>
@@ -7233,7 +7247,7 @@
       <c r="H206" s="4"/>
       <c r="I206" s="4"/>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A207" s="2">
         <f t="shared" si="3"/>
         <v>206</v>
@@ -7249,7 +7263,7 @@
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
     </row>
-    <row r="208" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="208" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A208" s="9">
         <f t="shared" si="3"/>
         <v>207</v>
@@ -7267,7 +7281,7 @@
       <c r="H208" s="8"/>
       <c r="I208" s="8"/>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A209" s="2">
         <f t="shared" si="3"/>
         <v>208</v>
@@ -7283,7 +7297,7 @@
       <c r="H209" s="4"/>
       <c r="I209" s="4"/>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A210" s="2">
         <f t="shared" si="3"/>
         <v>209</v>
@@ -7299,7 +7313,7 @@
       <c r="H210" s="4"/>
       <c r="I210" s="4"/>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A211" s="2">
         <f t="shared" si="3"/>
         <v>210</v>
@@ -7315,7 +7329,7 @@
       <c r="H211" s="4"/>
       <c r="I211" s="4"/>
     </row>
-    <row r="212" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="212" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A212" s="9">
         <f t="shared" si="3"/>
         <v>211</v>
@@ -7333,7 +7347,7 @@
       <c r="H212" s="8"/>
       <c r="I212" s="8"/>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A213" s="2">
         <f t="shared" si="3"/>
         <v>212</v>
@@ -7349,7 +7363,7 @@
       <c r="H213" s="4"/>
       <c r="I213" s="4"/>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A214" s="2">
         <f t="shared" si="3"/>
         <v>213</v>
@@ -7365,7 +7379,7 @@
       <c r="H214" s="4"/>
       <c r="I214" s="4"/>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A215" s="2">
         <f t="shared" si="3"/>
         <v>214</v>
@@ -7381,7 +7395,7 @@
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
     </row>
-    <row r="216" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="216" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A216" s="9">
         <f t="shared" si="3"/>
         <v>215</v>
@@ -7399,7 +7413,7 @@
       <c r="H216" s="8"/>
       <c r="I216" s="8"/>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A217" s="2">
         <f t="shared" si="3"/>
         <v>216</v>
@@ -7415,7 +7429,7 @@
       <c r="H217" s="4"/>
       <c r="I217" s="4"/>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A218" s="2">
         <f t="shared" si="3"/>
         <v>217</v>
@@ -7431,7 +7445,7 @@
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
     </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A219" s="2">
         <f t="shared" si="3"/>
         <v>218</v>
@@ -7447,7 +7461,7 @@
       <c r="H219" s="4"/>
       <c r="I219" s="4"/>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A220" s="2">
         <f t="shared" si="3"/>
         <v>219</v>
@@ -7463,7 +7477,7 @@
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A221" s="2">
         <f t="shared" si="3"/>
         <v>220</v>
@@ -7479,7 +7493,7 @@
       <c r="H221" s="4"/>
       <c r="I221" s="4"/>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A222" s="2">
         <f t="shared" si="3"/>
         <v>221</v>
@@ -7495,7 +7509,7 @@
       <c r="H222" s="4"/>
       <c r="I222" s="4"/>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A223" s="2">
         <f t="shared" si="3"/>
         <v>222</v>
@@ -7511,7 +7525,7 @@
       <c r="H223" s="4"/>
       <c r="I223" s="4"/>
     </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A224" s="2">
         <f t="shared" si="3"/>
         <v>223</v>
@@ -7527,7 +7541,7 @@
       <c r="H224" s="4"/>
       <c r="I224" s="4"/>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A225" s="2">
         <f t="shared" si="3"/>
         <v>224</v>
@@ -7543,7 +7557,7 @@
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
     </row>
-    <row r="226" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="226" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A226" s="9">
         <f t="shared" si="3"/>
         <v>225</v>
@@ -7561,7 +7575,7 @@
       <c r="H226" s="8"/>
       <c r="I226" s="8"/>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A227" s="2">
         <f t="shared" si="3"/>
         <v>226</v>
@@ -7577,7 +7591,7 @@
       <c r="H227" s="4"/>
       <c r="I227" s="4"/>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A228" s="2">
         <f t="shared" si="3"/>
         <v>227</v>
@@ -7593,7 +7607,7 @@
       <c r="H228" s="4"/>
       <c r="I228" s="4"/>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A229" s="2">
         <f t="shared" si="3"/>
         <v>228</v>
@@ -7609,7 +7623,7 @@
       <c r="H229" s="4"/>
       <c r="I229" s="4"/>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
         <f t="shared" si="3"/>
         <v>229</v>
@@ -7625,7 +7639,7 @@
       <c r="H230" s="4"/>
       <c r="I230" s="4"/>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A231" s="2">
         <f t="shared" si="3"/>
         <v>230</v>
@@ -7641,7 +7655,7 @@
       <c r="H231" s="4"/>
       <c r="I231" s="4"/>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A232" s="2">
         <f t="shared" si="3"/>
         <v>231</v>
@@ -7657,7 +7671,7 @@
       <c r="H232" s="4"/>
       <c r="I232" s="4"/>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A233" s="2">
         <f t="shared" si="3"/>
         <v>232</v>
@@ -7673,7 +7687,7 @@
       <c r="H233" s="4"/>
       <c r="I233" s="4"/>
     </row>
-    <row r="234" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="234" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A234" s="9">
         <f t="shared" si="3"/>
         <v>233</v>
@@ -7691,7 +7705,7 @@
       <c r="H234" s="8"/>
       <c r="I234" s="8"/>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A235" s="2">
         <f t="shared" si="3"/>
         <v>234</v>
@@ -7707,7 +7721,7 @@
       <c r="H235" s="4"/>
       <c r="I235" s="4"/>
     </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A236" s="2">
         <f t="shared" si="3"/>
         <v>235</v>
@@ -7723,7 +7737,7 @@
       <c r="H236" s="4"/>
       <c r="I236" s="4"/>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A237" s="2">
         <f t="shared" si="3"/>
         <v>236</v>
@@ -7739,7 +7753,7 @@
       <c r="H237" s="4"/>
       <c r="I237" s="4"/>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A238" s="2">
         <f t="shared" si="3"/>
         <v>237</v>
@@ -7755,7 +7769,7 @@
       <c r="H238" s="4"/>
       <c r="I238" s="4"/>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A239" s="2">
         <f t="shared" si="3"/>
         <v>238</v>
@@ -7771,7 +7785,7 @@
       <c r="H239" s="4"/>
       <c r="I239" s="4"/>
     </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A240" s="2">
         <f t="shared" si="3"/>
         <v>239</v>
@@ -7787,7 +7801,7 @@
       <c r="H240" s="4"/>
       <c r="I240" s="4"/>
     </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A241" s="2">
         <f t="shared" si="3"/>
         <v>240</v>
@@ -7803,7 +7817,7 @@
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
     </row>
-    <row r="242" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="242" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A242" s="2">
         <f t="shared" si="3"/>
         <v>241</v>
@@ -7821,7 +7835,7 @@
       <c r="H242" s="8"/>
       <c r="I242" s="8"/>
     </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A243" s="2">
         <f t="shared" si="3"/>
         <v>242</v>
@@ -7837,7 +7851,7 @@
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
     </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A244" s="2">
         <f t="shared" si="3"/>
         <v>243</v>
@@ -7853,7 +7867,7 @@
       <c r="H244" s="4"/>
       <c r="I244" s="4"/>
     </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A245" s="2">
         <f t="shared" si="3"/>
         <v>244</v>
@@ -7869,7 +7883,7 @@
       <c r="H245" s="4"/>
       <c r="I245" s="4"/>
     </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A246" s="2">
         <f t="shared" si="3"/>
         <v>245</v>
@@ -7885,7 +7899,7 @@
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
     </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A247" s="2">
         <f t="shared" si="3"/>
         <v>246</v>
@@ -7901,7 +7915,7 @@
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
     </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A248" s="2">
         <f t="shared" si="3"/>
         <v>247</v>
@@ -7917,7 +7931,7 @@
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
     </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A249" s="2">
         <f t="shared" si="3"/>
         <v>248</v>
@@ -7933,7 +7947,7 @@
       <c r="H249" s="4"/>
       <c r="I249" s="4"/>
     </row>
-    <row r="250" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="250" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A250" s="2">
         <f t="shared" si="3"/>
         <v>249</v>
@@ -7951,7 +7965,7 @@
       <c r="H250" s="8"/>
       <c r="I250" s="8"/>
     </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A251" s="2">
         <f t="shared" si="3"/>
         <v>250</v>
@@ -7967,7 +7981,7 @@
       <c r="H251" s="4"/>
       <c r="I251" s="4"/>
     </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A252" s="2">
         <f t="shared" si="3"/>
         <v>251</v>
@@ -7983,7 +7997,7 @@
       <c r="H252" s="4"/>
       <c r="I252" s="4"/>
     </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A253" s="2">
         <f t="shared" si="3"/>
         <v>252</v>
@@ -7999,7 +8013,7 @@
       <c r="H253" s="4"/>
       <c r="I253" s="4"/>
     </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A254" s="2">
         <f t="shared" si="3"/>
         <v>253</v>
@@ -8015,7 +8029,7 @@
       <c r="H254" s="4"/>
       <c r="I254" s="4"/>
     </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A255" s="2">
         <f t="shared" si="3"/>
         <v>254</v>
@@ -8031,7 +8045,7 @@
       <c r="H255" s="4"/>
       <c r="I255" s="4"/>
     </row>
-    <row r="256" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="256" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A256" s="2">
         <f t="shared" si="3"/>
         <v>255</v>
@@ -8049,7 +8063,7 @@
       <c r="H256" s="8"/>
       <c r="I256" s="8"/>
     </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A257" s="2">
         <f t="shared" si="3"/>
         <v>256</v>
@@ -8065,7 +8079,7 @@
       <c r="H257" s="4"/>
       <c r="I257" s="4"/>
     </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A258" s="2">
         <f t="shared" si="3"/>
         <v>257</v>
@@ -8081,7 +8095,7 @@
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
     </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A259" s="2">
         <f t="shared" si="3"/>
         <v>258</v>
@@ -8097,7 +8111,7 @@
       <c r="H259" s="4"/>
       <c r="I259" s="4"/>
     </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A260" s="2">
         <f t="shared" si="3"/>
         <v>259</v>
@@ -8113,7 +8127,7 @@
       <c r="H260" s="4"/>
       <c r="I260" s="4"/>
     </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A261" s="2">
         <f t="shared" si="3"/>
         <v>260</v>
@@ -8129,7 +8143,7 @@
       <c r="H261" s="4"/>
       <c r="I261" s="4"/>
     </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A262" s="2">
         <f t="shared" si="3"/>
         <v>261</v>
@@ -8145,7 +8159,7 @@
       <c r="H262" s="4"/>
       <c r="I262" s="4"/>
     </row>
-    <row r="263" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="263" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A263" s="2">
         <f t="shared" si="3"/>
         <v>262</v>
@@ -8163,7 +8177,7 @@
       <c r="H263" s="8"/>
       <c r="I263" s="8"/>
     </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A264" s="2">
         <f t="shared" si="3"/>
         <v>263</v>
@@ -8179,7 +8193,7 @@
       <c r="H264" s="4"/>
       <c r="I264" s="4"/>
     </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A265" s="2">
         <f t="shared" ref="A265:A295" si="4">A264+1</f>
         <v>264</v>
@@ -8195,7 +8209,7 @@
       <c r="H265" s="4"/>
       <c r="I265" s="4"/>
     </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A266" s="2">
         <f t="shared" si="4"/>
         <v>265</v>
@@ -8211,7 +8225,7 @@
       <c r="H266" s="4"/>
       <c r="I266" s="4"/>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A267" s="2">
         <f t="shared" si="4"/>
         <v>266</v>
@@ -8227,7 +8241,7 @@
       <c r="H267" s="4"/>
       <c r="I267" s="4"/>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A268" s="2">
         <f t="shared" si="4"/>
         <v>267</v>
@@ -8243,7 +8257,7 @@
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
     </row>
-    <row r="269" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="269" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A269" s="9">
         <f t="shared" si="4"/>
         <v>268</v>
@@ -8261,7 +8275,7 @@
       <c r="H269" s="8"/>
       <c r="I269" s="8"/>
     </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A270" s="2">
         <f t="shared" si="4"/>
         <v>269</v>
@@ -8277,7 +8291,7 @@
       <c r="H270" s="4"/>
       <c r="I270" s="4"/>
     </row>
-    <row r="271" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="271" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A271" s="9">
         <f t="shared" si="4"/>
         <v>270</v>
@@ -8295,7 +8309,7 @@
       <c r="H271" s="8"/>
       <c r="I271" s="8"/>
     </row>
-    <row r="272" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A272" s="2">
         <f t="shared" si="4"/>
         <v>271</v>
@@ -8311,7 +8325,7 @@
       <c r="H272" s="4"/>
       <c r="I272" s="4"/>
     </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A273" s="2">
         <f t="shared" si="4"/>
         <v>272</v>
@@ -8327,7 +8341,7 @@
       <c r="H273" s="4"/>
       <c r="I273" s="4"/>
     </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A274" s="2">
         <f t="shared" si="4"/>
         <v>273</v>
@@ -8343,7 +8357,7 @@
       <c r="H274" s="4"/>
       <c r="I274" s="4"/>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A275" s="2">
         <f t="shared" si="4"/>
         <v>274</v>
@@ -8359,7 +8373,7 @@
       <c r="H275" s="4"/>
       <c r="I275" s="4"/>
     </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A276" s="2">
         <f t="shared" si="4"/>
         <v>275</v>
@@ -8375,7 +8389,7 @@
       <c r="H276" s="4"/>
       <c r="I276" s="4"/>
     </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A277" s="2">
         <f t="shared" si="4"/>
         <v>276</v>
@@ -8391,7 +8405,7 @@
       <c r="H277" s="4"/>
       <c r="I277" s="4"/>
     </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A278" s="2">
         <f t="shared" si="4"/>
         <v>277</v>
@@ -8407,7 +8421,7 @@
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
     </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A279" s="2">
         <f t="shared" si="4"/>
         <v>278</v>
@@ -8423,7 +8437,7 @@
       <c r="H279" s="4"/>
       <c r="I279" s="4"/>
     </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A280" s="2">
         <f t="shared" si="4"/>
         <v>279</v>
@@ -8439,7 +8453,7 @@
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
     </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A281" s="2">
         <f t="shared" si="4"/>
         <v>280</v>
@@ -8455,7 +8469,7 @@
       <c r="H281" s="4"/>
       <c r="I281" s="4"/>
     </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A282" s="2">
         <f t="shared" si="4"/>
         <v>281</v>
@@ -8471,7 +8485,7 @@
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
     </row>
-    <row r="283" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="283" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A283" s="9">
         <f t="shared" si="4"/>
         <v>282</v>
@@ -8489,7 +8503,7 @@
       <c r="H283" s="8"/>
       <c r="I283" s="8"/>
     </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A284" s="2">
         <f t="shared" si="4"/>
         <v>283</v>
@@ -8505,7 +8519,7 @@
       <c r="H284" s="4"/>
       <c r="I284" s="4"/>
     </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A285" s="2">
         <f t="shared" si="4"/>
         <v>284</v>
@@ -8521,7 +8535,7 @@
       <c r="H285" s="4"/>
       <c r="I285" s="4"/>
     </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A286" s="2">
         <f t="shared" si="4"/>
         <v>285</v>
@@ -8537,7 +8551,7 @@
       <c r="H286" s="4"/>
       <c r="I286" s="4"/>
     </row>
-    <row r="287" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A287" s="2">
         <f t="shared" si="4"/>
         <v>286</v>
@@ -8553,7 +8567,7 @@
       <c r="H287" s="4"/>
       <c r="I287" s="4"/>
     </row>
-    <row r="288" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A288" s="2">
         <f t="shared" si="4"/>
         <v>287</v>
@@ -8569,7 +8583,7 @@
       <c r="H288" s="4"/>
       <c r="I288" s="4"/>
     </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A289" s="2">
         <f t="shared" si="4"/>
         <v>288</v>
@@ -8585,7 +8599,7 @@
       <c r="H289" s="4"/>
       <c r="I289" s="4"/>
     </row>
-    <row r="290" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A290" s="2">
         <f t="shared" si="4"/>
         <v>289</v>
@@ -8601,7 +8615,7 @@
       <c r="H290" s="4"/>
       <c r="I290" s="4"/>
     </row>
-    <row r="291" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A291" s="2">
         <f t="shared" si="4"/>
         <v>290</v>
@@ -8617,7 +8631,7 @@
       <c r="H291" s="4"/>
       <c r="I291" s="4"/>
     </row>
-    <row r="292" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A292" s="2">
         <f t="shared" si="4"/>
         <v>291</v>
@@ -8633,7 +8647,7 @@
       <c r="H292" s="4"/>
       <c r="I292" s="4"/>
     </row>
-    <row r="293" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A293" s="2">
         <f t="shared" si="4"/>
         <v>292</v>
@@ -8649,7 +8663,7 @@
       <c r="H293" s="4"/>
       <c r="I293" s="4"/>
     </row>
-    <row r="294" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
       <c r="A294" s="2">
         <f t="shared" si="4"/>
         <v>293</v>
@@ -8665,7 +8679,7 @@
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
     </row>
-    <row r="295" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="295" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A295" s="9">
         <f t="shared" si="4"/>
         <v>294</v>
@@ -8684,6 +8698,13 @@
       <c r="I295" s="8"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I295" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}">
+    <filterColumn colId="4">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D154:D160 D162:D164 D166:D191 D201:D207 D209:D211 D213:D215 D217:D225 D227:D233 D235:D241 D243:D249 D251:D255 D257:D262 D264:D268 D270 D272:D282 D284:D294 D52:D56 D133:D152">
     <cfRule type="cellIs" dxfId="83" priority="111" operator="equal">
       <formula>"Fail"</formula>

</xml_diff>

<commit_message>
Fix deep zoom UI: Add status bar indicator and enable by default
- Added missing status bar column displaying view dimensions and deep zoom indicator
- Deep zoom indicator shows '- Deep Zoom mode' in brown (SaddleBrown) when zoom >= 1e10
- Changed UseDeepZoom default from false to true (for fresh installs/no persisted settings)
- User's deep zoom preference continues to be persisted and restored
- Fixes issue where deep zoom text was not appearing on status bar
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D040530-6C3C-4F8B-AF18-8A9F73E8353D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{964255C4-2A3A-4CBA-82CF-781B4F7038ED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2617,7 +2617,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:I295"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -2662,7 +2661,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2680,7 +2679,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <f>A2+1</f>
         <v>2</v>
@@ -2699,7 +2698,7 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
@@ -2718,7 +2717,7 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2737,7 +2736,7 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2756,7 +2755,7 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2775,7 +2774,7 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2795,7 +2794,7 @@
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
     </row>
-    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2815,7 +2814,7 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2835,7 +2834,7 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2855,7 +2854,7 @@
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2875,7 +2874,7 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2895,7 +2894,7 @@
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="9">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2915,7 +2914,7 @@
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2935,7 +2934,7 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2977,7 +2976,7 @@
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -3019,7 +3018,7 @@
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
     </row>
-    <row r="20" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="9">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3039,7 +3038,7 @@
       <c r="H20" s="8"/>
       <c r="I20" s="8"/>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3058,7 +3057,7 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
     </row>
-    <row r="22" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="22" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="9">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3078,7 +3077,7 @@
       <c r="H22" s="8"/>
       <c r="I22" s="8"/>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3098,7 +3097,7 @@
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3118,7 +3117,7 @@
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3138,7 +3137,7 @@
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
     </row>
-    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -3158,7 +3157,7 @@
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
     </row>
-    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -3178,7 +3177,7 @@
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -3198,7 +3197,7 @@
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
     </row>
-    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -3218,7 +3217,7 @@
       <c r="H29" s="4"/>
       <c r="I29" s="4"/>
     </row>
-    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -3238,7 +3237,7 @@
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
     </row>
-    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -3258,7 +3257,7 @@
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" s="2">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -3278,7 +3277,7 @@
       <c r="H32" s="4"/>
       <c r="I32" s="4"/>
     </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A33" s="2">
         <f t="shared" si="0"/>
         <v>32</v>
@@ -3320,7 +3319,7 @@
       <c r="H34" s="8"/>
       <c r="I34" s="8"/>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -3348,7 +3347,7 @@
         <v>0.81325301205</v>
       </c>
     </row>
-    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -3376,7 +3375,7 @@
         <v>86.837976550999997</v>
       </c>
     </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" s="2">
         <f t="shared" si="0"/>
         <v>36</v>
@@ -3396,7 +3395,7 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
     </row>
-    <row r="38" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="38" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A38" s="9">
         <f t="shared" si="0"/>
         <v>37</v>
@@ -3416,7 +3415,7 @@
       <c r="H38" s="8"/>
       <c r="I38" s="8"/>
     </row>
-    <row r="39" spans="1:9" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <f t="shared" si="0"/>
         <v>38</v>
@@ -3444,7 +3443,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
@@ -3463,7 +3462,7 @@
       <c r="H40" s="4"/>
       <c r="I40" s="4"/>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A41" s="22">
         <f t="shared" si="0"/>
         <v>40</v>
@@ -3490,7 +3489,7 @@
         <v>5.5981979492000002</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
         <f t="shared" si="0"/>
         <v>41</v>
@@ -3518,7 +3517,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="43" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A43" s="9">
         <f t="shared" si="0"/>
         <v>42</v>
@@ -3538,7 +3537,7 @@
       <c r="H43" s="8"/>
       <c r="I43" s="8"/>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A44" s="2">
         <f t="shared" si="0"/>
         <v>43</v>
@@ -3557,7 +3556,7 @@
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A45" s="2">
         <f t="shared" si="0"/>
         <v>44</v>
@@ -3576,7 +3575,7 @@
       <c r="H45" s="23"/>
       <c r="I45" s="23"/>
     </row>
-    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A46" s="2">
         <f t="shared" si="0"/>
         <v>45</v>
@@ -3595,7 +3594,7 @@
       <c r="H46" s="23"/>
       <c r="I46" s="23"/>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A47" s="22">
         <f t="shared" si="0"/>
         <v>46</v>
@@ -3622,7 +3621,7 @@
         <v>21.35734072</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A48" s="2">
         <f t="shared" si="0"/>
         <v>47</v>
@@ -3641,7 +3640,7 @@
       <c r="H48" s="23"/>
       <c r="I48" s="23"/>
     </row>
-    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -3660,7 +3659,7 @@
       <c r="H49" s="23"/>
       <c r="I49" s="23"/>
     </row>
-    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -3679,7 +3678,7 @@
       <c r="H50" s="23"/>
       <c r="I50" s="23"/>
     </row>
-    <row r="51" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A51" s="9">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -3699,7 +3698,7 @@
       <c r="H51" s="24"/>
       <c r="I51" s="24"/>
     </row>
-    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -3718,7 +3717,7 @@
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
     </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -3737,7 +3736,7 @@
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -3756,7 +3755,7 @@
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
     </row>
-    <row r="55" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="55" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A55" s="9">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -3776,7 +3775,7 @@
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
     </row>
-    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" s="22">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -3803,7 +3802,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -3831,7 +3830,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3859,7 +3858,7 @@
         <v>2.3420689813000002</v>
       </c>
     </row>
-    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A59" s="2">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -3887,7 +3886,7 @@
         <v>1.8436548223</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -3915,7 +3914,7 @@
         <v>2.3309644980000002</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -3965,7 +3964,7 @@
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
     </row>
-    <row r="63" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="63" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A63" s="9">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -3993,7 +3992,7 @@
         <v>0.28801632742</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" s="2">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -4021,7 +4020,7 @@
         <v>1.4659263959</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -4039,7 +4038,7 @@
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
     </row>
-    <row r="66" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="66" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A66" s="9">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -4067,7 +4066,7 @@
         <v>2.397631133</v>
       </c>
     </row>
-    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <f t="shared" si="0"/>
         <v>66</v>
@@ -4095,7 +4094,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A68" s="22">
         <f t="shared" ref="A68:A131" si="1">A67+1</f>
         <v>67</v>
@@ -4122,7 +4121,7 @@
         <v>8.4375</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -4142,7 +4141,7 @@
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A70" s="2">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -4170,7 +4169,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A71" s="2">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -4190,7 +4189,7 @@
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
     </row>
-    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A72" s="2">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -4218,7 +4217,7 @@
         <v>6.75</v>
       </c>
     </row>
-    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A73" s="2">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -4246,7 +4245,7 @@
         <v>21.025059204000002</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -4274,7 +4273,7 @@
         <v>0.2109375</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -4302,7 +4301,7 @@
         <v>1.0884495317</v>
       </c>
     </row>
-    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A76" s="2">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -4330,7 +4329,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A77" s="2">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -4358,7 +4357,7 @@
         <v>1.4678492578</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="78" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A78" s="9">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -4386,7 +4385,7 @@
         <v>0.84375</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -4406,7 +4405,7 @@
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
     </row>
-    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -4426,7 +4425,7 @@
       <c r="H80" s="4"/>
       <c r="I80" s="4"/>
     </row>
-    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
         <f t="shared" si="1"/>
         <v>80</v>
@@ -4454,7 +4453,7 @@
         <v>3.8068369917</v>
       </c>
     </row>
-    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A82" s="2">
         <f t="shared" si="1"/>
         <v>81</v>
@@ -4504,7 +4503,7 @@
       <c r="H83" s="4"/>
       <c r="I83" s="4"/>
     </row>
-    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
         <f t="shared" si="1"/>
         <v>83</v>
@@ -4532,7 +4531,7 @@
         <v>2.2090805910000002</v>
       </c>
     </row>
-    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
         <f t="shared" si="1"/>
         <v>84</v>
@@ -4552,7 +4551,7 @@
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
     </row>
-    <row r="86" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="86" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A86" s="9">
         <f t="shared" si="1"/>
         <v>85</v>
@@ -4572,7 +4571,7 @@
       <c r="H86" s="21"/>
       <c r="I86" s="21"/>
     </row>
-    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <f t="shared" si="1"/>
         <v>86</v>
@@ -4600,7 +4599,7 @@
         <v>3.7408990110000002</v>
       </c>
     </row>
-    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A88" s="2">
         <f t="shared" si="1"/>
         <v>87</v>
@@ -4628,7 +4627,7 @@
         <v>2.1342925659</v>
       </c>
     </row>
-    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A89" s="2">
         <f t="shared" si="1"/>
         <v>88</v>
@@ -4656,7 +4655,7 @@
         <v>2.4107142857000001</v>
       </c>
     </row>
-    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A90" s="2">
         <f t="shared" si="1"/>
         <v>89</v>
@@ -4684,7 +4683,7 @@
         <v>2.3556012803000002</v>
       </c>
     </row>
-    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
         <f t="shared" si="1"/>
         <v>90</v>
@@ -4712,7 +4711,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
         <f t="shared" si="1"/>
         <v>91</v>
@@ -4740,7 +4739,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
         <f t="shared" si="1"/>
         <v>92</v>
@@ -4768,7 +4767,7 @@
         <v>3.2040082611999998</v>
       </c>
     </row>
-    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
         <f t="shared" si="1"/>
         <v>93</v>
@@ -4796,7 +4795,7 @@
         <v>11.181911864</v>
       </c>
     </row>
-    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
         <f t="shared" si="1"/>
         <v>94</v>
@@ -4824,7 +4823,7 @@
         <v>2.542651593</v>
       </c>
     </row>
-    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
         <f t="shared" si="1"/>
         <v>95</v>
@@ -4852,7 +4851,7 @@
         <v>4.6783144913000001</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <f t="shared" si="1"/>
         <v>96</v>
@@ -4872,7 +4871,7 @@
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <f t="shared" si="1"/>
         <v>97</v>
@@ -4900,7 +4899,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -4928,7 +4927,7 @@
         <v>6.1130526660999998</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A100" s="2">
         <f t="shared" si="1"/>
         <v>99</v>
@@ -4956,7 +4955,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="20.65" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:9" ht="20.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -4984,7 +4983,7 @@
         <v>4.21875</v>
       </c>
     </row>
-    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -5012,7 +5011,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
         <f t="shared" si="1"/>
         <v>102</v>
@@ -5040,7 +5039,7 @@
         <v>1.0194922309000001</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="104" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A104" s="9">
         <f t="shared" si="1"/>
         <v>103</v>
@@ -5068,7 +5067,7 @@
         <v>2.3396227092999999</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
         <f t="shared" si="1"/>
         <v>104</v>
@@ -5096,7 +5095,7 @@
         <v>11.028960818</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
         <f t="shared" si="1"/>
         <v>105</v>
@@ -5124,7 +5123,7 @@
         <v>1.1422222222</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
         <f t="shared" si="1"/>
         <v>106</v>
@@ -5152,7 +5151,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
         <f t="shared" si="1"/>
         <v>107</v>
@@ -5180,7 +5179,7 @@
         <v>1.125</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="109" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A109" s="9">
         <f t="shared" si="1"/>
         <v>108</v>
@@ -5208,7 +5207,7 @@
         <v>0.82935879629999998</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
         <f t="shared" si="1"/>
         <v>109</v>
@@ -5236,7 +5235,7 @@
         <v>2.4900562852000001</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -5264,7 +5263,7 @@
         <v>2.2581613508</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -5292,7 +5291,7 @@
         <v>2.956097561</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A113" s="2">
         <f t="shared" si="1"/>
         <v>112</v>
@@ -5320,7 +5319,7 @@
         <v>2.4279250753000001</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A114" s="2">
         <f t="shared" si="1"/>
         <v>113</v>
@@ -5339,7 +5338,7 @@
       <c r="H114" s="4"/>
       <c r="I114" s="4"/>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A115" s="2">
         <f t="shared" si="1"/>
         <v>114</v>
@@ -5366,7 +5365,7 @@
         <v>2.4135156878999999</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A116" s="2">
         <f t="shared" si="1"/>
         <v>115</v>
@@ -5393,7 +5392,7 @@
         <v>2.2134956765</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A117" s="2">
         <f t="shared" si="1"/>
         <v>116</v>
@@ -5420,7 +5419,7 @@
         <v>2.5144496681000001</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A118" s="2">
         <f t="shared" si="1"/>
         <v>117</v>
@@ -5447,7 +5446,7 @@
         <v>2.4081908582999998</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A119" s="2">
         <f t="shared" si="1"/>
         <v>118</v>
@@ -5474,7 +5473,7 @@
         <v>1.9245172044000001</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
         <f t="shared" si="1"/>
         <v>119</v>
@@ -5501,7 +5500,7 @@
         <v>2.2422422422000001</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
         <f t="shared" si="1"/>
         <v>120</v>
@@ -5528,7 +5527,7 @@
         <v>2.4078947367999999</v>
       </c>
     </row>
-    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
         <f t="shared" si="1"/>
         <v>121</v>
@@ -5555,7 +5554,7 @@
         <v>1.9986149583999999</v>
       </c>
     </row>
-    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
         <f t="shared" si="1"/>
         <v>122</v>
@@ -5582,7 +5581,7 @@
         <v>2.2622149836999998</v>
       </c>
     </row>
-    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
         <f t="shared" si="1"/>
         <v>123</v>
@@ -5609,7 +5608,7 @@
         <v>2.3257329176999999</v>
       </c>
     </row>
-    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
         <f t="shared" si="1"/>
         <v>124</v>
@@ -5636,7 +5635,7 @@
         <v>2.0472313449000001</v>
       </c>
     </row>
-    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
         <f t="shared" si="1"/>
         <v>125</v>
@@ -5663,7 +5662,7 @@
         <v>2.4332247557</v>
       </c>
     </row>
-    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
         <f t="shared" si="1"/>
         <v>126</v>
@@ -5690,7 +5689,7 @@
         <v>1.836565097</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
         <f t="shared" si="1"/>
         <v>127</v>
@@ -5717,7 +5716,7 @@
         <v>2.3746537395999998</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <f t="shared" si="1"/>
         <v>128</v>
@@ -5744,7 +5743,7 @@
         <v>2.4515236091000001</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <f t="shared" si="1"/>
         <v>129</v>
@@ -5771,7 +5770,7 @@
         <v>2.2475570032999999</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <f t="shared" si="1"/>
         <v>130</v>
@@ -5798,7 +5797,7 @@
         <v>2.237534626</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="132" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A132" s="9">
         <f t="shared" ref="A132:A204" si="2">A131+1</f>
         <v>131</v>
@@ -5826,7 +5825,7 @@
         <v>2.3891966918</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
         <f t="shared" si="2"/>
         <v>132</v>
@@ -5845,7 +5844,7 @@
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A134" s="2">
         <f t="shared" si="2"/>
         <v>133</v>
@@ -5872,7 +5871,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
         <f t="shared" si="2"/>
         <v>134</v>
@@ -5899,7 +5898,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
         <f t="shared" si="2"/>
         <v>135</v>
@@ -5918,7 +5917,7 @@
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A137" s="2">
         <f t="shared" si="2"/>
         <v>136</v>
@@ -5945,7 +5944,7 @@
         <v>2.5051334684</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A138" s="2">
         <f t="shared" si="2"/>
         <v>137</v>
@@ -5972,7 +5971,7 @@
         <v>2.2266695994000001</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A139" s="2">
         <f t="shared" si="2"/>
         <v>138</v>
@@ -5991,7 +5990,7 @@
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
     </row>
-    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A140" s="2">
         <f t="shared" si="2"/>
         <v>139</v>
@@ -6078,7 +6077,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A143" s="2">
         <f t="shared" si="2"/>
         <v>142</v>
@@ -6105,7 +6104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A144" s="2">
         <f t="shared" si="2"/>
         <v>143</v>
@@ -6162,7 +6161,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A146" s="2">
         <f t="shared" si="2"/>
         <v>145</v>
@@ -6249,7 +6248,7 @@
         <v>3.3313313309999999</v>
       </c>
     </row>
-    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A149" s="2">
         <f t="shared" si="2"/>
         <v>148</v>
@@ -6276,7 +6275,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A150" s="2">
         <f t="shared" si="2"/>
         <v>149</v>
@@ -6363,7 +6362,7 @@
         <v>12.595945386</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="153" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A153" s="9">
         <f t="shared" si="2"/>
         <v>152</v>
@@ -6391,7 +6390,7 @@
         <v>1.808617718</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A154" s="2">
         <f t="shared" si="2"/>
         <v>153</v>
@@ -6407,7 +6406,7 @@
       <c r="H154" s="4"/>
       <c r="I154" s="4"/>
     </row>
-    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A155" s="2">
         <f t="shared" si="2"/>
         <v>154</v>
@@ -6423,7 +6422,7 @@
       <c r="H155" s="4"/>
       <c r="I155" s="4"/>
     </row>
-    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A156" s="2">
         <f t="shared" si="2"/>
         <v>155</v>
@@ -6439,7 +6438,7 @@
       <c r="H156" s="4"/>
       <c r="I156" s="4"/>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A157" s="2">
         <f t="shared" si="2"/>
         <v>156</v>
@@ -6455,7 +6454,7 @@
       <c r="H157" s="4"/>
       <c r="I157" s="4"/>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A158" s="2">
         <f t="shared" si="2"/>
         <v>157</v>
@@ -6471,7 +6470,7 @@
       <c r="H158" s="4"/>
       <c r="I158" s="4"/>
     </row>
-    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A159" s="2">
         <f t="shared" si="2"/>
         <v>158</v>
@@ -6487,7 +6486,7 @@
       <c r="H159" s="4"/>
       <c r="I159" s="4"/>
     </row>
-    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A160" s="2">
         <f t="shared" si="2"/>
         <v>159</v>
@@ -6503,7 +6502,7 @@
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
     </row>
-    <row r="161" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="161" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A161" s="9">
         <f t="shared" si="2"/>
         <v>160</v>
@@ -6521,7 +6520,7 @@
       <c r="H161" s="8"/>
       <c r="I161" s="8"/>
     </row>
-    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A162" s="2">
         <f t="shared" si="2"/>
         <v>161</v>
@@ -6537,7 +6536,7 @@
       <c r="H162" s="4"/>
       <c r="I162" s="4"/>
     </row>
-    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A163" s="2">
         <f t="shared" si="2"/>
         <v>162</v>
@@ -6553,7 +6552,7 @@
       <c r="H163" s="4"/>
       <c r="I163" s="4"/>
     </row>
-    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A164" s="2">
         <f t="shared" si="2"/>
         <v>163</v>
@@ -6569,7 +6568,7 @@
       <c r="H164" s="4"/>
       <c r="I164" s="4"/>
     </row>
-    <row r="165" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="165" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A165" s="9">
         <f t="shared" si="2"/>
         <v>164</v>
@@ -6587,7 +6586,7 @@
       <c r="H165" s="8"/>
       <c r="I165" s="8"/>
     </row>
-    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A166" s="2">
         <f t="shared" si="2"/>
         <v>165</v>
@@ -6603,7 +6602,7 @@
       <c r="H166" s="4"/>
       <c r="I166" s="4"/>
     </row>
-    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A167" s="25">
         <f t="shared" si="2"/>
         <v>166</v>
@@ -6619,7 +6618,7 @@
       <c r="H167" s="4"/>
       <c r="I167" s="4"/>
     </row>
-    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A168" s="2">
         <f t="shared" si="2"/>
         <v>167</v>
@@ -6635,7 +6634,7 @@
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
     </row>
-    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A169" s="2">
         <f t="shared" si="2"/>
         <v>168</v>
@@ -6651,7 +6650,7 @@
       <c r="H169" s="4"/>
       <c r="I169" s="4"/>
     </row>
-    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A170" s="2">
         <f t="shared" si="2"/>
         <v>169</v>
@@ -6667,7 +6666,7 @@
       <c r="H170" s="4"/>
       <c r="I170" s="4"/>
     </row>
-    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A171" s="2">
         <f t="shared" si="2"/>
         <v>170</v>
@@ -6683,7 +6682,7 @@
       <c r="H171" s="4"/>
       <c r="I171" s="4"/>
     </row>
-    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A172" s="2">
         <f t="shared" si="2"/>
         <v>171</v>
@@ -6699,7 +6698,7 @@
       <c r="H172" s="4"/>
       <c r="I172" s="4"/>
     </row>
-    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A173" s="2">
         <f t="shared" si="2"/>
         <v>172</v>
@@ -6715,7 +6714,7 @@
       <c r="H173" s="4"/>
       <c r="I173" s="4"/>
     </row>
-    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A174" s="2">
         <f t="shared" si="2"/>
         <v>173</v>
@@ -6731,7 +6730,7 @@
       <c r="H174" s="4"/>
       <c r="I174" s="4"/>
     </row>
-    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A175" s="2">
         <f t="shared" si="2"/>
         <v>174</v>
@@ -6747,7 +6746,7 @@
       <c r="H175" s="4"/>
       <c r="I175" s="4"/>
     </row>
-    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A176" s="2">
         <f t="shared" si="2"/>
         <v>175</v>
@@ -6763,7 +6762,7 @@
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
     </row>
-    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A177" s="2">
         <f t="shared" si="2"/>
         <v>176</v>
@@ -6779,7 +6778,7 @@
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
     </row>
-    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A178" s="2">
         <f t="shared" si="2"/>
         <v>177</v>
@@ -6795,7 +6794,7 @@
       <c r="H178" s="4"/>
       <c r="I178" s="4"/>
     </row>
-    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A179" s="2">
         <f t="shared" si="2"/>
         <v>178</v>
@@ -6811,7 +6810,7 @@
       <c r="H179" s="4"/>
       <c r="I179" s="4"/>
     </row>
-    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A180" s="2">
         <f t="shared" si="2"/>
         <v>179</v>
@@ -6827,7 +6826,7 @@
       <c r="H180" s="4"/>
       <c r="I180" s="4"/>
     </row>
-    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A181" s="2">
         <f t="shared" si="2"/>
         <v>180</v>
@@ -6843,7 +6842,7 @@
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
     </row>
-    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A182" s="2">
         <f t="shared" si="2"/>
         <v>181</v>
@@ -6859,7 +6858,7 @@
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
     </row>
-    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A183" s="2">
         <f t="shared" si="2"/>
         <v>182</v>
@@ -6875,7 +6874,7 @@
       <c r="H183" s="4"/>
       <c r="I183" s="4"/>
     </row>
-    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A184" s="2">
         <f t="shared" si="2"/>
         <v>183</v>
@@ -6891,7 +6890,7 @@
       <c r="H184" s="4"/>
       <c r="I184" s="4"/>
     </row>
-    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A185" s="2">
         <f t="shared" si="2"/>
         <v>184</v>
@@ -6907,7 +6906,7 @@
       <c r="H185" s="4"/>
       <c r="I185" s="4"/>
     </row>
-    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A186" s="2">
         <f t="shared" si="2"/>
         <v>185</v>
@@ -6923,7 +6922,7 @@
       <c r="H186" s="4"/>
       <c r="I186" s="4"/>
     </row>
-    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A187" s="2">
         <f t="shared" si="2"/>
         <v>186</v>
@@ -6939,7 +6938,7 @@
       <c r="H187" s="4"/>
       <c r="I187" s="4"/>
     </row>
-    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A188" s="2">
         <f t="shared" si="2"/>
         <v>187</v>
@@ -6955,7 +6954,7 @@
       <c r="H188" s="4"/>
       <c r="I188" s="4"/>
     </row>
-    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A189" s="2">
         <f t="shared" si="2"/>
         <v>188</v>
@@ -6971,7 +6970,7 @@
       <c r="H189" s="4"/>
       <c r="I189" s="4"/>
     </row>
-    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A190" s="2">
         <f t="shared" si="2"/>
         <v>189</v>
@@ -6987,7 +6986,7 @@
       <c r="H190" s="4"/>
       <c r="I190" s="4"/>
     </row>
-    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A191" s="2">
         <f t="shared" si="2"/>
         <v>190</v>
@@ -7003,7 +7002,7 @@
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
     </row>
-    <row r="192" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="192" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A192" s="9">
         <f t="shared" si="2"/>
         <v>191</v>
@@ -7021,7 +7020,7 @@
       <c r="H192" s="8"/>
       <c r="I192" s="8"/>
     </row>
-    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A193" s="9">
         <f t="shared" si="2"/>
         <v>192</v>
@@ -7037,7 +7036,7 @@
       <c r="H193" s="4"/>
       <c r="I193" s="4"/>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A194" s="9">
         <f t="shared" si="2"/>
         <v>193</v>
@@ -7053,7 +7052,7 @@
       <c r="H194" s="4"/>
       <c r="I194" s="4"/>
     </row>
-    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A195" s="9">
         <f t="shared" si="2"/>
         <v>194</v>
@@ -7069,7 +7068,7 @@
       <c r="H195" s="4"/>
       <c r="I195" s="4"/>
     </row>
-    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A196" s="9">
         <f t="shared" si="2"/>
         <v>195</v>
@@ -7085,7 +7084,7 @@
       <c r="H196" s="4"/>
       <c r="I196" s="4"/>
     </row>
-    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A197" s="9">
         <f t="shared" si="2"/>
         <v>196</v>
@@ -7101,7 +7100,7 @@
       <c r="H197" s="4"/>
       <c r="I197" s="4"/>
     </row>
-    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A198" s="9">
         <f t="shared" si="2"/>
         <v>197</v>
@@ -7117,7 +7116,7 @@
       <c r="H198" s="4"/>
       <c r="I198" s="4"/>
     </row>
-    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A199" s="9">
         <f t="shared" si="2"/>
         <v>198</v>
@@ -7133,7 +7132,7 @@
       <c r="H199" s="4"/>
       <c r="I199" s="4"/>
     </row>
-    <row r="200" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="200" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A200" s="9">
         <f t="shared" si="2"/>
         <v>199</v>
@@ -7151,7 +7150,7 @@
       <c r="H200" s="8"/>
       <c r="I200" s="8"/>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A201" s="9">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -7167,7 +7166,7 @@
       <c r="H201" s="4"/>
       <c r="I201" s="4"/>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A202" s="9">
         <f t="shared" si="2"/>
         <v>201</v>
@@ -7183,7 +7182,7 @@
       <c r="H202" s="4"/>
       <c r="I202" s="4"/>
     </row>
-    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A203" s="2">
         <f t="shared" si="2"/>
         <v>202</v>
@@ -7199,7 +7198,7 @@
       <c r="H203" s="4"/>
       <c r="I203" s="4"/>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A204" s="2">
         <f t="shared" si="2"/>
         <v>203</v>
@@ -7215,7 +7214,7 @@
       <c r="H204" s="4"/>
       <c r="I204" s="4"/>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A205" s="2">
         <f t="shared" ref="A205:A264" si="3">A204+1</f>
         <v>204</v>
@@ -7231,7 +7230,7 @@
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
     </row>
-    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A206" s="2">
         <f t="shared" si="3"/>
         <v>205</v>
@@ -7247,7 +7246,7 @@
       <c r="H206" s="4"/>
       <c r="I206" s="4"/>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A207" s="2">
         <f t="shared" si="3"/>
         <v>206</v>
@@ -7263,7 +7262,7 @@
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
     </row>
-    <row r="208" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="208" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A208" s="9">
         <f t="shared" si="3"/>
         <v>207</v>
@@ -7281,7 +7280,7 @@
       <c r="H208" s="8"/>
       <c r="I208" s="8"/>
     </row>
-    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A209" s="2">
         <f t="shared" si="3"/>
         <v>208</v>
@@ -7297,7 +7296,7 @@
       <c r="H209" s="4"/>
       <c r="I209" s="4"/>
     </row>
-    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A210" s="2">
         <f t="shared" si="3"/>
         <v>209</v>
@@ -7313,7 +7312,7 @@
       <c r="H210" s="4"/>
       <c r="I210" s="4"/>
     </row>
-    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A211" s="2">
         <f t="shared" si="3"/>
         <v>210</v>
@@ -7329,7 +7328,7 @@
       <c r="H211" s="4"/>
       <c r="I211" s="4"/>
     </row>
-    <row r="212" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="212" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A212" s="9">
         <f t="shared" si="3"/>
         <v>211</v>
@@ -7347,7 +7346,7 @@
       <c r="H212" s="8"/>
       <c r="I212" s="8"/>
     </row>
-    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A213" s="2">
         <f t="shared" si="3"/>
         <v>212</v>
@@ -7363,7 +7362,7 @@
       <c r="H213" s="4"/>
       <c r="I213" s="4"/>
     </row>
-    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A214" s="2">
         <f t="shared" si="3"/>
         <v>213</v>
@@ -7379,7 +7378,7 @@
       <c r="H214" s="4"/>
       <c r="I214" s="4"/>
     </row>
-    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A215" s="2">
         <f t="shared" si="3"/>
         <v>214</v>
@@ -7395,7 +7394,7 @@
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
     </row>
-    <row r="216" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="216" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A216" s="9">
         <f t="shared" si="3"/>
         <v>215</v>
@@ -7413,7 +7412,7 @@
       <c r="H216" s="8"/>
       <c r="I216" s="8"/>
     </row>
-    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A217" s="2">
         <f t="shared" si="3"/>
         <v>216</v>
@@ -7429,7 +7428,7 @@
       <c r="H217" s="4"/>
       <c r="I217" s="4"/>
     </row>
-    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A218" s="2">
         <f t="shared" si="3"/>
         <v>217</v>
@@ -7445,7 +7444,7 @@
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
     </row>
-    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A219" s="2">
         <f t="shared" si="3"/>
         <v>218</v>
@@ -7461,7 +7460,7 @@
       <c r="H219" s="4"/>
       <c r="I219" s="4"/>
     </row>
-    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A220" s="2">
         <f t="shared" si="3"/>
         <v>219</v>
@@ -7477,7 +7476,7 @@
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
     </row>
-    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A221" s="2">
         <f t="shared" si="3"/>
         <v>220</v>
@@ -7493,7 +7492,7 @@
       <c r="H221" s="4"/>
       <c r="I221" s="4"/>
     </row>
-    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A222" s="2">
         <f t="shared" si="3"/>
         <v>221</v>
@@ -7509,7 +7508,7 @@
       <c r="H222" s="4"/>
       <c r="I222" s="4"/>
     </row>
-    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A223" s="2">
         <f t="shared" si="3"/>
         <v>222</v>
@@ -7525,7 +7524,7 @@
       <c r="H223" s="4"/>
       <c r="I223" s="4"/>
     </row>
-    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A224" s="2">
         <f t="shared" si="3"/>
         <v>223</v>
@@ -7541,7 +7540,7 @@
       <c r="H224" s="4"/>
       <c r="I224" s="4"/>
     </row>
-    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A225" s="2">
         <f t="shared" si="3"/>
         <v>224</v>
@@ -7557,7 +7556,7 @@
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
     </row>
-    <row r="226" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="226" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A226" s="9">
         <f t="shared" si="3"/>
         <v>225</v>
@@ -7575,7 +7574,7 @@
       <c r="H226" s="8"/>
       <c r="I226" s="8"/>
     </row>
-    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A227" s="2">
         <f t="shared" si="3"/>
         <v>226</v>
@@ -7591,7 +7590,7 @@
       <c r="H227" s="4"/>
       <c r="I227" s="4"/>
     </row>
-    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A228" s="2">
         <f t="shared" si="3"/>
         <v>227</v>
@@ -7607,7 +7606,7 @@
       <c r="H228" s="4"/>
       <c r="I228" s="4"/>
     </row>
-    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A229" s="2">
         <f t="shared" si="3"/>
         <v>228</v>
@@ -7623,7 +7622,7 @@
       <c r="H229" s="4"/>
       <c r="I229" s="4"/>
     </row>
-    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
         <f t="shared" si="3"/>
         <v>229</v>
@@ -7639,7 +7638,7 @@
       <c r="H230" s="4"/>
       <c r="I230" s="4"/>
     </row>
-    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A231" s="2">
         <f t="shared" si="3"/>
         <v>230</v>
@@ -7655,7 +7654,7 @@
       <c r="H231" s="4"/>
       <c r="I231" s="4"/>
     </row>
-    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A232" s="2">
         <f t="shared" si="3"/>
         <v>231</v>
@@ -7671,7 +7670,7 @@
       <c r="H232" s="4"/>
       <c r="I232" s="4"/>
     </row>
-    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A233" s="2">
         <f t="shared" si="3"/>
         <v>232</v>
@@ -7687,7 +7686,7 @@
       <c r="H233" s="4"/>
       <c r="I233" s="4"/>
     </row>
-    <row r="234" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="234" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A234" s="9">
         <f t="shared" si="3"/>
         <v>233</v>
@@ -7705,7 +7704,7 @@
       <c r="H234" s="8"/>
       <c r="I234" s="8"/>
     </row>
-    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A235" s="2">
         <f t="shared" si="3"/>
         <v>234</v>
@@ -7721,7 +7720,7 @@
       <c r="H235" s="4"/>
       <c r="I235" s="4"/>
     </row>
-    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A236" s="2">
         <f t="shared" si="3"/>
         <v>235</v>
@@ -7737,7 +7736,7 @@
       <c r="H236" s="4"/>
       <c r="I236" s="4"/>
     </row>
-    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A237" s="2">
         <f t="shared" si="3"/>
         <v>236</v>
@@ -7753,7 +7752,7 @@
       <c r="H237" s="4"/>
       <c r="I237" s="4"/>
     </row>
-    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A238" s="2">
         <f t="shared" si="3"/>
         <v>237</v>
@@ -7769,7 +7768,7 @@
       <c r="H238" s="4"/>
       <c r="I238" s="4"/>
     </row>
-    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A239" s="2">
         <f t="shared" si="3"/>
         <v>238</v>
@@ -7785,7 +7784,7 @@
       <c r="H239" s="4"/>
       <c r="I239" s="4"/>
     </row>
-    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A240" s="2">
         <f t="shared" si="3"/>
         <v>239</v>
@@ -7801,7 +7800,7 @@
       <c r="H240" s="4"/>
       <c r="I240" s="4"/>
     </row>
-    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A241" s="2">
         <f t="shared" si="3"/>
         <v>240</v>
@@ -7817,7 +7816,7 @@
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
     </row>
-    <row r="242" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="242" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A242" s="2">
         <f t="shared" si="3"/>
         <v>241</v>
@@ -7835,7 +7834,7 @@
       <c r="H242" s="8"/>
       <c r="I242" s="8"/>
     </row>
-    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A243" s="2">
         <f t="shared" si="3"/>
         <v>242</v>
@@ -7851,7 +7850,7 @@
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
     </row>
-    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A244" s="2">
         <f t="shared" si="3"/>
         <v>243</v>
@@ -7867,7 +7866,7 @@
       <c r="H244" s="4"/>
       <c r="I244" s="4"/>
     </row>
-    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A245" s="2">
         <f t="shared" si="3"/>
         <v>244</v>
@@ -7883,7 +7882,7 @@
       <c r="H245" s="4"/>
       <c r="I245" s="4"/>
     </row>
-    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A246" s="2">
         <f t="shared" si="3"/>
         <v>245</v>
@@ -7899,7 +7898,7 @@
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
     </row>
-    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A247" s="2">
         <f t="shared" si="3"/>
         <v>246</v>
@@ -7915,7 +7914,7 @@
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
     </row>
-    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A248" s="2">
         <f t="shared" si="3"/>
         <v>247</v>
@@ -7931,7 +7930,7 @@
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
     </row>
-    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A249" s="2">
         <f t="shared" si="3"/>
         <v>248</v>
@@ -7947,7 +7946,7 @@
       <c r="H249" s="4"/>
       <c r="I249" s="4"/>
     </row>
-    <row r="250" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="250" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A250" s="2">
         <f t="shared" si="3"/>
         <v>249</v>
@@ -7965,7 +7964,7 @@
       <c r="H250" s="8"/>
       <c r="I250" s="8"/>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A251" s="2">
         <f t="shared" si="3"/>
         <v>250</v>
@@ -7981,7 +7980,7 @@
       <c r="H251" s="4"/>
       <c r="I251" s="4"/>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A252" s="2">
         <f t="shared" si="3"/>
         <v>251</v>
@@ -7997,7 +7996,7 @@
       <c r="H252" s="4"/>
       <c r="I252" s="4"/>
     </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A253" s="2">
         <f t="shared" si="3"/>
         <v>252</v>
@@ -8013,7 +8012,7 @@
       <c r="H253" s="4"/>
       <c r="I253" s="4"/>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A254" s="2">
         <f t="shared" si="3"/>
         <v>253</v>
@@ -8029,7 +8028,7 @@
       <c r="H254" s="4"/>
       <c r="I254" s="4"/>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A255" s="2">
         <f t="shared" si="3"/>
         <v>254</v>
@@ -8045,7 +8044,7 @@
       <c r="H255" s="4"/>
       <c r="I255" s="4"/>
     </row>
-    <row r="256" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="256" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A256" s="2">
         <f t="shared" si="3"/>
         <v>255</v>
@@ -8063,7 +8062,7 @@
       <c r="H256" s="8"/>
       <c r="I256" s="8"/>
     </row>
-    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A257" s="2">
         <f t="shared" si="3"/>
         <v>256</v>
@@ -8079,7 +8078,7 @@
       <c r="H257" s="4"/>
       <c r="I257" s="4"/>
     </row>
-    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A258" s="2">
         <f t="shared" si="3"/>
         <v>257</v>
@@ -8095,7 +8094,7 @@
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
     </row>
-    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A259" s="2">
         <f t="shared" si="3"/>
         <v>258</v>
@@ -8111,7 +8110,7 @@
       <c r="H259" s="4"/>
       <c r="I259" s="4"/>
     </row>
-    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A260" s="2">
         <f t="shared" si="3"/>
         <v>259</v>
@@ -8127,7 +8126,7 @@
       <c r="H260" s="4"/>
       <c r="I260" s="4"/>
     </row>
-    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A261" s="2">
         <f t="shared" si="3"/>
         <v>260</v>
@@ -8143,7 +8142,7 @@
       <c r="H261" s="4"/>
       <c r="I261" s="4"/>
     </row>
-    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A262" s="2">
         <f t="shared" si="3"/>
         <v>261</v>
@@ -8159,7 +8158,7 @@
       <c r="H262" s="4"/>
       <c r="I262" s="4"/>
     </row>
-    <row r="263" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="263" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A263" s="2">
         <f t="shared" si="3"/>
         <v>262</v>
@@ -8177,7 +8176,7 @@
       <c r="H263" s="8"/>
       <c r="I263" s="8"/>
     </row>
-    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A264" s="2">
         <f t="shared" si="3"/>
         <v>263</v>
@@ -8193,7 +8192,7 @@
       <c r="H264" s="4"/>
       <c r="I264" s="4"/>
     </row>
-    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A265" s="2">
         <f t="shared" ref="A265:A295" si="4">A264+1</f>
         <v>264</v>
@@ -8209,7 +8208,7 @@
       <c r="H265" s="4"/>
       <c r="I265" s="4"/>
     </row>
-    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A266" s="2">
         <f t="shared" si="4"/>
         <v>265</v>
@@ -8225,7 +8224,7 @@
       <c r="H266" s="4"/>
       <c r="I266" s="4"/>
     </row>
-    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A267" s="2">
         <f t="shared" si="4"/>
         <v>266</v>
@@ -8241,7 +8240,7 @@
       <c r="H267" s="4"/>
       <c r="I267" s="4"/>
     </row>
-    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A268" s="2">
         <f t="shared" si="4"/>
         <v>267</v>
@@ -8257,7 +8256,7 @@
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
     </row>
-    <row r="269" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="269" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A269" s="9">
         <f t="shared" si="4"/>
         <v>268</v>
@@ -8275,7 +8274,7 @@
       <c r="H269" s="8"/>
       <c r="I269" s="8"/>
     </row>
-    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A270" s="2">
         <f t="shared" si="4"/>
         <v>269</v>
@@ -8291,7 +8290,7 @@
       <c r="H270" s="4"/>
       <c r="I270" s="4"/>
     </row>
-    <row r="271" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="271" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A271" s="9">
         <f t="shared" si="4"/>
         <v>270</v>
@@ -8309,7 +8308,7 @@
       <c r="H271" s="8"/>
       <c r="I271" s="8"/>
     </row>
-    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A272" s="2">
         <f t="shared" si="4"/>
         <v>271</v>
@@ -8325,7 +8324,7 @@
       <c r="H272" s="4"/>
       <c r="I272" s="4"/>
     </row>
-    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A273" s="2">
         <f t="shared" si="4"/>
         <v>272</v>
@@ -8341,7 +8340,7 @@
       <c r="H273" s="4"/>
       <c r="I273" s="4"/>
     </row>
-    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A274" s="2">
         <f t="shared" si="4"/>
         <v>273</v>
@@ -8357,7 +8356,7 @@
       <c r="H274" s="4"/>
       <c r="I274" s="4"/>
     </row>
-    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A275" s="2">
         <f t="shared" si="4"/>
         <v>274</v>
@@ -8373,7 +8372,7 @@
       <c r="H275" s="4"/>
       <c r="I275" s="4"/>
     </row>
-    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A276" s="2">
         <f t="shared" si="4"/>
         <v>275</v>
@@ -8389,7 +8388,7 @@
       <c r="H276" s="4"/>
       <c r="I276" s="4"/>
     </row>
-    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A277" s="2">
         <f t="shared" si="4"/>
         <v>276</v>
@@ -8405,7 +8404,7 @@
       <c r="H277" s="4"/>
       <c r="I277" s="4"/>
     </row>
-    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A278" s="2">
         <f t="shared" si="4"/>
         <v>277</v>
@@ -8421,7 +8420,7 @@
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
     </row>
-    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A279" s="2">
         <f t="shared" si="4"/>
         <v>278</v>
@@ -8437,7 +8436,7 @@
       <c r="H279" s="4"/>
       <c r="I279" s="4"/>
     </row>
-    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A280" s="2">
         <f t="shared" si="4"/>
         <v>279</v>
@@ -8453,7 +8452,7 @@
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
     </row>
-    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A281" s="2">
         <f t="shared" si="4"/>
         <v>280</v>
@@ -8469,7 +8468,7 @@
       <c r="H281" s="4"/>
       <c r="I281" s="4"/>
     </row>
-    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A282" s="2">
         <f t="shared" si="4"/>
         <v>281</v>
@@ -8485,7 +8484,7 @@
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
     </row>
-    <row r="283" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="283" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A283" s="9">
         <f t="shared" si="4"/>
         <v>282</v>
@@ -8503,7 +8502,7 @@
       <c r="H283" s="8"/>
       <c r="I283" s="8"/>
     </row>
-    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A284" s="2">
         <f t="shared" si="4"/>
         <v>283</v>
@@ -8519,7 +8518,7 @@
       <c r="H284" s="4"/>
       <c r="I284" s="4"/>
     </row>
-    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A285" s="2">
         <f t="shared" si="4"/>
         <v>284</v>
@@ -8535,7 +8534,7 @@
       <c r="H285" s="4"/>
       <c r="I285" s="4"/>
     </row>
-    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A286" s="2">
         <f t="shared" si="4"/>
         <v>285</v>
@@ -8551,7 +8550,7 @@
       <c r="H286" s="4"/>
       <c r="I286" s="4"/>
     </row>
-    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A287" s="2">
         <f t="shared" si="4"/>
         <v>286</v>
@@ -8567,7 +8566,7 @@
       <c r="H287" s="4"/>
       <c r="I287" s="4"/>
     </row>
-    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A288" s="2">
         <f t="shared" si="4"/>
         <v>287</v>
@@ -8583,7 +8582,7 @@
       <c r="H288" s="4"/>
       <c r="I288" s="4"/>
     </row>
-    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A289" s="2">
         <f t="shared" si="4"/>
         <v>288</v>
@@ -8599,7 +8598,7 @@
       <c r="H289" s="4"/>
       <c r="I289" s="4"/>
     </row>
-    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A290" s="2">
         <f t="shared" si="4"/>
         <v>289</v>
@@ -8615,7 +8614,7 @@
       <c r="H290" s="4"/>
       <c r="I290" s="4"/>
     </row>
-    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A291" s="2">
         <f t="shared" si="4"/>
         <v>290</v>
@@ -8631,7 +8630,7 @@
       <c r="H291" s="4"/>
       <c r="I291" s="4"/>
     </row>
-    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A292" s="2">
         <f t="shared" si="4"/>
         <v>291</v>
@@ -8647,7 +8646,7 @@
       <c r="H292" s="4"/>
       <c r="I292" s="4"/>
     </row>
-    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A293" s="2">
         <f t="shared" si="4"/>
         <v>292</v>
@@ -8663,7 +8662,7 @@
       <c r="H293" s="4"/>
       <c r="I293" s="4"/>
     </row>
-    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.45">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A294" s="2">
         <f t="shared" si="4"/>
         <v>293</v>
@@ -8679,7 +8678,7 @@
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
     </row>
-    <row r="295" spans="1:9" ht="14.65" hidden="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="295" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A295" s="9">
         <f t="shared" si="4"/>
         <v>294</v>
@@ -8698,13 +8697,7 @@
       <c r="I295" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I295" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}">
-    <filterColumn colId="4">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I295" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}"/>
   <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D154:D160 D162:D164 D166:D191 D201:D207 D209:D211 D213:D215 D217:D225 D227:D233 D235:D241 D243:D249 D251:D255 D257:D262 D264:D268 D270 D272:D282 D284:D294 D52:D56 D133:D152">
     <cfRule type="cellIs" dxfId="83" priority="111" operator="equal">
       <formula>"Fail"</formula>

</xml_diff>

<commit_message>
Docs: Update FractalRegistry.xlsx architecture documentation
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{964255C4-2A3A-4CBA-82CF-781B4F7038ED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA39C264-9DB7-400E-8D44-5A30DE0315A2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,15 +16,15 @@
     <sheet name="FractalRegistry" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$I$295</definedName>
-    <definedName name="Data">FractalRegistry!$A$1:$I$295</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$I$296</definedName>
+    <definedName name="Data">FractalRegistry!$A$1:$I$296</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="761" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="352">
   <si>
     <t>Group Name</t>
   </si>
@@ -1071,6 +1071,15 @@
   </si>
   <si>
     <t>boring black pentagon - still boring</t>
+  </si>
+  <si>
+    <t>double mandelbrot</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>black screen, no structure</t>
   </si>
 </sst>
 </file>
@@ -1216,7 +1225,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1414,6 +1423,9 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="lightUp"/>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -1604,7 +1616,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1673,6 +1685,13 @@
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2617,17 +2636,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I295"/>
+  <dimension ref="A1:I296"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.3984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="20.3984375" customWidth="1"/>
-    <col min="3" max="3" width="22.1328125" customWidth="1"/>
+    <col min="2" max="2" width="14.06640625" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" customWidth="1"/>
     <col min="4" max="4" width="6.46484375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="40.53125" customWidth="1"/>
+    <col min="5" max="5" width="19.46484375" customWidth="1"/>
     <col min="6" max="6" width="6.3984375" customWidth="1"/>
     <col min="7" max="7" width="6.46484375" customWidth="1"/>
-    <col min="8" max="8" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.53125" customWidth="1"/>
     <col min="9" max="9" width="17.265625" customWidth="1"/>
     <col min="10" max="10" width="2.3984375" customWidth="1"/>
   </cols>
@@ -5799,7 +5818,7 @@
     </row>
     <row r="132" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A132" s="9">
-        <f t="shared" ref="A132:A204" si="2">A131+1</f>
+        <f t="shared" ref="A132:A205" si="2">A131+1</f>
         <v>131</v>
       </c>
       <c r="B132" s="6" t="s">
@@ -6391,47 +6410,62 @@
       </c>
     </row>
     <row r="154" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A154" s="2">
-        <f t="shared" si="2"/>
-        <v>153</v>
-      </c>
-      <c r="B154" t="s">
-        <v>167</v>
-      </c>
-      <c r="C154" t="s">
-        <v>168</v>
-      </c>
-      <c r="F154" s="3"/>
-      <c r="G154" s="3"/>
-      <c r="H154" s="4"/>
-      <c r="I154" s="4"/>
+      <c r="A154" s="9"/>
+      <c r="B154" s="30"/>
+      <c r="C154" s="30"/>
+      <c r="D154" s="31"/>
+      <c r="E154" s="30"/>
+      <c r="F154" s="32"/>
+      <c r="G154" s="32"/>
+      <c r="H154" s="33"/>
+      <c r="I154" s="33"/>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A155" s="2">
-        <f t="shared" si="2"/>
-        <v>154</v>
+        <f>A153+1</f>
+        <v>153</v>
       </c>
       <c r="B155" t="s">
         <v>167</v>
       </c>
       <c r="C155" t="s">
-        <v>169</v>
-      </c>
-      <c r="F155" s="3"/>
-      <c r="G155" s="3"/>
-      <c r="H155" s="4"/>
-      <c r="I155" s="4"/>
+        <v>168</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E155" t="s">
+        <v>349</v>
+      </c>
+      <c r="F155" s="3">
+        <v>0.99843749999999898</v>
+      </c>
+      <c r="G155" s="3">
+        <v>-1.40625E-2</v>
+      </c>
+      <c r="H155" s="4">
+        <v>6</v>
+      </c>
+      <c r="I155" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A156" s="2">
         <f t="shared" si="2"/>
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B156" t="s">
         <v>167</v>
       </c>
       <c r="C156" t="s">
-        <v>170</v>
+        <v>169</v>
+      </c>
+      <c r="D156" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E156" t="s">
+        <v>351</v>
       </c>
       <c r="F156" s="3"/>
       <c r="G156" s="3"/>
@@ -6441,13 +6475,19 @@
     <row r="157" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A157" s="2">
         <f t="shared" si="2"/>
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B157" t="s">
         <v>167</v>
       </c>
       <c r="C157" t="s">
-        <v>171</v>
+        <v>170</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E157" s="34" t="s">
+        <v>351</v>
       </c>
       <c r="F157" s="3"/>
       <c r="G157" s="3"/>
@@ -6457,13 +6497,19 @@
     <row r="158" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A158" s="2">
         <f t="shared" si="2"/>
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B158" t="s">
         <v>167</v>
       </c>
       <c r="C158" t="s">
-        <v>172</v>
+        <v>171</v>
+      </c>
+      <c r="D158" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E158" t="s">
+        <v>351</v>
       </c>
       <c r="F158" s="3"/>
       <c r="G158" s="3"/>
@@ -6473,13 +6519,19 @@
     <row r="159" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A159" s="2">
         <f t="shared" si="2"/>
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B159" t="s">
         <v>167</v>
       </c>
       <c r="C159" t="s">
-        <v>173</v>
+        <v>172</v>
+      </c>
+      <c r="D159" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E159" t="s">
+        <v>351</v>
       </c>
       <c r="F159" s="3"/>
       <c r="G159" s="3"/>
@@ -6489,257 +6541,404 @@
     <row r="160" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A160" s="2">
         <f t="shared" si="2"/>
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B160" t="s">
         <v>167</v>
       </c>
       <c r="C160" t="s">
-        <v>174</v>
+        <v>173</v>
+      </c>
+      <c r="D160" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E160" t="s">
+        <v>351</v>
       </c>
       <c r="F160" s="3"/>
       <c r="G160" s="3"/>
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
     </row>
-    <row r="161" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A161" s="9">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A161" s="2">
+        <f t="shared" si="2"/>
+        <v>159</v>
+      </c>
+      <c r="B161" t="s">
+        <v>167</v>
+      </c>
+      <c r="C161" t="s">
+        <v>174</v>
+      </c>
+      <c r="D161" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E161" t="s">
+        <v>351</v>
+      </c>
+      <c r="F161" s="3"/>
+      <c r="G161" s="3"/>
+      <c r="H161" s="4"/>
+      <c r="I161" s="4"/>
+    </row>
+    <row r="162" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A162" s="9">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-      <c r="B161" s="6" t="s">
+      <c r="B162" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="C161" s="6" t="s">
+      <c r="C162" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D161" s="5"/>
-      <c r="E161" s="6"/>
-      <c r="F161" s="7"/>
-      <c r="G161" s="7"/>
-      <c r="H161" s="8"/>
-      <c r="I161" s="8"/>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A162" s="2">
-        <f t="shared" si="2"/>
-        <v>161</v>
-      </c>
-      <c r="B162" t="s">
-        <v>176</v>
-      </c>
-      <c r="C162" t="s">
-        <v>177</v>
-      </c>
-      <c r="F162" s="3"/>
-      <c r="G162" s="3"/>
-      <c r="H162" s="4"/>
-      <c r="I162" s="4"/>
+      <c r="D162" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="E162" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="F162" s="7"/>
+      <c r="G162" s="7"/>
+      <c r="H162" s="8"/>
+      <c r="I162" s="8"/>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A163" s="2">
         <f t="shared" si="2"/>
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B163" t="s">
         <v>176</v>
       </c>
       <c r="C163" t="s">
-        <v>178</v>
-      </c>
-      <c r="F163" s="3"/>
-      <c r="G163" s="3"/>
-      <c r="H163" s="4"/>
-      <c r="I163" s="4"/>
+        <v>177</v>
+      </c>
+      <c r="D163" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F163" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G163" s="3">
+        <v>0</v>
+      </c>
+      <c r="H163" s="4">
+        <v>11.708916568099999</v>
+      </c>
+      <c r="I163" s="4">
+        <v>6.586265569</v>
+      </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A164" s="2">
         <f t="shared" si="2"/>
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B164" t="s">
         <v>176</v>
       </c>
       <c r="C164" t="s">
+        <v>178</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F164" s="3">
+        <v>1.0506908049146E-3</v>
+      </c>
+      <c r="G164" s="3">
+        <v>6.1209568601377003E-2</v>
+      </c>
+      <c r="H164" s="4">
+        <v>15.913224864</v>
+      </c>
+      <c r="I164" s="4">
+        <v>8.9511889862</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A165" s="2">
+        <f t="shared" si="2"/>
+        <v>163</v>
+      </c>
+      <c r="B165" t="s">
+        <v>176</v>
+      </c>
+      <c r="C165" t="s">
         <v>179</v>
       </c>
-      <c r="F164" s="3"/>
-      <c r="G164" s="3"/>
-      <c r="H164" s="4"/>
-      <c r="I164" s="4"/>
-    </row>
-    <row r="165" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A165" s="9">
+      <c r="D165" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F165" s="3">
+        <v>-0.63635085849499495</v>
+      </c>
+      <c r="G165" s="3">
+        <v>0.100125156445557</v>
+      </c>
+      <c r="H165" s="4">
+        <v>20.325406911000002</v>
+      </c>
+      <c r="I165" s="4">
+        <v>5.5349445396999999E-2</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A166" s="9">
         <f t="shared" si="2"/>
         <v>164</v>
       </c>
-      <c r="B165" s="6" t="s">
+      <c r="B166" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C165" s="6" t="s">
+      <c r="C166" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D165" s="5"/>
-      <c r="E165" s="6"/>
-      <c r="F165" s="7"/>
-      <c r="G165" s="7"/>
-      <c r="H165" s="8"/>
-      <c r="I165" s="8"/>
-    </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A166" s="2">
+      <c r="D166" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="E166" s="6"/>
+      <c r="F166" s="7">
+        <v>-2.05467938553257</v>
+      </c>
+      <c r="G166" s="7">
+        <v>-0.387706856852924</v>
+      </c>
+      <c r="H166" s="8">
+        <v>1.9784731066000001</v>
+      </c>
+      <c r="I166" s="8">
+        <v>5.6862031442999998E-2</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A167" s="2">
         <f t="shared" si="2"/>
         <v>165</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B167" t="s">
         <v>181</v>
       </c>
-      <c r="C166" t="s">
+      <c r="C167" t="s">
         <v>182</v>
       </c>
-      <c r="F166" s="3"/>
-      <c r="G166" s="3"/>
-      <c r="H166" s="4"/>
-      <c r="I166" s="4"/>
-    </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A167" s="25">
+      <c r="D167" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F167" s="3">
+        <v>-0.5</v>
+      </c>
+      <c r="G167" s="3">
+        <v>-0.5</v>
+      </c>
+      <c r="H167" s="4">
+        <v>2.109375</v>
+      </c>
+      <c r="I167" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A168" s="25">
         <f t="shared" si="2"/>
         <v>166</v>
       </c>
-      <c r="B167" t="s">
-        <v>181</v>
-      </c>
-      <c r="C167" t="s">
-        <v>337</v>
-      </c>
-      <c r="F167" s="3"/>
-      <c r="G167" s="3"/>
-      <c r="H167" s="4"/>
-      <c r="I167" s="4"/>
-    </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A168" s="2">
-        <f t="shared" si="2"/>
-        <v>167</v>
-      </c>
       <c r="B168" t="s">
         <v>181</v>
       </c>
       <c r="C168" t="s">
-        <v>183</v>
-      </c>
-      <c r="F168" s="3"/>
-      <c r="G168" s="3"/>
-      <c r="H168" s="4"/>
-      <c r="I168" s="4"/>
+        <v>337</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F168" s="3">
+        <v>-0.28988974570550302</v>
+      </c>
+      <c r="G168" s="3">
+        <v>-0.561744537960148</v>
+      </c>
+      <c r="H168" s="4">
+        <v>2.3864853865</v>
+      </c>
+      <c r="I168" s="4">
+        <v>0.35355339059000002</v>
+      </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A169" s="2">
         <f t="shared" si="2"/>
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B169" t="s">
         <v>181</v>
       </c>
       <c r="C169" t="s">
-        <v>184</v>
-      </c>
-      <c r="F169" s="3"/>
-      <c r="G169" s="3"/>
-      <c r="H169" s="4"/>
-      <c r="I169" s="4"/>
+        <v>183</v>
+      </c>
+      <c r="D169" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F169" s="3">
+        <v>-0.54094642857142805</v>
+      </c>
+      <c r="G169" s="3">
+        <v>4.0113707983192998E-2</v>
+      </c>
+      <c r="H169" s="4">
+        <v>3.6257142857</v>
+      </c>
+      <c r="I169" s="4">
+        <v>0.31028368794</v>
+      </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A170" s="2">
         <f t="shared" si="2"/>
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B170" t="s">
         <v>181</v>
       </c>
       <c r="C170" t="s">
-        <v>185</v>
-      </c>
-      <c r="F170" s="3"/>
-      <c r="G170" s="3"/>
-      <c r="H170" s="4"/>
-      <c r="I170" s="4"/>
+        <v>184</v>
+      </c>
+      <c r="D170" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F170" s="3">
+        <v>-0.45390625000000001</v>
+      </c>
+      <c r="G170" s="3">
+        <v>-3.90624999999999E-3</v>
+      </c>
+      <c r="H170" s="4">
+        <v>2</v>
+      </c>
+      <c r="I170" s="4">
+        <v>1.125</v>
+      </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A171" s="2">
         <f t="shared" si="2"/>
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B171" t="s">
         <v>181</v>
       </c>
       <c r="C171" t="s">
-        <v>186</v>
-      </c>
-      <c r="F171" s="3"/>
-      <c r="G171" s="3"/>
-      <c r="H171" s="4"/>
-      <c r="I171" s="4"/>
+        <v>185</v>
+      </c>
+      <c r="D171" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F171" s="3">
+        <v>0</v>
+      </c>
+      <c r="G171" s="3">
+        <v>0</v>
+      </c>
+      <c r="H171" s="4">
+        <v>4.9481546653999997</v>
+      </c>
+      <c r="I171" s="4">
+        <v>2.7833369992999999</v>
+      </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A172" s="2">
         <f t="shared" si="2"/>
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B172" t="s">
         <v>181</v>
       </c>
       <c r="C172" t="s">
-        <v>187</v>
-      </c>
-      <c r="F172" s="3"/>
-      <c r="G172" s="3"/>
-      <c r="H172" s="4"/>
-      <c r="I172" s="4"/>
+        <v>186</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F172" s="3">
+        <v>0</v>
+      </c>
+      <c r="G172" s="3">
+        <v>0</v>
+      </c>
+      <c r="H172" s="4">
+        <v>7.9170474646000004</v>
+      </c>
+      <c r="I172" s="4">
+        <v>4.4533391989000002</v>
+      </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A173" s="2">
         <f t="shared" si="2"/>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B173" t="s">
         <v>181</v>
       </c>
       <c r="C173" t="s">
-        <v>188</v>
-      </c>
-      <c r="F173" s="3"/>
-      <c r="G173" s="3"/>
-      <c r="H173" s="4"/>
-      <c r="I173" s="4"/>
+        <v>187</v>
+      </c>
+      <c r="D173" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F173" s="3">
+        <v>0</v>
+      </c>
+      <c r="G173" s="3">
+        <v>0</v>
+      </c>
+      <c r="H173" s="4">
+        <v>6</v>
+      </c>
+      <c r="I173" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A174" s="2">
         <f t="shared" si="2"/>
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B174" t="s">
         <v>181</v>
       </c>
       <c r="C174" t="s">
-        <v>189</v>
-      </c>
-      <c r="F174" s="3"/>
-      <c r="G174" s="3"/>
-      <c r="H174" s="4"/>
-      <c r="I174" s="4"/>
+        <v>188</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F174" s="3">
+        <v>0</v>
+      </c>
+      <c r="G174" s="3">
+        <v>0</v>
+      </c>
+      <c r="H174" s="4">
+        <v>4.0191504844999999</v>
+      </c>
+      <c r="I174" s="4">
+        <v>2.2607721475</v>
+      </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A175" s="2">
         <f t="shared" si="2"/>
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B175" t="s">
         <v>181</v>
       </c>
       <c r="C175" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F175" s="3"/>
       <c r="G175" s="3"/>
@@ -6749,13 +6948,13 @@
     <row r="176" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A176" s="2">
         <f t="shared" si="2"/>
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B176" t="s">
         <v>181</v>
       </c>
       <c r="C176" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F176" s="3"/>
       <c r="G176" s="3"/>
@@ -6765,13 +6964,13 @@
     <row r="177" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A177" s="2">
         <f t="shared" si="2"/>
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B177" t="s">
         <v>181</v>
       </c>
       <c r="C177" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F177" s="3"/>
       <c r="G177" s="3"/>
@@ -6781,13 +6980,13 @@
     <row r="178" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A178" s="2">
         <f t="shared" si="2"/>
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B178" t="s">
         <v>181</v>
       </c>
       <c r="C178" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F178" s="3"/>
       <c r="G178" s="3"/>
@@ -6797,13 +6996,13 @@
     <row r="179" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A179" s="2">
         <f t="shared" si="2"/>
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B179" t="s">
         <v>181</v>
       </c>
       <c r="C179" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F179" s="3"/>
       <c r="G179" s="3"/>
@@ -6813,13 +7012,13 @@
     <row r="180" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A180" s="2">
         <f t="shared" si="2"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B180" t="s">
         <v>181</v>
       </c>
       <c r="C180" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F180" s="3"/>
       <c r="G180" s="3"/>
@@ -6829,13 +7028,13 @@
     <row r="181" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A181" s="2">
         <f t="shared" si="2"/>
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B181" t="s">
         <v>181</v>
       </c>
       <c r="C181" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F181" s="3"/>
       <c r="G181" s="3"/>
@@ -6845,13 +7044,13 @@
     <row r="182" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A182" s="2">
         <f t="shared" si="2"/>
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B182" t="s">
         <v>181</v>
       </c>
       <c r="C182" t="s">
-        <v>319</v>
+        <v>196</v>
       </c>
       <c r="F182" s="3"/>
       <c r="G182" s="3"/>
@@ -6861,13 +7060,13 @@
     <row r="183" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A183" s="2">
         <f t="shared" si="2"/>
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B183" t="s">
         <v>181</v>
       </c>
       <c r="C183" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F183" s="3"/>
       <c r="G183" s="3"/>
@@ -6877,13 +7076,13 @@
     <row r="184" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A184" s="2">
         <f t="shared" si="2"/>
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B184" t="s">
         <v>181</v>
       </c>
       <c r="C184" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F184" s="3"/>
       <c r="G184" s="3"/>
@@ -6893,13 +7092,13 @@
     <row r="185" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A185" s="2">
         <f t="shared" si="2"/>
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B185" t="s">
         <v>181</v>
       </c>
       <c r="C185" t="s">
-        <v>197</v>
+        <v>321</v>
       </c>
       <c r="F185" s="3"/>
       <c r="G185" s="3"/>
@@ -6909,13 +7108,13 @@
     <row r="186" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A186" s="2">
         <f t="shared" si="2"/>
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B186" t="s">
         <v>181</v>
       </c>
       <c r="C186" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F186" s="3"/>
       <c r="G186" s="3"/>
@@ -6925,13 +7124,13 @@
     <row r="187" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A187" s="2">
         <f t="shared" si="2"/>
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B187" t="s">
         <v>181</v>
       </c>
       <c r="C187" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F187" s="3"/>
       <c r="G187" s="3"/>
@@ -6941,13 +7140,13 @@
     <row r="188" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A188" s="2">
         <f t="shared" si="2"/>
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B188" t="s">
         <v>181</v>
       </c>
       <c r="C188" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F188" s="3"/>
       <c r="G188" s="3"/>
@@ -6957,13 +7156,13 @@
     <row r="189" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A189" s="2">
         <f t="shared" si="2"/>
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B189" t="s">
         <v>181</v>
       </c>
       <c r="C189" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F189" s="3"/>
       <c r="G189" s="3"/>
@@ -6973,13 +7172,13 @@
     <row r="190" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A190" s="2">
         <f t="shared" si="2"/>
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B190" t="s">
         <v>181</v>
       </c>
       <c r="C190" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F190" s="3"/>
       <c r="G190" s="3"/>
@@ -6989,63 +7188,63 @@
     <row r="191" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A191" s="2">
         <f t="shared" si="2"/>
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B191" t="s">
         <v>181</v>
       </c>
       <c r="C191" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F191" s="3"/>
       <c r="G191" s="3"/>
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
     </row>
-    <row r="192" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A192" s="9">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A192" s="2">
+        <f t="shared" si="2"/>
+        <v>190</v>
+      </c>
+      <c r="B192" t="s">
+        <v>181</v>
+      </c>
+      <c r="C192" t="s">
+        <v>203</v>
+      </c>
+      <c r="F192" s="3"/>
+      <c r="G192" s="3"/>
+      <c r="H192" s="4"/>
+      <c r="I192" s="4"/>
+    </row>
+    <row r="193" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A193" s="9">
         <f t="shared" si="2"/>
         <v>191</v>
       </c>
-      <c r="B192" s="6" t="s">
+      <c r="B193" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="C192" s="6" t="s">
+      <c r="C193" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D192" s="5"/>
-      <c r="E192" s="6"/>
-      <c r="F192" s="7"/>
-      <c r="G192" s="7"/>
-      <c r="H192" s="8"/>
-      <c r="I192" s="8"/>
-    </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A193" s="9">
-        <f t="shared" si="2"/>
-        <v>192</v>
-      </c>
-      <c r="B193" t="s">
-        <v>314</v>
-      </c>
-      <c r="C193" t="s">
-        <v>245</v>
-      </c>
-      <c r="F193" s="3"/>
-      <c r="G193" s="3"/>
-      <c r="H193" s="4"/>
-      <c r="I193" s="4"/>
+      <c r="D193" s="5"/>
+      <c r="E193" s="6"/>
+      <c r="F193" s="7"/>
+      <c r="G193" s="7"/>
+      <c r="H193" s="8"/>
+      <c r="I193" s="8"/>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A194" s="9">
         <f t="shared" si="2"/>
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B194" t="s">
         <v>314</v>
       </c>
       <c r="C194" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F194" s="3"/>
       <c r="G194" s="3"/>
@@ -7055,13 +7254,13 @@
     <row r="195" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A195" s="9">
         <f t="shared" si="2"/>
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B195" t="s">
         <v>314</v>
       </c>
       <c r="C195" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F195" s="3"/>
       <c r="G195" s="3"/>
@@ -7071,13 +7270,13 @@
     <row r="196" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A196" s="9">
         <f t="shared" si="2"/>
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B196" t="s">
         <v>314</v>
       </c>
       <c r="C196" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F196" s="3"/>
       <c r="G196" s="3"/>
@@ -7087,13 +7286,13 @@
     <row r="197" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A197" s="9">
         <f t="shared" si="2"/>
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B197" t="s">
         <v>314</v>
       </c>
       <c r="C197" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F197" s="3"/>
       <c r="G197" s="3"/>
@@ -7103,13 +7302,13 @@
     <row r="198" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A198" s="9">
         <f t="shared" si="2"/>
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B198" t="s">
         <v>314</v>
       </c>
       <c r="C198" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F198" s="3"/>
       <c r="G198" s="3"/>
@@ -7119,63 +7318,63 @@
     <row r="199" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A199" s="9">
         <f t="shared" si="2"/>
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B199" t="s">
         <v>314</v>
       </c>
       <c r="C199" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F199" s="3"/>
       <c r="G199" s="3"/>
       <c r="H199" s="4"/>
       <c r="I199" s="4"/>
     </row>
-    <row r="200" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A200" s="9">
         <f t="shared" si="2"/>
-        <v>199</v>
-      </c>
-      <c r="B200" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="B200" t="s">
         <v>314</v>
       </c>
-      <c r="C200" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="D200" s="5"/>
-      <c r="E200" s="6"/>
-      <c r="F200" s="7"/>
-      <c r="G200" s="7"/>
-      <c r="H200" s="8"/>
-      <c r="I200" s="8"/>
-    </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="C200" t="s">
+        <v>251</v>
+      </c>
+      <c r="F200" s="3"/>
+      <c r="G200" s="3"/>
+      <c r="H200" s="4"/>
+      <c r="I200" s="4"/>
+    </row>
+    <row r="201" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A201" s="9">
         <f t="shared" si="2"/>
-        <v>200</v>
-      </c>
-      <c r="B201" t="s">
-        <v>205</v>
-      </c>
-      <c r="C201" t="s">
-        <v>324</v>
-      </c>
-      <c r="F201" s="3"/>
-      <c r="G201" s="3"/>
-      <c r="H201" s="4"/>
-      <c r="I201" s="4"/>
+        <v>199</v>
+      </c>
+      <c r="B201" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="C201" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="D201" s="5"/>
+      <c r="E201" s="6"/>
+      <c r="F201" s="7"/>
+      <c r="G201" s="7"/>
+      <c r="H201" s="8"/>
+      <c r="I201" s="8"/>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A202" s="9">
         <f t="shared" si="2"/>
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B202" t="s">
         <v>205</v>
       </c>
       <c r="C202" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F202" s="3"/>
       <c r="G202" s="3"/>
@@ -7183,15 +7382,15 @@
       <c r="I202" s="4"/>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A203" s="2">
+      <c r="A203" s="9">
         <f t="shared" si="2"/>
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B203" t="s">
         <v>205</v>
       </c>
       <c r="C203" t="s">
-        <v>206</v>
+        <v>325</v>
       </c>
       <c r="F203" s="3"/>
       <c r="G203" s="3"/>
@@ -7201,13 +7400,13 @@
     <row r="204" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A204" s="2">
         <f t="shared" si="2"/>
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B204" t="s">
         <v>205</v>
       </c>
       <c r="C204" t="s">
-        <v>326</v>
+        <v>206</v>
       </c>
       <c r="F204" s="3"/>
       <c r="G204" s="3"/>
@@ -7216,14 +7415,14 @@
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A205" s="2">
-        <f t="shared" ref="A205:A264" si="3">A204+1</f>
-        <v>204</v>
+        <f t="shared" si="2"/>
+        <v>203</v>
       </c>
       <c r="B205" t="s">
         <v>205</v>
       </c>
       <c r="C205" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F205" s="3"/>
       <c r="G205" s="3"/>
@@ -7232,14 +7431,14 @@
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A206" s="2">
-        <f t="shared" si="3"/>
-        <v>205</v>
+        <f t="shared" ref="A206:A265" si="3">A205+1</f>
+        <v>204</v>
       </c>
       <c r="B206" t="s">
         <v>205</v>
       </c>
       <c r="C206" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="F206" s="3"/>
       <c r="G206" s="3"/>
@@ -7249,63 +7448,63 @@
     <row r="207" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A207" s="2">
         <f t="shared" si="3"/>
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B207" t="s">
         <v>205</v>
       </c>
       <c r="C207" t="s">
-        <v>207</v>
+        <v>328</v>
       </c>
       <c r="F207" s="3"/>
       <c r="G207" s="3"/>
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
     </row>
-    <row r="208" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A208" s="9">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A208" s="2">
+        <f t="shared" si="3"/>
+        <v>206</v>
+      </c>
+      <c r="B208" t="s">
+        <v>205</v>
+      </c>
+      <c r="C208" t="s">
+        <v>207</v>
+      </c>
+      <c r="F208" s="3"/>
+      <c r="G208" s="3"/>
+      <c r="H208" s="4"/>
+      <c r="I208" s="4"/>
+    </row>
+    <row r="209" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A209" s="9">
         <f t="shared" si="3"/>
         <v>207</v>
       </c>
-      <c r="B208" s="6" t="s">
+      <c r="B209" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="C208" s="6" t="s">
+      <c r="C209" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="D208" s="5"/>
-      <c r="E208" s="6"/>
-      <c r="F208" s="7"/>
-      <c r="G208" s="7"/>
-      <c r="H208" s="8"/>
-      <c r="I208" s="8"/>
-    </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A209" s="2">
-        <f t="shared" si="3"/>
-        <v>208</v>
-      </c>
-      <c r="B209" t="s">
-        <v>209</v>
-      </c>
-      <c r="C209" t="s">
-        <v>210</v>
-      </c>
-      <c r="F209" s="3"/>
-      <c r="G209" s="3"/>
-      <c r="H209" s="4"/>
-      <c r="I209" s="4"/>
+      <c r="D209" s="5"/>
+      <c r="E209" s="6"/>
+      <c r="F209" s="7"/>
+      <c r="G209" s="7"/>
+      <c r="H209" s="8"/>
+      <c r="I209" s="8"/>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A210" s="2">
         <f t="shared" si="3"/>
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B210" t="s">
         <v>209</v>
       </c>
       <c r="C210" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F210" s="3"/>
       <c r="G210" s="3"/>
@@ -7315,63 +7514,63 @@
     <row r="211" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A211" s="2">
         <f t="shared" si="3"/>
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B211" t="s">
         <v>209</v>
       </c>
       <c r="C211" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F211" s="3"/>
       <c r="G211" s="3"/>
       <c r="H211" s="4"/>
       <c r="I211" s="4"/>
     </row>
-    <row r="212" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A212" s="9">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A212" s="2">
+        <f t="shared" si="3"/>
+        <v>210</v>
+      </c>
+      <c r="B212" t="s">
+        <v>209</v>
+      </c>
+      <c r="C212" t="s">
+        <v>212</v>
+      </c>
+      <c r="F212" s="3"/>
+      <c r="G212" s="3"/>
+      <c r="H212" s="4"/>
+      <c r="I212" s="4"/>
+    </row>
+    <row r="213" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A213" s="9">
         <f t="shared" si="3"/>
         <v>211</v>
       </c>
-      <c r="B212" s="6" t="s">
+      <c r="B213" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="C212" s="6" t="s">
+      <c r="C213" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="D212" s="5"/>
-      <c r="E212" s="6"/>
-      <c r="F212" s="7"/>
-      <c r="G212" s="7"/>
-      <c r="H212" s="8"/>
-      <c r="I212" s="8"/>
-    </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A213" s="2">
-        <f t="shared" si="3"/>
-        <v>212</v>
-      </c>
-      <c r="B213" t="s">
-        <v>214</v>
-      </c>
-      <c r="C213" t="s">
-        <v>215</v>
-      </c>
-      <c r="F213" s="3"/>
-      <c r="G213" s="3"/>
-      <c r="H213" s="4"/>
-      <c r="I213" s="4"/>
+      <c r="D213" s="5"/>
+      <c r="E213" s="6"/>
+      <c r="F213" s="7"/>
+      <c r="G213" s="7"/>
+      <c r="H213" s="8"/>
+      <c r="I213" s="8"/>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A214" s="2">
         <f t="shared" si="3"/>
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B214" t="s">
         <v>214</v>
       </c>
       <c r="C214" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F214" s="3"/>
       <c r="G214" s="3"/>
@@ -7381,63 +7580,63 @@
     <row r="215" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A215" s="2">
         <f t="shared" si="3"/>
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B215" t="s">
         <v>214</v>
       </c>
       <c r="C215" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F215" s="3"/>
       <c r="G215" s="3"/>
       <c r="H215" s="4"/>
       <c r="I215" s="4"/>
     </row>
-    <row r="216" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A216" s="9">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A216" s="2">
+        <f t="shared" si="3"/>
+        <v>214</v>
+      </c>
+      <c r="B216" t="s">
+        <v>214</v>
+      </c>
+      <c r="C216" t="s">
+        <v>217</v>
+      </c>
+      <c r="F216" s="3"/>
+      <c r="G216" s="3"/>
+      <c r="H216" s="4"/>
+      <c r="I216" s="4"/>
+    </row>
+    <row r="217" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A217" s="9">
         <f t="shared" si="3"/>
         <v>215</v>
       </c>
-      <c r="B216" s="6" t="s">
+      <c r="B217" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="C216" s="6" t="s">
+      <c r="C217" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="D216" s="5"/>
-      <c r="E216" s="6"/>
-      <c r="F216" s="7"/>
-      <c r="G216" s="7"/>
-      <c r="H216" s="8"/>
-      <c r="I216" s="8"/>
-    </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A217" s="2">
-        <f t="shared" si="3"/>
-        <v>216</v>
-      </c>
-      <c r="B217" t="s">
-        <v>219</v>
-      </c>
-      <c r="C217" t="s">
-        <v>220</v>
-      </c>
-      <c r="F217" s="3"/>
-      <c r="G217" s="3"/>
-      <c r="H217" s="4"/>
-      <c r="I217" s="4"/>
+      <c r="D217" s="5"/>
+      <c r="E217" s="6"/>
+      <c r="F217" s="7"/>
+      <c r="G217" s="7"/>
+      <c r="H217" s="8"/>
+      <c r="I217" s="8"/>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A218" s="2">
         <f t="shared" si="3"/>
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B218" t="s">
         <v>219</v>
       </c>
       <c r="C218" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F218" s="3"/>
       <c r="G218" s="3"/>
@@ -7447,13 +7646,13 @@
     <row r="219" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A219" s="2">
         <f t="shared" si="3"/>
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B219" t="s">
         <v>219</v>
       </c>
       <c r="C219" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F219" s="3"/>
       <c r="G219" s="3"/>
@@ -7463,13 +7662,13 @@
     <row r="220" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A220" s="2">
         <f t="shared" si="3"/>
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B220" t="s">
         <v>219</v>
       </c>
       <c r="C220" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F220" s="3"/>
       <c r="G220" s="3"/>
@@ -7479,13 +7678,13 @@
     <row r="221" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A221" s="2">
         <f t="shared" si="3"/>
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B221" t="s">
         <v>219</v>
       </c>
       <c r="C221" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F221" s="3"/>
       <c r="G221" s="3"/>
@@ -7495,13 +7694,13 @@
     <row r="222" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A222" s="2">
         <f t="shared" si="3"/>
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B222" t="s">
         <v>219</v>
       </c>
       <c r="C222" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F222" s="3"/>
       <c r="G222" s="3"/>
@@ -7511,13 +7710,13 @@
     <row r="223" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A223" s="2">
         <f t="shared" si="3"/>
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B223" t="s">
         <v>219</v>
       </c>
       <c r="C223" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F223" s="3"/>
       <c r="G223" s="3"/>
@@ -7527,13 +7726,13 @@
     <row r="224" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A224" s="2">
         <f t="shared" si="3"/>
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B224" t="s">
         <v>219</v>
       </c>
       <c r="C224" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F224" s="3"/>
       <c r="G224" s="3"/>
@@ -7543,63 +7742,63 @@
     <row r="225" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A225" s="2">
         <f t="shared" si="3"/>
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B225" t="s">
         <v>219</v>
       </c>
       <c r="C225" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F225" s="3"/>
       <c r="G225" s="3"/>
       <c r="H225" s="4"/>
       <c r="I225" s="4"/>
     </row>
-    <row r="226" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A226" s="9">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A226" s="2">
+        <f t="shared" si="3"/>
+        <v>224</v>
+      </c>
+      <c r="B226" t="s">
+        <v>219</v>
+      </c>
+      <c r="C226" t="s">
+        <v>228</v>
+      </c>
+      <c r="F226" s="3"/>
+      <c r="G226" s="3"/>
+      <c r="H226" s="4"/>
+      <c r="I226" s="4"/>
+    </row>
+    <row r="227" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A227" s="9">
         <f t="shared" si="3"/>
         <v>225</v>
       </c>
-      <c r="B226" s="6" t="s">
+      <c r="B227" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="C226" s="6" t="s">
+      <c r="C227" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D226" s="5"/>
-      <c r="E226" s="6"/>
-      <c r="F226" s="7"/>
-      <c r="G226" s="7"/>
-      <c r="H226" s="8"/>
-      <c r="I226" s="8"/>
-    </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A227" s="2">
-        <f t="shared" si="3"/>
-        <v>226</v>
-      </c>
-      <c r="B227" t="s">
-        <v>230</v>
-      </c>
-      <c r="C227" t="s">
-        <v>231</v>
-      </c>
-      <c r="F227" s="3"/>
-      <c r="G227" s="3"/>
-      <c r="H227" s="4"/>
-      <c r="I227" s="4"/>
+      <c r="D227" s="5"/>
+      <c r="E227" s="6"/>
+      <c r="F227" s="7"/>
+      <c r="G227" s="7"/>
+      <c r="H227" s="8"/>
+      <c r="I227" s="8"/>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A228" s="2">
         <f t="shared" si="3"/>
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B228" t="s">
         <v>230</v>
       </c>
       <c r="C228" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F228" s="3"/>
       <c r="G228" s="3"/>
@@ -7609,13 +7808,13 @@
     <row r="229" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A229" s="2">
         <f t="shared" si="3"/>
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B229" t="s">
         <v>230</v>
       </c>
       <c r="C229" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F229" s="3"/>
       <c r="G229" s="3"/>
@@ -7625,13 +7824,13 @@
     <row r="230" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
         <f t="shared" si="3"/>
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B230" t="s">
         <v>230</v>
       </c>
       <c r="C230" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F230" s="3"/>
       <c r="G230" s="3"/>
@@ -7641,13 +7840,13 @@
     <row r="231" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A231" s="2">
         <f t="shared" si="3"/>
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B231" t="s">
         <v>230</v>
       </c>
       <c r="C231" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F231" s="3"/>
       <c r="G231" s="3"/>
@@ -7657,13 +7856,13 @@
     <row r="232" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A232" s="2">
         <f t="shared" si="3"/>
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B232" t="s">
         <v>230</v>
       </c>
       <c r="C232" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F232" s="3"/>
       <c r="G232" s="3"/>
@@ -7673,63 +7872,63 @@
     <row r="233" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A233" s="2">
         <f t="shared" si="3"/>
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B233" t="s">
         <v>230</v>
       </c>
       <c r="C233" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F233" s="3"/>
       <c r="G233" s="3"/>
       <c r="H233" s="4"/>
       <c r="I233" s="4"/>
     </row>
-    <row r="234" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A234" s="9">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A234" s="2">
+        <f t="shared" si="3"/>
+        <v>232</v>
+      </c>
+      <c r="B234" t="s">
+        <v>230</v>
+      </c>
+      <c r="C234" t="s">
+        <v>237</v>
+      </c>
+      <c r="F234" s="3"/>
+      <c r="G234" s="3"/>
+      <c r="H234" s="4"/>
+      <c r="I234" s="4"/>
+    </row>
+    <row r="235" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A235" s="9">
         <f t="shared" si="3"/>
         <v>233</v>
       </c>
-      <c r="B234" s="6" t="s">
+      <c r="B235" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="C234" s="6" t="s">
+      <c r="C235" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="D234" s="5"/>
-      <c r="E234" s="6"/>
-      <c r="F234" s="7"/>
-      <c r="G234" s="7"/>
-      <c r="H234" s="8"/>
-      <c r="I234" s="8"/>
-    </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A235" s="2">
-        <f t="shared" si="3"/>
-        <v>234</v>
-      </c>
-      <c r="B235" t="s">
-        <v>315</v>
-      </c>
-      <c r="C235" t="s">
-        <v>239</v>
-      </c>
-      <c r="F235" s="3"/>
-      <c r="G235" s="3"/>
-      <c r="H235" s="4"/>
-      <c r="I235" s="4"/>
+      <c r="D235" s="5"/>
+      <c r="E235" s="6"/>
+      <c r="F235" s="7"/>
+      <c r="G235" s="7"/>
+      <c r="H235" s="8"/>
+      <c r="I235" s="8"/>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A236" s="2">
         <f t="shared" si="3"/>
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B236" t="s">
         <v>315</v>
       </c>
       <c r="C236" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F236" s="3"/>
       <c r="G236" s="3"/>
@@ -7739,13 +7938,13 @@
     <row r="237" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A237" s="2">
         <f t="shared" si="3"/>
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B237" t="s">
         <v>315</v>
       </c>
       <c r="C237" t="s">
-        <v>322</v>
+        <v>240</v>
       </c>
       <c r="F237" s="3"/>
       <c r="G237" s="3"/>
@@ -7755,13 +7954,13 @@
     <row r="238" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A238" s="2">
         <f t="shared" si="3"/>
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B238" t="s">
         <v>315</v>
       </c>
       <c r="C238" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F238" s="3"/>
       <c r="G238" s="3"/>
@@ -7771,13 +7970,13 @@
     <row r="239" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A239" s="2">
         <f t="shared" si="3"/>
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B239" t="s">
         <v>315</v>
       </c>
       <c r="C239" t="s">
-        <v>241</v>
+        <v>323</v>
       </c>
       <c r="F239" s="3"/>
       <c r="G239" s="3"/>
@@ -7787,13 +7986,13 @@
     <row r="240" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A240" s="2">
         <f t="shared" si="3"/>
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B240" t="s">
         <v>315</v>
       </c>
       <c r="C240" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F240" s="3"/>
       <c r="G240" s="3"/>
@@ -7803,63 +8002,63 @@
     <row r="241" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A241" s="2">
         <f t="shared" si="3"/>
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B241" t="s">
         <v>315</v>
       </c>
       <c r="C241" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F241" s="3"/>
       <c r="G241" s="3"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
     </row>
-    <row r="242" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A242" s="2">
         <f t="shared" si="3"/>
-        <v>241</v>
-      </c>
-      <c r="B242" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="B242" t="s">
         <v>315</v>
       </c>
-      <c r="C242" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="D242" s="5"/>
-      <c r="E242" s="6"/>
-      <c r="F242" s="7"/>
-      <c r="G242" s="7"/>
-      <c r="H242" s="8"/>
-      <c r="I242" s="8"/>
-    </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="C242" t="s">
+        <v>243</v>
+      </c>
+      <c r="F242" s="3"/>
+      <c r="G242" s="3"/>
+      <c r="H242" s="4"/>
+      <c r="I242" s="4"/>
+    </row>
+    <row r="243" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A243" s="2">
         <f t="shared" si="3"/>
-        <v>242</v>
-      </c>
-      <c r="B243" t="s">
-        <v>253</v>
-      </c>
-      <c r="C243" t="s">
-        <v>329</v>
-      </c>
-      <c r="F243" s="3"/>
-      <c r="G243" s="3"/>
-      <c r="H243" s="4"/>
-      <c r="I243" s="4"/>
+        <v>241</v>
+      </c>
+      <c r="B243" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="C243" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="D243" s="5"/>
+      <c r="E243" s="6"/>
+      <c r="F243" s="7"/>
+      <c r="G243" s="7"/>
+      <c r="H243" s="8"/>
+      <c r="I243" s="8"/>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A244" s="2">
         <f t="shared" si="3"/>
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B244" t="s">
         <v>253</v>
       </c>
       <c r="C244" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F244" s="3"/>
       <c r="G244" s="3"/>
@@ -7869,13 +8068,13 @@
     <row r="245" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A245" s="2">
         <f t="shared" si="3"/>
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B245" t="s">
         <v>253</v>
       </c>
       <c r="C245" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F245" s="3"/>
       <c r="G245" s="3"/>
@@ -7885,13 +8084,13 @@
     <row r="246" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A246" s="2">
         <f t="shared" si="3"/>
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B246" t="s">
         <v>253</v>
       </c>
       <c r="C246" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F246" s="3"/>
       <c r="G246" s="3"/>
@@ -7901,13 +8100,13 @@
     <row r="247" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A247" s="2">
         <f t="shared" si="3"/>
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B247" t="s">
         <v>253</v>
       </c>
       <c r="C247" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F247" s="3"/>
       <c r="G247" s="3"/>
@@ -7917,13 +8116,13 @@
     <row r="248" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A248" s="2">
         <f t="shared" si="3"/>
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B248" t="s">
         <v>253</v>
       </c>
       <c r="C248" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="F248" s="3"/>
       <c r="G248" s="3"/>
@@ -7933,63 +8132,63 @@
     <row r="249" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A249" s="2">
         <f t="shared" si="3"/>
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B249" t="s">
         <v>253</v>
       </c>
       <c r="C249" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="F249" s="3"/>
       <c r="G249" s="3"/>
       <c r="H249" s="4"/>
       <c r="I249" s="4"/>
     </row>
-    <row r="250" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A250" s="2">
         <f t="shared" si="3"/>
-        <v>249</v>
-      </c>
-      <c r="B250" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B250" t="s">
         <v>253</v>
       </c>
       <c r="C250" t="s">
-        <v>336</v>
-      </c>
-      <c r="D250" s="5"/>
-      <c r="E250" s="6"/>
-      <c r="F250" s="7"/>
-      <c r="G250" s="7"/>
-      <c r="H250" s="8"/>
-      <c r="I250" s="8"/>
-    </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.45">
+        <v>335</v>
+      </c>
+      <c r="F250" s="3"/>
+      <c r="G250" s="3"/>
+      <c r="H250" s="4"/>
+      <c r="I250" s="4"/>
+    </row>
+    <row r="251" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A251" s="2">
         <f t="shared" si="3"/>
-        <v>250</v>
-      </c>
-      <c r="B251" t="s">
-        <v>254</v>
+        <v>249</v>
+      </c>
+      <c r="B251" s="6" t="s">
+        <v>253</v>
       </c>
       <c r="C251" t="s">
-        <v>255</v>
-      </c>
-      <c r="F251" s="3"/>
-      <c r="G251" s="3"/>
-      <c r="H251" s="4"/>
-      <c r="I251" s="4"/>
+        <v>336</v>
+      </c>
+      <c r="D251" s="5"/>
+      <c r="E251" s="6"/>
+      <c r="F251" s="7"/>
+      <c r="G251" s="7"/>
+      <c r="H251" s="8"/>
+      <c r="I251" s="8"/>
     </row>
     <row r="252" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A252" s="2">
         <f t="shared" si="3"/>
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B252" t="s">
         <v>254</v>
       </c>
       <c r="C252" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F252" s="3"/>
       <c r="G252" s="3"/>
@@ -7999,13 +8198,13 @@
     <row r="253" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A253" s="2">
         <f t="shared" si="3"/>
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B253" t="s">
         <v>254</v>
       </c>
       <c r="C253" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F253" s="3"/>
       <c r="G253" s="3"/>
@@ -8015,13 +8214,13 @@
     <row r="254" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A254" s="2">
         <f t="shared" si="3"/>
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B254" t="s">
         <v>254</v>
       </c>
       <c r="C254" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F254" s="3"/>
       <c r="G254" s="3"/>
@@ -8031,63 +8230,63 @@
     <row r="255" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A255" s="2">
         <f t="shared" si="3"/>
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B255" t="s">
         <v>254</v>
       </c>
       <c r="C255" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F255" s="3"/>
       <c r="G255" s="3"/>
       <c r="H255" s="4"/>
       <c r="I255" s="4"/>
     </row>
-    <row r="256" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A256" s="2">
         <f t="shared" si="3"/>
-        <v>255</v>
-      </c>
-      <c r="B256" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="C256" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="D256" s="5"/>
-      <c r="E256" s="6"/>
-      <c r="F256" s="7"/>
-      <c r="G256" s="7"/>
-      <c r="H256" s="8"/>
-      <c r="I256" s="8"/>
-    </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="B256" t="s">
+        <v>254</v>
+      </c>
+      <c r="C256" t="s">
+        <v>259</v>
+      </c>
+      <c r="F256" s="3"/>
+      <c r="G256" s="3"/>
+      <c r="H256" s="4"/>
+      <c r="I256" s="4"/>
+    </row>
+    <row r="257" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A257" s="2">
         <f t="shared" si="3"/>
-        <v>256</v>
-      </c>
-      <c r="B257" t="s">
-        <v>261</v>
-      </c>
-      <c r="C257" t="s">
-        <v>262</v>
-      </c>
-      <c r="F257" s="3"/>
-      <c r="G257" s="3"/>
-      <c r="H257" s="4"/>
-      <c r="I257" s="4"/>
+        <v>255</v>
+      </c>
+      <c r="B257" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C257" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="D257" s="5"/>
+      <c r="E257" s="6"/>
+      <c r="F257" s="7"/>
+      <c r="G257" s="7"/>
+      <c r="H257" s="8"/>
+      <c r="I257" s="8"/>
     </row>
     <row r="258" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A258" s="2">
         <f t="shared" si="3"/>
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B258" t="s">
         <v>261</v>
       </c>
       <c r="C258" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F258" s="3"/>
       <c r="G258" s="3"/>
@@ -8097,13 +8296,13 @@
     <row r="259" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A259" s="2">
         <f t="shared" si="3"/>
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B259" t="s">
         <v>261</v>
       </c>
       <c r="C259" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F259" s="3"/>
       <c r="G259" s="3"/>
@@ -8113,13 +8312,13 @@
     <row r="260" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A260" s="2">
         <f t="shared" si="3"/>
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B260" t="s">
         <v>261</v>
       </c>
       <c r="C260" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F260" s="3"/>
       <c r="G260" s="3"/>
@@ -8129,13 +8328,13 @@
     <row r="261" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A261" s="2">
         <f t="shared" si="3"/>
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B261" t="s">
         <v>261</v>
       </c>
       <c r="C261" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F261" s="3"/>
       <c r="G261" s="3"/>
@@ -8145,63 +8344,63 @@
     <row r="262" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A262" s="2">
         <f t="shared" si="3"/>
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B262" t="s">
         <v>261</v>
       </c>
       <c r="C262" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F262" s="3"/>
       <c r="G262" s="3"/>
       <c r="H262" s="4"/>
       <c r="I262" s="4"/>
     </row>
-    <row r="263" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A263" s="2">
         <f t="shared" si="3"/>
-        <v>262</v>
-      </c>
-      <c r="B263" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="C263" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="D263" s="5"/>
-      <c r="E263" s="6"/>
-      <c r="F263" s="7"/>
-      <c r="G263" s="7"/>
-      <c r="H263" s="8"/>
-      <c r="I263" s="8"/>
-    </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="B263" t="s">
+        <v>261</v>
+      </c>
+      <c r="C263" t="s">
+        <v>267</v>
+      </c>
+      <c r="F263" s="3"/>
+      <c r="G263" s="3"/>
+      <c r="H263" s="4"/>
+      <c r="I263" s="4"/>
+    </row>
+    <row r="264" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A264" s="2">
         <f t="shared" si="3"/>
-        <v>263</v>
-      </c>
-      <c r="B264" t="s">
-        <v>269</v>
-      </c>
-      <c r="C264" t="s">
-        <v>270</v>
-      </c>
-      <c r="F264" s="3"/>
-      <c r="G264" s="3"/>
-      <c r="H264" s="4"/>
-      <c r="I264" s="4"/>
+        <v>262</v>
+      </c>
+      <c r="B264" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="C264" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D264" s="5"/>
+      <c r="E264" s="6"/>
+      <c r="F264" s="7"/>
+      <c r="G264" s="7"/>
+      <c r="H264" s="8"/>
+      <c r="I264" s="8"/>
     </row>
     <row r="265" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A265" s="2">
-        <f t="shared" ref="A265:A295" si="4">A264+1</f>
-        <v>264</v>
+        <f t="shared" si="3"/>
+        <v>263</v>
       </c>
       <c r="B265" t="s">
         <v>269</v>
       </c>
       <c r="C265" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F265" s="3"/>
       <c r="G265" s="3"/>
@@ -8210,14 +8409,14 @@
     </row>
     <row r="266" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A266" s="2">
-        <f t="shared" si="4"/>
-        <v>265</v>
+        <f t="shared" ref="A266:A296" si="4">A265+1</f>
+        <v>264</v>
       </c>
       <c r="B266" t="s">
         <v>269</v>
       </c>
       <c r="C266" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F266" s="3"/>
       <c r="G266" s="3"/>
@@ -8227,13 +8426,13 @@
     <row r="267" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A267" s="2">
         <f t="shared" si="4"/>
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B267" t="s">
         <v>269</v>
       </c>
       <c r="C267" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F267" s="3"/>
       <c r="G267" s="3"/>
@@ -8243,97 +8442,97 @@
     <row r="268" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A268" s="2">
         <f t="shared" si="4"/>
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B268" t="s">
         <v>269</v>
       </c>
       <c r="C268" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F268" s="3"/>
       <c r="G268" s="3"/>
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
     </row>
-    <row r="269" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A269" s="9">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A269" s="2">
+        <f t="shared" si="4"/>
+        <v>267</v>
+      </c>
+      <c r="B269" t="s">
+        <v>269</v>
+      </c>
+      <c r="C269" t="s">
+        <v>274</v>
+      </c>
+      <c r="F269" s="3"/>
+      <c r="G269" s="3"/>
+      <c r="H269" s="4"/>
+      <c r="I269" s="4"/>
+    </row>
+    <row r="270" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A270" s="9">
         <f t="shared" si="4"/>
         <v>268</v>
       </c>
-      <c r="B269" s="6" t="s">
+      <c r="B270" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="C269" s="6" t="s">
+      <c r="C270" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="D269" s="5"/>
-      <c r="E269" s="6"/>
-      <c r="F269" s="7"/>
-      <c r="G269" s="7"/>
-      <c r="H269" s="8"/>
-      <c r="I269" s="8"/>
-    </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A270" s="2">
+      <c r="D270" s="5"/>
+      <c r="E270" s="6"/>
+      <c r="F270" s="7"/>
+      <c r="G270" s="7"/>
+      <c r="H270" s="8"/>
+      <c r="I270" s="8"/>
+    </row>
+    <row r="271" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A271" s="2">
         <f t="shared" si="4"/>
         <v>269</v>
       </c>
-      <c r="B270" t="s">
+      <c r="B271" t="s">
         <v>276</v>
       </c>
-      <c r="C270" t="s">
+      <c r="C271" t="s">
         <v>277</v>
       </c>
-      <c r="F270" s="3"/>
-      <c r="G270" s="3"/>
-      <c r="H270" s="4"/>
-      <c r="I270" s="4"/>
-    </row>
-    <row r="271" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A271" s="9">
+      <c r="F271" s="3"/>
+      <c r="G271" s="3"/>
+      <c r="H271" s="4"/>
+      <c r="I271" s="4"/>
+    </row>
+    <row r="272" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A272" s="9">
         <f t="shared" si="4"/>
         <v>270</v>
       </c>
-      <c r="B271" s="6" t="s">
+      <c r="B272" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="C271" s="6" t="s">
+      <c r="C272" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="D271" s="5"/>
-      <c r="E271" s="6"/>
-      <c r="F271" s="7"/>
-      <c r="G271" s="7"/>
-      <c r="H271" s="8"/>
-      <c r="I271" s="8"/>
-    </row>
-    <row r="272" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A272" s="2">
-        <f t="shared" si="4"/>
-        <v>271</v>
-      </c>
-      <c r="B272" t="s">
-        <v>279</v>
-      </c>
-      <c r="C272" t="s">
-        <v>280</v>
-      </c>
-      <c r="F272" s="3"/>
-      <c r="G272" s="3"/>
-      <c r="H272" s="4"/>
-      <c r="I272" s="4"/>
+      <c r="D272" s="5"/>
+      <c r="E272" s="6"/>
+      <c r="F272" s="7"/>
+      <c r="G272" s="7"/>
+      <c r="H272" s="8"/>
+      <c r="I272" s="8"/>
     </row>
     <row r="273" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A273" s="2">
         <f t="shared" si="4"/>
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B273" t="s">
         <v>279</v>
       </c>
       <c r="C273" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F273" s="3"/>
       <c r="G273" s="3"/>
@@ -8343,13 +8542,13 @@
     <row r="274" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A274" s="2">
         <f t="shared" si="4"/>
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B274" t="s">
         <v>279</v>
       </c>
       <c r="C274" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F274" s="3"/>
       <c r="G274" s="3"/>
@@ -8359,13 +8558,13 @@
     <row r="275" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A275" s="2">
         <f t="shared" si="4"/>
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B275" t="s">
         <v>279</v>
       </c>
       <c r="C275" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F275" s="3"/>
       <c r="G275" s="3"/>
@@ -8375,13 +8574,13 @@
     <row r="276" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A276" s="2">
         <f t="shared" si="4"/>
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B276" t="s">
         <v>279</v>
       </c>
       <c r="C276" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F276" s="3"/>
       <c r="G276" s="3"/>
@@ -8391,13 +8590,13 @@
     <row r="277" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A277" s="2">
         <f t="shared" si="4"/>
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B277" t="s">
         <v>279</v>
       </c>
       <c r="C277" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F277" s="3"/>
       <c r="G277" s="3"/>
@@ -8407,13 +8606,13 @@
     <row r="278" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A278" s="2">
         <f t="shared" si="4"/>
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B278" t="s">
         <v>279</v>
       </c>
       <c r="C278" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F278" s="3"/>
       <c r="G278" s="3"/>
@@ -8423,13 +8622,13 @@
     <row r="279" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A279" s="2">
         <f t="shared" si="4"/>
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B279" t="s">
         <v>279</v>
       </c>
       <c r="C279" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F279" s="3"/>
       <c r="G279" s="3"/>
@@ -8439,13 +8638,13 @@
     <row r="280" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A280" s="2">
         <f t="shared" si="4"/>
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B280" t="s">
         <v>279</v>
       </c>
       <c r="C280" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F280" s="3"/>
       <c r="G280" s="3"/>
@@ -8455,13 +8654,13 @@
     <row r="281" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A281" s="2">
         <f t="shared" si="4"/>
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B281" t="s">
         <v>279</v>
       </c>
       <c r="C281" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F281" s="3"/>
       <c r="G281" s="3"/>
@@ -8471,63 +8670,63 @@
     <row r="282" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A282" s="2">
         <f t="shared" si="4"/>
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B282" t="s">
         <v>279</v>
       </c>
       <c r="C282" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F282" s="3"/>
       <c r="G282" s="3"/>
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
     </row>
-    <row r="283" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A283" s="9">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A283" s="2">
+        <f t="shared" si="4"/>
+        <v>281</v>
+      </c>
+      <c r="B283" t="s">
+        <v>279</v>
+      </c>
+      <c r="C283" t="s">
+        <v>290</v>
+      </c>
+      <c r="F283" s="3"/>
+      <c r="G283" s="3"/>
+      <c r="H283" s="4"/>
+      <c r="I283" s="4"/>
+    </row>
+    <row r="284" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A284" s="9">
         <f t="shared" si="4"/>
         <v>282</v>
       </c>
-      <c r="B283" s="6" t="s">
+      <c r="B284" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="C283" s="6" t="s">
+      <c r="C284" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="D283" s="5"/>
-      <c r="E283" s="6"/>
-      <c r="F283" s="7"/>
-      <c r="G283" s="7"/>
-      <c r="H283" s="8"/>
-      <c r="I283" s="8"/>
-    </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A284" s="2">
-        <f t="shared" si="4"/>
-        <v>283</v>
-      </c>
-      <c r="B284" t="s">
-        <v>292</v>
-      </c>
-      <c r="C284" t="s">
-        <v>293</v>
-      </c>
-      <c r="F284" s="3"/>
-      <c r="G284" s="3"/>
-      <c r="H284" s="4"/>
-      <c r="I284" s="4"/>
+      <c r="D284" s="5"/>
+      <c r="E284" s="6"/>
+      <c r="F284" s="7"/>
+      <c r="G284" s="7"/>
+      <c r="H284" s="8"/>
+      <c r="I284" s="8"/>
     </row>
     <row r="285" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A285" s="2">
         <f t="shared" si="4"/>
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B285" t="s">
         <v>292</v>
       </c>
       <c r="C285" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F285" s="3"/>
       <c r="G285" s="3"/>
@@ -8537,13 +8736,13 @@
     <row r="286" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A286" s="2">
         <f t="shared" si="4"/>
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B286" t="s">
         <v>292</v>
       </c>
       <c r="C286" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F286" s="3"/>
       <c r="G286" s="3"/>
@@ -8553,13 +8752,13 @@
     <row r="287" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A287" s="2">
         <f t="shared" si="4"/>
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B287" t="s">
         <v>292</v>
       </c>
       <c r="C287" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F287" s="3"/>
       <c r="G287" s="3"/>
@@ -8569,13 +8768,13 @@
     <row r="288" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A288" s="2">
         <f t="shared" si="4"/>
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B288" t="s">
         <v>292</v>
       </c>
       <c r="C288" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F288" s="3"/>
       <c r="G288" s="3"/>
@@ -8585,13 +8784,13 @@
     <row r="289" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A289" s="2">
         <f t="shared" si="4"/>
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B289" t="s">
         <v>292</v>
       </c>
       <c r="C289" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F289" s="3"/>
       <c r="G289" s="3"/>
@@ -8601,13 +8800,13 @@
     <row r="290" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A290" s="2">
         <f t="shared" si="4"/>
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B290" t="s">
         <v>292</v>
       </c>
       <c r="C290" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F290" s="3"/>
       <c r="G290" s="3"/>
@@ -8617,13 +8816,13 @@
     <row r="291" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A291" s="2">
         <f t="shared" si="4"/>
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B291" t="s">
         <v>292</v>
       </c>
       <c r="C291" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F291" s="3"/>
       <c r="G291" s="3"/>
@@ -8633,13 +8832,13 @@
     <row r="292" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A292" s="2">
         <f t="shared" si="4"/>
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B292" t="s">
         <v>292</v>
       </c>
       <c r="C292" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F292" s="3"/>
       <c r="G292" s="3"/>
@@ -8649,13 +8848,13 @@
     <row r="293" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A293" s="2">
         <f t="shared" si="4"/>
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B293" t="s">
         <v>292</v>
       </c>
       <c r="C293" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F293" s="3"/>
       <c r="G293" s="3"/>
@@ -8665,40 +8864,56 @@
     <row r="294" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A294" s="2">
         <f t="shared" si="4"/>
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B294" t="s">
         <v>292</v>
       </c>
       <c r="C294" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F294" s="3"/>
       <c r="G294" s="3"/>
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
     </row>
-    <row r="295" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A295" s="9">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A295" s="2">
+        <f t="shared" si="4"/>
+        <v>293</v>
+      </c>
+      <c r="B295" t="s">
+        <v>292</v>
+      </c>
+      <c r="C295" t="s">
+        <v>303</v>
+      </c>
+      <c r="F295" s="3"/>
+      <c r="G295" s="3"/>
+      <c r="H295" s="4"/>
+      <c r="I295" s="4"/>
+    </row>
+    <row r="296" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A296" s="9">
         <f t="shared" si="4"/>
         <v>294</v>
       </c>
-      <c r="B295" s="6" t="s">
+      <c r="B296" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="C295" s="6" t="s">
+      <c r="C296" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="D295" s="5"/>
-      <c r="E295" s="6"/>
-      <c r="F295" s="7"/>
-      <c r="G295" s="7"/>
-      <c r="H295" s="8"/>
-      <c r="I295" s="8"/>
+      <c r="D296" s="5"/>
+      <c r="E296" s="6"/>
+      <c r="F296" s="7"/>
+      <c r="G296" s="7"/>
+      <c r="H296" s="8"/>
+      <c r="I296" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I295" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}"/>
-  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D154:D160 D162:D164 D166:D191 D201:D207 D209:D211 D213:D215 D217:D225 D227:D233 D235:D241 D243:D249 D251:D255 D257:D262 D264:D268 D270 D272:D282 D284:D294 D52:D56 D133:D152">
+  <autoFilter ref="A1:I296" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}"/>
+  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D155:D161 D163:D165 D167:D192 D202:D208 D210:D212 D214:D216 D218:D226 D228:D234 D236:D242 D244:D250 D252:D256 D258:D263 D265:D269 D271 D273:D283 D285:D295 D52:D56 D133:D152">
     <cfRule type="cellIs" dxfId="83" priority="111" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8706,7 +8921,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D295">
+  <conditionalFormatting sqref="D296">
     <cfRule type="cellIs" dxfId="81" priority="43" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8738,7 +8953,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D153">
+  <conditionalFormatting sqref="D153:D154">
     <cfRule type="cellIs" dxfId="73" priority="77" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8746,7 +8961,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D161">
+  <conditionalFormatting sqref="D162">
     <cfRule type="cellIs" dxfId="71" priority="75" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8754,7 +8969,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D165">
+  <conditionalFormatting sqref="D166">
     <cfRule type="cellIs" dxfId="69" priority="73" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8762,7 +8977,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D192">
+  <conditionalFormatting sqref="D193">
     <cfRule type="cellIs" dxfId="67" priority="71" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8770,7 +8985,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D200">
+  <conditionalFormatting sqref="D201">
     <cfRule type="cellIs" dxfId="65" priority="39" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8778,7 +8993,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D208">
+  <conditionalFormatting sqref="D209">
     <cfRule type="cellIs" dxfId="63" priority="69" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8786,7 +9001,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D212">
+  <conditionalFormatting sqref="D213">
     <cfRule type="cellIs" dxfId="61" priority="67" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8794,7 +9009,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D216">
+  <conditionalFormatting sqref="D217">
     <cfRule type="cellIs" dxfId="59" priority="65" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8802,7 +9017,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D226">
+  <conditionalFormatting sqref="D227">
     <cfRule type="cellIs" dxfId="57" priority="63" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8810,7 +9025,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D234">
+  <conditionalFormatting sqref="D235">
     <cfRule type="cellIs" dxfId="55" priority="61" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8818,7 +9033,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D242">
+  <conditionalFormatting sqref="D243">
     <cfRule type="cellIs" dxfId="53" priority="59" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8826,7 +9041,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D250">
+  <conditionalFormatting sqref="D251">
     <cfRule type="cellIs" dxfId="51" priority="55" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8834,7 +9049,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D256">
+  <conditionalFormatting sqref="D257">
     <cfRule type="cellIs" dxfId="49" priority="53" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8842,7 +9057,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D263">
+  <conditionalFormatting sqref="D264">
     <cfRule type="cellIs" dxfId="47" priority="51" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8850,7 +9065,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D269">
+  <conditionalFormatting sqref="D270">
     <cfRule type="cellIs" dxfId="45" priority="49" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8858,7 +9073,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D271">
+  <conditionalFormatting sqref="D272">
     <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8866,7 +9081,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D283">
+  <conditionalFormatting sqref="D284">
     <cfRule type="cellIs" dxfId="41" priority="45" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8874,7 +9089,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D193:D199">
+  <conditionalFormatting sqref="D194:D200">
     <cfRule type="cellIs" dxfId="39" priority="41" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9035,7 +9250,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D41 D43:D56 D68 D114:D295" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D41 D43:D56 D68 D114:D296" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D39 D42 D57:D67 D69:D113" xr:uid="{00000000-0002-0000-0000-000001000000}">

</xml_diff>

<commit_message>
Add metadata planning documentation and fractal family analysis
- Add ATTRIBUTION_INTEGRATION_SUMMARY.md: Documentation for attribution metadata in images
- Add FRACTAL_FAMILY_NAME_METADATA_UPDATE.md: Detailed analysis and implementation plan for fractal family names
- Add FractalMetadataRecommendations.md: Best practices for fractal image metadata
- Add ImageMetadataProperties.csv: Comprehensive list of PNG/JPEG metadata properties
- Update FractalRegistry.xlsx: Enhanced fractal categorization and family structure
- Support research and planning for fractal family name feature implementation
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA39C264-9DB7-400E-8D44-5A30DE0315A2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B3B3F2-7C79-4272-9767-1A822803F5AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="361">
   <si>
     <t>Group Name</t>
   </si>
@@ -1080,6 +1080,33 @@
   </si>
   <si>
     <t>black screen, no structure</t>
+  </si>
+  <si>
+    <t>no difference with previous?</t>
+  </si>
+  <si>
+    <t>nice</t>
+  </si>
+  <si>
+    <t>only concentric circles at very small scale</t>
+  </si>
+  <si>
+    <t>nothing but concentric circles</t>
+  </si>
+  <si>
+    <t>amazing full screen of texture</t>
+  </si>
+  <si>
+    <t>solid color screen no structure</t>
+  </si>
+  <si>
+    <t>yet another mandelbrot</t>
+  </si>
+  <si>
+    <t>this is not the Buddahbrot shape.  It is the classic Mandelbrot shape</t>
+  </si>
+  <si>
+    <t>Are we supposed to see vertical bands of colors, only?</t>
   </si>
 </sst>
 </file>
@@ -1737,7 +1764,21 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="84">
+  <dxfs count="86">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color theme="9" tint="-0.24994659260841701"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -2636,14 +2677,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I296"/>
+  <dimension ref="A1:I303"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.3984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.06640625" customWidth="1"/>
-    <col min="3" max="3" width="22.3984375" customWidth="1"/>
+    <col min="2" max="2" width="19.9296875" customWidth="1"/>
+    <col min="3" max="3" width="16.46484375" customWidth="1"/>
     <col min="4" max="4" width="6.46484375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="19.46484375" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" customWidth="1"/>
     <col min="6" max="6" width="6.3984375" customWidth="1"/>
     <col min="7" max="7" width="6.46484375" customWidth="1"/>
     <col min="8" max="8" width="17.53125" customWidth="1"/>
@@ -6940,6 +6981,12 @@
       <c r="C175" t="s">
         <v>189</v>
       </c>
+      <c r="D175" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E175" t="s">
+        <v>351</v>
+      </c>
       <c r="F175" s="3"/>
       <c r="G175" s="3"/>
       <c r="H175" s="4"/>
@@ -6956,6 +7003,9 @@
       <c r="C176" t="s">
         <v>190</v>
       </c>
+      <c r="D176" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F176" s="3"/>
       <c r="G176" s="3"/>
       <c r="H176" s="4"/>
@@ -6972,6 +7022,9 @@
       <c r="C177" t="s">
         <v>191</v>
       </c>
+      <c r="D177" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F177" s="3"/>
       <c r="G177" s="3"/>
       <c r="H177" s="4"/>
@@ -6988,10 +7041,21 @@
       <c r="C178" t="s">
         <v>192</v>
       </c>
-      <c r="F178" s="3"/>
-      <c r="G178" s="3"/>
-      <c r="H178" s="4"/>
-      <c r="I178" s="4"/>
+      <c r="D178" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F178" s="3">
+        <v>-0.36210937499999901</v>
+      </c>
+      <c r="G178" s="3">
+        <v>-4.6874999999999903E-3</v>
+      </c>
+      <c r="H178" s="4">
+        <v>4.2426406870999998</v>
+      </c>
+      <c r="I178" s="4">
+        <v>2.3864853865</v>
+      </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A179" s="2">
@@ -7004,10 +7068,24 @@
       <c r="C179" t="s">
         <v>193</v>
       </c>
-      <c r="F179" s="3"/>
-      <c r="G179" s="3"/>
-      <c r="H179" s="4"/>
-      <c r="I179" s="4"/>
+      <c r="D179" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E179" t="s">
+        <v>352</v>
+      </c>
+      <c r="F179" s="3">
+        <v>-0.36784607040524497</v>
+      </c>
+      <c r="G179" s="3">
+        <v>-1.0777737655028299E-3</v>
+      </c>
+      <c r="H179" s="4">
+        <v>3.6934332400000001</v>
+      </c>
+      <c r="I179" s="4">
+        <v>2.0775561974999999</v>
+      </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A180" s="2">
@@ -7020,10 +7098,21 @@
       <c r="C180" t="s">
         <v>194</v>
       </c>
-      <c r="F180" s="3"/>
-      <c r="G180" s="3"/>
-      <c r="H180" s="4"/>
-      <c r="I180" s="4"/>
+      <c r="D180" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F180" s="3">
+        <v>0</v>
+      </c>
+      <c r="G180" s="3">
+        <v>0</v>
+      </c>
+      <c r="H180" s="4">
+        <v>4</v>
+      </c>
+      <c r="I180" s="4">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A181" s="2">
@@ -7036,10 +7125,21 @@
       <c r="C181" t="s">
         <v>195</v>
       </c>
-      <c r="F181" s="3"/>
-      <c r="G181" s="3"/>
-      <c r="H181" s="4"/>
-      <c r="I181" s="4"/>
+      <c r="D181" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F181" s="3">
+        <v>0</v>
+      </c>
+      <c r="G181" s="3">
+        <v>0</v>
+      </c>
+      <c r="H181" s="4">
+        <v>4.2870938500999998</v>
+      </c>
+      <c r="I181" s="4">
+        <v>2.4114902907000002</v>
+      </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A182" s="2">
@@ -7052,10 +7152,21 @@
       <c r="C182" t="s">
         <v>196</v>
       </c>
-      <c r="F182" s="3"/>
-      <c r="G182" s="3"/>
-      <c r="H182" s="4"/>
-      <c r="I182" s="4"/>
+      <c r="D182" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F182" s="3">
+        <v>0</v>
+      </c>
+      <c r="G182" s="3">
+        <v>0</v>
+      </c>
+      <c r="H182" s="4">
+        <v>4</v>
+      </c>
+      <c r="I182" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A183" s="2">
@@ -7068,10 +7179,21 @@
       <c r="C183" t="s">
         <v>319</v>
       </c>
-      <c r="F183" s="3"/>
-      <c r="G183" s="3"/>
-      <c r="H183" s="4"/>
-      <c r="I183" s="4"/>
+      <c r="D183" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F183" s="3">
+        <v>-0.15712696055775799</v>
+      </c>
+      <c r="G183" s="3">
+        <v>5.5483965529608704E-3</v>
+      </c>
+      <c r="H183" s="4">
+        <v>5.4524630516999997</v>
+      </c>
+      <c r="I183" s="4">
+        <v>3.0670104666000002</v>
+      </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A184" s="2">
@@ -7084,10 +7206,21 @@
       <c r="C184" t="s">
         <v>320</v>
       </c>
-      <c r="F184" s="3"/>
-      <c r="G184" s="3"/>
-      <c r="H184" s="4"/>
-      <c r="I184" s="4"/>
+      <c r="D184" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F184" s="3">
+        <v>0</v>
+      </c>
+      <c r="G184" s="3">
+        <v>0</v>
+      </c>
+      <c r="H184" s="4">
+        <v>4.2857142857000001</v>
+      </c>
+      <c r="I184" s="4">
+        <v>2.4107142857000001</v>
+      </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A185" s="2">
@@ -7100,10 +7233,21 @@
       <c r="C185" t="s">
         <v>321</v>
       </c>
-      <c r="F185" s="3"/>
-      <c r="G185" s="3"/>
-      <c r="H185" s="4"/>
-      <c r="I185" s="4"/>
+      <c r="D185" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F185" s="3">
+        <v>0</v>
+      </c>
+      <c r="G185" s="3">
+        <v>0</v>
+      </c>
+      <c r="H185" s="4">
+        <v>4.6153846154</v>
+      </c>
+      <c r="I185" s="4">
+        <v>2.5961538462</v>
+      </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A186" s="2">
@@ -7116,10 +7260,21 @@
       <c r="C186" t="s">
         <v>197</v>
       </c>
-      <c r="F186" s="3"/>
-      <c r="G186" s="3"/>
-      <c r="H186" s="4"/>
-      <c r="I186" s="4"/>
+      <c r="D186" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F186" s="3">
+        <v>-0.148758993771477</v>
+      </c>
+      <c r="G186" s="3">
+        <v>0.62955326460480998</v>
+      </c>
+      <c r="H186" s="4">
+        <v>4.5794579574999998</v>
+      </c>
+      <c r="I186" s="4">
+        <v>2.5759451010999999</v>
+      </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A187" s="2">
@@ -7132,10 +7287,21 @@
       <c r="C187" t="s">
         <v>198</v>
       </c>
-      <c r="F187" s="3"/>
-      <c r="G187" s="3"/>
-      <c r="H187" s="4"/>
-      <c r="I187" s="4"/>
+      <c r="D187" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F187" s="3">
+        <v>0</v>
+      </c>
+      <c r="G187" s="3">
+        <v>0</v>
+      </c>
+      <c r="H187" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="I187" s="4">
+        <v>0.28125</v>
+      </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A188" s="2">
@@ -7148,10 +7314,24 @@
       <c r="C188" t="s">
         <v>199</v>
       </c>
-      <c r="F188" s="3"/>
-      <c r="G188" s="3"/>
-      <c r="H188" s="4"/>
-      <c r="I188" s="4"/>
+      <c r="D188" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E188" t="s">
+        <v>353</v>
+      </c>
+      <c r="F188" s="3">
+        <v>-0.58828124999999898</v>
+      </c>
+      <c r="G188" s="3">
+        <v>-4.6874999999999903E-3</v>
+      </c>
+      <c r="H188" s="4">
+        <v>3</v>
+      </c>
+      <c r="I188" s="4">
+        <v>1.6875</v>
+      </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A189" s="2">
@@ -7164,10 +7344,21 @@
       <c r="C189" t="s">
         <v>200</v>
       </c>
-      <c r="F189" s="3"/>
-      <c r="G189" s="3"/>
-      <c r="H189" s="4"/>
-      <c r="I189" s="4"/>
+      <c r="D189" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F189" s="3">
+        <v>-0.249609374999999</v>
+      </c>
+      <c r="G189" s="3">
+        <v>-1.6406250000000001E-2</v>
+      </c>
+      <c r="H189" s="4">
+        <v>4.8735143555000002</v>
+      </c>
+      <c r="I189" s="4">
+        <v>2.7413518250000002</v>
+      </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A190" s="2">
@@ -7180,10 +7371,21 @@
       <c r="C190" t="s">
         <v>201</v>
       </c>
-      <c r="F190" s="3"/>
-      <c r="G190" s="3"/>
-      <c r="H190" s="4"/>
-      <c r="I190" s="4"/>
+      <c r="D190" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F190" s="3">
+        <v>-0.2109375</v>
+      </c>
+      <c r="G190" s="3">
+        <v>-1.8749999999999899E-2</v>
+      </c>
+      <c r="H190" s="4">
+        <v>6</v>
+      </c>
+      <c r="I190" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A191" s="2">
@@ -7196,6 +7398,12 @@
       <c r="C191" t="s">
         <v>202</v>
       </c>
+      <c r="D191" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E191" t="s">
+        <v>354</v>
+      </c>
       <c r="F191" s="3"/>
       <c r="G191" s="3"/>
       <c r="H191" s="4"/>
@@ -7212,10 +7420,21 @@
       <c r="C192" t="s">
         <v>203</v>
       </c>
-      <c r="F192" s="3"/>
-      <c r="G192" s="3"/>
-      <c r="H192" s="4"/>
-      <c r="I192" s="4"/>
+      <c r="D192" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F192" s="3">
+        <v>-0.248521008366511</v>
+      </c>
+      <c r="G192" s="3">
+        <v>3.6650423737307002E-2</v>
+      </c>
+      <c r="H192" s="4">
+        <v>6.9643507080999996</v>
+      </c>
+      <c r="I192" s="4">
+        <v>3.9174472733000001</v>
+      </c>
     </row>
     <row r="193" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A193" s="9">
@@ -7228,12 +7447,22 @@
       <c r="C193" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="D193" s="5"/>
+      <c r="D193" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E193" s="6"/>
-      <c r="F193" s="7"/>
-      <c r="G193" s="7"/>
-      <c r="H193" s="8"/>
-      <c r="I193" s="8"/>
+      <c r="F193" s="7">
+        <v>-0.109897735001431</v>
+      </c>
+      <c r="G193" s="7">
+        <v>-4.35438144329897E-2</v>
+      </c>
+      <c r="H193" s="8">
+        <v>5.7768613975000003</v>
+      </c>
+      <c r="I193" s="8">
+        <v>3.2494845361000002</v>
+      </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A194" s="9">
@@ -7246,10 +7475,21 @@
       <c r="C194" t="s">
         <v>245</v>
       </c>
-      <c r="F194" s="3"/>
-      <c r="G194" s="3"/>
-      <c r="H194" s="4"/>
-      <c r="I194" s="4"/>
+      <c r="D194" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F194" s="3">
+        <v>-0.214285714285714</v>
+      </c>
+      <c r="G194" s="3">
+        <v>-0.57756696428571397</v>
+      </c>
+      <c r="H194" s="4">
+        <v>4.2857142857000001</v>
+      </c>
+      <c r="I194" s="4">
+        <v>2.4107142857000001</v>
+      </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A195" s="9">
@@ -7262,10 +7502,21 @@
       <c r="C195" t="s">
         <v>246</v>
       </c>
-      <c r="F195" s="3"/>
-      <c r="G195" s="3"/>
-      <c r="H195" s="4"/>
-      <c r="I195" s="4"/>
+      <c r="D195" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F195" s="3">
+        <v>0</v>
+      </c>
+      <c r="G195" s="3">
+        <v>0</v>
+      </c>
+      <c r="H195" s="4">
+        <v>4</v>
+      </c>
+      <c r="I195" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A196" s="9">
@@ -7278,10 +7529,21 @@
       <c r="C196" t="s">
         <v>247</v>
       </c>
-      <c r="F196" s="3"/>
-      <c r="G196" s="3"/>
-      <c r="H196" s="4"/>
-      <c r="I196" s="4"/>
+      <c r="D196" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F196" s="3">
+        <v>-0.19380004332237499</v>
+      </c>
+      <c r="G196" s="3">
+        <v>1.8667670377751001E-2</v>
+      </c>
+      <c r="H196" s="4">
+        <v>5.4524630516999997</v>
+      </c>
+      <c r="I196" s="4">
+        <v>3.0670104666000002</v>
+      </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A197" s="9">
@@ -7294,10 +7556,21 @@
       <c r="C197" t="s">
         <v>248</v>
       </c>
-      <c r="F197" s="3"/>
-      <c r="G197" s="3"/>
-      <c r="H197" s="4"/>
-      <c r="I197" s="4"/>
+      <c r="D197" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F197" s="3">
+        <v>-0.114484592013889</v>
+      </c>
+      <c r="G197" s="3">
+        <v>4.7308132875143504E-3</v>
+      </c>
+      <c r="H197" s="4">
+        <v>4.1530355096999996</v>
+      </c>
+      <c r="I197" s="4">
+        <v>2.3360824741999999</v>
+      </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A198" s="9">
@@ -7310,10 +7583,21 @@
       <c r="C198" t="s">
         <v>249</v>
       </c>
-      <c r="F198" s="3"/>
-      <c r="G198" s="3"/>
-      <c r="H198" s="4"/>
-      <c r="I198" s="4"/>
+      <c r="D198" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F198" s="3">
+        <v>7.5036966004140407E-2</v>
+      </c>
+      <c r="G198" s="3">
+        <v>-2.21804600992744E-2</v>
+      </c>
+      <c r="H198" s="4">
+        <v>3.9984726995000002</v>
+      </c>
+      <c r="I198" s="4">
+        <v>2.2491408934999999</v>
+      </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A199" s="9">
@@ -7326,10 +7610,21 @@
       <c r="C199" t="s">
         <v>250</v>
       </c>
-      <c r="F199" s="3"/>
-      <c r="G199" s="3"/>
-      <c r="H199" s="4"/>
-      <c r="I199" s="4"/>
+      <c r="D199" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F199" s="3">
+        <v>-1.2357903888167401E-2</v>
+      </c>
+      <c r="G199" s="3">
+        <v>-4.4905939034107098E-2</v>
+      </c>
+      <c r="H199" s="4">
+        <v>4.1758745694000003</v>
+      </c>
+      <c r="I199" s="4">
+        <v>2.3489294453</v>
+      </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A200" s="9">
@@ -7342,10 +7637,21 @@
       <c r="C200" t="s">
         <v>251</v>
       </c>
-      <c r="F200" s="3"/>
-      <c r="G200" s="3"/>
-      <c r="H200" s="4"/>
-      <c r="I200" s="4"/>
+      <c r="D200" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F200" s="3">
+        <v>0</v>
+      </c>
+      <c r="G200" s="3">
+        <v>0</v>
+      </c>
+      <c r="H200" s="4">
+        <v>3.9987128208999998</v>
+      </c>
+      <c r="I200" s="4">
+        <v>2.2492759617</v>
+      </c>
     </row>
     <row r="201" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A201" s="9">
@@ -7358,12 +7664,22 @@
       <c r="C201" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="D201" s="5"/>
+      <c r="D201" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E201" s="6"/>
-      <c r="F201" s="7"/>
-      <c r="G201" s="7"/>
-      <c r="H201" s="8"/>
-      <c r="I201" s="8"/>
+      <c r="F201" s="7">
+        <v>0</v>
+      </c>
+      <c r="G201" s="7">
+        <v>0</v>
+      </c>
+      <c r="H201" s="8">
+        <v>6.5975395538999999</v>
+      </c>
+      <c r="I201" s="8">
+        <v>3.711115999</v>
+      </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A202" s="9">
@@ -7376,6 +7692,9 @@
       <c r="C202" t="s">
         <v>324</v>
       </c>
+      <c r="D202" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F202" s="3"/>
       <c r="G202" s="3"/>
       <c r="H202" s="4"/>
@@ -7392,6 +7711,9 @@
       <c r="C203" t="s">
         <v>325</v>
       </c>
+      <c r="D203" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F203" s="3"/>
       <c r="G203" s="3"/>
       <c r="H203" s="4"/>
@@ -7408,6 +7730,12 @@
       <c r="C204" t="s">
         <v>206</v>
       </c>
+      <c r="D204" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E204" t="s">
+        <v>355</v>
+      </c>
       <c r="F204" s="3"/>
       <c r="G204" s="3"/>
       <c r="H204" s="4"/>
@@ -7424,6 +7752,9 @@
       <c r="C205" t="s">
         <v>326</v>
       </c>
+      <c r="D205" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F205" s="3"/>
       <c r="G205" s="3"/>
       <c r="H205" s="4"/>
@@ -7440,6 +7771,9 @@
       <c r="C206" t="s">
         <v>327</v>
       </c>
+      <c r="D206" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F206" s="3"/>
       <c r="G206" s="3"/>
       <c r="H206" s="4"/>
@@ -7456,6 +7790,9 @@
       <c r="C207" t="s">
         <v>328</v>
       </c>
+      <c r="D207" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F207" s="3"/>
       <c r="G207" s="3"/>
       <c r="H207" s="4"/>
@@ -7472,10 +7809,24 @@
       <c r="C208" t="s">
         <v>207</v>
       </c>
-      <c r="F208" s="3"/>
-      <c r="G208" s="3"/>
-      <c r="H208" s="4"/>
-      <c r="I208" s="4"/>
+      <c r="D208" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E208" t="s">
+        <v>356</v>
+      </c>
+      <c r="F208" s="3">
+        <v>0</v>
+      </c>
+      <c r="G208" s="3">
+        <v>0</v>
+      </c>
+      <c r="H208" s="4">
+        <v>96</v>
+      </c>
+      <c r="I208" s="4">
+        <v>54</v>
+      </c>
     </row>
     <row r="209" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A209" s="9">
@@ -7488,12 +7839,22 @@
       <c r="C209" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="D209" s="5"/>
+      <c r="D209" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E209" s="6"/>
-      <c r="F209" s="7"/>
-      <c r="G209" s="7"/>
-      <c r="H209" s="8"/>
-      <c r="I209" s="8"/>
+      <c r="F209" s="7">
+        <v>-0.55139768622793595</v>
+      </c>
+      <c r="G209" s="7">
+        <v>2.63177386339149E-2</v>
+      </c>
+      <c r="H209" s="8">
+        <v>2.2207857502000001</v>
+      </c>
+      <c r="I209" s="8">
+        <v>1.2491919844999999</v>
+      </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A210" s="2">
@@ -7506,10 +7867,21 @@
       <c r="C210" t="s">
         <v>210</v>
       </c>
-      <c r="F210" s="3"/>
-      <c r="G210" s="3"/>
-      <c r="H210" s="4"/>
-      <c r="I210" s="4"/>
+      <c r="D210" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F210" s="3">
+        <v>0</v>
+      </c>
+      <c r="G210" s="3">
+        <v>0</v>
+      </c>
+      <c r="H210" s="4">
+        <v>6</v>
+      </c>
+      <c r="I210" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A211" s="2">
@@ -7522,10 +7894,21 @@
       <c r="C211" t="s">
         <v>211</v>
       </c>
-      <c r="F211" s="3"/>
-      <c r="G211" s="3"/>
-      <c r="H211" s="4"/>
-      <c r="I211" s="4"/>
+      <c r="D211" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F211" s="3">
+        <v>0</v>
+      </c>
+      <c r="G211" s="3">
+        <v>0</v>
+      </c>
+      <c r="H211" s="4">
+        <v>6</v>
+      </c>
+      <c r="I211" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A212" s="2">
@@ -7538,10 +7921,21 @@
       <c r="C212" t="s">
         <v>212</v>
       </c>
-      <c r="F212" s="3"/>
-      <c r="G212" s="3"/>
-      <c r="H212" s="4"/>
-      <c r="I212" s="4"/>
+      <c r="D212" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F212" s="3">
+        <v>0</v>
+      </c>
+      <c r="G212" s="3">
+        <v>0</v>
+      </c>
+      <c r="H212" s="4">
+        <v>6</v>
+      </c>
+      <c r="I212" s="4">
+        <v>3.375</v>
+      </c>
     </row>
     <row r="213" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A213" s="9">
@@ -7554,8 +7948,12 @@
       <c r="C213" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="D213" s="5"/>
-      <c r="E213" s="6"/>
+      <c r="D213" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="E213" s="6" t="s">
+        <v>357</v>
+      </c>
       <c r="F213" s="7"/>
       <c r="G213" s="7"/>
       <c r="H213" s="8"/>
@@ -7572,12 +7970,23 @@
       <c r="C214" t="s">
         <v>215</v>
       </c>
-      <c r="F214" s="3"/>
-      <c r="G214" s="3"/>
-      <c r="H214" s="4"/>
-      <c r="I214" s="4"/>
-    </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="D214" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F214" s="3">
+        <v>-0.37968749999999901</v>
+      </c>
+      <c r="G214" s="3">
+        <v>-1.7578125E-2</v>
+      </c>
+      <c r="H214" s="4">
+        <v>3</v>
+      </c>
+      <c r="I214" s="4">
+        <v>1.6875</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A215" s="2">
         <f t="shared" si="3"/>
         <v>213</v>
@@ -7587,6 +7996,12 @@
       </c>
       <c r="C215" t="s">
         <v>216</v>
+      </c>
+      <c r="D215" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E215" s="6" t="s">
+        <v>357</v>
       </c>
       <c r="F215" s="3"/>
       <c r="G215" s="3"/>
@@ -7604,6 +8019,12 @@
       <c r="C216" t="s">
         <v>217</v>
       </c>
+      <c r="D216" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E216" t="s">
+        <v>357</v>
+      </c>
       <c r="F216" s="3"/>
       <c r="G216" s="3"/>
       <c r="H216" s="4"/>
@@ -7620,12 +8041,22 @@
       <c r="C217" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="D217" s="5"/>
+      <c r="D217" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E217" s="6"/>
-      <c r="F217" s="7"/>
-      <c r="G217" s="7"/>
-      <c r="H217" s="8"/>
-      <c r="I217" s="8"/>
+      <c r="F217" s="7">
+        <v>-0.16662704558133701</v>
+      </c>
+      <c r="G217" s="7">
+        <v>6.5052130349130199E-19</v>
+      </c>
+      <c r="H217" s="8">
+        <v>4.0238269362999999</v>
+      </c>
+      <c r="I217" s="8">
+        <v>2.2634026516999999</v>
+      </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A218" s="2">
@@ -7638,10 +8069,21 @@
       <c r="C218" t="s">
         <v>220</v>
       </c>
-      <c r="F218" s="3"/>
-      <c r="G218" s="3"/>
-      <c r="H218" s="4"/>
-      <c r="I218" s="4"/>
+      <c r="D218" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F218" s="3">
+        <v>-8.8863350609925396E-2</v>
+      </c>
+      <c r="G218" s="3">
+        <v>-2.49544228749192E-2</v>
+      </c>
+      <c r="H218" s="4">
+        <v>4.1707022676000003</v>
+      </c>
+      <c r="I218" s="4">
+        <v>2.3460200255000001</v>
+      </c>
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A219" s="2">
@@ -7654,10 +8096,21 @@
       <c r="C219" t="s">
         <v>221</v>
       </c>
-      <c r="F219" s="3"/>
-      <c r="G219" s="3"/>
-      <c r="H219" s="4"/>
-      <c r="I219" s="4"/>
+      <c r="D219" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F219" s="3">
+        <v>0</v>
+      </c>
+      <c r="G219" s="3">
+        <v>0</v>
+      </c>
+      <c r="H219" s="4">
+        <v>15</v>
+      </c>
+      <c r="I219" s="4">
+        <v>8.4375</v>
+      </c>
     </row>
     <row r="220" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A220" s="2">
@@ -7670,10 +8123,21 @@
       <c r="C220" t="s">
         <v>222</v>
       </c>
-      <c r="F220" s="3"/>
-      <c r="G220" s="3"/>
-      <c r="H220" s="4"/>
-      <c r="I220" s="4"/>
+      <c r="D220" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F220" s="3">
+        <v>0</v>
+      </c>
+      <c r="G220" s="3">
+        <v>0</v>
+      </c>
+      <c r="H220" s="4">
+        <v>15</v>
+      </c>
+      <c r="I220" s="4">
+        <v>8.4375</v>
+      </c>
     </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A221" s="2">
@@ -7686,10 +8150,21 @@
       <c r="C221" t="s">
         <v>223</v>
       </c>
-      <c r="F221" s="3"/>
-      <c r="G221" s="3"/>
-      <c r="H221" s="4"/>
-      <c r="I221" s="4"/>
+      <c r="D221" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F221" s="3">
+        <v>0</v>
+      </c>
+      <c r="G221" s="3">
+        <v>0</v>
+      </c>
+      <c r="H221" s="4">
+        <v>15</v>
+      </c>
+      <c r="I221" s="4">
+        <v>8.4375</v>
+      </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A222" s="2">
@@ -7702,10 +8177,21 @@
       <c r="C222" t="s">
         <v>224</v>
       </c>
-      <c r="F222" s="3"/>
-      <c r="G222" s="3"/>
-      <c r="H222" s="4"/>
-      <c r="I222" s="4"/>
+      <c r="D222" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F222" s="3">
+        <v>0</v>
+      </c>
+      <c r="G222" s="3">
+        <v>0</v>
+      </c>
+      <c r="H222" s="4">
+        <v>3.75</v>
+      </c>
+      <c r="I222" s="4">
+        <v>2.109375</v>
+      </c>
     </row>
     <row r="223" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A223" s="2">
@@ -7718,10 +8204,21 @@
       <c r="C223" t="s">
         <v>225</v>
       </c>
-      <c r="F223" s="3"/>
-      <c r="G223" s="3"/>
-      <c r="H223" s="4"/>
-      <c r="I223" s="4"/>
+      <c r="D223" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F223" s="3">
+        <v>0</v>
+      </c>
+      <c r="G223" s="3">
+        <v>0</v>
+      </c>
+      <c r="H223" s="4">
+        <v>3.75</v>
+      </c>
+      <c r="I223" s="4">
+        <v>2.109375</v>
+      </c>
     </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A224" s="2">
@@ -7734,10 +8231,21 @@
       <c r="C224" t="s">
         <v>226</v>
       </c>
-      <c r="F224" s="3"/>
-      <c r="G224" s="3"/>
-      <c r="H224" s="4"/>
-      <c r="I224" s="4"/>
+      <c r="D224" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F224" s="3">
+        <v>-0.251953125</v>
+      </c>
+      <c r="G224" s="3">
+        <v>-8.7890625E-3</v>
+      </c>
+      <c r="H224" s="4">
+        <v>3.75</v>
+      </c>
+      <c r="I224" s="4">
+        <v>2.109375</v>
+      </c>
     </row>
     <row r="225" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A225" s="2">
@@ -7750,10 +8258,24 @@
       <c r="C225" t="s">
         <v>227</v>
       </c>
-      <c r="F225" s="3"/>
-      <c r="G225" s="3"/>
-      <c r="H225" s="4"/>
-      <c r="I225" s="4"/>
+      <c r="D225" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E225" t="s">
+        <v>358</v>
+      </c>
+      <c r="F225" s="3">
+        <v>-0.15487041477869101</v>
+      </c>
+      <c r="G225" s="3">
+        <v>-1.36663693622268E-2</v>
+      </c>
+      <c r="H225" s="4">
+        <v>4.0779891939999997</v>
+      </c>
+      <c r="I225" s="4">
+        <v>2.2938689218000001</v>
+      </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A226" s="2">
@@ -7766,10 +8288,21 @@
       <c r="C226" t="s">
         <v>228</v>
       </c>
-      <c r="F226" s="3"/>
-      <c r="G226" s="3"/>
-      <c r="H226" s="4"/>
-      <c r="I226" s="4"/>
+      <c r="D226" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F226" s="3">
+        <v>-0.1787109375</v>
+      </c>
+      <c r="G226" s="3">
+        <v>1.46484375E-3</v>
+      </c>
+      <c r="H226" s="4">
+        <v>3.75</v>
+      </c>
+      <c r="I226" s="4">
+        <v>2.109375</v>
+      </c>
     </row>
     <row r="227" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A227" s="9">
@@ -7782,12 +8315,22 @@
       <c r="C227" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D227" s="5"/>
+      <c r="D227" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E227" s="6"/>
-      <c r="F227" s="7"/>
-      <c r="G227" s="7"/>
-      <c r="H227" s="8"/>
-      <c r="I227" s="8"/>
+      <c r="F227" s="7">
+        <v>-0.34130859375</v>
+      </c>
+      <c r="G227" s="7">
+        <v>-1.46484375E-3</v>
+      </c>
+      <c r="H227" s="8">
+        <v>15</v>
+      </c>
+      <c r="I227" s="8">
+        <v>8.4375</v>
+      </c>
     </row>
     <row r="228" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A228" s="2">
@@ -7800,10 +8343,21 @@
       <c r="C228" t="s">
         <v>231</v>
       </c>
-      <c r="F228" s="3"/>
-      <c r="G228" s="3"/>
-      <c r="H228" s="4"/>
-      <c r="I228" s="4"/>
+      <c r="D228" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F228" s="3">
+        <v>-0.18535125895255999</v>
+      </c>
+      <c r="G228" s="3">
+        <v>1.5132638679150301E-2</v>
+      </c>
+      <c r="H228" s="4">
+        <v>2.9396959630000001</v>
+      </c>
+      <c r="I228" s="4">
+        <v>1.6535789792</v>
+      </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A229" s="2">
@@ -7816,10 +8370,21 @@
       <c r="C229" t="s">
         <v>232</v>
       </c>
-      <c r="F229" s="3"/>
-      <c r="G229" s="3"/>
-      <c r="H229" s="4"/>
-      <c r="I229" s="4"/>
+      <c r="D229" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F229" s="3">
+        <v>0</v>
+      </c>
+      <c r="G229" s="3">
+        <v>0</v>
+      </c>
+      <c r="H229" s="4">
+        <v>22.973967099999999</v>
+      </c>
+      <c r="I229" s="4">
+        <v>12.922856493999999</v>
+      </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
@@ -7832,10 +8397,21 @@
       <c r="C230" t="s">
         <v>233</v>
       </c>
-      <c r="F230" s="3"/>
-      <c r="G230" s="3"/>
-      <c r="H230" s="4"/>
-      <c r="I230" s="4"/>
+      <c r="D230" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F230" s="3">
+        <v>0</v>
+      </c>
+      <c r="G230" s="3">
+        <v>0</v>
+      </c>
+      <c r="H230" s="4">
+        <v>3.2645646124000001</v>
+      </c>
+      <c r="I230" s="4">
+        <v>1.8363175945000001</v>
+      </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A231" s="2">
@@ -7848,10 +8424,21 @@
       <c r="C231" t="s">
         <v>234</v>
       </c>
-      <c r="F231" s="3"/>
-      <c r="G231" s="3"/>
-      <c r="H231" s="4"/>
-      <c r="I231" s="4"/>
+      <c r="D231" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F231" s="3">
+        <v>-0.16611516952966299</v>
+      </c>
+      <c r="G231" s="3">
+        <v>6.6816265541818395E-2</v>
+      </c>
+      <c r="H231" s="4">
+        <v>5.6568542495000003</v>
+      </c>
+      <c r="I231" s="4">
+        <v>3.1819805152999998</v>
+      </c>
     </row>
     <row r="232" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A232" s="2">
@@ -7864,10 +8451,21 @@
       <c r="C232" t="s">
         <v>235</v>
       </c>
-      <c r="F232" s="3"/>
-      <c r="G232" s="3"/>
-      <c r="H232" s="4"/>
-      <c r="I232" s="4"/>
+      <c r="D232" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F232" s="3">
+        <v>0.6</v>
+      </c>
+      <c r="G232" s="3">
+        <v>0</v>
+      </c>
+      <c r="H232" s="4">
+        <v>4.8735143781000003</v>
+      </c>
+      <c r="I232" s="4">
+        <v>2.7413518376999999</v>
+      </c>
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A233" s="2">
@@ -7880,10 +8478,21 @@
       <c r="C233" t="s">
         <v>236</v>
       </c>
-      <c r="F233" s="3"/>
-      <c r="G233" s="3"/>
-      <c r="H233" s="4"/>
-      <c r="I233" s="4"/>
+      <c r="D233" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F233" s="3">
+        <v>-0.19383352385890201</v>
+      </c>
+      <c r="G233" s="3">
+        <v>3.4005881378754801E-3</v>
+      </c>
+      <c r="H233" s="4">
+        <v>4.3527528164999998</v>
+      </c>
+      <c r="I233" s="4">
+        <v>2.4484234592999998</v>
+      </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A234" s="2">
@@ -7896,6 +8505,9 @@
       <c r="C234" t="s">
         <v>237</v>
       </c>
+      <c r="D234" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F234" s="3"/>
       <c r="G234" s="3"/>
       <c r="H234" s="4"/>
@@ -7912,12 +8524,22 @@
       <c r="C235" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="D235" s="5"/>
+      <c r="D235" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E235" s="6"/>
-      <c r="F235" s="7"/>
-      <c r="G235" s="7"/>
-      <c r="H235" s="8"/>
-      <c r="I235" s="8"/>
+      <c r="F235" s="7">
+        <v>0</v>
+      </c>
+      <c r="G235" s="7">
+        <v>0</v>
+      </c>
+      <c r="H235" s="8">
+        <v>8</v>
+      </c>
+      <c r="I235" s="8">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="236" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A236" s="2">
@@ -7930,10 +8552,21 @@
       <c r="C236" t="s">
         <v>239</v>
       </c>
-      <c r="F236" s="3"/>
-      <c r="G236" s="3"/>
-      <c r="H236" s="4"/>
-      <c r="I236" s="4"/>
+      <c r="D236" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F236" s="3">
+        <v>-0.57070312499999998</v>
+      </c>
+      <c r="G236" s="3">
+        <v>2.6953124999999901E-2</v>
+      </c>
+      <c r="H236" s="4">
+        <v>3.6934332400000001</v>
+      </c>
+      <c r="I236" s="4">
+        <v>2.0775561974999999</v>
+      </c>
     </row>
     <row r="237" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A237" s="2">
@@ -7946,10 +8579,21 @@
       <c r="C237" t="s">
         <v>240</v>
       </c>
-      <c r="F237" s="3"/>
-      <c r="G237" s="3"/>
-      <c r="H237" s="4"/>
-      <c r="I237" s="4"/>
+      <c r="D237" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F237" s="3">
+        <v>0</v>
+      </c>
+      <c r="G237" s="3">
+        <v>0</v>
+      </c>
+      <c r="H237" s="4">
+        <v>5</v>
+      </c>
+      <c r="I237" s="4">
+        <v>2.8125</v>
+      </c>
     </row>
     <row r="238" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A238" s="2">
@@ -7962,10 +8606,21 @@
       <c r="C238" t="s">
         <v>322</v>
       </c>
-      <c r="F238" s="3"/>
-      <c r="G238" s="3"/>
-      <c r="H238" s="4"/>
-      <c r="I238" s="4"/>
+      <c r="D238" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F238" s="3">
+        <v>0</v>
+      </c>
+      <c r="G238" s="3">
+        <v>0</v>
+      </c>
+      <c r="H238" s="4">
+        <v>2.4622888267</v>
+      </c>
+      <c r="I238" s="4">
+        <v>1.3850374649999999</v>
+      </c>
     </row>
     <row r="239" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A239" s="2">
@@ -7978,10 +8633,21 @@
       <c r="C239" t="s">
         <v>323</v>
       </c>
-      <c r="F239" s="3"/>
-      <c r="G239" s="3"/>
-      <c r="H239" s="4"/>
-      <c r="I239" s="4"/>
+      <c r="D239" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F239" s="3">
+        <v>0</v>
+      </c>
+      <c r="G239" s="3">
+        <v>0</v>
+      </c>
+      <c r="H239" s="4">
+        <v>4</v>
+      </c>
+      <c r="I239" s="4">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="240" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A240" s="2">
@@ -7994,10 +8660,21 @@
       <c r="C240" t="s">
         <v>241</v>
       </c>
-      <c r="F240" s="3"/>
-      <c r="G240" s="3"/>
-      <c r="H240" s="4"/>
-      <c r="I240" s="4"/>
+      <c r="D240" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F240" s="3">
+        <v>0</v>
+      </c>
+      <c r="G240" s="3">
+        <v>0</v>
+      </c>
+      <c r="H240" s="4">
+        <v>4.3063061147999999</v>
+      </c>
+      <c r="I240" s="4">
+        <v>2.4222971896000001</v>
+      </c>
     </row>
     <row r="241" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A241" s="2">
@@ -8010,10 +8687,21 @@
       <c r="C241" t="s">
         <v>242</v>
       </c>
-      <c r="F241" s="3"/>
-      <c r="G241" s="3"/>
-      <c r="H241" s="4"/>
-      <c r="I241" s="4"/>
+      <c r="D241" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F241" s="3">
+        <v>-0.168898568184977</v>
+      </c>
+      <c r="G241" s="3">
+        <v>2.1546730920717301E-2</v>
+      </c>
+      <c r="H241" s="4">
+        <v>3.5586858811000002</v>
+      </c>
+      <c r="I241" s="4">
+        <v>2.0017608080999998</v>
+      </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A242" s="2">
@@ -8026,10 +8714,21 @@
       <c r="C242" t="s">
         <v>243</v>
       </c>
-      <c r="F242" s="3"/>
-      <c r="G242" s="3"/>
-      <c r="H242" s="4"/>
-      <c r="I242" s="4"/>
+      <c r="D242" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F242" s="3">
+        <v>0</v>
+      </c>
+      <c r="G242" s="3">
+        <v>0</v>
+      </c>
+      <c r="H242" s="4">
+        <v>32</v>
+      </c>
+      <c r="I242" s="4">
+        <v>18</v>
+      </c>
     </row>
     <row r="243" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A243" s="2">
@@ -8042,12 +8741,22 @@
       <c r="C243" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="D243" s="5"/>
+      <c r="D243" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E243" s="6"/>
-      <c r="F243" s="7"/>
-      <c r="G243" s="7"/>
-      <c r="H243" s="8"/>
-      <c r="I243" s="8"/>
+      <c r="F243" s="7">
+        <v>0</v>
+      </c>
+      <c r="G243" s="7">
+        <v>0</v>
+      </c>
+      <c r="H243" s="8">
+        <v>4</v>
+      </c>
+      <c r="I243" s="8">
+        <v>2.25</v>
+      </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A244" s="2">
@@ -8060,10 +8769,21 @@
       <c r="C244" t="s">
         <v>329</v>
       </c>
-      <c r="F244" s="3"/>
-      <c r="G244" s="3"/>
-      <c r="H244" s="4"/>
-      <c r="I244" s="4"/>
+      <c r="D244" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F244" s="3">
+        <v>0</v>
+      </c>
+      <c r="G244" s="3">
+        <v>0</v>
+      </c>
+      <c r="H244" s="4">
+        <v>80</v>
+      </c>
+      <c r="I244" s="4">
+        <v>45</v>
+      </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A245" s="2">
@@ -8076,10 +8796,21 @@
       <c r="C245" t="s">
         <v>330</v>
       </c>
-      <c r="F245" s="3"/>
-      <c r="G245" s="3"/>
-      <c r="H245" s="4"/>
-      <c r="I245" s="4"/>
+      <c r="D245" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F245" s="3">
+        <v>-2.3551547802465</v>
+      </c>
+      <c r="G245" s="3">
+        <v>1.49625973078175E-2</v>
+      </c>
+      <c r="H245" s="4">
+        <v>7.3868664801000001</v>
+      </c>
+      <c r="I245" s="4">
+        <v>4.1551123949999997</v>
+      </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A246" s="2">
@@ -8092,10 +8823,21 @@
       <c r="C246" t="s">
         <v>331</v>
       </c>
-      <c r="F246" s="3"/>
-      <c r="G246" s="3"/>
-      <c r="H246" s="4"/>
-      <c r="I246" s="4"/>
+      <c r="D246" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F246" s="3">
+        <v>0</v>
+      </c>
+      <c r="G246" s="3">
+        <v>0</v>
+      </c>
+      <c r="H246" s="4">
+        <v>5</v>
+      </c>
+      <c r="I246" s="4">
+        <v>2.8125</v>
+      </c>
     </row>
     <row r="247" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A247" s="2">
@@ -8108,10 +8850,21 @@
       <c r="C247" t="s">
         <v>332</v>
       </c>
-      <c r="F247" s="3"/>
-      <c r="G247" s="3"/>
-      <c r="H247" s="4"/>
-      <c r="I247" s="4"/>
+      <c r="D247" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F247" s="3">
+        <v>0</v>
+      </c>
+      <c r="G247" s="3">
+        <v>0</v>
+      </c>
+      <c r="H247" s="4">
+        <v>5</v>
+      </c>
+      <c r="I247" s="4">
+        <v>2.8125</v>
+      </c>
     </row>
     <row r="248" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A248" s="2">
@@ -8124,10 +8877,21 @@
       <c r="C248" t="s">
         <v>333</v>
       </c>
-      <c r="F248" s="3"/>
-      <c r="G248" s="3"/>
-      <c r="H248" s="4"/>
-      <c r="I248" s="4"/>
+      <c r="D248" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F248" s="3">
+        <v>0</v>
+      </c>
+      <c r="G248" s="3">
+        <v>0</v>
+      </c>
+      <c r="H248" s="4">
+        <v>5</v>
+      </c>
+      <c r="I248" s="4">
+        <v>2.8125</v>
+      </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A249" s="2">
@@ -8140,10 +8904,21 @@
       <c r="C249" t="s">
         <v>334</v>
       </c>
-      <c r="F249" s="3"/>
-      <c r="G249" s="3"/>
-      <c r="H249" s="4"/>
-      <c r="I249" s="4"/>
+      <c r="D249" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F249" s="3">
+        <v>4.0254603399433702</v>
+      </c>
+      <c r="G249" s="3">
+        <v>0.144673630783757</v>
+      </c>
+      <c r="H249" s="4">
+        <v>12</v>
+      </c>
+      <c r="I249" s="4">
+        <v>6.75</v>
+      </c>
     </row>
     <row r="250" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A250" s="2">
@@ -8156,10 +8931,21 @@
       <c r="C250" t="s">
         <v>335</v>
       </c>
-      <c r="F250" s="3"/>
-      <c r="G250" s="3"/>
-      <c r="H250" s="4"/>
-      <c r="I250" s="4"/>
+      <c r="D250" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F250" s="3">
+        <v>-6.2910553801410293E-2</v>
+      </c>
+      <c r="G250" s="3">
+        <v>-0.133920889728255</v>
+      </c>
+      <c r="H250" s="4">
+        <v>3.008288742</v>
+      </c>
+      <c r="I250" s="4">
+        <v>1.6921624174000001</v>
+      </c>
     </row>
     <row r="251" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A251" s="2">
@@ -8172,12 +8958,22 @@
       <c r="C251" t="s">
         <v>336</v>
       </c>
-      <c r="D251" s="5"/>
+      <c r="D251" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E251" s="6"/>
-      <c r="F251" s="7"/>
-      <c r="G251" s="7"/>
-      <c r="H251" s="8"/>
-      <c r="I251" s="8"/>
+      <c r="F251" s="7">
+        <v>9.1841731880125899E-2</v>
+      </c>
+      <c r="G251" s="7">
+        <v>-0.17277720945686001</v>
+      </c>
+      <c r="H251" s="8">
+        <v>1.8494037001999999</v>
+      </c>
+      <c r="I251" s="8">
+        <v>1.0402895813999999</v>
+      </c>
     </row>
     <row r="252" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A252" s="2">
@@ -8190,6 +8986,9 @@
       <c r="C252" t="s">
         <v>255</v>
       </c>
+      <c r="D252" s="2" t="s">
+        <v>313</v>
+      </c>
       <c r="F252" s="3"/>
       <c r="G252" s="3"/>
       <c r="H252" s="4"/>
@@ -8206,6 +9005,12 @@
       <c r="C253" t="s">
         <v>256</v>
       </c>
+      <c r="D253" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E253" t="s">
+        <v>359</v>
+      </c>
       <c r="F253" s="3"/>
       <c r="G253" s="3"/>
       <c r="H253" s="4"/>
@@ -8222,6 +9027,12 @@
       <c r="C254" t="s">
         <v>257</v>
       </c>
+      <c r="D254" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E254" t="s">
+        <v>360</v>
+      </c>
       <c r="F254" s="3"/>
       <c r="G254" s="3"/>
       <c r="H254" s="4"/>
@@ -8238,10 +9049,21 @@
       <c r="C255" t="s">
         <v>258</v>
       </c>
-      <c r="F255" s="3"/>
-      <c r="G255" s="3"/>
-      <c r="H255" s="4"/>
-      <c r="I255" s="4"/>
+      <c r="D255" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F255" s="3">
+        <v>-5.6126062322933903E-3</v>
+      </c>
+      <c r="G255" s="3">
+        <v>1.19068696883983E-3</v>
+      </c>
+      <c r="H255" s="4">
+        <v>19.494057513000001</v>
+      </c>
+      <c r="I255" s="4">
+        <v>10.965407351</v>
+      </c>
     </row>
     <row r="256" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A256" s="2">
@@ -8254,10 +9076,21 @@
       <c r="C256" t="s">
         <v>259</v>
       </c>
-      <c r="F256" s="3"/>
-      <c r="G256" s="3"/>
-      <c r="H256" s="4"/>
-      <c r="I256" s="4"/>
+      <c r="D256" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F256" s="3">
+        <v>0</v>
+      </c>
+      <c r="G256" s="3">
+        <v>0</v>
+      </c>
+      <c r="H256" s="4">
+        <v>4.8735143781000003</v>
+      </c>
+      <c r="I256" s="4">
+        <v>2.7413518376999999</v>
+      </c>
     </row>
     <row r="257" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A257" s="2">
@@ -8270,12 +9103,22 @@
       <c r="C257" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="D257" s="5"/>
+      <c r="D257" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E257" s="6"/>
-      <c r="F257" s="7"/>
-      <c r="G257" s="7"/>
-      <c r="H257" s="8"/>
-      <c r="I257" s="8"/>
+      <c r="F257" s="7">
+        <v>-0.22203909754190099</v>
+      </c>
+      <c r="G257" s="7">
+        <v>5.2512073606900397E-2</v>
+      </c>
+      <c r="H257" s="8">
+        <v>12.489770531</v>
+      </c>
+      <c r="I257" s="8">
+        <v>7.0254959236000003</v>
+      </c>
     </row>
     <row r="258" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A258" s="2">
@@ -8824,10 +9667,21 @@
       <c r="C291" t="s">
         <v>299</v>
       </c>
-      <c r="F291" s="3"/>
-      <c r="G291" s="3"/>
-      <c r="H291" s="4"/>
-      <c r="I291" s="4"/>
+      <c r="D291" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F291" s="3">
+        <v>0</v>
+      </c>
+      <c r="G291" s="3">
+        <v>0</v>
+      </c>
+      <c r="H291" s="4">
+        <v>12</v>
+      </c>
+      <c r="I291" s="4">
+        <v>6.75</v>
+      </c>
     </row>
     <row r="292" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A292" s="2">
@@ -8911,25 +9765,39 @@
       <c r="H296" s="8"/>
       <c r="I296" s="8"/>
     </row>
+    <row r="303" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="E303">
+        <f>294-244</f>
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I296" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}"/>
-  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D155:D161 D163:D165 D167:D192 D202:D208 D210:D212 D214:D216 D218:D226 D228:D234 D236:D242 D244:D250 D252:D256 D258:D263 D265:D269 D271 D273:D283 D285:D295 D52:D56 D133:D152">
-    <cfRule type="cellIs" dxfId="83" priority="111" operator="equal">
+  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D155:D161 D163:D165 D167:D174 D202:D208 D210:D212 D214:D216 D218:D226 D228:D234 D236:D242 D244:D250 D252:D256 D258:D263 D265:D269 D271 D273:D283 D285:D295 D52:D56 D133:D152 D176:D192">
+    <cfRule type="cellIs" dxfId="85" priority="113" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="112" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="114" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D296">
-    <cfRule type="cellIs" dxfId="81" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="45" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="46" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D43">
+    <cfRule type="cellIs" dxfId="81" priority="99" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="80" priority="100" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D51">
     <cfRule type="cellIs" dxfId="79" priority="97" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8937,15 +9805,15 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D51">
-    <cfRule type="cellIs" dxfId="77" priority="95" operator="equal">
+  <conditionalFormatting sqref="D132">
+    <cfRule type="cellIs" dxfId="77" priority="81" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="96" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="82" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D132">
+  <conditionalFormatting sqref="D153:D154">
     <cfRule type="cellIs" dxfId="75" priority="79" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8953,7 +9821,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D153:D154">
+  <conditionalFormatting sqref="D162">
     <cfRule type="cellIs" dxfId="73" priority="77" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8961,7 +9829,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D162">
+  <conditionalFormatting sqref="D166">
     <cfRule type="cellIs" dxfId="71" priority="75" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8969,7 +9837,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D166">
+  <conditionalFormatting sqref="D193">
     <cfRule type="cellIs" dxfId="69" priority="73" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -8977,23 +9845,23 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D193">
-    <cfRule type="cellIs" dxfId="67" priority="71" operator="equal">
+  <conditionalFormatting sqref="D201">
+    <cfRule type="cellIs" dxfId="67" priority="41" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="72" operator="equal">
-      <formula>"Pass"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D201">
-    <cfRule type="cellIs" dxfId="65" priority="39" operator="equal">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="40" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="42" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D209">
+    <cfRule type="cellIs" dxfId="65" priority="71" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="72" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D213">
     <cfRule type="cellIs" dxfId="63" priority="69" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9001,7 +9869,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D213">
+  <conditionalFormatting sqref="D217">
     <cfRule type="cellIs" dxfId="61" priority="67" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9009,7 +9877,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D217">
+  <conditionalFormatting sqref="D227">
     <cfRule type="cellIs" dxfId="59" priority="65" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9017,7 +9885,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D227">
+  <conditionalFormatting sqref="D235">
     <cfRule type="cellIs" dxfId="57" priority="63" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9025,7 +9893,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D235">
+  <conditionalFormatting sqref="D243">
     <cfRule type="cellIs" dxfId="55" priority="61" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9033,15 +9901,15 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D243">
-    <cfRule type="cellIs" dxfId="53" priority="59" operator="equal">
+  <conditionalFormatting sqref="D251">
+    <cfRule type="cellIs" dxfId="53" priority="57" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="60" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="58" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D251">
+  <conditionalFormatting sqref="D257">
     <cfRule type="cellIs" dxfId="51" priority="55" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9049,7 +9917,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D257">
+  <conditionalFormatting sqref="D264">
     <cfRule type="cellIs" dxfId="49" priority="53" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9057,7 +9925,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D264">
+  <conditionalFormatting sqref="D270">
     <cfRule type="cellIs" dxfId="47" priority="51" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9065,7 +9933,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D270">
+  <conditionalFormatting sqref="D272">
     <cfRule type="cellIs" dxfId="45" priority="49" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9073,7 +9941,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D272">
+  <conditionalFormatting sqref="D284">
     <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9081,23 +9949,23 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D284">
-    <cfRule type="cellIs" dxfId="41" priority="45" operator="equal">
+  <conditionalFormatting sqref="D194:D200">
+    <cfRule type="cellIs" dxfId="41" priority="43" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="46" operator="equal">
-      <formula>"Pass"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D194:D200">
-    <cfRule type="cellIs" dxfId="39" priority="41" operator="equal">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="44" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D8">
+    <cfRule type="cellIs" dxfId="39" priority="39" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="40" operator="equal">
+      <formula>"Pass"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9:D13 D15:D16 D18:D19">
     <cfRule type="cellIs" dxfId="37" priority="37" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9105,7 +9973,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D9:D13 D15:D16 D18:D19">
+  <conditionalFormatting sqref="D20">
     <cfRule type="cellIs" dxfId="35" priority="35" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9113,7 +9981,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D20">
+  <conditionalFormatting sqref="D14">
     <cfRule type="cellIs" dxfId="33" priority="33" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9121,7 +9989,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D14">
+  <conditionalFormatting sqref="D17">
     <cfRule type="cellIs" dxfId="31" priority="31" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9129,7 +9997,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D17">
+  <conditionalFormatting sqref="D21:D22">
     <cfRule type="cellIs" dxfId="29" priority="29" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9137,7 +10005,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D21:D22">
+  <conditionalFormatting sqref="D23:D34">
     <cfRule type="cellIs" dxfId="27" priority="27" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9145,7 +10013,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D23:D34">
+  <conditionalFormatting sqref="D35:D38">
     <cfRule type="cellIs" dxfId="25" priority="25" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9153,7 +10021,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D35:D38">
+  <conditionalFormatting sqref="D39">
     <cfRule type="cellIs" dxfId="23" priority="23" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9161,7 +10029,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D39">
+  <conditionalFormatting sqref="D42">
     <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9169,7 +10037,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D42">
+  <conditionalFormatting sqref="D57:D63">
     <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9177,7 +10045,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D57:D63">
+  <conditionalFormatting sqref="D64:D66">
     <cfRule type="cellIs" dxfId="17" priority="17" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9185,7 +10053,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D64:D66">
+  <conditionalFormatting sqref="D67">
     <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9193,7 +10061,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D67">
+  <conditionalFormatting sqref="D69:D74 D76:D78">
     <cfRule type="cellIs" dxfId="13" priority="13" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9201,7 +10069,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D69:D74 D76:D78">
+  <conditionalFormatting sqref="D75">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9209,7 +10077,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D75">
+  <conditionalFormatting sqref="D79:D86">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9217,7 +10085,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D79:D86">
+  <conditionalFormatting sqref="D87:D104">
     <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9225,7 +10093,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D87:D104">
+  <conditionalFormatting sqref="D105:D109">
     <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9233,7 +10101,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D105:D109">
+  <conditionalFormatting sqref="D110:D113">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9241,7 +10109,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D110:D113">
+  <conditionalFormatting sqref="D175">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Modifications to center coordinates and viewport scale (a.k.a, Viewport Tuning) for fractals numbered #153 thru #262 .  Purpose is to start the user at the top level of a visualization, where the structure is just beginning to emerge.  The assumption is that the user wants to see from the start, down to smaller scales, how the fractal is structured.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B3B3F2-7C79-4272-9767-1A822803F5AB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA3C202B-4365-4054-BB14-9FF95974417D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FractalRegistry" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$I$296</definedName>
-    <definedName name="Data">FractalRegistry!$A$1:$I$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$K$297</definedName>
+    <definedName name="Data">FractalRegistry!$A$1:$K$297</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="885" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="372">
   <si>
     <t>Group Name</t>
   </si>
@@ -1076,37 +1077,70 @@
     <t>double mandelbrot</t>
   </si>
   <si>
+    <t>no difference with previous?</t>
+  </si>
+  <si>
+    <t>nice</t>
+  </si>
+  <si>
+    <t>amazing full screen of texture</t>
+  </si>
+  <si>
+    <t>yet another mandelbrot</t>
+  </si>
+  <si>
+    <t>VP Tuning Status</t>
+  </si>
+  <si>
+    <t>APPLIED</t>
+  </si>
+  <si>
+    <t>FORMULA FIXED</t>
+  </si>
+  <si>
+    <t>NOT APPLIED</t>
+  </si>
+  <si>
+    <t>N/A (no coordinates)</t>
+  </si>
+  <si>
+    <t>IMPROVED + NOT APPLIED</t>
+  </si>
+  <si>
+    <t>Resubmit with same numbers</t>
+  </si>
+  <si>
+    <t>Do not resubmit or Take no action</t>
+  </si>
+  <si>
+    <t>Resubmit with NEW numbers</t>
+  </si>
+  <si>
+    <t>Do not resubmit, action finished</t>
+  </si>
+  <si>
+    <t>full screen coverage</t>
+  </si>
+  <si>
+    <t>glowing green and blue Mandelbrot</t>
+  </si>
+  <si>
+    <t>this is not the Buddahbrot shape.  It is the classic Mandelbrot shape, but's worth saving somehow</t>
+  </si>
+  <si>
+    <t>Resubmit with NEW numbers; generated</t>
+  </si>
+  <si>
+    <t>looks identical to Minimum Distance</t>
+  </si>
+  <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>black screen, no structure</t>
-  </si>
-  <si>
-    <t>no difference with previous?</t>
-  </si>
-  <si>
-    <t>nice</t>
-  </si>
-  <si>
-    <t>only concentric circles at very small scale</t>
-  </si>
-  <si>
-    <t>nothing but concentric circles</t>
-  </si>
-  <si>
-    <t>amazing full screen of texture</t>
-  </si>
-  <si>
-    <t>solid color screen no structure</t>
-  </si>
-  <si>
-    <t>yet another mandelbrot</t>
-  </si>
-  <si>
-    <t>this is not the Buddahbrot shape.  It is the classic Mandelbrot shape</t>
-  </si>
-  <si>
-    <t>Are we supposed to see vertical bands of colors, only?</t>
+    <t>check the computations; black disk with a green crescent edge.  No fine structure; original Bessel disk with waves and striations is gone</t>
+  </si>
+  <si>
+    <t>Mark's Action?</t>
   </si>
 </sst>
 </file>
@@ -1252,7 +1286,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="37">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1453,6 +1487,9 @@
     <fill>
       <patternFill patternType="lightUp"/>
     </fill>
+    <fill>
+      <patternFill patternType="lightDown"/>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -1643,7 +1680,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1719,6 +1756,19 @@
     <xf numFmtId="2" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2677,22 +2727,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I303"/>
+  <dimension ref="A1:K304"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.3984375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="19.9296875" customWidth="1"/>
-    <col min="3" max="3" width="16.46484375" customWidth="1"/>
+    <col min="2" max="2" width="15.1328125" customWidth="1"/>
+    <col min="3" max="3" width="17.59765625" customWidth="1"/>
     <col min="4" max="4" width="6.46484375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.6640625" customWidth="1"/>
+    <col min="5" max="5" width="5.796875" customWidth="1"/>
     <col min="6" max="6" width="6.3984375" customWidth="1"/>
     <col min="7" max="7" width="6.46484375" customWidth="1"/>
-    <col min="8" max="8" width="17.53125" customWidth="1"/>
-    <col min="9" max="9" width="17.265625" customWidth="1"/>
-    <col min="10" max="10" width="2.3984375" customWidth="1"/>
+    <col min="8" max="8" width="16.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.86328125" customWidth="1"/>
+    <col min="10" max="10" width="21.9296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.9" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
         <v>305</v>
       </c>
@@ -2720,8 +2771,14 @@
       <c r="I1" s="1" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J1" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="K1" s="36" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -2739,7 +2796,7 @@
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <f>A2+1</f>
         <v>2</v>
@@ -2758,7 +2815,7 @@
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <f t="shared" ref="A4:A67" si="0">A3+1</f>
         <v>3</v>
@@ -2777,7 +2834,7 @@
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2796,7 +2853,7 @@
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2815,7 +2872,7 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2834,7 +2891,7 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2854,7 +2911,7 @@
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2874,7 +2931,7 @@
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2894,7 +2951,7 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2914,7 +2971,7 @@
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2934,7 +2991,7 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2954,7 +3011,7 @@
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="14" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A14" s="9">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2974,7 +3031,7 @@
       <c r="H14" s="8"/>
       <c r="I14" s="8"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2994,7 +3051,7 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -3700,7 +3757,7 @@
       <c r="H48" s="23"/>
       <c r="I48" s="23"/>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A49" s="2">
         <f t="shared" si="0"/>
         <v>48</v>
@@ -3719,7 +3776,7 @@
       <c r="H49" s="23"/>
       <c r="I49" s="23"/>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <f t="shared" si="0"/>
         <v>49</v>
@@ -3738,7 +3795,7 @@
       <c r="H50" s="23"/>
       <c r="I50" s="23"/>
     </row>
-    <row r="51" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="51" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A51" s="9">
         <f t="shared" si="0"/>
         <v>50</v>
@@ -3758,7 +3815,7 @@
       <c r="H51" s="24"/>
       <c r="I51" s="24"/>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <f t="shared" si="0"/>
         <v>51</v>
@@ -3777,7 +3834,7 @@
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <f t="shared" si="0"/>
         <v>52</v>
@@ -3796,7 +3853,7 @@
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <f t="shared" si="0"/>
         <v>53</v>
@@ -3815,7 +3872,7 @@
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
     </row>
-    <row r="55" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="55" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A55" s="9">
         <f t="shared" si="0"/>
         <v>54</v>
@@ -3835,7 +3892,7 @@
       <c r="H55" s="8"/>
       <c r="I55" s="8"/>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A56" s="22">
         <f t="shared" si="0"/>
         <v>55</v>
@@ -3862,7 +3919,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <f t="shared" si="0"/>
         <v>56</v>
@@ -3890,7 +3947,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3918,7 +3975,7 @@
         <v>2.3420689813000002</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A59" s="2">
         <f t="shared" si="0"/>
         <v>58</v>
@@ -3946,7 +4003,7 @@
         <v>1.8436548223</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <f t="shared" si="0"/>
         <v>59</v>
@@ -3974,7 +4031,7 @@
         <v>2.3309644980000002</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <f t="shared" si="0"/>
         <v>60</v>
@@ -4002,7 +4059,7 @@
         <v>1.4659263959</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2">
         <f t="shared" si="0"/>
         <v>61</v>
@@ -4024,7 +4081,7 @@
       <c r="H62" s="4"/>
       <c r="I62" s="4"/>
     </row>
-    <row r="63" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="63" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A63" s="9">
         <f t="shared" si="0"/>
         <v>62</v>
@@ -4051,8 +4108,9 @@
       <c r="I63" s="8">
         <v>0.28801632742</v>
       </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J63" s="6"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A64" s="2">
         <f t="shared" si="0"/>
         <v>63</v>
@@ -4080,7 +4138,7 @@
         <v>1.4659263959</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <f t="shared" si="0"/>
         <v>64</v>
@@ -4098,7 +4156,7 @@
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
     </row>
-    <row r="66" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="66" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A66" s="9">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -4125,8 +4183,9 @@
       <c r="I66" s="8">
         <v>2.397631133</v>
       </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J66" s="6"/>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <f t="shared" si="0"/>
         <v>66</v>
@@ -4154,7 +4213,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A68" s="22">
         <f t="shared" ref="A68:A131" si="1">A67+1</f>
         <v>67</v>
@@ -4181,7 +4240,7 @@
         <v>8.4375</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <f t="shared" si="1"/>
         <v>68</v>
@@ -4201,7 +4260,7 @@
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A70" s="2">
         <f t="shared" si="1"/>
         <v>69</v>
@@ -4229,7 +4288,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A71" s="2">
         <f t="shared" si="1"/>
         <v>70</v>
@@ -4249,7 +4308,7 @@
       <c r="H71" s="4"/>
       <c r="I71" s="4"/>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A72" s="2">
         <f t="shared" si="1"/>
         <v>71</v>
@@ -4277,7 +4336,7 @@
         <v>6.75</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A73" s="2">
         <f t="shared" si="1"/>
         <v>72</v>
@@ -4305,7 +4364,7 @@
         <v>21.025059204000002</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <f t="shared" si="1"/>
         <v>73</v>
@@ -4333,7 +4392,7 @@
         <v>0.2109375</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A75" s="2">
         <f t="shared" si="1"/>
         <v>74</v>
@@ -4361,7 +4420,7 @@
         <v>1.0884495317</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A76" s="2">
         <f t="shared" si="1"/>
         <v>75</v>
@@ -4389,7 +4448,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A77" s="2">
         <f t="shared" si="1"/>
         <v>76</v>
@@ -4417,7 +4476,7 @@
         <v>1.4678492578</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="78" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A78" s="9">
         <f t="shared" si="1"/>
         <v>77</v>
@@ -4444,8 +4503,9 @@
       <c r="I78" s="8">
         <v>0.84375</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J78" s="6"/>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <f t="shared" si="1"/>
         <v>78</v>
@@ -4465,7 +4525,7 @@
       <c r="H79" s="4"/>
       <c r="I79" s="4"/>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <f t="shared" si="1"/>
         <v>79</v>
@@ -4911,7 +4971,7 @@
         <v>4.6783144913000001</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <f t="shared" si="1"/>
         <v>96</v>
@@ -4931,7 +4991,7 @@
       <c r="H97" s="4"/>
       <c r="I97" s="4"/>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <f t="shared" si="1"/>
         <v>97</v>
@@ -4959,7 +5019,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <f t="shared" si="1"/>
         <v>98</v>
@@ -4987,7 +5047,7 @@
         <v>6.1130526660999998</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A100" s="2">
         <f t="shared" si="1"/>
         <v>99</v>
@@ -5015,7 +5075,7 @@
         <v>11.25</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="20.65" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:10" ht="20.65" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <f t="shared" si="1"/>
         <v>100</v>
@@ -5043,7 +5103,7 @@
         <v>4.21875</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
         <f t="shared" si="1"/>
         <v>101</v>
@@ -5071,7 +5131,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
         <f t="shared" si="1"/>
         <v>102</v>
@@ -5099,7 +5159,7 @@
         <v>1.0194922309000001</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="104" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A104" s="9">
         <f t="shared" si="1"/>
         <v>103</v>
@@ -5126,8 +5186,9 @@
       <c r="I104" s="8">
         <v>2.3396227092999999</v>
       </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J104" s="6"/>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
         <f t="shared" si="1"/>
         <v>104</v>
@@ -5155,7 +5216,7 @@
         <v>11.028960818</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
         <f t="shared" si="1"/>
         <v>105</v>
@@ -5183,7 +5244,7 @@
         <v>1.1422222222</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
         <f t="shared" si="1"/>
         <v>106</v>
@@ -5211,7 +5272,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
         <f t="shared" si="1"/>
         <v>107</v>
@@ -5239,7 +5300,7 @@
         <v>1.125</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="109" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A109" s="9">
         <f t="shared" si="1"/>
         <v>108</v>
@@ -5266,8 +5327,9 @@
       <c r="I109" s="8">
         <v>0.82935879629999998</v>
       </c>
-    </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J109" s="6"/>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
         <f t="shared" si="1"/>
         <v>109</v>
@@ -5295,7 +5357,7 @@
         <v>2.4900562852000001</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
         <f t="shared" si="1"/>
         <v>110</v>
@@ -5323,7 +5385,7 @@
         <v>2.2581613508</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
         <f t="shared" si="1"/>
         <v>111</v>
@@ -5776,7 +5838,7 @@
         <v>2.3746537395999998</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <f t="shared" si="1"/>
         <v>128</v>
@@ -5803,7 +5865,7 @@
         <v>2.4515236091000001</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <f t="shared" si="1"/>
         <v>129</v>
@@ -5830,7 +5892,7 @@
         <v>2.2475570032999999</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <f t="shared" si="1"/>
         <v>130</v>
@@ -5857,7 +5919,7 @@
         <v>2.237534626</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="132" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A132" s="9">
         <f t="shared" ref="A132:A205" si="2">A131+1</f>
         <v>131</v>
@@ -5884,8 +5946,9 @@
       <c r="I132" s="8">
         <v>2.3891966918</v>
       </c>
-    </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J132" s="6"/>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A133" s="2">
         <f t="shared" si="2"/>
         <v>132</v>
@@ -5904,7 +5967,7 @@
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A134" s="2">
         <f t="shared" si="2"/>
         <v>133</v>
@@ -5931,7 +5994,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A135" s="2">
         <f t="shared" si="2"/>
         <v>134</v>
@@ -5958,7 +6021,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A136" s="2">
         <f t="shared" si="2"/>
         <v>135</v>
@@ -5977,7 +6040,7 @@
       <c r="H136" s="4"/>
       <c r="I136" s="4"/>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A137" s="2">
         <f t="shared" si="2"/>
         <v>136</v>
@@ -6004,7 +6067,7 @@
         <v>2.5051334684</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A138" s="2">
         <f t="shared" si="2"/>
         <v>137</v>
@@ -6031,7 +6094,7 @@
         <v>2.2266695994000001</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A139" s="2">
         <f t="shared" si="2"/>
         <v>138</v>
@@ -6050,7 +6113,7 @@
       <c r="H139" s="4"/>
       <c r="I139" s="4"/>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A140" s="2">
         <f t="shared" si="2"/>
         <v>139</v>
@@ -6077,7 +6140,7 @@
         <v>21.621621621999999</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A141" s="29">
         <f t="shared" si="2"/>
         <v>140</v>
@@ -6107,7 +6170,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A142" s="29">
         <f t="shared" si="2"/>
         <v>141</v>
@@ -6137,7 +6200,7 @@
         <v>3.375</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A143" s="2">
         <f t="shared" si="2"/>
         <v>142</v>
@@ -6164,7 +6227,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A144" s="2">
         <f t="shared" si="2"/>
         <v>143</v>
@@ -6191,7 +6254,7 @@
         <v>2.4114902907000002</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A145" s="29">
         <f t="shared" si="2"/>
         <v>144</v>
@@ -6221,7 +6284,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A146" s="2">
         <f t="shared" si="2"/>
         <v>145</v>
@@ -6248,7 +6311,7 @@
         <v>3.3313313312999999</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" s="29">
         <f t="shared" si="2"/>
         <v>146</v>
@@ -6278,7 +6341,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A148" s="2">
         <f t="shared" si="2"/>
         <v>147</v>
@@ -6308,7 +6371,7 @@
         <v>3.3313313309999999</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A149" s="2">
         <f t="shared" si="2"/>
         <v>148</v>
@@ -6335,7 +6398,7 @@
         <v>1.6875</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A150" s="2">
         <f t="shared" si="2"/>
         <v>149</v>
@@ -6362,7 +6425,7 @@
         <v>2.0775561974999999</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A151" s="2">
         <f t="shared" si="2"/>
         <v>150</v>
@@ -6392,7 +6455,7 @@
         <v>2.0775561974999999</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A152" s="2">
         <f t="shared" si="2"/>
         <v>151</v>
@@ -6422,7 +6485,7 @@
         <v>12.595945386</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="153" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A153" s="9">
         <f t="shared" si="2"/>
         <v>152</v>
@@ -6450,7 +6513,7 @@
         <v>1.808617718</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:11" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="A154" s="9"/>
       <c r="B154" s="30"/>
       <c r="C154" s="30"/>
@@ -6461,7 +6524,7 @@
       <c r="H154" s="33"/>
       <c r="I154" s="33"/>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A155" s="2">
         <f>A153+1</f>
         <v>153</v>
@@ -6490,8 +6553,14 @@
       <c r="I155" s="4">
         <v>3.375</v>
       </c>
-    </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J155" t="s">
+        <v>355</v>
+      </c>
+      <c r="K155" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A156" s="2">
         <f t="shared" si="2"/>
         <v>154</v>
@@ -6503,17 +6572,28 @@
         <v>169</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E156" t="s">
-        <v>351</v>
-      </c>
-      <c r="F156" s="3"/>
-      <c r="G156" s="3"/>
-      <c r="H156" s="4"/>
-      <c r="I156" s="4"/>
-    </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F156" s="3">
+        <v>-3.9525691699608904E-3</v>
+      </c>
+      <c r="G156" s="3">
+        <v>6.9169960474309402E-3</v>
+      </c>
+      <c r="H156" s="4">
+        <v>6</v>
+      </c>
+      <c r="I156" s="4">
+        <v>3.375</v>
+      </c>
+      <c r="J156" t="s">
+        <v>356</v>
+      </c>
+      <c r="K156" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A157" s="2">
         <f t="shared" si="2"/>
         <v>155</v>
@@ -6525,17 +6605,29 @@
         <v>170</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E157" s="34" t="s">
-        <v>351</v>
-      </c>
-      <c r="F157" s="3"/>
-      <c r="G157" s="3"/>
-      <c r="H157" s="4"/>
-      <c r="I157" s="4"/>
-    </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="E157" s="34"/>
+      <c r="F157" s="3">
+        <v>0.80330705765450305</v>
+      </c>
+      <c r="G157" s="3">
+        <v>7.0312499999999898E-3</v>
+      </c>
+      <c r="H157" s="4">
+        <v>5.2233033797999999</v>
+      </c>
+      <c r="I157" s="4">
+        <v>2.9381081510999998</v>
+      </c>
+      <c r="J157" t="s">
+        <v>356</v>
+      </c>
+      <c r="K157" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A158" s="2">
         <f t="shared" si="2"/>
         <v>156</v>
@@ -6547,17 +6639,28 @@
         <v>171</v>
       </c>
       <c r="D158" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E158" t="s">
-        <v>351</v>
-      </c>
-      <c r="F158" s="3"/>
-      <c r="G158" s="3"/>
-      <c r="H158" s="4"/>
-      <c r="I158" s="4"/>
-    </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F158" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G158" s="3">
+        <v>0</v>
+      </c>
+      <c r="H158" s="4">
+        <v>25.722563100999999</v>
+      </c>
+      <c r="I158" s="4">
+        <v>14.468941744</v>
+      </c>
+      <c r="J158" t="s">
+        <v>356</v>
+      </c>
+      <c r="K158" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="159" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A159" s="2">
         <f t="shared" si="2"/>
         <v>157</v>
@@ -6569,17 +6672,28 @@
         <v>172</v>
       </c>
       <c r="D159" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E159" t="s">
-        <v>351</v>
-      </c>
-      <c r="F159" s="3"/>
-      <c r="G159" s="3"/>
-      <c r="H159" s="4"/>
-      <c r="I159" s="4"/>
-    </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F159" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="G159" s="3">
+        <v>0</v>
+      </c>
+      <c r="H159" s="4">
+        <v>55.137521040000003</v>
+      </c>
+      <c r="I159" s="4">
+        <v>31.014855584999999</v>
+      </c>
+      <c r="J159" t="s">
+        <v>356</v>
+      </c>
+      <c r="K159" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="160" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A160" s="2">
         <f t="shared" si="2"/>
         <v>158</v>
@@ -6591,17 +6705,28 @@
         <v>173</v>
       </c>
       <c r="D160" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E160" t="s">
-        <v>351</v>
-      </c>
-      <c r="F160" s="3"/>
-      <c r="G160" s="3"/>
-      <c r="H160" s="4"/>
-      <c r="I160" s="4"/>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F160" s="3">
+        <v>-6.9169960474308206E-2</v>
+      </c>
+      <c r="G160" s="3">
+        <v>8.8932806324111005E-2</v>
+      </c>
+      <c r="H160" s="4">
+        <v>12</v>
+      </c>
+      <c r="I160" s="4">
+        <v>6.75</v>
+      </c>
+      <c r="J160" t="s">
+        <v>356</v>
+      </c>
+      <c r="K160" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="161" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A161" s="2">
         <f t="shared" si="2"/>
         <v>159</v>
@@ -6613,17 +6738,28 @@
         <v>174</v>
       </c>
       <c r="D161" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E161" t="s">
-        <v>351</v>
-      </c>
-      <c r="F161" s="3"/>
-      <c r="G161" s="3"/>
-      <c r="H161" s="4"/>
-      <c r="I161" s="4"/>
-    </row>
-    <row r="162" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>313</v>
+      </c>
+      <c r="F161" s="3">
+        <v>-5.1937595141288803E-2</v>
+      </c>
+      <c r="G161" s="3">
+        <v>4.36566380910271E-2</v>
+      </c>
+      <c r="H161" s="4">
+        <v>2.6986537192000002</v>
+      </c>
+      <c r="I161" s="4">
+        <v>15.179927169999999</v>
+      </c>
+      <c r="J161" t="s">
+        <v>356</v>
+      </c>
+      <c r="K161" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A162" s="9">
         <f t="shared" si="2"/>
         <v>160</v>
@@ -6635,17 +6771,29 @@
         <v>175</v>
       </c>
       <c r="D162" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="E162" s="6" t="s">
-        <v>351</v>
-      </c>
-      <c r="F162" s="7"/>
-      <c r="G162" s="7"/>
-      <c r="H162" s="8"/>
-      <c r="I162" s="8"/>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="E162" s="6"/>
+      <c r="F162" s="7">
+        <v>-5.0217764515757303E-2</v>
+      </c>
+      <c r="G162" s="7">
+        <v>2.9605211767096198E-2</v>
+      </c>
+      <c r="H162" s="8">
+        <v>29.512516469000001</v>
+      </c>
+      <c r="I162" s="8">
+        <v>16.600790514</v>
+      </c>
+      <c r="J162" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="K162" s="6" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="163" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A163" s="2">
         <f t="shared" si="2"/>
         <v>161</v>
@@ -6671,8 +6819,14 @@
       <c r="I163" s="4">
         <v>6.586265569</v>
       </c>
-    </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J163" t="s">
+        <v>357</v>
+      </c>
+      <c r="K163" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A164" s="2">
         <f t="shared" si="2"/>
         <v>162</v>
@@ -6698,8 +6852,14 @@
       <c r="I164" s="4">
         <v>8.9511889862</v>
       </c>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J164" t="s">
+        <v>357</v>
+      </c>
+      <c r="K164" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A165" s="2">
         <f t="shared" si="2"/>
         <v>163</v>
@@ -6725,8 +6885,14 @@
       <c r="I165" s="4">
         <v>5.5349445396999999E-2</v>
       </c>
-    </row>
-    <row r="166" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J165" t="s">
+        <v>357</v>
+      </c>
+      <c r="K165" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="166" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A166" s="9">
         <f t="shared" si="2"/>
         <v>164</v>
@@ -6753,8 +6919,14 @@
       <c r="I166" s="8">
         <v>5.6862031442999998E-2</v>
       </c>
-    </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J166" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K166" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="167" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A167" s="2">
         <f t="shared" si="2"/>
         <v>165</v>
@@ -6780,8 +6952,14 @@
       <c r="I167" s="4">
         <v>1</v>
       </c>
-    </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J167" t="s">
+        <v>357</v>
+      </c>
+      <c r="K167" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A168" s="25">
         <f t="shared" si="2"/>
         <v>166</v>
@@ -6807,8 +6985,14 @@
       <c r="I168" s="4">
         <v>0.35355339059000002</v>
       </c>
-    </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J168" t="s">
+        <v>357</v>
+      </c>
+      <c r="K168" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="169" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A169" s="2">
         <f t="shared" si="2"/>
         <v>167</v>
@@ -6834,8 +7018,14 @@
       <c r="I169" s="4">
         <v>0.31028368794</v>
       </c>
-    </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J169" t="s">
+        <v>357</v>
+      </c>
+      <c r="K169" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A170" s="2">
         <f t="shared" si="2"/>
         <v>168</v>
@@ -6861,8 +7051,14 @@
       <c r="I170" s="4">
         <v>1.125</v>
       </c>
-    </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J170" t="s">
+        <v>357</v>
+      </c>
+      <c r="K170" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="171" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A171" s="2">
         <f t="shared" si="2"/>
         <v>169</v>
@@ -6888,8 +7084,14 @@
       <c r="I171" s="4">
         <v>2.7833369992999999</v>
       </c>
-    </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J171" t="s">
+        <v>357</v>
+      </c>
+      <c r="K171" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="172" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A172" s="2">
         <f t="shared" si="2"/>
         <v>170</v>
@@ -6915,8 +7117,14 @@
       <c r="I172" s="4">
         <v>4.4533391989000002</v>
       </c>
-    </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J172" t="s">
+        <v>357</v>
+      </c>
+      <c r="K172" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="173" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A173" s="2">
         <f t="shared" si="2"/>
         <v>171</v>
@@ -6942,8 +7150,14 @@
       <c r="I173" s="4">
         <v>3.375</v>
       </c>
-    </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J173" t="s">
+        <v>357</v>
+      </c>
+      <c r="K173" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="174" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A174" s="2">
         <f t="shared" si="2"/>
         <v>172</v>
@@ -6969,8 +7183,14 @@
       <c r="I174" s="4">
         <v>2.2607721475</v>
       </c>
-    </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J174" t="s">
+        <v>357</v>
+      </c>
+      <c r="K174" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="175" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A175" s="2">
         <f t="shared" si="2"/>
         <v>173</v>
@@ -6982,17 +7202,28 @@
         <v>189</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E175" t="s">
-        <v>351</v>
-      </c>
-      <c r="F175" s="3"/>
-      <c r="G175" s="3"/>
-      <c r="H175" s="4"/>
-      <c r="I175" s="4"/>
-    </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F175" s="3">
+        <v>0.99957651044607498</v>
+      </c>
+      <c r="G175" s="3">
+        <v>6.3523433088651503E-3</v>
+      </c>
+      <c r="H175" s="4">
+        <v>6.0609152673000004</v>
+      </c>
+      <c r="I175" s="4">
+        <v>3.4092648378999999</v>
+      </c>
+      <c r="J175" t="s">
+        <v>356</v>
+      </c>
+      <c r="K175" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A176" s="2">
         <f t="shared" si="2"/>
         <v>174</v>
@@ -7010,8 +7241,14 @@
       <c r="G176" s="3"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
-    </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J176" t="s">
+        <v>358</v>
+      </c>
+      <c r="K176" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="177" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A177" s="2">
         <f t="shared" si="2"/>
         <v>175</v>
@@ -7029,8 +7266,14 @@
       <c r="G177" s="3"/>
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
-    </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J177" t="s">
+        <v>358</v>
+      </c>
+      <c r="K177" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="178" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A178" s="2">
         <f t="shared" si="2"/>
         <v>176</v>
@@ -7056,8 +7299,14 @@
       <c r="I178" s="4">
         <v>2.3864853865</v>
       </c>
-    </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J178" t="s">
+        <v>357</v>
+      </c>
+      <c r="K178" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="179" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A179" s="2">
         <f t="shared" si="2"/>
         <v>177</v>
@@ -7072,13 +7321,13 @@
         <v>313</v>
       </c>
       <c r="E179" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F179" s="3">
-        <v>-0.36784607040524497</v>
+        <v>-0.394574846588925</v>
       </c>
       <c r="G179" s="3">
-        <v>-1.0777737655028299E-3</v>
+        <v>-1.6110981627733001E-3</v>
       </c>
       <c r="H179" s="4">
         <v>3.6934332400000001</v>
@@ -7086,8 +7335,14 @@
       <c r="I179" s="4">
         <v>2.0775561974999999</v>
       </c>
-    </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J179" t="s">
+        <v>359</v>
+      </c>
+      <c r="K179" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="180" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A180" s="2">
         <f t="shared" si="2"/>
         <v>178</v>
@@ -7113,8 +7368,14 @@
       <c r="I180" s="4">
         <v>2.5</v>
       </c>
-    </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J180" t="s">
+        <v>357</v>
+      </c>
+      <c r="K180" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="181" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A181" s="2">
         <f t="shared" si="2"/>
         <v>179</v>
@@ -7140,8 +7401,14 @@
       <c r="I181" s="4">
         <v>2.4114902907000002</v>
       </c>
-    </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J181" t="s">
+        <v>357</v>
+      </c>
+      <c r="K181" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="182" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A182" s="2">
         <f t="shared" si="2"/>
         <v>180</v>
@@ -7167,8 +7434,14 @@
       <c r="I182" s="4">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J182" t="s">
+        <v>357</v>
+      </c>
+      <c r="K182" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="183" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A183" s="2">
         <f t="shared" si="2"/>
         <v>181</v>
@@ -7194,8 +7467,14 @@
       <c r="I183" s="4">
         <v>3.0670104666000002</v>
       </c>
-    </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J183" t="s">
+        <v>357</v>
+      </c>
+      <c r="K183" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="184" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A184" s="2">
         <f t="shared" si="2"/>
         <v>182</v>
@@ -7221,8 +7500,14 @@
       <c r="I184" s="4">
         <v>2.4107142857000001</v>
       </c>
-    </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J184" t="s">
+        <v>357</v>
+      </c>
+      <c r="K184" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="185" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A185" s="2">
         <f t="shared" si="2"/>
         <v>183</v>
@@ -7248,8 +7533,14 @@
       <c r="I185" s="4">
         <v>2.5961538462</v>
       </c>
-    </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J185" t="s">
+        <v>357</v>
+      </c>
+      <c r="K185" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="186" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A186" s="2">
         <f t="shared" si="2"/>
         <v>184</v>
@@ -7275,8 +7566,14 @@
       <c r="I186" s="4">
         <v>2.5759451010999999</v>
       </c>
-    </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J186" t="s">
+        <v>357</v>
+      </c>
+      <c r="K186" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="187" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A187" s="2">
         <f t="shared" si="2"/>
         <v>185</v>
@@ -7302,8 +7599,14 @@
       <c r="I187" s="4">
         <v>0.28125</v>
       </c>
-    </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J187" t="s">
+        <v>357</v>
+      </c>
+      <c r="K187" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="188" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A188" s="2">
         <f t="shared" si="2"/>
         <v>186</v>
@@ -7318,7 +7621,7 @@
         <v>313</v>
       </c>
       <c r="E188" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F188" s="3">
         <v>-0.58828124999999898</v>
@@ -7332,8 +7635,14 @@
       <c r="I188" s="4">
         <v>1.6875</v>
       </c>
-    </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J188" t="s">
+        <v>357</v>
+      </c>
+      <c r="K188" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="189" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A189" s="2">
         <f t="shared" si="2"/>
         <v>187</v>
@@ -7359,8 +7668,14 @@
       <c r="I189" s="4">
         <v>2.7413518250000002</v>
       </c>
-    </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J189" t="s">
+        <v>357</v>
+      </c>
+      <c r="K189" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="190" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A190" s="2">
         <f t="shared" si="2"/>
         <v>188</v>
@@ -7386,8 +7701,14 @@
       <c r="I190" s="4">
         <v>3.375</v>
       </c>
-    </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J190" t="s">
+        <v>357</v>
+      </c>
+      <c r="K190" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="191" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A191" s="2">
         <f t="shared" si="2"/>
         <v>189</v>
@@ -7399,17 +7720,28 @@
         <v>202</v>
       </c>
       <c r="D191" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E191" t="s">
-        <v>354</v>
-      </c>
-      <c r="F191" s="3"/>
-      <c r="G191" s="3"/>
-      <c r="H191" s="4"/>
-      <c r="I191" s="4"/>
-    </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F191" s="3">
+        <v>-1.8681088587872701E-3</v>
+      </c>
+      <c r="G191" s="3">
+        <v>1.45213559590144E-3</v>
+      </c>
+      <c r="H191" s="4">
+        <v>0.87583915586000005</v>
+      </c>
+      <c r="I191" s="4">
+        <v>0.49265952517</v>
+      </c>
+      <c r="J191" t="s">
+        <v>356</v>
+      </c>
+      <c r="K191" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="192" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A192" s="2">
         <f t="shared" si="2"/>
         <v>190</v>
@@ -7435,8 +7767,14 @@
       <c r="I192" s="4">
         <v>3.9174472733000001</v>
       </c>
-    </row>
-    <row r="193" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J192" t="s">
+        <v>357</v>
+      </c>
+      <c r="K192" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="193" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A193" s="9">
         <f t="shared" si="2"/>
         <v>191</v>
@@ -7463,8 +7801,14 @@
       <c r="I193" s="8">
         <v>3.2494845361000002</v>
       </c>
-    </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J193" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K193" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="194" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A194" s="9">
         <f t="shared" si="2"/>
         <v>192</v>
@@ -7490,8 +7834,14 @@
       <c r="I194" s="4">
         <v>2.4107142857000001</v>
       </c>
-    </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J194" t="s">
+        <v>357</v>
+      </c>
+      <c r="K194" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="195" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A195" s="9">
         <f t="shared" si="2"/>
         <v>193</v>
@@ -7517,8 +7867,14 @@
       <c r="I195" s="4">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J195" t="s">
+        <v>357</v>
+      </c>
+      <c r="K195" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A196" s="9">
         <f t="shared" si="2"/>
         <v>194</v>
@@ -7544,8 +7900,14 @@
       <c r="I196" s="4">
         <v>3.0670104666000002</v>
       </c>
-    </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J196" t="s">
+        <v>357</v>
+      </c>
+      <c r="K196" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A197" s="9">
         <f t="shared" si="2"/>
         <v>195</v>
@@ -7571,8 +7933,14 @@
       <c r="I197" s="4">
         <v>2.3360824741999999</v>
       </c>
-    </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J197" t="s">
+        <v>357</v>
+      </c>
+      <c r="K197" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A198" s="9">
         <f t="shared" si="2"/>
         <v>196</v>
@@ -7598,8 +7966,14 @@
       <c r="I198" s="4">
         <v>2.2491408934999999</v>
       </c>
-    </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J198" t="s">
+        <v>357</v>
+      </c>
+      <c r="K198" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A199" s="9">
         <f t="shared" si="2"/>
         <v>197</v>
@@ -7625,8 +7999,14 @@
       <c r="I199" s="4">
         <v>2.3489294453</v>
       </c>
-    </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J199" t="s">
+        <v>357</v>
+      </c>
+      <c r="K199" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="200" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A200" s="9">
         <f t="shared" si="2"/>
         <v>198</v>
@@ -7652,8 +8032,14 @@
       <c r="I200" s="4">
         <v>2.2492759617</v>
       </c>
-    </row>
-    <row r="201" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J200" t="s">
+        <v>357</v>
+      </c>
+      <c r="K200" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="201" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A201" s="9">
         <f t="shared" si="2"/>
         <v>199</v>
@@ -7680,8 +8066,14 @@
       <c r="I201" s="8">
         <v>3.711115999</v>
       </c>
-    </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J201" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K201" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A202" s="9">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -7699,8 +8091,14 @@
       <c r="G202" s="3"/>
       <c r="H202" s="4"/>
       <c r="I202" s="4"/>
-    </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J202" t="s">
+        <v>358</v>
+      </c>
+      <c r="K202" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A203" s="9">
         <f t="shared" si="2"/>
         <v>201</v>
@@ -7718,8 +8116,14 @@
       <c r="G203" s="3"/>
       <c r="H203" s="4"/>
       <c r="I203" s="4"/>
-    </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J203" t="s">
+        <v>358</v>
+      </c>
+      <c r="K203" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A204" s="2">
         <f t="shared" si="2"/>
         <v>202</v>
@@ -7731,17 +8135,31 @@
         <v>206</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>350</v>
+        <v>313</v>
       </c>
       <c r="E204" t="s">
-        <v>355</v>
-      </c>
-      <c r="F204" s="3"/>
-      <c r="G204" s="3"/>
-      <c r="H204" s="4"/>
-      <c r="I204" s="4"/>
-    </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.45">
+        <v>364</v>
+      </c>
+      <c r="F204" s="3">
+        <v>0</v>
+      </c>
+      <c r="G204" s="3">
+        <v>0</v>
+      </c>
+      <c r="H204" s="4">
+        <v>20</v>
+      </c>
+      <c r="I204" s="4">
+        <v>11.25</v>
+      </c>
+      <c r="J204" t="s">
+        <v>356</v>
+      </c>
+      <c r="K204" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A205" s="2">
         <f t="shared" si="2"/>
         <v>203</v>
@@ -7759,10 +8177,16 @@
       <c r="G205" s="3"/>
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
-    </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J205" t="s">
+        <v>358</v>
+      </c>
+      <c r="K205" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A206" s="2">
-        <f t="shared" ref="A206:A265" si="3">A205+1</f>
+        <f t="shared" ref="A206:A264" si="3">A205+1</f>
         <v>204</v>
       </c>
       <c r="B206" t="s">
@@ -7778,8 +8202,14 @@
       <c r="G206" s="3"/>
       <c r="H206" s="4"/>
       <c r="I206" s="4"/>
-    </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J206" t="s">
+        <v>358</v>
+      </c>
+      <c r="K206" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A207" s="2">
         <f t="shared" si="3"/>
         <v>205</v>
@@ -7797,8 +8227,14 @@
       <c r="G207" s="3"/>
       <c r="H207" s="4"/>
       <c r="I207" s="4"/>
-    </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J207" t="s">
+        <v>358</v>
+      </c>
+      <c r="K207" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A208" s="2">
         <f t="shared" si="3"/>
         <v>206</v>
@@ -7813,7 +8249,7 @@
         <v>313</v>
       </c>
       <c r="E208" t="s">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="F208" s="3">
         <v>0</v>
@@ -7827,8 +8263,14 @@
       <c r="I208" s="4">
         <v>54</v>
       </c>
-    </row>
-    <row r="209" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J208" t="s">
+        <v>355</v>
+      </c>
+      <c r="K208" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="209" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A209" s="9">
         <f t="shared" si="3"/>
         <v>207</v>
@@ -7855,8 +8297,14 @@
       <c r="I209" s="8">
         <v>1.2491919844999999</v>
       </c>
-    </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J209" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K209" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A210" s="2">
         <f t="shared" si="3"/>
         <v>208</v>
@@ -7882,8 +8330,14 @@
       <c r="I210" s="4">
         <v>3.375</v>
       </c>
-    </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J210" t="s">
+        <v>357</v>
+      </c>
+      <c r="K210" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="211" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A211" s="2">
         <f t="shared" si="3"/>
         <v>209</v>
@@ -7909,8 +8363,14 @@
       <c r="I211" s="4">
         <v>3.375</v>
       </c>
-    </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J211" t="s">
+        <v>357</v>
+      </c>
+      <c r="K211" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="212" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A212" s="2">
         <f t="shared" si="3"/>
         <v>210</v>
@@ -7936,8 +8396,14 @@
       <c r="I212" s="4">
         <v>3.375</v>
       </c>
-    </row>
-    <row r="213" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J212" t="s">
+        <v>357</v>
+      </c>
+      <c r="K212" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="213" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A213" s="9">
         <f t="shared" si="3"/>
         <v>211</v>
@@ -7949,17 +8415,29 @@
         <v>213</v>
       </c>
       <c r="D213" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="E213" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="F213" s="7"/>
-      <c r="G213" s="7"/>
-      <c r="H213" s="8"/>
-      <c r="I213" s="8"/>
-    </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="E213" s="6"/>
+      <c r="F213" s="7">
+        <v>-0.24257812499999901</v>
+      </c>
+      <c r="G213" s="7">
+        <v>-3.5156249999999901E-3</v>
+      </c>
+      <c r="H213" s="8">
+        <v>3</v>
+      </c>
+      <c r="I213" s="8">
+        <v>1.6875</v>
+      </c>
+      <c r="J213" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="K213" s="6" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="214" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A214" s="2">
         <f t="shared" si="3"/>
         <v>212</v>
@@ -7985,8 +8463,14 @@
       <c r="I214" s="4">
         <v>1.6875</v>
       </c>
-    </row>
-    <row r="215" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J214" t="s">
+        <v>357</v>
+      </c>
+      <c r="K214" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="215" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A215" s="2">
         <f t="shared" si="3"/>
         <v>213</v>
@@ -7998,17 +8482,31 @@
         <v>216</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E215" s="6" t="s">
-        <v>357</v>
-      </c>
-      <c r="F215" s="3"/>
-      <c r="G215" s="3"/>
-      <c r="H215" s="4"/>
-      <c r="I215" s="4"/>
-    </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="E215" s="35" t="s">
+        <v>368</v>
+      </c>
+      <c r="F215" s="7">
+        <v>-0.24257812499999901</v>
+      </c>
+      <c r="G215" s="7">
+        <v>-3.5156249999999901E-3</v>
+      </c>
+      <c r="H215" s="4">
+        <v>3</v>
+      </c>
+      <c r="I215" s="4">
+        <v>1.6875</v>
+      </c>
+      <c r="J215" t="s">
+        <v>356</v>
+      </c>
+      <c r="K215" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="216" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A216" s="2">
         <f t="shared" si="3"/>
         <v>214</v>
@@ -8020,17 +8518,31 @@
         <v>217</v>
       </c>
       <c r="D216" s="2" t="s">
-        <v>350</v>
+        <v>313</v>
       </c>
       <c r="E216" t="s">
-        <v>357</v>
-      </c>
-      <c r="F216" s="3"/>
-      <c r="G216" s="3"/>
-      <c r="H216" s="4"/>
-      <c r="I216" s="4"/>
-    </row>
-    <row r="217" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+        <v>365</v>
+      </c>
+      <c r="F216" s="3">
+        <v>0</v>
+      </c>
+      <c r="G216" s="3">
+        <v>0</v>
+      </c>
+      <c r="H216" s="4">
+        <v>3</v>
+      </c>
+      <c r="I216" s="4">
+        <v>1.6875</v>
+      </c>
+      <c r="J216" t="s">
+        <v>356</v>
+      </c>
+      <c r="K216" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="217" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A217" s="9">
         <f t="shared" si="3"/>
         <v>215</v>
@@ -8057,8 +8569,14 @@
       <c r="I217" s="8">
         <v>2.2634026516999999</v>
       </c>
-    </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J217" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K217" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="218" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A218" s="2">
         <f t="shared" si="3"/>
         <v>216</v>
@@ -8084,8 +8602,14 @@
       <c r="I218" s="4">
         <v>2.3460200255000001</v>
       </c>
-    </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J218" t="s">
+        <v>357</v>
+      </c>
+      <c r="K218" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="219" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A219" s="2">
         <f t="shared" si="3"/>
         <v>217</v>
@@ -8111,8 +8635,14 @@
       <c r="I219" s="4">
         <v>8.4375</v>
       </c>
-    </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J219" t="s">
+        <v>357</v>
+      </c>
+      <c r="K219" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="220" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A220" s="2">
         <f t="shared" si="3"/>
         <v>218</v>
@@ -8138,8 +8668,14 @@
       <c r="I220" s="4">
         <v>8.4375</v>
       </c>
-    </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J220" t="s">
+        <v>357</v>
+      </c>
+      <c r="K220" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="221" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A221" s="2">
         <f t="shared" si="3"/>
         <v>219</v>
@@ -8165,8 +8701,14 @@
       <c r="I221" s="4">
         <v>8.4375</v>
       </c>
-    </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J221" t="s">
+        <v>357</v>
+      </c>
+      <c r="K221" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="222" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A222" s="2">
         <f t="shared" si="3"/>
         <v>220</v>
@@ -8192,8 +8734,14 @@
       <c r="I222" s="4">
         <v>2.109375</v>
       </c>
-    </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J222" t="s">
+        <v>357</v>
+      </c>
+      <c r="K222" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="223" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A223" s="2">
         <f t="shared" si="3"/>
         <v>221</v>
@@ -8219,8 +8767,14 @@
       <c r="I223" s="4">
         <v>2.109375</v>
       </c>
-    </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J223" t="s">
+        <v>357</v>
+      </c>
+      <c r="K223" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="224" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A224" s="2">
         <f t="shared" si="3"/>
         <v>222</v>
@@ -8246,8 +8800,14 @@
       <c r="I224" s="4">
         <v>2.109375</v>
       </c>
-    </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J224" t="s">
+        <v>357</v>
+      </c>
+      <c r="K224" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="225" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A225" s="2">
         <f t="shared" si="3"/>
         <v>223</v>
@@ -8262,7 +8822,7 @@
         <v>313</v>
       </c>
       <c r="E225" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="F225" s="3">
         <v>-0.15487041477869101</v>
@@ -8276,8 +8836,14 @@
       <c r="I225" s="4">
         <v>2.2938689218000001</v>
       </c>
-    </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J225" t="s">
+        <v>357</v>
+      </c>
+      <c r="K225" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="226" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A226" s="2">
         <f t="shared" si="3"/>
         <v>224</v>
@@ -8303,8 +8869,14 @@
       <c r="I226" s="4">
         <v>2.109375</v>
       </c>
-    </row>
-    <row r="227" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J226" t="s">
+        <v>357</v>
+      </c>
+      <c r="K226" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="227" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A227" s="9">
         <f t="shared" si="3"/>
         <v>225</v>
@@ -8331,8 +8903,14 @@
       <c r="I227" s="8">
         <v>8.4375</v>
       </c>
-    </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J227" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K227" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="228" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A228" s="2">
         <f t="shared" si="3"/>
         <v>226</v>
@@ -8358,8 +8936,14 @@
       <c r="I228" s="4">
         <v>1.6535789792</v>
       </c>
-    </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J228" t="s">
+        <v>357</v>
+      </c>
+      <c r="K228" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="229" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A229" s="2">
         <f t="shared" si="3"/>
         <v>227</v>
@@ -8385,8 +8969,14 @@
       <c r="I229" s="4">
         <v>12.922856493999999</v>
       </c>
-    </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J229" t="s">
+        <v>357</v>
+      </c>
+      <c r="K229" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="230" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
         <f t="shared" si="3"/>
         <v>228</v>
@@ -8412,8 +9002,14 @@
       <c r="I230" s="4">
         <v>1.8363175945000001</v>
       </c>
-    </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J230" t="s">
+        <v>357</v>
+      </c>
+      <c r="K230" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="231" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A231" s="2">
         <f t="shared" si="3"/>
         <v>229</v>
@@ -8439,8 +9035,14 @@
       <c r="I231" s="4">
         <v>3.1819805152999998</v>
       </c>
-    </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J231" t="s">
+        <v>357</v>
+      </c>
+      <c r="K231" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="232" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A232" s="2">
         <f t="shared" si="3"/>
         <v>230</v>
@@ -8466,8 +9068,14 @@
       <c r="I232" s="4">
         <v>2.7413518376999999</v>
       </c>
-    </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J232" t="s">
+        <v>357</v>
+      </c>
+      <c r="K232" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="233" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A233" s="2">
         <f t="shared" si="3"/>
         <v>231</v>
@@ -8493,8 +9101,14 @@
       <c r="I233" s="4">
         <v>2.4484234592999998</v>
       </c>
-    </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J233" t="s">
+        <v>357</v>
+      </c>
+      <c r="K233" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="234" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A234" s="2">
         <f t="shared" si="3"/>
         <v>232</v>
@@ -8512,8 +9126,14 @@
       <c r="G234" s="3"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
-    </row>
-    <row r="235" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J234" t="s">
+        <v>358</v>
+      </c>
+      <c r="K234" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="235" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A235" s="9">
         <f t="shared" si="3"/>
         <v>233</v>
@@ -8540,8 +9160,14 @@
       <c r="I235" s="8">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J235" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K235" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="236" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A236" s="2">
         <f t="shared" si="3"/>
         <v>234</v>
@@ -8567,8 +9193,14 @@
       <c r="I236" s="4">
         <v>2.0775561974999999</v>
       </c>
-    </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J236" t="s">
+        <v>357</v>
+      </c>
+      <c r="K236" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="237" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A237" s="2">
         <f t="shared" si="3"/>
         <v>235</v>
@@ -8594,8 +9226,14 @@
       <c r="I237" s="4">
         <v>2.8125</v>
       </c>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J237" t="s">
+        <v>357</v>
+      </c>
+      <c r="K237" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="238" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A238" s="2">
         <f t="shared" si="3"/>
         <v>236</v>
@@ -8621,8 +9259,14 @@
       <c r="I238" s="4">
         <v>1.3850374649999999</v>
       </c>
-    </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J238" t="s">
+        <v>357</v>
+      </c>
+      <c r="K238" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="239" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A239" s="2">
         <f t="shared" si="3"/>
         <v>237</v>
@@ -8648,8 +9292,14 @@
       <c r="I239" s="4">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J239" t="s">
+        <v>357</v>
+      </c>
+      <c r="K239" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="240" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A240" s="2">
         <f t="shared" si="3"/>
         <v>238</v>
@@ -8675,8 +9325,14 @@
       <c r="I240" s="4">
         <v>2.4222971896000001</v>
       </c>
-    </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J240" t="s">
+        <v>357</v>
+      </c>
+      <c r="K240" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="241" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A241" s="2">
         <f t="shared" si="3"/>
         <v>239</v>
@@ -8702,8 +9358,14 @@
       <c r="I241" s="4">
         <v>2.0017608080999998</v>
       </c>
-    </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J241" t="s">
+        <v>357</v>
+      </c>
+      <c r="K241" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="242" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A242" s="2">
         <f t="shared" si="3"/>
         <v>240</v>
@@ -8729,8 +9391,14 @@
       <c r="I242" s="4">
         <v>18</v>
       </c>
-    </row>
-    <row r="243" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J242" t="s">
+        <v>357</v>
+      </c>
+      <c r="K242" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="243" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A243" s="2">
         <f t="shared" si="3"/>
         <v>241</v>
@@ -8757,8 +9425,14 @@
       <c r="I243" s="8">
         <v>2.25</v>
       </c>
-    </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J243" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K243" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="244" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A244" s="2">
         <f t="shared" si="3"/>
         <v>242</v>
@@ -8784,8 +9458,14 @@
       <c r="I244" s="4">
         <v>45</v>
       </c>
-    </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J244" t="s">
+        <v>357</v>
+      </c>
+      <c r="K244" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="245" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A245" s="2">
         <f t="shared" si="3"/>
         <v>243</v>
@@ -8811,8 +9491,14 @@
       <c r="I245" s="4">
         <v>4.1551123949999997</v>
       </c>
-    </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J245" t="s">
+        <v>357</v>
+      </c>
+      <c r="K245" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="246" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A246" s="2">
         <f t="shared" si="3"/>
         <v>244</v>
@@ -8838,8 +9524,14 @@
       <c r="I246" s="4">
         <v>2.8125</v>
       </c>
-    </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J246" t="s">
+        <v>357</v>
+      </c>
+      <c r="K246" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="247" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A247" s="2">
         <f t="shared" si="3"/>
         <v>245</v>
@@ -8865,8 +9557,14 @@
       <c r="I247" s="4">
         <v>2.8125</v>
       </c>
-    </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J247" t="s">
+        <v>357</v>
+      </c>
+      <c r="K247" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="248" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A248" s="2">
         <f t="shared" si="3"/>
         <v>246</v>
@@ -8892,8 +9590,14 @@
       <c r="I248" s="4">
         <v>2.8125</v>
       </c>
-    </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J248" t="s">
+        <v>357</v>
+      </c>
+      <c r="K248" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="249" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A249" s="2">
         <f t="shared" si="3"/>
         <v>247</v>
@@ -8919,8 +9623,14 @@
       <c r="I249" s="4">
         <v>6.75</v>
       </c>
-    </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J249" t="s">
+        <v>357</v>
+      </c>
+      <c r="K249" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="250" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A250" s="2">
         <f t="shared" si="3"/>
         <v>248</v>
@@ -8946,8 +9656,14 @@
       <c r="I250" s="4">
         <v>1.6921624174000001</v>
       </c>
-    </row>
-    <row r="251" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J250" t="s">
+        <v>357</v>
+      </c>
+      <c r="K250" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="251" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A251" s="2">
         <f t="shared" si="3"/>
         <v>249</v>
@@ -8974,8 +9690,14 @@
       <c r="I251" s="8">
         <v>1.0402895813999999</v>
       </c>
-    </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J251" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K251" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="252" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A252" s="2">
         <f t="shared" si="3"/>
         <v>250</v>
@@ -8993,8 +9715,14 @@
       <c r="G252" s="3"/>
       <c r="H252" s="4"/>
       <c r="I252" s="4"/>
-    </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J252" t="s">
+        <v>358</v>
+      </c>
+      <c r="K252" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="253" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A253" s="2">
         <f t="shared" si="3"/>
         <v>251</v>
@@ -9006,17 +9734,31 @@
         <v>256</v>
       </c>
       <c r="D253" s="2" t="s">
-        <v>350</v>
+        <v>313</v>
       </c>
       <c r="E253" t="s">
-        <v>359</v>
-      </c>
-      <c r="F253" s="3"/>
-      <c r="G253" s="3"/>
-      <c r="H253" s="4"/>
-      <c r="I253" s="4"/>
-    </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.45">
+        <v>366</v>
+      </c>
+      <c r="F253" s="3">
+        <v>-0.33226284584980198</v>
+      </c>
+      <c r="G253" s="3">
+        <v>2.5321146245059298E-2</v>
+      </c>
+      <c r="H253" s="4">
+        <v>3.75</v>
+      </c>
+      <c r="I253" s="4">
+        <v>2.109375</v>
+      </c>
+      <c r="J253" t="s">
+        <v>356</v>
+      </c>
+      <c r="K253" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="254" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A254" s="2">
         <f t="shared" si="3"/>
         <v>252</v>
@@ -9028,17 +9770,28 @@
         <v>257</v>
       </c>
       <c r="D254" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="E254" t="s">
-        <v>360</v>
-      </c>
-      <c r="F254" s="3"/>
-      <c r="G254" s="3"/>
-      <c r="H254" s="4"/>
-      <c r="I254" s="4"/>
-    </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.45">
+        <v>313</v>
+      </c>
+      <c r="F254" s="3">
+        <v>0.38923542490118201</v>
+      </c>
+      <c r="G254" s="3">
+        <v>-0.43648097826086701</v>
+      </c>
+      <c r="H254" s="4">
+        <v>150</v>
+      </c>
+      <c r="I254" s="4">
+        <v>84.375</v>
+      </c>
+      <c r="J254" t="s">
+        <v>356</v>
+      </c>
+      <c r="K254" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="255" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A255" s="2">
         <f t="shared" si="3"/>
         <v>253</v>
@@ -9064,8 +9817,14 @@
       <c r="I255" s="4">
         <v>10.965407351</v>
       </c>
-    </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J255" t="s">
+        <v>357</v>
+      </c>
+      <c r="K255" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="256" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A256" s="2">
         <f t="shared" si="3"/>
         <v>254</v>
@@ -9091,8 +9850,14 @@
       <c r="I256" s="4">
         <v>2.7413518376999999</v>
       </c>
-    </row>
-    <row r="257" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J256" t="s">
+        <v>357</v>
+      </c>
+      <c r="K256" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="257" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A257" s="2">
         <f t="shared" si="3"/>
         <v>255</v>
@@ -9119,8 +9884,14 @@
       <c r="I257" s="8">
         <v>7.0254959236000003</v>
       </c>
-    </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J257" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K257" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="258" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A258" s="2">
         <f t="shared" si="3"/>
         <v>256</v>
@@ -9130,13 +9901,25 @@
       </c>
       <c r="C258" t="s">
         <v>262</v>
+      </c>
+      <c r="D258" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E258" t="s">
+        <v>370</v>
       </c>
       <c r="F258" s="3"/>
       <c r="G258" s="3"/>
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
-    </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="J258" t="s">
+        <v>359</v>
+      </c>
+      <c r="K258" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="259" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A259" s="2">
         <f t="shared" si="3"/>
         <v>257</v>
@@ -9147,12 +9930,29 @@
       <c r="C259" t="s">
         <v>263</v>
       </c>
-      <c r="F259" s="3"/>
-      <c r="G259" s="3"/>
-      <c r="H259" s="4"/>
-      <c r="I259" s="4"/>
-    </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="D259" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F259" s="3">
+        <v>-3.6467902022801</v>
+      </c>
+      <c r="G259" s="3">
+        <v>-0.57021594101123496</v>
+      </c>
+      <c r="H259" s="4">
+        <v>7.3108614232000004</v>
+      </c>
+      <c r="I259" s="4">
+        <v>4.1123595505999999</v>
+      </c>
+      <c r="J259" t="s">
+        <v>357</v>
+      </c>
+      <c r="K259" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="260" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A260" s="2">
         <f t="shared" si="3"/>
         <v>258</v>
@@ -9163,12 +9963,29 @@
       <c r="C260" t="s">
         <v>264</v>
       </c>
-      <c r="F260" s="3"/>
-      <c r="G260" s="3"/>
-      <c r="H260" s="4"/>
-      <c r="I260" s="4"/>
-    </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="D260" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F260" s="3">
+        <v>-2.8385181470369503E-4</v>
+      </c>
+      <c r="G260" s="3">
+        <v>4.9965455276017201E-2</v>
+      </c>
+      <c r="H260" s="4">
+        <v>37.269492073999999</v>
+      </c>
+      <c r="I260" s="4">
+        <v>20.964089291000001</v>
+      </c>
+      <c r="J260" t="s">
+        <v>357</v>
+      </c>
+      <c r="K260" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="261" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A261" s="2">
         <f t="shared" si="3"/>
         <v>259</v>
@@ -9179,12 +9996,29 @@
       <c r="C261" t="s">
         <v>265</v>
       </c>
-      <c r="F261" s="3"/>
-      <c r="G261" s="3"/>
-      <c r="H261" s="4"/>
-      <c r="I261" s="4"/>
-    </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="D261" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F261" s="3">
+        <v>-1.125</v>
+      </c>
+      <c r="G261" s="3">
+        <v>-6.640625E-2</v>
+      </c>
+      <c r="H261" s="4">
+        <v>10</v>
+      </c>
+      <c r="I261" s="4">
+        <v>5.625</v>
+      </c>
+      <c r="J261" t="s">
+        <v>357</v>
+      </c>
+      <c r="K261" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="262" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A262" s="2">
         <f t="shared" si="3"/>
         <v>260</v>
@@ -9195,12 +10029,29 @@
       <c r="C262" t="s">
         <v>266</v>
       </c>
-      <c r="F262" s="3"/>
-      <c r="G262" s="3"/>
-      <c r="H262" s="4"/>
-      <c r="I262" s="4"/>
-    </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="D262" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F262" s="3">
+        <v>-1.6356183941933999</v>
+      </c>
+      <c r="G262" s="3">
+        <v>2.4050322445418201E-2</v>
+      </c>
+      <c r="H262" s="4">
+        <v>7.6224545954999998</v>
+      </c>
+      <c r="I262" s="4">
+        <v>4.2876307100000002</v>
+      </c>
+      <c r="J262" t="s">
+        <v>357</v>
+      </c>
+      <c r="K262" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="263" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A263" s="2">
         <f t="shared" si="3"/>
         <v>261</v>
@@ -9211,12 +10062,29 @@
       <c r="C263" t="s">
         <v>267</v>
       </c>
-      <c r="F263" s="3"/>
-      <c r="G263" s="3"/>
-      <c r="H263" s="4"/>
-      <c r="I263" s="4"/>
-    </row>
-    <row r="264" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D263" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F263" s="3">
+        <v>2.5644984865162299</v>
+      </c>
+      <c r="G263" s="3">
+        <v>0.150454045129335</v>
+      </c>
+      <c r="H263" s="4">
+        <v>36.376444689000003</v>
+      </c>
+      <c r="I263" s="4">
+        <v>20.461750137999999</v>
+      </c>
+      <c r="J263" t="s">
+        <v>357</v>
+      </c>
+      <c r="K263" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="264" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A264" s="2">
         <f t="shared" si="3"/>
         <v>262</v>
@@ -9227,553 +10095,586 @@
       <c r="C264" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="D264" s="5"/>
+      <c r="D264" s="5" t="s">
+        <v>313</v>
+      </c>
       <c r="E264" s="6"/>
-      <c r="F264" s="7"/>
-      <c r="G264" s="7"/>
-      <c r="H264" s="8"/>
-      <c r="I264" s="8"/>
-    </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A265" s="2">
-        <f t="shared" si="3"/>
+      <c r="F264" s="7">
+        <v>1</v>
+      </c>
+      <c r="G264" s="7">
+        <v>0</v>
+      </c>
+      <c r="H264" s="8">
+        <v>37.399899974</v>
+      </c>
+      <c r="I264" s="8">
+        <v>21.037443736</v>
+      </c>
+      <c r="J264" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="K264" s="6" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="265" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A265" s="37"/>
+      <c r="B265" s="38"/>
+      <c r="C265" s="38"/>
+      <c r="D265" s="39"/>
+      <c r="E265" s="38"/>
+      <c r="F265" s="40"/>
+      <c r="G265" s="40"/>
+      <c r="H265" s="41"/>
+      <c r="I265" s="41"/>
+      <c r="J265" s="38"/>
+      <c r="K265" s="38"/>
+    </row>
+    <row r="266" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A266" s="2">
+        <f>A264+1</f>
         <v>263</v>
-      </c>
-      <c r="B265" t="s">
-        <v>269</v>
-      </c>
-      <c r="C265" t="s">
-        <v>270</v>
-      </c>
-      <c r="F265" s="3"/>
-      <c r="G265" s="3"/>
-      <c r="H265" s="4"/>
-      <c r="I265" s="4"/>
-    </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A266" s="2">
-        <f t="shared" ref="A266:A296" si="4">A265+1</f>
-        <v>264</v>
       </c>
       <c r="B266" t="s">
         <v>269</v>
       </c>
       <c r="C266" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F266" s="3"/>
       <c r="G266" s="3"/>
       <c r="H266" s="4"/>
       <c r="I266" s="4"/>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="267" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A267" s="2">
-        <f t="shared" si="4"/>
-        <v>265</v>
+        <f t="shared" ref="A267:A297" si="4">A266+1</f>
+        <v>264</v>
       </c>
       <c r="B267" t="s">
         <v>269</v>
       </c>
       <c r="C267" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F267" s="3"/>
       <c r="G267" s="3"/>
       <c r="H267" s="4"/>
       <c r="I267" s="4"/>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="268" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A268" s="2">
         <f t="shared" si="4"/>
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B268" t="s">
         <v>269</v>
       </c>
       <c r="C268" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F268" s="3"/>
       <c r="G268" s="3"/>
       <c r="H268" s="4"/>
       <c r="I268" s="4"/>
     </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="269" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A269" s="2">
         <f t="shared" si="4"/>
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B269" t="s">
         <v>269</v>
       </c>
       <c r="C269" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F269" s="3"/>
       <c r="G269" s="3"/>
       <c r="H269" s="4"/>
       <c r="I269" s="4"/>
     </row>
-    <row r="270" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A270" s="9">
+    <row r="270" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A270" s="2">
+        <f t="shared" si="4"/>
+        <v>267</v>
+      </c>
+      <c r="B270" t="s">
+        <v>269</v>
+      </c>
+      <c r="C270" t="s">
+        <v>274</v>
+      </c>
+      <c r="F270" s="3"/>
+      <c r="G270" s="3"/>
+      <c r="H270" s="4"/>
+      <c r="I270" s="4"/>
+    </row>
+    <row r="271" spans="1:11" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A271" s="9">
         <f t="shared" si="4"/>
         <v>268</v>
       </c>
-      <c r="B270" s="6" t="s">
+      <c r="B271" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="C270" s="6" t="s">
+      <c r="C271" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="D270" s="5"/>
-      <c r="E270" s="6"/>
-      <c r="F270" s="7"/>
-      <c r="G270" s="7"/>
-      <c r="H270" s="8"/>
-      <c r="I270" s="8"/>
-    </row>
-    <row r="271" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A271" s="2">
+      <c r="D271" s="5"/>
+      <c r="E271" s="6"/>
+      <c r="F271" s="7"/>
+      <c r="G271" s="7"/>
+      <c r="H271" s="8"/>
+      <c r="I271" s="8"/>
+      <c r="J271" s="6"/>
+    </row>
+    <row r="272" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A272" s="2">
         <f t="shared" si="4"/>
         <v>269</v>
       </c>
-      <c r="B271" t="s">
+      <c r="B272" t="s">
         <v>276</v>
       </c>
-      <c r="C271" t="s">
+      <c r="C272" t="s">
         <v>277</v>
       </c>
-      <c r="F271" s="3"/>
-      <c r="G271" s="3"/>
-      <c r="H271" s="4"/>
-      <c r="I271" s="4"/>
-    </row>
-    <row r="272" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A272" s="9">
+      <c r="F272" s="3"/>
+      <c r="G272" s="3"/>
+      <c r="H272" s="4"/>
+      <c r="I272" s="4"/>
+    </row>
+    <row r="273" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A273" s="9">
         <f t="shared" si="4"/>
         <v>270</v>
       </c>
-      <c r="B272" s="6" t="s">
+      <c r="B273" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="C272" s="6" t="s">
+      <c r="C273" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="D272" s="5"/>
-      <c r="E272" s="6"/>
-      <c r="F272" s="7"/>
-      <c r="G272" s="7"/>
-      <c r="H272" s="8"/>
-      <c r="I272" s="8"/>
-    </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A273" s="2">
+      <c r="D273" s="5"/>
+      <c r="E273" s="6"/>
+      <c r="F273" s="7"/>
+      <c r="G273" s="7"/>
+      <c r="H273" s="8"/>
+      <c r="I273" s="8"/>
+      <c r="J273" s="6"/>
+    </row>
+    <row r="274" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A274" s="2">
         <f t="shared" si="4"/>
         <v>271</v>
       </c>
-      <c r="B273" t="s">
-        <v>279</v>
-      </c>
-      <c r="C273" t="s">
-        <v>280</v>
-      </c>
-      <c r="F273" s="3"/>
-      <c r="G273" s="3"/>
-      <c r="H273" s="4"/>
-      <c r="I273" s="4"/>
-    </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A274" s="2">
-        <f t="shared" si="4"/>
-        <v>272</v>
-      </c>
       <c r="B274" t="s">
         <v>279</v>
       </c>
       <c r="C274" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F274" s="3"/>
       <c r="G274" s="3"/>
       <c r="H274" s="4"/>
       <c r="I274" s="4"/>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="275" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A275" s="2">
         <f t="shared" si="4"/>
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B275" t="s">
         <v>279</v>
       </c>
       <c r="C275" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F275" s="3"/>
       <c r="G275" s="3"/>
       <c r="H275" s="4"/>
       <c r="I275" s="4"/>
     </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="276" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A276" s="2">
         <f t="shared" si="4"/>
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B276" t="s">
         <v>279</v>
       </c>
       <c r="C276" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F276" s="3"/>
       <c r="G276" s="3"/>
       <c r="H276" s="4"/>
       <c r="I276" s="4"/>
     </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A277" s="2">
         <f t="shared" si="4"/>
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B277" t="s">
         <v>279</v>
       </c>
       <c r="C277" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F277" s="3"/>
       <c r="G277" s="3"/>
       <c r="H277" s="4"/>
       <c r="I277" s="4"/>
     </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A278" s="2">
         <f t="shared" si="4"/>
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B278" t="s">
         <v>279</v>
       </c>
       <c r="C278" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F278" s="3"/>
       <c r="G278" s="3"/>
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
     </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A279" s="2">
         <f t="shared" si="4"/>
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B279" t="s">
         <v>279</v>
       </c>
       <c r="C279" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F279" s="3"/>
       <c r="G279" s="3"/>
       <c r="H279" s="4"/>
       <c r="I279" s="4"/>
     </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A280" s="2">
         <f t="shared" si="4"/>
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B280" t="s">
         <v>279</v>
       </c>
       <c r="C280" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F280" s="3"/>
       <c r="G280" s="3"/>
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
     </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A281" s="2">
         <f t="shared" si="4"/>
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B281" t="s">
         <v>279</v>
       </c>
       <c r="C281" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F281" s="3"/>
       <c r="G281" s="3"/>
       <c r="H281" s="4"/>
       <c r="I281" s="4"/>
     </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A282" s="2">
         <f t="shared" si="4"/>
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B282" t="s">
         <v>279</v>
       </c>
       <c r="C282" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F282" s="3"/>
       <c r="G282" s="3"/>
       <c r="H282" s="4"/>
       <c r="I282" s="4"/>
     </row>
-    <row r="283" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="283" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A283" s="2">
         <f t="shared" si="4"/>
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B283" t="s">
         <v>279</v>
       </c>
       <c r="C283" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F283" s="3"/>
       <c r="G283" s="3"/>
       <c r="H283" s="4"/>
       <c r="I283" s="4"/>
     </row>
-    <row r="284" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A284" s="9">
+    <row r="284" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A284" s="2">
+        <f t="shared" si="4"/>
+        <v>281</v>
+      </c>
+      <c r="B284" t="s">
+        <v>279</v>
+      </c>
+      <c r="C284" t="s">
+        <v>290</v>
+      </c>
+      <c r="F284" s="3"/>
+      <c r="G284" s="3"/>
+      <c r="H284" s="4"/>
+      <c r="I284" s="4"/>
+    </row>
+    <row r="285" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A285" s="9">
         <f t="shared" si="4"/>
         <v>282</v>
       </c>
-      <c r="B284" s="6" t="s">
+      <c r="B285" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="C284" s="6" t="s">
+      <c r="C285" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="D284" s="5"/>
-      <c r="E284" s="6"/>
-      <c r="F284" s="7"/>
-      <c r="G284" s="7"/>
-      <c r="H284" s="8"/>
-      <c r="I284" s="8"/>
-    </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A285" s="2">
+      <c r="D285" s="5"/>
+      <c r="E285" s="6"/>
+      <c r="F285" s="7"/>
+      <c r="G285" s="7"/>
+      <c r="H285" s="8"/>
+      <c r="I285" s="8"/>
+      <c r="J285" s="6"/>
+    </row>
+    <row r="286" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A286" s="2">
         <f t="shared" si="4"/>
         <v>283</v>
       </c>
-      <c r="B285" t="s">
-        <v>292</v>
-      </c>
-      <c r="C285" t="s">
-        <v>293</v>
-      </c>
-      <c r="F285" s="3"/>
-      <c r="G285" s="3"/>
-      <c r="H285" s="4"/>
-      <c r="I285" s="4"/>
-    </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A286" s="2">
-        <f t="shared" si="4"/>
-        <v>284</v>
-      </c>
       <c r="B286" t="s">
         <v>292</v>
       </c>
       <c r="C286" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F286" s="3"/>
       <c r="G286" s="3"/>
       <c r="H286" s="4"/>
       <c r="I286" s="4"/>
     </row>
-    <row r="287" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="287" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A287" s="2">
         <f t="shared" si="4"/>
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B287" t="s">
         <v>292</v>
       </c>
       <c r="C287" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F287" s="3"/>
       <c r="G287" s="3"/>
       <c r="H287" s="4"/>
       <c r="I287" s="4"/>
     </row>
-    <row r="288" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="288" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A288" s="2">
         <f t="shared" si="4"/>
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B288" t="s">
         <v>292</v>
       </c>
       <c r="C288" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F288" s="3"/>
       <c r="G288" s="3"/>
       <c r="H288" s="4"/>
       <c r="I288" s="4"/>
     </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="289" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A289" s="2">
         <f t="shared" si="4"/>
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B289" t="s">
         <v>292</v>
       </c>
       <c r="C289" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F289" s="3"/>
       <c r="G289" s="3"/>
       <c r="H289" s="4"/>
       <c r="I289" s="4"/>
     </row>
-    <row r="290" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A290" s="2">
         <f t="shared" si="4"/>
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B290" t="s">
         <v>292</v>
       </c>
       <c r="C290" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F290" s="3"/>
       <c r="G290" s="3"/>
       <c r="H290" s="4"/>
       <c r="I290" s="4"/>
     </row>
-    <row r="291" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A291" s="2">
         <f t="shared" si="4"/>
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B291" t="s">
         <v>292</v>
       </c>
       <c r="C291" t="s">
-        <v>299</v>
-      </c>
-      <c r="D291" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="F291" s="3">
-        <v>0</v>
-      </c>
-      <c r="G291" s="3">
-        <v>0</v>
-      </c>
-      <c r="H291" s="4">
-        <v>12</v>
-      </c>
-      <c r="I291" s="4">
-        <v>6.75</v>
-      </c>
-    </row>
-    <row r="292" spans="1:9" x14ac:dyDescent="0.45">
+        <v>298</v>
+      </c>
+      <c r="F291" s="3"/>
+      <c r="G291" s="3"/>
+      <c r="H291" s="4"/>
+      <c r="I291" s="4"/>
+    </row>
+    <row r="292" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A292" s="2">
         <f t="shared" si="4"/>
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B292" t="s">
         <v>292</v>
       </c>
       <c r="C292" t="s">
-        <v>300</v>
-      </c>
-      <c r="F292" s="3"/>
-      <c r="G292" s="3"/>
-      <c r="H292" s="4"/>
-      <c r="I292" s="4"/>
-    </row>
-    <row r="293" spans="1:9" x14ac:dyDescent="0.45">
+        <v>299</v>
+      </c>
+      <c r="D292" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="F292" s="3">
+        <v>0</v>
+      </c>
+      <c r="G292" s="3">
+        <v>0</v>
+      </c>
+      <c r="H292" s="4">
+        <v>12</v>
+      </c>
+      <c r="I292" s="4">
+        <v>6.75</v>
+      </c>
+    </row>
+    <row r="293" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A293" s="2">
         <f t="shared" si="4"/>
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B293" t="s">
         <v>292</v>
       </c>
       <c r="C293" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F293" s="3"/>
       <c r="G293" s="3"/>
       <c r="H293" s="4"/>
       <c r="I293" s="4"/>
     </row>
-    <row r="294" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A294" s="2">
         <f t="shared" si="4"/>
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B294" t="s">
         <v>292</v>
       </c>
       <c r="C294" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F294" s="3"/>
       <c r="G294" s="3"/>
       <c r="H294" s="4"/>
       <c r="I294" s="4"/>
     </row>
-    <row r="295" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A295" s="2">
         <f t="shared" si="4"/>
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B295" t="s">
         <v>292</v>
       </c>
       <c r="C295" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F295" s="3"/>
       <c r="G295" s="3"/>
       <c r="H295" s="4"/>
       <c r="I295" s="4"/>
     </row>
-    <row r="296" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A296" s="9">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A296" s="2">
+        <f t="shared" si="4"/>
+        <v>293</v>
+      </c>
+      <c r="B296" t="s">
+        <v>292</v>
+      </c>
+      <c r="C296" t="s">
+        <v>303</v>
+      </c>
+      <c r="F296" s="3"/>
+      <c r="G296" s="3"/>
+      <c r="H296" s="4"/>
+      <c r="I296" s="4"/>
+    </row>
+    <row r="297" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A297" s="9">
         <f t="shared" si="4"/>
         <v>294</v>
       </c>
-      <c r="B296" s="6" t="s">
+      <c r="B297" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="C296" s="6" t="s">
+      <c r="C297" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="D296" s="5"/>
-      <c r="E296" s="6"/>
-      <c r="F296" s="7"/>
-      <c r="G296" s="7"/>
-      <c r="H296" s="8"/>
-      <c r="I296" s="8"/>
-    </row>
-    <row r="303" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="E303">
+      <c r="D297" s="5"/>
+      <c r="E297" s="6"/>
+      <c r="F297" s="7"/>
+      <c r="G297" s="7"/>
+      <c r="H297" s="8"/>
+      <c r="I297" s="8"/>
+      <c r="J297" s="6"/>
+    </row>
+    <row r="304" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="E304">
         <f>294-244</f>
         <v>50</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I296" xr:uid="{191F369C-B93F-4EDC-AE58-562397A4F805}"/>
-  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D155:D161 D163:D165 D167:D174 D202:D208 D210:D212 D214:D216 D218:D226 D228:D234 D236:D242 D244:D250 D252:D256 D258:D263 D265:D269 D271 D273:D283 D285:D295 D52:D56 D133:D152 D176:D192">
+  <autoFilter ref="A1:K297" xr:uid="{DDCD0A24-47A3-4D2D-80DF-18729F910C8C}"/>
+  <conditionalFormatting sqref="D40:D41 D44:D50 D68 D114:D131 D155:D161 D163:D165 D167:D174 D202:D208 D210:D212 D214:D216 D218:D226 D228:D234 D236:D242 D244:D250 D252:D256 D258:D263 D266:D270 D272 D274:D284 D286:D296 D52:D56 D133:D152 D176:D192">
     <cfRule type="cellIs" dxfId="85" priority="113" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9781,7 +10682,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D296">
+  <conditionalFormatting sqref="D297">
     <cfRule type="cellIs" dxfId="83" priority="45" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9917,7 +10818,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D264">
+  <conditionalFormatting sqref="D264:D265">
     <cfRule type="cellIs" dxfId="49" priority="53" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9925,7 +10826,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D270">
+  <conditionalFormatting sqref="D271">
     <cfRule type="cellIs" dxfId="47" priority="51" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9933,7 +10834,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D272">
+  <conditionalFormatting sqref="D273">
     <cfRule type="cellIs" dxfId="45" priority="49" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -9941,7 +10842,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D284">
+  <conditionalFormatting sqref="D285">
     <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -10117,8 +11018,8 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D41 D43:D56 D68 D114:D296" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations disablePrompts="1" count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D40:D41 D43:D56 D68 D114:D297" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D39 D42 D57:D67 D69:D113" xr:uid="{00000000-0002-0000-0000-000001000000}">
@@ -10128,4 +11029,58 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CA8A3E1-4185-4723-8E90-0367393E96D6}">
+  <dimension ref="C3:D7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="3" max="3" width="24.86328125" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C3" t="s">
+        <v>355</v>
+      </c>
+      <c r="D3" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C4" t="s">
+        <v>358</v>
+      </c>
+      <c r="D4" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C5" t="s">
+        <v>357</v>
+      </c>
+      <c r="D5" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C6" t="s">
+        <v>359</v>
+      </c>
+      <c r="D6" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.45">
+      <c r="C7" t="s">
+        <v>356</v>
+      </c>
+      <c r="D7" t="s">
+        <v>362</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Finished viewport tuning through Exotic Fractals.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB7D1E11-19A3-4F6E-BADB-561D3185D3C7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38228DE1-7EC0-42C2-A166-12E3122A227D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3963,13 +3963,13 @@
   <cols>
     <col min="1" max="1" width="4.59765625" style="2" customWidth="1"/>
     <col min="2" max="2" width="13.73046875" customWidth="1"/>
-    <col min="3" max="3" width="10.86328125" customWidth="1"/>
-    <col min="4" max="4" width="13.73046875" customWidth="1"/>
-    <col min="5" max="5" width="18.796875" customWidth="1"/>
+    <col min="3" max="3" width="10.86328125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="17.73046875" customWidth="1"/>
+    <col min="5" max="5" width="18.1328125" customWidth="1"/>
     <col min="6" max="6" width="4.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="108.86328125" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="5.796875" customWidth="1"/>
-    <col min="9" max="9" width="4.9296875" customWidth="1"/>
+    <col min="9" max="9" width="6.53125" customWidth="1"/>
     <col min="10" max="10" width="17.73046875" style="2" customWidth="1"/>
     <col min="11" max="11" width="11.1328125" customWidth="1"/>
     <col min="12" max="12" width="21.06640625" hidden="1" customWidth="1"/>
@@ -5967,11 +5967,14 @@
       <c r="F59" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H59" s="3"/>
-      <c r="I59" s="3"/>
-      <c r="J59" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H59" s="3">
+        <v>-0.31913395904436798</v>
+      </c>
+      <c r="I59" s="3">
+        <v>-0.45826311860068097</v>
+      </c>
+      <c r="J59" s="13">
+        <v>0.5</v>
       </c>
       <c r="L59" t="s">
         <v>638</v>
@@ -5997,11 +6000,14 @@
       <c r="F60" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H60" s="3"/>
-      <c r="I60" s="3"/>
-      <c r="J60" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H60" s="3">
+        <v>0</v>
+      </c>
+      <c r="I60" s="3">
+        <v>0</v>
+      </c>
+      <c r="J60" s="13">
+        <v>0.87055056599362002</v>
       </c>
       <c r="L60" t="s">
         <v>638</v>
@@ -6028,11 +6034,14 @@
         <v>302</v>
       </c>
       <c r="G61" s="15"/>
-      <c r="H61" s="20"/>
-      <c r="I61" s="20"/>
-      <c r="J61" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H61" s="20">
+        <v>-0.70955631399317298</v>
+      </c>
+      <c r="I61" s="20">
+        <v>6.6552901023890698E-3</v>
+      </c>
+      <c r="J61" s="24">
+        <v>0.66896378133148504</v>
       </c>
       <c r="K61" s="15"/>
       <c r="L61" t="s">
@@ -6060,11 +6069,14 @@
         <v>302</v>
       </c>
       <c r="G62" s="5"/>
-      <c r="H62" s="6"/>
-      <c r="I62" s="6"/>
-      <c r="J62" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H62" s="6">
+        <v>0</v>
+      </c>
+      <c r="I62" s="6">
+        <v>0</v>
+      </c>
+      <c r="J62" s="23">
+        <v>0.30354871978195103</v>
       </c>
       <c r="K62" s="5"/>
       <c r="L62" s="5" t="s">
@@ -6096,11 +6108,10 @@
         <v>4.3229257991153E-3</v>
       </c>
       <c r="I63" s="20">
-        <v>4.3608552897599802E-2</v>
-      </c>
-      <c r="J63" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.04</v>
+      </c>
+      <c r="J63" s="24">
+        <v>0.152613636</v>
       </c>
       <c r="L63" t="s">
         <v>638</v>
@@ -6128,14 +6139,13 @@
       </c>
       <c r="G64" s="5"/>
       <c r="H64" s="6">
-        <v>-7.0846644629357796</v>
+        <v>-7.08</v>
       </c>
       <c r="I64" s="6">
-        <v>0.148191759883506</v>
-      </c>
-      <c r="J64" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.149999999999999</v>
+      </c>
+      <c r="J64" s="23">
+        <v>0.19299538999999899</v>
       </c>
       <c r="K64" s="5"/>
       <c r="L64" s="5" t="s">
@@ -6168,9 +6178,8 @@
       <c r="I65" s="10">
         <v>0</v>
       </c>
-      <c r="J65" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J65" s="13">
+        <v>6.25E-2</v>
       </c>
       <c r="L65" t="s">
         <v>638</v>
@@ -6198,14 +6207,13 @@
       </c>
       <c r="G66" s="9"/>
       <c r="H66" s="11">
-        <v>-0.5</v>
+        <v>-0.75864646064601704</v>
       </c>
       <c r="I66" s="11">
-        <v>0</v>
-      </c>
-      <c r="J66" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>2.8800335472748802E-2</v>
+      </c>
+      <c r="J66" s="24">
+        <v>0.46402327582432901</v>
       </c>
       <c r="K66" s="15"/>
       <c r="L66" s="15" t="s">
@@ -6234,14 +6242,13 @@
       </c>
       <c r="G67" s="8"/>
       <c r="H67" s="10">
-        <v>-0.6</v>
+        <v>-0.65324232081911204</v>
       </c>
       <c r="I67" s="10">
-        <v>0</v>
-      </c>
-      <c r="J67" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>1.9453924914675701E-2</v>
+      </c>
+      <c r="J67" s="13">
+        <v>0.5</v>
       </c>
       <c r="L67" t="s">
         <v>638</v>
@@ -6269,14 +6276,13 @@
       </c>
       <c r="G68" s="9"/>
       <c r="H68" s="11">
-        <v>-0.4</v>
+        <v>-0.37894317752393802</v>
       </c>
       <c r="I68" s="11">
-        <v>-0.3</v>
-      </c>
-      <c r="J68" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.59552795736415698</v>
+      </c>
+      <c r="J68" s="24">
+        <v>0.61557220381133104</v>
       </c>
       <c r="K68" s="15"/>
       <c r="L68" s="15" t="s">
@@ -6305,14 +6311,13 @@
       </c>
       <c r="G69" s="8"/>
       <c r="H69" s="10">
-        <v>-0.8</v>
+        <v>-0.78381274654266098</v>
       </c>
       <c r="I69" s="10">
-        <v>-0.5</v>
-      </c>
-      <c r="J69" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.63759165438737397</v>
+      </c>
+      <c r="J69" s="13">
+        <v>0.72394924999999899</v>
       </c>
       <c r="L69" t="s">
         <v>638</v>
@@ -6340,14 +6345,13 @@
       </c>
       <c r="G70" s="8"/>
       <c r="H70" s="10">
-        <v>-0.5</v>
+        <v>-0.58551237312633797</v>
       </c>
       <c r="I70" s="10">
-        <v>0</v>
-      </c>
-      <c r="J70" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>1.0180044419802301E-3</v>
+      </c>
+      <c r="J70" s="13">
+        <v>1.3223231894474801</v>
       </c>
       <c r="L70" t="s">
         <v>638</v>
@@ -6376,11 +6380,14 @@
       <c r="G71" s="8" t="s">
         <v>332</v>
       </c>
-      <c r="H71" s="10"/>
-      <c r="I71" s="10"/>
-      <c r="J71" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H71" s="10">
+        <v>-1.2163822525597201</v>
+      </c>
+      <c r="I71" s="10">
+        <v>5.1194539249150802E-4</v>
+      </c>
+      <c r="J71" s="13">
+        <v>0.93952275052405798</v>
       </c>
       <c r="L71" t="s">
         <v>638</v>
@@ -6413,9 +6420,8 @@
       <c r="I72" s="6">
         <v>0</v>
       </c>
-      <c r="J72" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J72" s="23">
+        <v>5.8590428369999898</v>
       </c>
       <c r="K72" s="5"/>
       <c r="L72" s="5" t="s">
@@ -6444,14 +6450,13 @@
       </c>
       <c r="G73" s="8"/>
       <c r="H73" s="10">
-        <v>-0.5</v>
+        <v>1.2006302738052901</v>
       </c>
       <c r="I73" s="10">
-        <v>0</v>
-      </c>
-      <c r="J73" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>1.24523137203316E-2</v>
+      </c>
+      <c r="J73" s="13">
+        <v>0.36426867103350702</v>
       </c>
       <c r="L73" t="s">
         <v>638</v>
@@ -6475,11 +6480,14 @@
         <v>302</v>
       </c>
       <c r="G74" s="8"/>
-      <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
-      <c r="J74" s="2" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H74" s="2">
+        <v>0.71640358361774703</v>
+      </c>
+      <c r="I74" s="2">
+        <v>-1.5206377986348E-2</v>
+      </c>
+      <c r="J74" s="2">
+        <v>0.5</v>
       </c>
       <c r="L74" t="s">
         <v>638</v>
@@ -6512,9 +6520,8 @@
       <c r="I75" s="6">
         <v>0</v>
       </c>
-      <c r="J75" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J75" s="23">
+        <v>0.35190984450000001</v>
       </c>
       <c r="K75" s="5"/>
       <c r="L75" s="5" t="s">

</xml_diff>

<commit_message>
Added initial conditions (viewport tuning) for all fractals through Mechanical Engineering.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460553B5-9820-4A76-B1DC-A0CA09A2F504}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B2BD8E-69F9-4428-8BED-D16342021454}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2841,7 +2841,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="118">
+  <dxfs count="114">
     <dxf>
       <font>
         <b/>
@@ -2910,20 +2910,6 @@
         <b/>
         <i val="0"/>
         <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
       </font>
     </dxf>
     <dxf>
@@ -3654,20 +3640,6 @@
         <color rgb="FFFF0000"/>
       </font>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color theme="9" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3984,11 +3956,11 @@
     <col min="1" max="1" width="5.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.9296875" customWidth="1"/>
     <col min="3" max="3" width="6.640625E-2" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="23.3984375" customWidth="1"/>
-    <col min="5" max="5" width="18.1328125" customWidth="1"/>
+    <col min="4" max="4" width="20.73046875" customWidth="1"/>
+    <col min="5" max="5" width="18.86328125" customWidth="1"/>
     <col min="6" max="6" width="4.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="108.86328125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="5.796875" customWidth="1"/>
+    <col min="8" max="8" width="5.53125" customWidth="1"/>
     <col min="9" max="9" width="6.53125" customWidth="1"/>
     <col min="10" max="10" width="17.73046875" style="2" customWidth="1"/>
     <col min="11" max="11" width="11.1328125" customWidth="1"/>
@@ -9944,14 +9916,13 @@
       </c>
       <c r="G176" s="15"/>
       <c r="H176" s="20">
-        <v>-0.5</v>
+        <v>-0.50164794921900702</v>
       </c>
       <c r="I176" s="20">
-        <v>-0.5</v>
-      </c>
-      <c r="J176" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.57415771485533595</v>
+      </c>
+      <c r="J176" s="24">
+        <v>0.71111111100000002</v>
       </c>
       <c r="K176" s="15"/>
       <c r="L176" s="5" t="s">
@@ -9980,14 +9951,13 @@
       </c>
       <c r="G177" s="15"/>
       <c r="H177" s="20">
-        <v>-0.28988974570550302</v>
+        <v>-0.27917647429924902</v>
       </c>
       <c r="I177" s="20">
-        <v>-0.561744537960148</v>
-      </c>
-      <c r="J177" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.60484032076025196</v>
+      </c>
+      <c r="J177" s="24">
+        <v>0.75789767833516897</v>
       </c>
       <c r="K177" s="15"/>
       <c r="L177" s="15" t="s">
@@ -10015,14 +9985,13 @@
         <v>302</v>
       </c>
       <c r="H178" s="3">
-        <v>-0.54094642857142805</v>
+        <v>-0.54</v>
       </c>
       <c r="I178" s="3">
-        <v>4.0113707983192998E-2</v>
-      </c>
-      <c r="J178" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.04</v>
+      </c>
+      <c r="J178" s="13">
+        <v>0.82742316800000004</v>
       </c>
       <c r="L178" t="s">
         <v>635</v>
@@ -10049,14 +10018,13 @@
         <v>302</v>
       </c>
       <c r="H179" s="3">
-        <v>-0.45390625000000001</v>
+        <v>-0.65324232100000001</v>
       </c>
       <c r="I179" s="3">
-        <v>-3.90624999999999E-3</v>
-      </c>
-      <c r="J179" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>1.945392E-2</v>
+      </c>
+      <c r="J179" s="13">
+        <v>0.85856543936414798</v>
       </c>
       <c r="L179" t="s">
         <v>635</v>
@@ -10088,9 +10056,8 @@
       <c r="I180" s="3">
         <v>0</v>
       </c>
-      <c r="J180" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J180" s="13">
+        <v>0.65887281301927803</v>
       </c>
       <c r="L180" t="s">
         <v>635</v>
@@ -10122,9 +10089,8 @@
       <c r="I181" s="3">
         <v>0</v>
       </c>
-      <c r="J181" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J181" s="13">
+        <v>0.74642639300000002</v>
       </c>
       <c r="L181" t="s">
         <v>635</v>
@@ -10156,9 +10122,8 @@
       <c r="I182" s="3">
         <v>0</v>
       </c>
-      <c r="J182" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J182" s="13">
+        <v>0.5</v>
       </c>
       <c r="L182" t="s">
         <v>635</v>
@@ -10190,9 +10155,8 @@
       <c r="I183" s="3">
         <v>0</v>
       </c>
-      <c r="J183" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J183" s="13">
+        <v>0.5</v>
       </c>
       <c r="L183" t="s">
         <v>635</v>
@@ -10219,14 +10183,13 @@
         <v>302</v>
       </c>
       <c r="H184" s="3">
-        <v>0.99957651044607498</v>
+        <v>1</v>
       </c>
       <c r="I184" s="3">
-        <v>6.3523433088651503E-3</v>
-      </c>
-      <c r="J184" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.01</v>
+      </c>
+      <c r="J184" s="13">
+        <v>0.49497474699999899</v>
       </c>
       <c r="L184" t="s">
         <v>635</v>
@@ -10252,11 +10215,14 @@
       <c r="F185" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H185" s="3"/>
-      <c r="I185" s="3"/>
-      <c r="J185" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H185" s="3">
+        <v>0</v>
+      </c>
+      <c r="I185" s="3">
+        <v>0</v>
+      </c>
+      <c r="J185" s="13">
+        <v>1</v>
       </c>
       <c r="L185" t="s">
         <v>635</v>
@@ -10282,11 +10248,14 @@
       <c r="F186" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H186" s="3"/>
-      <c r="I186" s="3"/>
-      <c r="J186" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H186" s="3">
+        <v>0</v>
+      </c>
+      <c r="I186" s="3">
+        <v>0</v>
+      </c>
+      <c r="J186" s="13">
+        <v>0.97265494801506103</v>
       </c>
       <c r="L186" t="s">
         <v>635</v>
@@ -10313,14 +10282,13 @@
         <v>302</v>
       </c>
       <c r="H187" s="3">
-        <v>-0.36210937499999901</v>
+        <v>-0.35999999999999899</v>
       </c>
       <c r="I187" s="3">
-        <v>-4.6874999999999903E-3</v>
-      </c>
-      <c r="J187" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J187" s="13">
+        <v>0.70710678100000002</v>
       </c>
       <c r="L187" t="s">
         <v>635</v>
@@ -10350,14 +10318,13 @@
         <v>337</v>
       </c>
       <c r="H188" s="3">
-        <v>-0.394574846588925</v>
+        <v>-0.39</v>
       </c>
       <c r="I188" s="3">
-        <v>-1.6110981627733001E-3</v>
-      </c>
-      <c r="J188" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J188" s="13">
+        <v>0.81225239599999899</v>
       </c>
       <c r="L188" t="s">
         <v>635</v>
@@ -10384,14 +10351,13 @@
         <v>302</v>
       </c>
       <c r="H189" s="3">
-        <v>-0.15712696055775799</v>
+        <v>-0.16</v>
       </c>
       <c r="I189" s="3">
-        <v>5.5483965529608704E-3</v>
-      </c>
-      <c r="J189" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.01</v>
+      </c>
+      <c r="J189" s="13">
+        <v>0.57756467465400496</v>
       </c>
       <c r="L189" t="s">
         <v>635</v>
@@ -10423,9 +10389,8 @@
       <c r="I190" s="3">
         <v>0</v>
       </c>
-      <c r="J190" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J190" s="13">
+        <v>0.69999999999999896</v>
       </c>
       <c r="L190" t="s">
         <v>635</v>
@@ -10457,9 +10422,8 @@
       <c r="I191" s="3">
         <v>0</v>
       </c>
-      <c r="J191" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J191" s="13">
+        <v>0.83422682876299004</v>
       </c>
       <c r="L191" t="s">
         <v>635</v>
@@ -10491,9 +10455,8 @@
       <c r="I192" s="3">
         <v>0</v>
       </c>
-      <c r="J192" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J192" s="13">
+        <v>0.75</v>
       </c>
       <c r="L192" t="s">
         <v>635</v>
@@ -10525,9 +10488,8 @@
       <c r="I193" s="3">
         <v>0</v>
       </c>
-      <c r="J193" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J193" s="13">
+        <v>0.72445224649207995</v>
       </c>
       <c r="L193" t="s">
         <v>635</v>
@@ -10559,9 +10521,8 @@
       <c r="I194" s="3">
         <v>0</v>
       </c>
-      <c r="J194" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J194" s="13">
+        <v>0.75</v>
       </c>
       <c r="L194" t="s">
         <v>635</v>
@@ -10588,14 +10549,13 @@
         <v>302</v>
       </c>
       <c r="H195" s="3">
-        <v>-0.148758993771477</v>
+        <v>-0.40369149330892101</v>
       </c>
       <c r="I195" s="3">
-        <v>0.62955326460480998</v>
-      </c>
-      <c r="J195" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.45913101847251803</v>
+      </c>
+      <c r="J195" s="13">
+        <v>0.64617641181263497</v>
       </c>
       <c r="L195" t="s">
         <v>635</v>
@@ -10627,9 +10587,8 @@
       <c r="I196" s="3">
         <v>0</v>
       </c>
-      <c r="J196" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J196" s="13">
+        <v>6</v>
       </c>
       <c r="L196" t="s">
         <v>635</v>
@@ -10659,14 +10618,13 @@
         <v>338</v>
       </c>
       <c r="H197" s="3">
-        <v>-0.58828124999999898</v>
+        <v>-0.58999999999999897</v>
       </c>
       <c r="I197" s="3">
-        <v>-4.6874999999999903E-3</v>
-      </c>
-      <c r="J197" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J197" s="13">
+        <v>1</v>
       </c>
       <c r="L197" t="s">
         <v>635</v>
@@ -10693,14 +10651,13 @@
         <v>302</v>
       </c>
       <c r="H198" s="3">
-        <v>-0.249609374999999</v>
+        <v>-0.25</v>
       </c>
       <c r="I198" s="3">
-        <v>-1.6406250000000001E-2</v>
-      </c>
-      <c r="J198" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.02</v>
+      </c>
+      <c r="J198" s="13">
+        <v>0.61557220999999895</v>
       </c>
       <c r="L198" t="s">
         <v>635</v>
@@ -10727,14 +10684,13 @@
         <v>302</v>
       </c>
       <c r="H199" s="3">
-        <v>-0.2109375</v>
+        <v>-0.20999999999999899</v>
       </c>
       <c r="I199" s="3">
-        <v>-1.8749999999999899E-2</v>
-      </c>
-      <c r="J199" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.02</v>
+      </c>
+      <c r="J199" s="13">
+        <v>0.5</v>
       </c>
       <c r="L199" t="s">
         <v>635</v>
@@ -10761,14 +10717,13 @@
         <v>302</v>
       </c>
       <c r="H200" s="3">
-        <v>-1.8681088587872701E-3</v>
+        <v>0</v>
       </c>
       <c r="I200" s="3">
-        <v>1.45213559590144E-3</v>
-      </c>
-      <c r="J200" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J200" s="13">
+        <v>3.425286458</v>
       </c>
       <c r="L200" t="s">
         <v>635</v>
@@ -10795,51 +10750,49 @@
         <v>302</v>
       </c>
       <c r="H201" s="3">
-        <v>-0.248521008366511</v>
+        <v>-0.25</v>
       </c>
       <c r="I201" s="3">
-        <v>3.6650423737307002E-2</v>
-      </c>
-      <c r="J201" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.04</v>
+      </c>
+      <c r="J201" s="13">
+        <v>0.43076521099999898</v>
       </c>
       <c r="L201" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A202" s="2">
         <f t="shared" si="4"/>
         <v>200</v>
       </c>
-      <c r="B202" s="15" t="s">
+      <c r="B202" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="C202" s="15" t="s">
+      <c r="C202" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="D202" s="15" t="s">
+      <c r="D202" s="5" t="s">
         <v>201</v>
       </c>
-      <c r="E202" s="15" t="s">
+      <c r="E202" s="5" t="s">
         <v>492</v>
       </c>
-      <c r="F202" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G202" s="15"/>
-      <c r="H202" s="20">
-        <v>-0.109897735001431</v>
-      </c>
-      <c r="I202" s="20">
-        <v>-4.35438144329897E-2</v>
-      </c>
-      <c r="J202" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K202" s="15"/>
+      <c r="F202" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G202" s="5"/>
+      <c r="H202" s="6">
+        <v>-0.11</v>
+      </c>
+      <c r="I202" s="6">
+        <v>-0.04</v>
+      </c>
+      <c r="J202" s="23">
+        <v>0.59241357983800402</v>
+      </c>
+      <c r="K202" s="5"/>
       <c r="L202" s="15" t="s">
         <v>635</v>
       </c>
@@ -10870,7 +10823,7 @@
         <v>0</v>
       </c>
       <c r="J203" s="24">
-        <v>0.57434917749851699</v>
+        <v>0.57434917699999899</v>
       </c>
       <c r="K203" s="15"/>
       <c r="L203" s="15"/>
@@ -10895,13 +10848,13 @@
       </c>
       <c r="G204" s="15"/>
       <c r="H204" s="20">
-        <v>1.8813865629474899E-3</v>
+        <v>0</v>
       </c>
       <c r="I204" s="20">
-        <v>-1.7929192851177101E-3</v>
+        <v>0</v>
       </c>
       <c r="J204" s="24">
-        <v>0.80907390083999897</v>
+        <v>0.80900000000000005</v>
       </c>
       <c r="K204" s="15"/>
       <c r="L204" s="15"/>
@@ -10932,7 +10885,7 @@
         <v>0</v>
       </c>
       <c r="J205" s="24">
-        <v>0.54829886274714601</v>
+        <v>0.54829886299999897</v>
       </c>
       <c r="K205" s="15"/>
       <c r="L205" s="15"/>
@@ -10961,40 +10914,40 @@
         <v>0</v>
       </c>
       <c r="J206" s="24">
-        <v>0.107725135666983</v>
+        <v>0.108</v>
       </c>
       <c r="K206" s="15"/>
       <c r="L206" s="15"/>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A207" s="2">
         <f t="shared" si="4"/>
         <v>205</v>
       </c>
-      <c r="B207" s="21" t="s">
+      <c r="B207" s="22" t="s">
         <v>712</v>
       </c>
-      <c r="C207" s="15"/>
-      <c r="D207" s="15" t="s">
+      <c r="C207" s="5"/>
+      <c r="D207" s="5" t="s">
         <v>720</v>
       </c>
-      <c r="E207" t="s">
+      <c r="E207" s="5" t="s">
         <v>721</v>
       </c>
-      <c r="F207" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G207" s="15"/>
-      <c r="H207" s="20">
-        <v>-0.31954390776346397</v>
-      </c>
-      <c r="I207" s="20">
-        <v>3.4974955078587999E-2</v>
-      </c>
-      <c r="J207" s="24">
-        <v>0.737134613670553</v>
-      </c>
-      <c r="K207" s="15"/>
+      <c r="F207" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G207" s="5"/>
+      <c r="H207" s="6">
+        <v>-0.32</v>
+      </c>
+      <c r="I207" s="6">
+        <v>2.9999999999999898E-2</v>
+      </c>
+      <c r="J207" s="23">
+        <v>0.73699999999999899</v>
+      </c>
+      <c r="K207" s="5"/>
       <c r="L207" s="15"/>
     </row>
     <row r="208" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -14663,306 +14616,306 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="F78 F124:F141 F165:F171 F173:F175 F177:F184 F217:F223 F225:F227 F229:F231 F233:F241 F243:F249 F251:F257 F259:F265 F267:F271 F273:F285 F289:F293 F295 F58:F60 F186:F207 F297:F303 F62:F66 F305:F314 F42 F49:F53 F47 F143:F162">
-    <cfRule type="cellIs" dxfId="117" priority="191" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="191" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="116" priority="192" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="192" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F209:F215">
-    <cfRule type="cellIs" dxfId="115" priority="121" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="121" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="122" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="122" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F164">
-    <cfRule type="cellIs" dxfId="113" priority="157" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="157" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="158" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="158" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F272">
-    <cfRule type="cellIs" dxfId="109" priority="133" operator="equal">
+    <cfRule type="cellIs" dxfId="107" priority="133" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="134" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="134" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F288">
-    <cfRule type="cellIs" dxfId="107" priority="131" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="131" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="132" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="132" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F8 F89:F92 F97:F113">
-    <cfRule type="cellIs" dxfId="105" priority="117" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="117" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="118" operator="equal">
+    <cfRule type="cellIs" dxfId="102" priority="118" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:F13 F15:F17">
-    <cfRule type="cellIs" dxfId="103" priority="115" operator="equal">
+    <cfRule type="cellIs" dxfId="101" priority="115" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="116" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="116" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F114">
-    <cfRule type="cellIs" dxfId="101" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="49" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="98" priority="50" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F142">
-    <cfRule type="cellIs" dxfId="99" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="45" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="46" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="46" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F19">
-    <cfRule type="cellIs" dxfId="97" priority="107" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="107" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="108" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="108" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F21:F31">
-    <cfRule type="cellIs" dxfId="95" priority="105" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="105" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="106" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="106" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F33:F35">
-    <cfRule type="cellIs" dxfId="93" priority="103" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="103" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="104" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="104" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F41">
-    <cfRule type="cellIs" dxfId="91" priority="101" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="101" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="102" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="102" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F44">
-    <cfRule type="cellIs" dxfId="89" priority="99" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="99" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="100" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="100" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F67:F72">
-    <cfRule type="cellIs" dxfId="87" priority="97" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="97" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="98" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="98" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F74:F75">
-    <cfRule type="cellIs" dxfId="85" priority="95" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="95" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="96" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="96" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F77">
-    <cfRule type="cellIs" dxfId="83" priority="93" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="93" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="94" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="94" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F79:F84 F86:F87">
-    <cfRule type="cellIs" dxfId="81" priority="91" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="91" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="92" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="92" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F85">
-    <cfRule type="cellIs" dxfId="79" priority="89" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="89" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="90" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="90" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F94:F95">
-    <cfRule type="cellIs" dxfId="77" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="87" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="88" operator="equal">
+    <cfRule type="cellIs" dxfId="74" priority="88" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F115:F118">
-    <cfRule type="cellIs" dxfId="75" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="83" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="84" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F120:F123">
-    <cfRule type="cellIs" dxfId="73" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="81" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="82" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F185">
-    <cfRule type="cellIs" dxfId="71" priority="79" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="79" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="68" priority="80" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F14">
-    <cfRule type="cellIs" dxfId="69" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="67" priority="77" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="78" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F18">
-    <cfRule type="cellIs" dxfId="67" priority="75" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="75" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="76" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F20">
-    <cfRule type="cellIs" dxfId="65" priority="73" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="73" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="62" priority="74" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F32">
-    <cfRule type="cellIs" dxfId="63" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="71" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="72" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F36:F40">
-    <cfRule type="cellIs" dxfId="61" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="69" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="70" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="70" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F45">
-    <cfRule type="cellIs" dxfId="59" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="67" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="68" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="68" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F46">
-    <cfRule type="cellIs" dxfId="57" priority="65" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="65" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="66" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="66" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F54:F57">
-    <cfRule type="cellIs" dxfId="55" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="63" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="64" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F61">
-    <cfRule type="cellIs" dxfId="53" priority="61" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="61" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="50" priority="62" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F73">
-    <cfRule type="cellIs" dxfId="51" priority="57" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="57" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="58" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="58" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F76">
-    <cfRule type="cellIs" dxfId="49" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="55" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="56" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F88">
-    <cfRule type="cellIs" dxfId="47" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="53" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="54" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96">
-    <cfRule type="cellIs" dxfId="45" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="43" priority="51" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="52" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F119">
-    <cfRule type="cellIs" dxfId="43" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="47" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="48" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F163">
-    <cfRule type="cellIs" dxfId="41" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="43" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="44" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15118,7 +15071,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F78 F42:F43 F45:F66 F124:F314" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
More initial conditions provided.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B2BD8E-69F9-4428-8BED-D16342021454}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74E9D4A-9731-4AAA-9642-CE33CEC99E97}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2556,7 +2556,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -2691,6 +2691,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2736,7 +2745,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2794,6 +2803,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -10972,16 +10989,15 @@
       </c>
       <c r="G208" s="15"/>
       <c r="H208" s="20">
-        <v>-0.214285714285714</v>
+        <v>-0.41008784481774602</v>
       </c>
       <c r="I208" s="20">
-        <v>-0.57756696428571397</v>
-      </c>
-      <c r="J208" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K208" s="5"/>
+        <v>-0.53266733831739099</v>
+      </c>
+      <c r="J208" s="24">
+        <v>0.66434290282825004</v>
+      </c>
+      <c r="K208" s="27"/>
       <c r="L208" s="5" t="s">
         <v>635</v>
       </c>
@@ -11012,9 +11028,8 @@
       <c r="I209" s="3">
         <v>0</v>
       </c>
-      <c r="J209" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J209" s="13">
+        <v>0.75</v>
       </c>
       <c r="L209" t="s">
         <v>635</v>
@@ -11041,14 +11056,13 @@
         <v>302</v>
       </c>
       <c r="H210" s="3">
-        <v>-0.19380004332237499</v>
+        <v>-0.19</v>
       </c>
       <c r="I210" s="3">
-        <v>1.8667670377751001E-2</v>
-      </c>
-      <c r="J210" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.02</v>
+      </c>
+      <c r="J210" s="13">
+        <v>0.55021005599999895</v>
       </c>
       <c r="L210" t="s">
         <v>635</v>
@@ -11075,14 +11089,13 @@
         <v>302</v>
       </c>
       <c r="H211" s="3">
-        <v>-0.114484592013889</v>
+        <v>-0.11</v>
       </c>
       <c r="I211" s="3">
-        <v>4.7308132875143504E-3</v>
-      </c>
-      <c r="J211" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J211" s="13">
+        <v>0.72236319500000001</v>
       </c>
       <c r="L211" t="s">
         <v>635</v>
@@ -11109,14 +11122,13 @@
         <v>302</v>
       </c>
       <c r="H212" s="3">
-        <v>7.5036966004140407E-2</v>
+        <v>0.08</v>
       </c>
       <c r="I212" s="3">
-        <v>-2.21804600992744E-2</v>
-      </c>
-      <c r="J212" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.02</v>
+      </c>
+      <c r="J212" s="13">
+        <v>0.75028647800000003</v>
       </c>
       <c r="L212" t="s">
         <v>635</v>
@@ -11143,14 +11155,13 @@
         <v>302</v>
       </c>
       <c r="H213" s="3">
-        <v>-1.2357903888167401E-2</v>
+        <v>-0.01</v>
       </c>
       <c r="I213" s="3">
-        <v>-4.4905939034107098E-2</v>
-      </c>
-      <c r="J213" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.04</v>
+      </c>
+      <c r="J213" s="13">
+        <v>0.71841238299999899</v>
       </c>
       <c r="L213" t="s">
         <v>635</v>
@@ -11182,46 +11193,44 @@
       <c r="I214" s="3">
         <v>0</v>
       </c>
-      <c r="J214" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J214" s="13">
+        <v>0.75024142400000005</v>
       </c>
       <c r="L214" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A215" s="2">
         <f t="shared" si="4"/>
         <v>213</v>
       </c>
-      <c r="B215" s="15" t="s">
+      <c r="B215" s="5" t="s">
         <v>303</v>
       </c>
-      <c r="C215" s="15" t="s">
+      <c r="C215" s="5" t="s">
         <v>676</v>
       </c>
-      <c r="D215" s="15" t="s">
+      <c r="D215" s="5" t="s">
         <v>249</v>
       </c>
-      <c r="E215" s="15" t="s">
+      <c r="E215" s="5" t="s">
         <v>500</v>
       </c>
-      <c r="F215" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G215" s="15"/>
-      <c r="H215" s="20">
-        <v>0</v>
-      </c>
-      <c r="I215" s="20">
-        <v>0</v>
-      </c>
-      <c r="J215" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K215" s="15"/>
+      <c r="F215" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G215" s="5"/>
+      <c r="H215" s="6">
+        <v>0</v>
+      </c>
+      <c r="I215" s="6">
+        <v>0</v>
+      </c>
+      <c r="J215" s="23">
+        <v>0.45471497</v>
+      </c>
+      <c r="K215" s="5"/>
       <c r="L215" s="15" t="s">
         <v>635</v>
       </c>
@@ -11231,29 +11240,32 @@
         <f t="shared" si="4"/>
         <v>214</v>
       </c>
-      <c r="B216" s="5" t="s">
+      <c r="B216" s="27" t="s">
         <v>202</v>
       </c>
-      <c r="C216" s="5" t="s">
+      <c r="C216" s="27" t="s">
         <v>671</v>
       </c>
-      <c r="D216" s="5" t="s">
+      <c r="D216" s="27" t="s">
         <v>313</v>
       </c>
-      <c r="E216" s="5" t="s">
+      <c r="E216" s="27" t="s">
         <v>588</v>
       </c>
-      <c r="F216" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G216" s="5"/>
-      <c r="H216" s="6"/>
-      <c r="I216" s="6"/>
-      <c r="J216" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K216" s="5"/>
+      <c r="F216" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="G216" s="27"/>
+      <c r="H216" s="29">
+        <v>0</v>
+      </c>
+      <c r="I216" s="29">
+        <v>0</v>
+      </c>
+      <c r="J216" s="30">
+        <v>1</v>
+      </c>
+      <c r="K216" s="27"/>
       <c r="L216" s="5" t="s">
         <v>635</v>
       </c>
@@ -11278,11 +11290,14 @@
       <c r="F217" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H217" s="3"/>
-      <c r="I217" s="3"/>
-      <c r="J217" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H217" s="3">
+        <v>0</v>
+      </c>
+      <c r="I217" s="3">
+        <v>0</v>
+      </c>
+      <c r="J217" s="13">
+        <v>1</v>
       </c>
       <c r="L217" t="s">
         <v>635</v>
@@ -11317,9 +11332,8 @@
       <c r="I218" s="3">
         <v>0</v>
       </c>
-      <c r="J218" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J218" s="13">
+        <v>0.15</v>
       </c>
       <c r="L218" t="s">
         <v>635</v>
@@ -11345,11 +11359,14 @@
       <c r="F219" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H219" s="3"/>
-      <c r="I219" s="3"/>
-      <c r="J219" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H219" s="3">
+        <v>0</v>
+      </c>
+      <c r="I219" s="3">
+        <v>0</v>
+      </c>
+      <c r="J219" s="13">
+        <v>1</v>
       </c>
       <c r="L219" t="s">
         <v>635</v>
@@ -11375,11 +11392,14 @@
       <c r="F220" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H220" s="3"/>
-      <c r="I220" s="3"/>
-      <c r="J220" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H220" s="3">
+        <v>0</v>
+      </c>
+      <c r="I220" s="3">
+        <v>0</v>
+      </c>
+      <c r="J220" s="13">
+        <v>1</v>
       </c>
       <c r="L220" t="s">
         <v>635</v>
@@ -11405,11 +11425,14 @@
       <c r="F221" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="H221" s="3"/>
-      <c r="I221" s="3"/>
-      <c r="J221" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H221" s="3">
+        <v>0</v>
+      </c>
+      <c r="I221" s="3">
+        <v>0</v>
+      </c>
+      <c r="J221" s="13">
+        <v>1</v>
       </c>
       <c r="L221" t="s">
         <v>635</v>
@@ -11444,46 +11467,44 @@
       <c r="I222" s="3">
         <v>0</v>
       </c>
-      <c r="J222" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J222" s="13">
+        <v>7.8125E-3</v>
       </c>
       <c r="L222" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A223" s="2">
         <f t="shared" si="4"/>
         <v>221</v>
       </c>
-      <c r="B223" s="15" t="s">
+      <c r="B223" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C223" t="s">
+      <c r="C223" s="5" t="s">
         <v>671</v>
       </c>
-      <c r="D223" s="15" t="s">
+      <c r="D223" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="E223" s="15" t="s">
+      <c r="E223" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="F223" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G223" s="15"/>
-      <c r="H223" s="20">
-        <v>-0.55139768622793595</v>
-      </c>
-      <c r="I223" s="20">
-        <v>2.63177386339149E-2</v>
-      </c>
-      <c r="J223" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K223" s="15"/>
+      <c r="F223" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G223" s="5"/>
+      <c r="H223" s="6">
+        <v>-0.55000000000000004</v>
+      </c>
+      <c r="I223" s="6">
+        <v>2.9999999999999898E-2</v>
+      </c>
+      <c r="J223" s="23">
+        <v>1.3508732210000001</v>
+      </c>
+      <c r="K223" s="5"/>
       <c r="L223" s="15" t="s">
         <v>635</v>
       </c>
@@ -11493,33 +11514,32 @@
         <f t="shared" si="4"/>
         <v>222</v>
       </c>
-      <c r="B224" s="5" t="s">
+      <c r="B224" s="27" t="s">
         <v>206</v>
       </c>
-      <c r="C224" t="s">
+      <c r="C224" s="27" t="s">
         <v>673</v>
       </c>
-      <c r="D224" s="5" t="s">
+      <c r="D224" s="27" t="s">
         <v>207</v>
       </c>
-      <c r="E224" s="5" t="s">
+      <c r="E224" s="27" t="s">
         <v>502</v>
       </c>
-      <c r="F224" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G224" s="5"/>
-      <c r="H224" s="6">
-        <v>0</v>
-      </c>
-      <c r="I224" s="6">
-        <v>0</v>
-      </c>
-      <c r="J224" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K224" s="5"/>
+      <c r="F224" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="G224" s="27"/>
+      <c r="H224" s="29">
+        <v>0</v>
+      </c>
+      <c r="I224" s="29">
+        <v>0</v>
+      </c>
+      <c r="J224" s="30">
+        <v>0.5</v>
+      </c>
+      <c r="K224" s="27"/>
       <c r="L224" s="5" t="s">
         <v>635</v>
       </c>
@@ -11550,9 +11570,8 @@
       <c r="I225" s="3">
         <v>0</v>
       </c>
-      <c r="J225" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J225" s="13">
+        <v>0.5</v>
       </c>
       <c r="L225" t="s">
         <v>635</v>
@@ -11584,46 +11603,44 @@
       <c r="I226" s="3">
         <v>0</v>
       </c>
-      <c r="J226" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J226" s="13">
+        <v>0.5</v>
       </c>
       <c r="L226" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A227" s="2">
         <f t="shared" si="4"/>
         <v>225</v>
       </c>
-      <c r="B227" s="15" t="s">
+      <c r="B227" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C227" s="15" t="s">
+      <c r="C227" s="5" t="s">
         <v>673</v>
       </c>
-      <c r="D227" s="15" t="s">
+      <c r="D227" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="E227" s="15" t="s">
+      <c r="E227" s="5" t="s">
         <v>505</v>
       </c>
-      <c r="F227" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G227" s="15"/>
-      <c r="H227" s="20">
-        <v>-0.24257812499999901</v>
-      </c>
-      <c r="I227" s="20">
-        <v>-3.5156249999999901E-3</v>
-      </c>
-      <c r="J227" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K227" s="15"/>
+      <c r="F227" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G227" s="5"/>
+      <c r="H227" s="6">
+        <v>-0.23999999999999899</v>
+      </c>
+      <c r="I227" s="6">
+        <v>0</v>
+      </c>
+      <c r="J227" s="23">
+        <v>1</v>
+      </c>
+      <c r="K227" s="5"/>
       <c r="L227" s="15" t="s">
         <v>635</v>
       </c>
@@ -11633,33 +11650,33 @@
         <f t="shared" si="4"/>
         <v>226</v>
       </c>
-      <c r="B228" s="5" t="s">
+      <c r="B228" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="C228" s="5" t="s">
+      <c r="C228" s="27" t="s">
         <v>673</v>
       </c>
-      <c r="D228" s="5" t="s">
+      <c r="D228" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="E228" s="5" t="s">
+      <c r="E228" s="27" t="s">
         <v>506</v>
       </c>
-      <c r="F228" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G228" s="5"/>
-      <c r="H228" s="6">
+      <c r="F228" s="28" t="s">
+        <v>302</v>
+      </c>
+      <c r="G228" s="27"/>
+      <c r="H228" s="29">
         <v>-0.37968749999999901</v>
       </c>
-      <c r="I228" s="6">
+      <c r="I228" s="29">
         <v>-1.7578125E-2</v>
       </c>
-      <c r="J228" s="23" t="e">
+      <c r="J228" s="30" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K228" s="5"/>
+      <c r="K228" s="27"/>
       <c r="L228" s="5" t="s">
         <v>635</v>
       </c>
@@ -15071,7 +15088,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="2">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F78 F42:F43 F45:F66 F124:F314" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Finished initial conditions through Orbital Advanced.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74E9D4A-9731-4AAA-9642-CE33CEC99E97}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE20EFD5-8995-4B8F-883B-95A167D79719}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11672,9 +11672,8 @@
       <c r="I228" s="29">
         <v>-1.7578125E-2</v>
       </c>
-      <c r="J228" s="30" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J228" s="30">
+        <v>0.72698626384124199</v>
       </c>
       <c r="K228" s="27"/>
       <c r="L228" s="5" t="s">
@@ -11705,20 +11704,19 @@
         <v>354</v>
       </c>
       <c r="H229" s="20">
-        <v>-0.24257812499999901</v>
+        <v>-0.23999999999999899</v>
       </c>
       <c r="I229" s="20">
         <v>-3.5156249999999901E-3</v>
       </c>
-      <c r="J229" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J229" s="13">
+        <v>0.90125046470529702</v>
       </c>
       <c r="L229" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="230" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="230" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A230" s="2">
         <f t="shared" si="4"/>
         <v>228</v>
@@ -11741,52 +11739,50 @@
       <c r="G230" t="s">
         <v>352</v>
       </c>
-      <c r="H230" s="6">
-        <v>0</v>
-      </c>
-      <c r="I230" s="6">
-        <v>0</v>
-      </c>
-      <c r="J230" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H230" s="20">
+        <v>-0.44573109512926501</v>
+      </c>
+      <c r="I230" s="20">
+        <v>-1.1461656731895401E-2</v>
+      </c>
+      <c r="J230" s="13">
+        <v>0.92018765233565603</v>
       </c>
       <c r="L230" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="231" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A231" s="2">
         <f t="shared" si="4"/>
         <v>229</v>
       </c>
-      <c r="B231" s="15" t="s">
+      <c r="B231" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="C231" s="15" t="s">
+      <c r="C231" s="5" t="s">
         <v>673</v>
       </c>
-      <c r="D231" s="15" t="s">
+      <c r="D231" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="E231" s="15" t="s">
+      <c r="E231" s="5" t="s">
         <v>509</v>
       </c>
-      <c r="F231" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G231" s="15"/>
-      <c r="H231" s="20">
-        <v>-0.16662704558133701</v>
-      </c>
-      <c r="I231" s="20">
-        <v>6.5052130349130199E-19</v>
-      </c>
-      <c r="J231" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K231" s="15"/>
+      <c r="F231" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G231" s="5"/>
+      <c r="H231" s="6">
+        <v>-0.17</v>
+      </c>
+      <c r="I231" s="6">
+        <v>0</v>
+      </c>
+      <c r="J231" s="23">
+        <v>0.74555890400000002</v>
+      </c>
+      <c r="K231" s="5"/>
       <c r="L231" s="15" t="s">
         <v>635</v>
       </c>
@@ -11796,33 +11792,32 @@
         <f t="shared" si="4"/>
         <v>230</v>
       </c>
-      <c r="B232" s="5" t="s">
+      <c r="B232" s="15" t="s">
         <v>216</v>
       </c>
-      <c r="C232" s="22" t="s">
+      <c r="C232" s="21" t="s">
         <v>674</v>
       </c>
-      <c r="D232" s="5" t="s">
+      <c r="D232" s="15" t="s">
         <v>217</v>
       </c>
-      <c r="E232" s="5" t="s">
+      <c r="E232" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="F232" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G232" s="5"/>
-      <c r="H232" s="6">
-        <v>-8.8863350609925396E-2</v>
-      </c>
-      <c r="I232" s="6">
-        <v>-2.49544228749192E-2</v>
-      </c>
-      <c r="J232" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K232" s="5"/>
+      <c r="F232" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G232" s="15"/>
+      <c r="H232" s="20">
+        <v>-8.99999999999999E-2</v>
+      </c>
+      <c r="I232" s="20">
+        <v>-0.02</v>
+      </c>
+      <c r="J232" s="24">
+        <v>0.719303322999999</v>
+      </c>
+      <c r="K232" s="15"/>
       <c r="L232" s="22" t="s">
         <v>635</v>
       </c>
@@ -11854,9 +11849,8 @@
       <c r="I233" s="20">
         <v>0</v>
       </c>
-      <c r="J233" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J233" s="24">
+        <v>0.115668818014195</v>
       </c>
       <c r="K233" s="15"/>
       <c r="L233" s="21" t="s">
@@ -11889,9 +11883,8 @@
       <c r="I234" s="3">
         <v>0</v>
       </c>
-      <c r="J234" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J234" s="13">
+        <v>0.65887280646433599</v>
       </c>
       <c r="L234" s="21" t="s">
         <v>635</v>
@@ -11918,14 +11911,13 @@
         <v>302</v>
       </c>
       <c r="H235" s="3">
-        <v>0</v>
+        <v>-0.22469911352590899</v>
       </c>
       <c r="I235" s="3">
-        <v>0</v>
-      </c>
-      <c r="J235" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.114118895966029</v>
+      </c>
+      <c r="J235" s="13">
+        <v>0.62108828089326096</v>
       </c>
       <c r="L235" s="21" t="s">
         <v>635</v>
@@ -11952,14 +11944,13 @@
         <v>302</v>
       </c>
       <c r="H236" s="3">
-        <v>0</v>
+        <v>-0.51831205610004005</v>
       </c>
       <c r="I236" s="3">
-        <v>0</v>
-      </c>
-      <c r="J236" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-8.7623850934824193E-2</v>
+      </c>
+      <c r="J236" s="13">
+        <v>0.56369679707269804</v>
       </c>
       <c r="L236" s="21" t="s">
         <v>635</v>
@@ -11986,14 +11977,13 @@
         <v>302</v>
       </c>
       <c r="H237" s="3">
-        <v>0</v>
+        <v>-0.57059447983014799</v>
       </c>
       <c r="I237" s="3">
-        <v>0</v>
-      </c>
-      <c r="J237" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>1.9904458598727299E-3</v>
+      </c>
+      <c r="J237" s="13">
+        <v>0.68685235149131796</v>
       </c>
       <c r="L237" s="21" t="s">
         <v>635</v>
@@ -12020,14 +12010,13 @@
         <v>302</v>
       </c>
       <c r="H238" s="3">
-        <v>-0.251953125</v>
+        <v>-0.25</v>
       </c>
       <c r="I238" s="3">
-        <v>-8.7890625E-3</v>
-      </c>
-      <c r="J238" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.01</v>
+      </c>
+      <c r="J238" s="13">
+        <v>0.8</v>
       </c>
       <c r="L238" t="s">
         <v>635</v>
@@ -12057,14 +12046,13 @@
         <v>340</v>
       </c>
       <c r="H239" s="3">
-        <v>-0.15487041477869101</v>
+        <v>-0.149999999999999</v>
       </c>
       <c r="I239" s="3">
-        <v>-1.36663693622268E-2</v>
-      </c>
-      <c r="J239" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.01</v>
+      </c>
+      <c r="J239" s="13">
+        <v>0.73565668200000001</v>
       </c>
       <c r="L239" t="s">
         <v>635</v>
@@ -12091,51 +12079,49 @@
         <v>302</v>
       </c>
       <c r="H240" s="3">
-        <v>-0.1787109375</v>
+        <v>-0.17999999999999899</v>
       </c>
       <c r="I240" s="3">
-        <v>1.46484375E-3</v>
-      </c>
-      <c r="J240" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J240" s="13">
+        <v>0.8</v>
       </c>
       <c r="L240" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="241" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A241" s="2">
         <f t="shared" si="4"/>
         <v>239</v>
       </c>
-      <c r="B241" s="15" t="s">
+      <c r="B241" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="C241" s="15" t="s">
+      <c r="C241" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="D241" s="15" t="s">
+      <c r="D241" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="E241" s="15" t="s">
+      <c r="E241" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="F241" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G241" s="15"/>
-      <c r="H241" s="20">
-        <v>-0.34130859375</v>
-      </c>
-      <c r="I241" s="20">
-        <v>-1.46484375E-3</v>
-      </c>
-      <c r="J241" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K241" s="15"/>
+      <c r="F241" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G241" s="5"/>
+      <c r="H241" s="6">
+        <v>-0.34</v>
+      </c>
+      <c r="I241" s="6">
+        <v>0</v>
+      </c>
+      <c r="J241" s="23">
+        <v>0.2</v>
+      </c>
+      <c r="K241" s="5"/>
       <c r="L241" s="15" t="s">
         <v>635</v>
       </c>
@@ -12145,33 +12131,33 @@
         <f t="shared" si="4"/>
         <v>240</v>
       </c>
-      <c r="B242" s="5" t="s">
+      <c r="B242" s="15" t="s">
         <v>227</v>
       </c>
-      <c r="C242" s="5" t="s">
+      <c r="C242" s="15" t="s">
         <v>675</v>
       </c>
-      <c r="D242" s="5" t="s">
+      <c r="D242" s="15" t="s">
         <v>228</v>
       </c>
-      <c r="E242" s="5" t="s">
+      <c r="E242" s="15" t="s">
         <v>594</v>
       </c>
-      <c r="F242" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G242" s="5"/>
-      <c r="H242" s="6">
+      <c r="F242" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G242" s="15"/>
+      <c r="H242" s="20">
         <v>-0.18535125895255999</v>
       </c>
-      <c r="I242" s="6">
+      <c r="I242" s="20">
         <v>1.5132638679150301E-2</v>
       </c>
-      <c r="J242" s="23" t="e">
+      <c r="J242" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K242" s="5"/>
+      <c r="K242" s="15"/>
       <c r="L242" s="5" t="s">
         <v>635</v>
       </c>

</xml_diff>

<commit_message>
Finished initial conditions through Rational Function Fractals
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE20EFD5-8995-4B8F-883B-95A167D79719}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF0A825-5DD4-4878-A5D9-0EFFD0C961E8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3971,8 +3971,8 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.9296875" customWidth="1"/>
-    <col min="3" max="3" width="6.640625E-2" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="0.33203125" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="20.73046875" customWidth="1"/>
     <col min="5" max="5" width="18.86328125" customWidth="1"/>
     <col min="6" max="6" width="4.33203125" style="2" customWidth="1"/>
@@ -12148,14 +12148,13 @@
       </c>
       <c r="G242" s="15"/>
       <c r="H242" s="20">
-        <v>-0.18535125895255999</v>
+        <v>-0.19</v>
       </c>
       <c r="I242" s="20">
-        <v>1.5132638679150301E-2</v>
-      </c>
-      <c r="J242" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.02</v>
+      </c>
+      <c r="J242" s="24">
+        <v>1.0205136990000001</v>
       </c>
       <c r="K242" s="15"/>
       <c r="L242" s="5" t="s">
@@ -12188,9 +12187,8 @@
       <c r="I243" s="3">
         <v>0</v>
       </c>
-      <c r="J243" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J243" s="13">
+        <v>0.130582584</v>
       </c>
       <c r="L243" t="s">
         <v>635</v>
@@ -12217,14 +12215,13 @@
         <v>302</v>
       </c>
       <c r="H244" s="3">
-        <v>-0.16611516952966299</v>
+        <v>-0.17</v>
       </c>
       <c r="I244" s="3">
-        <v>6.6816265541818395E-2</v>
-      </c>
-      <c r="J244" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="J244" s="13">
+        <v>0.53033008599999998</v>
       </c>
       <c r="L244" t="s">
         <v>635</v>
@@ -12256,9 +12253,8 @@
       <c r="I245" s="3">
         <v>0</v>
       </c>
-      <c r="J245" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J245" s="13">
+        <v>0.61557220700000004</v>
       </c>
       <c r="L245" t="s">
         <v>635</v>
@@ -12285,14 +12281,13 @@
         <v>302</v>
       </c>
       <c r="H246" s="3">
-        <v>-0.19383352385890201</v>
+        <v>-0.19</v>
       </c>
       <c r="I246" s="3">
-        <v>3.4005881378754801E-3</v>
-      </c>
-      <c r="J246" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J246" s="13">
+        <v>0.68921901299999999</v>
       </c>
       <c r="L246" t="s">
         <v>635</v>
@@ -12324,9 +12319,8 @@
       <c r="I247" s="3">
         <v>0</v>
       </c>
-      <c r="J247" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J247" s="13">
+        <v>0.91895868400000003</v>
       </c>
       <c r="L247" t="s">
         <v>635</v>
@@ -12353,49 +12347,51 @@
         <v>302</v>
       </c>
       <c r="G248" s="15"/>
-      <c r="H248" s="20"/>
-      <c r="I248" s="20"/>
-      <c r="J248" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H248" s="20">
+        <v>0</v>
+      </c>
+      <c r="I248" s="20">
+        <v>0</v>
+      </c>
+      <c r="J248" s="24">
+        <v>1</v>
       </c>
       <c r="K248" s="15"/>
       <c r="L248" s="15" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="249" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A249" s="2">
         <f t="shared" si="4"/>
         <v>247</v>
       </c>
-      <c r="B249" s="15" t="s">
+      <c r="B249" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="C249" s="15" t="s">
+      <c r="C249" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="D249" s="15" t="s">
+      <c r="D249" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="E249" s="15" t="s">
+      <c r="E249" s="5" t="s">
         <v>598</v>
       </c>
-      <c r="F249" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G249" s="15"/>
-      <c r="H249" s="20">
-        <v>0</v>
-      </c>
-      <c r="I249" s="20">
-        <v>0</v>
-      </c>
-      <c r="J249" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K249" s="15"/>
+      <c r="F249" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G249" s="5"/>
+      <c r="H249" s="6">
+        <v>0</v>
+      </c>
+      <c r="I249" s="6">
+        <v>0</v>
+      </c>
+      <c r="J249" s="23">
+        <v>0.375</v>
+      </c>
+      <c r="K249" s="5"/>
       <c r="L249" s="15" t="s">
         <v>635</v>
       </c>
@@ -12405,33 +12401,32 @@
         <f t="shared" si="4"/>
         <v>248</v>
       </c>
-      <c r="B250" s="5" t="s">
+      <c r="B250" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="C250" s="5" t="s">
+      <c r="C250" s="15" t="s">
         <v>677</v>
       </c>
-      <c r="D250" s="5" t="s">
+      <c r="D250" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="E250" s="5" t="s">
+      <c r="E250" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="F250" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G250" s="5"/>
-      <c r="H250" s="6">
-        <v>-0.57070312499999998</v>
-      </c>
-      <c r="I250" s="6">
-        <v>2.6953124999999901E-2</v>
-      </c>
-      <c r="J250" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K250" s="5"/>
+      <c r="F250" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G250" s="15"/>
+      <c r="H250" s="20">
+        <v>-0.56999999999999895</v>
+      </c>
+      <c r="I250" s="20">
+        <v>2.9999999999999898E-2</v>
+      </c>
+      <c r="J250" s="24">
+        <v>0.81225239599999899</v>
+      </c>
+      <c r="K250" s="15"/>
       <c r="L250" s="5" t="s">
         <v>635</v>
       </c>
@@ -12462,9 +12457,8 @@
       <c r="I251" s="3">
         <v>0</v>
       </c>
-      <c r="J251" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J251" s="13">
+        <v>0.6</v>
       </c>
       <c r="L251" t="s">
         <v>635</v>
@@ -12496,9 +12490,8 @@
       <c r="I252" s="3">
         <v>0</v>
       </c>
-      <c r="J252" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J252" s="13">
+        <v>1.2183785949999999</v>
       </c>
       <c r="L252" t="s">
         <v>635</v>
@@ -12530,9 +12523,8 @@
       <c r="I253" s="3">
         <v>0</v>
       </c>
-      <c r="J253" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J253" s="13">
+        <v>0.75</v>
       </c>
       <c r="L253" t="s">
         <v>635</v>
@@ -12564,9 +12556,8 @@
       <c r="I254" s="3">
         <v>0</v>
       </c>
-      <c r="J254" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J254" s="13">
+        <v>0.69665275100000001</v>
       </c>
       <c r="L254" t="s">
         <v>635</v>
@@ -12593,14 +12584,13 @@
         <v>302</v>
       </c>
       <c r="H255" s="3">
-        <v>-0.168898568184977</v>
+        <v>-0.17</v>
       </c>
       <c r="I255" s="3">
-        <v>2.1546730920717301E-2</v>
-      </c>
-      <c r="J255" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.02</v>
+      </c>
+      <c r="J255" s="13">
+        <v>0.84300781199999997</v>
       </c>
       <c r="L255" t="s">
         <v>635</v>
@@ -12632,46 +12622,44 @@
       <c r="I256" s="3">
         <v>0</v>
       </c>
-      <c r="J256" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J256" s="13">
+        <v>9.375E-2</v>
       </c>
       <c r="L256" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="257" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A257" s="2">
         <f t="shared" si="4"/>
         <v>255</v>
       </c>
-      <c r="B257" s="15" t="s">
+      <c r="B257" s="5" t="s">
         <v>304</v>
       </c>
-      <c r="C257" s="15" t="s">
+      <c r="C257" s="5" t="s">
         <v>677</v>
       </c>
-      <c r="D257" s="15" t="s">
+      <c r="D257" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="E257" s="15" t="s">
+      <c r="E257" s="5" t="s">
         <v>603</v>
       </c>
-      <c r="F257" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G257" s="15"/>
-      <c r="H257" s="20">
-        <v>0</v>
-      </c>
-      <c r="I257" s="20">
-        <v>0</v>
-      </c>
-      <c r="J257" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K257" s="15"/>
+      <c r="F257" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G257" s="5"/>
+      <c r="H257" s="6">
+        <v>0</v>
+      </c>
+      <c r="I257" s="6">
+        <v>0</v>
+      </c>
+      <c r="J257" s="23">
+        <v>0.75</v>
+      </c>
+      <c r="K257" s="5"/>
       <c r="L257" s="15" t="s">
         <v>635</v>
       </c>
@@ -12681,33 +12669,32 @@
         <f t="shared" ref="A258:A314" si="5">A257+1</f>
         <v>256</v>
       </c>
-      <c r="B258" s="5" t="s">
+      <c r="B258" s="15" t="s">
         <v>250</v>
       </c>
-      <c r="C258" s="5" t="s">
+      <c r="C258" s="15" t="s">
         <v>679</v>
       </c>
-      <c r="D258" s="5" t="s">
+      <c r="D258" s="15" t="s">
         <v>318</v>
       </c>
-      <c r="E258" s="5" t="s">
+      <c r="E258" s="15" t="s">
         <v>604</v>
       </c>
-      <c r="F258" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G258" s="5"/>
-      <c r="H258" s="6">
-        <v>0</v>
-      </c>
-      <c r="I258" s="6">
-        <v>0</v>
-      </c>
-      <c r="J258" s="23" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="K258" s="5"/>
+      <c r="F258" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G258" s="15"/>
+      <c r="H258" s="20">
+        <v>0</v>
+      </c>
+      <c r="I258" s="20">
+        <v>0</v>
+      </c>
+      <c r="J258" s="24">
+        <v>3.7499999999999999E-2</v>
+      </c>
+      <c r="K258" s="15"/>
       <c r="L258" s="5" t="s">
         <v>635</v>
       </c>
@@ -12733,14 +12720,13 @@
         <v>302</v>
       </c>
       <c r="H259" s="3">
-        <v>-2.3551547802465</v>
+        <v>-2.36</v>
       </c>
       <c r="I259" s="3">
-        <v>1.49625973078175E-2</v>
-      </c>
-      <c r="J259" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.01</v>
+      </c>
+      <c r="J259" s="13">
+        <v>0.40612619799999999</v>
       </c>
       <c r="L259" t="s">
         <v>635</v>
@@ -12772,9 +12758,8 @@
       <c r="I260" s="3">
         <v>0</v>
       </c>
-      <c r="J260" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J260" s="13">
+        <v>0.6</v>
       </c>
       <c r="L260" t="s">
         <v>635</v>
@@ -12807,9 +12792,8 @@
       <c r="I261" s="20">
         <v>0</v>
       </c>
-      <c r="J261" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J261" s="24">
+        <v>0.6</v>
       </c>
       <c r="K261" s="15"/>
       <c r="L261" s="15" t="s">
@@ -12842,9 +12826,8 @@
       <c r="I262" s="3">
         <v>0</v>
       </c>
-      <c r="J262" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J262" s="13">
+        <v>0.6</v>
       </c>
       <c r="L262" t="s">
         <v>635</v>
@@ -12872,14 +12855,13 @@
       </c>
       <c r="G263" s="15"/>
       <c r="H263" s="20">
-        <v>9.1841731880125899E-2</v>
+        <v>0.09</v>
       </c>
       <c r="I263" s="20">
-        <v>-0.17277720945686001</v>
-      </c>
-      <c r="J263" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.17</v>
+      </c>
+      <c r="J263" s="24">
+        <v>1.6221444780000001</v>
       </c>
       <c r="K263" s="15"/>
       <c r="L263" s="15" t="s">
@@ -12908,50 +12890,50 @@
       </c>
       <c r="G264" s="15"/>
       <c r="H264" s="20">
-        <v>4.0254603399433702</v>
+        <v>4.03</v>
       </c>
       <c r="I264" s="20">
-        <v>0.144673630783757</v>
-      </c>
-      <c r="J264" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="J264" s="24">
+        <v>0.25</v>
       </c>
       <c r="K264" s="15"/>
       <c r="L264" s="15" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="265" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A265" s="2">
         <f t="shared" si="5"/>
         <v>263</v>
       </c>
-      <c r="B265" t="s">
+      <c r="B265" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="C265" t="s">
+      <c r="C265" s="5" t="s">
         <v>679</v>
       </c>
-      <c r="D265" t="s">
+      <c r="D265" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="E265" t="s">
+      <c r="E265" s="5" t="s">
         <v>610</v>
       </c>
-      <c r="F265" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H265" s="3">
-        <v>-6.2910553801410293E-2</v>
-      </c>
-      <c r="I265" s="3">
-        <v>-0.133920889728255</v>
-      </c>
-      <c r="J265" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
+      <c r="F265" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G265" s="5"/>
+      <c r="H265" s="6">
+        <v>-0.06</v>
+      </c>
+      <c r="I265" s="6">
+        <v>-0.13</v>
+      </c>
+      <c r="J265" s="23">
+        <v>0.99724469900000001</v>
+      </c>
+      <c r="K265" s="5"/>
       <c r="L265" t="s">
         <v>635</v>
       </c>
@@ -12961,35 +12943,35 @@
         <f t="shared" si="5"/>
         <v>264</v>
       </c>
-      <c r="B266" s="5" t="s">
+      <c r="B266" s="15" t="s">
         <v>251</v>
       </c>
-      <c r="C266" s="5" t="s">
+      <c r="C266" s="15" t="s">
         <v>681</v>
       </c>
-      <c r="D266" s="5" t="s">
+      <c r="D266" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="E266" s="5" t="s">
+      <c r="E266" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="F266" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G266" s="5" t="s">
+      <c r="F266" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G266" s="15" t="s">
         <v>353</v>
       </c>
-      <c r="H266" s="6">
+      <c r="H266" s="20">
         <v>-0.33226284584980198</v>
       </c>
-      <c r="I266" s="6">
+      <c r="I266" s="20">
         <v>2.5321146245059298E-2</v>
       </c>
-      <c r="J266" s="23" t="e">
+      <c r="J266" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K266" s="5"/>
+      <c r="K266" s="15"/>
       <c r="L266" s="5" t="s">
         <v>635</v>
       </c>
@@ -13128,38 +13110,38 @@
         <v>635</v>
       </c>
     </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="271" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A271" s="2">
         <f t="shared" si="5"/>
         <v>269</v>
       </c>
-      <c r="B271" s="15" t="s">
+      <c r="B271" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="C271" s="15" t="s">
+      <c r="C271" s="5" t="s">
         <v>681</v>
       </c>
-      <c r="D271" s="15" t="s">
+      <c r="D271" s="5" t="s">
         <v>257</v>
       </c>
-      <c r="E271" s="15" t="s">
+      <c r="E271" s="5" t="s">
         <v>526</v>
       </c>
-      <c r="F271" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G271" s="15"/>
-      <c r="H271" s="20">
+      <c r="F271" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G271" s="5"/>
+      <c r="H271" s="6">
         <v>-0.22203909754190099</v>
       </c>
-      <c r="I271" s="20">
+      <c r="I271" s="6">
         <v>5.2512073606900397E-2</v>
       </c>
-      <c r="J271" s="24" t="e">
+      <c r="J271" s="23" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K271" s="15"/>
+      <c r="K271" s="5"/>
       <c r="L271" s="15" t="s">
         <v>635</v>
       </c>
@@ -13169,34 +13151,34 @@
         <f t="shared" si="5"/>
         <v>270</v>
       </c>
-      <c r="B272" s="5" t="s">
+      <c r="B272" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="C272" s="5" t="s">
+      <c r="C272" s="15" t="s">
         <v>680</v>
       </c>
-      <c r="D272" s="5" t="s">
+      <c r="D272" s="15" t="s">
         <v>259</v>
       </c>
-      <c r="E272" s="5" t="s">
+      <c r="E272" s="15" t="s">
         <v>527</v>
       </c>
-      <c r="F272" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G272" s="5" t="s">
+      <c r="F272" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G272" s="15" t="s">
         <v>355</v>
       </c>
-      <c r="H272" s="6">
+      <c r="H272" s="20">
         <v>-0.69665929008750505</v>
       </c>
-      <c r="I272" s="6">
+      <c r="I272" s="20">
         <v>-0.57148811196592597</v>
       </c>
-      <c r="J272" s="23">
+      <c r="J272" s="24">
         <v>0.158807672173572</v>
       </c>
-      <c r="K272" s="5"/>
+      <c r="K272" s="15"/>
       <c r="L272" s="5" t="s">
         <v>635</v>
       </c>
@@ -13594,34 +13576,34 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="286" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A286" s="2">
         <f t="shared" si="5"/>
         <v>284</v>
       </c>
-      <c r="B286" s="15" t="s">
+      <c r="B286" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="C286" s="15" t="s">
+      <c r="C286" s="5" t="s">
         <v>680</v>
       </c>
-      <c r="D286" s="15" t="s">
+      <c r="D286" s="5" t="s">
         <v>689</v>
       </c>
-      <c r="E286" s="15" t="s">
+      <c r="E286" s="5" t="s">
         <v>533</v>
       </c>
-      <c r="F286" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G286" s="15"/>
-      <c r="H286" s="20">
+      <c r="F286" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G286" s="5"/>
+      <c r="H286" s="6">
         <v>-0.25343772240527501</v>
       </c>
-      <c r="I286" s="20">
+      <c r="I286" s="6">
         <v>2.8551421212316399E-3</v>
       </c>
-      <c r="J286" s="24">
+      <c r="J286" s="23">
         <v>0.325449642392387</v>
       </c>
       <c r="K286" s="15"/>
@@ -13634,33 +13616,33 @@
         <f t="shared" si="5"/>
         <v>285</v>
       </c>
-      <c r="B287" s="5" t="s">
+      <c r="B287" s="15" t="s">
         <v>266</v>
       </c>
-      <c r="C287" s="5" t="s">
+      <c r="C287" s="15" t="s">
         <v>682</v>
       </c>
-      <c r="D287" s="5" t="s">
+      <c r="D287" s="15" t="s">
         <v>267</v>
       </c>
-      <c r="E287" s="5" t="s">
+      <c r="E287" s="15" t="s">
         <v>613</v>
       </c>
-      <c r="F287" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G287" s="5"/>
-      <c r="H287" s="6">
-        <v>0</v>
-      </c>
-      <c r="I287" s="6">
-        <v>0</v>
-      </c>
-      <c r="J287" s="23" t="e">
+      <c r="F287" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G287" s="15"/>
+      <c r="H287" s="20">
+        <v>0</v>
+      </c>
+      <c r="I287" s="20">
+        <v>0</v>
+      </c>
+      <c r="J287" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K287" s="5"/>
+      <c r="K287" s="15"/>
       <c r="L287" s="5" t="s">
         <v>635</v>
       </c>
@@ -13803,38 +13785,38 @@
         <v>635</v>
       </c>
     </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="292" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A292" s="2">
         <f t="shared" si="5"/>
         <v>290</v>
       </c>
-      <c r="B292" s="15" t="s">
+      <c r="B292" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="C292" s="15" t="s">
+      <c r="C292" s="5" t="s">
         <v>682</v>
       </c>
-      <c r="D292" s="15" t="s">
+      <c r="D292" s="5" t="s">
         <v>272</v>
       </c>
-      <c r="E292" s="15" t="s">
+      <c r="E292" s="5" t="s">
         <v>617</v>
       </c>
-      <c r="F292" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G292" s="15"/>
-      <c r="H292" s="20">
+      <c r="F292" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G292" s="5"/>
+      <c r="H292" s="6">
         <v>-0.449612977602108</v>
       </c>
-      <c r="I292" s="20">
+      <c r="I292" s="6">
         <v>-0.53004776021080202</v>
       </c>
-      <c r="J292" s="24" t="e">
+      <c r="J292" s="23" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K292" s="15"/>
+      <c r="K292" s="5"/>
       <c r="L292" s="15" t="s">
         <v>635</v>
       </c>
@@ -13950,33 +13932,33 @@
         <f t="shared" si="5"/>
         <v>294</v>
       </c>
-      <c r="B296" s="5" t="s">
+      <c r="B296" s="15" t="s">
         <v>276</v>
       </c>
-      <c r="C296" s="5" t="s">
+      <c r="C296" s="15" t="s">
         <v>643</v>
       </c>
-      <c r="D296" s="5" t="s">
+      <c r="D296" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="E296" s="5" t="s">
+      <c r="E296" s="15" t="s">
         <v>535</v>
       </c>
-      <c r="F296" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G296" s="5"/>
-      <c r="H296" s="6">
+      <c r="F296" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G296" s="15"/>
+      <c r="H296" s="20">
         <v>-0.826954434020021</v>
       </c>
-      <c r="I296" s="6">
+      <c r="I296" s="20">
         <v>1.5896229075411601</v>
       </c>
-      <c r="J296" s="23" t="e">
+      <c r="J296" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K296" s="5"/>
+      <c r="K296" s="15"/>
       <c r="L296" s="5" t="s">
         <v>635</v>
       </c>
@@ -14154,40 +14136,40 @@
         <v>635</v>
       </c>
     </row>
-    <row r="302" spans="1:12" s="18" customFormat="1" x14ac:dyDescent="0.45">
+    <row r="302" spans="1:12" s="18" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A302" s="2">
         <f t="shared" si="5"/>
         <v>300</v>
       </c>
-      <c r="B302" s="15" t="s">
+      <c r="B302" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="C302" s="15" t="s">
+      <c r="C302" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="D302" s="15" t="s">
+      <c r="D302" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="E302" s="15" t="s">
+      <c r="E302" s="5" t="s">
         <v>538</v>
       </c>
-      <c r="F302" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G302" s="15" t="s">
+      <c r="F302" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G302" s="5" t="s">
         <v>358</v>
       </c>
-      <c r="H302" s="20">
-        <v>0</v>
-      </c>
-      <c r="I302" s="20">
-        <v>0</v>
-      </c>
-      <c r="J302" s="24" t="e">
+      <c r="H302" s="6">
+        <v>0</v>
+      </c>
+      <c r="I302" s="6">
+        <v>0</v>
+      </c>
+      <c r="J302" s="23" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K302" s="15"/>
+      <c r="K302" s="5"/>
       <c r="L302" s="15" t="s">
         <v>635</v>
       </c>
@@ -14231,33 +14213,33 @@
         <f t="shared" si="5"/>
         <v>302</v>
       </c>
-      <c r="B304" s="5" t="s">
+      <c r="B304" s="15" t="s">
         <v>284</v>
       </c>
-      <c r="C304" s="5" t="s">
+      <c r="C304" s="15" t="s">
         <v>683</v>
       </c>
-      <c r="D304" s="5" t="s">
+      <c r="D304" s="15" t="s">
         <v>287</v>
       </c>
-      <c r="E304" s="5" t="s">
+      <c r="E304" s="15" t="s">
         <v>626</v>
       </c>
-      <c r="F304" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G304" s="5"/>
-      <c r="H304" s="6">
-        <v>0</v>
-      </c>
-      <c r="I304" s="6">
-        <v>0</v>
-      </c>
-      <c r="J304" s="23" t="e">
+      <c r="F304" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G304" s="15"/>
+      <c r="H304" s="20">
+        <v>0</v>
+      </c>
+      <c r="I304" s="20">
+        <v>0</v>
+      </c>
+      <c r="J304" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K304" s="5"/>
+      <c r="K304" s="15"/>
       <c r="L304" s="5" t="s">
         <v>635</v>
       </c>

</xml_diff>

<commit_message>
feat: Add BuddhabrotBased fractal category and registrations
- Add FractalCategory::BuddhabrotBased enum to native and managed layers
- Register Buddhabrot (Classic) and Nebulabrot (Dramatic RGB) fractals
- Add detailed performance warnings and visual descriptions
- Update FractalRegistry documentation with new category
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EF0A825-5DD4-4878-A5D9-0EFFD0C961E8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5769AD4-731B-4472-BE4B-4C6222337B7B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,15 +17,15 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$L$314</definedName>
-    <definedName name="Data">FractalRegistry!$A$1:$L$314</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FractalRegistry!$A$1:$L$315</definedName>
+    <definedName name="Data">FractalRegistry!$A$1:$L$315</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1876" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1880" uniqueCount="732">
   <si>
     <t>Group Name</t>
   </si>
@@ -2218,6 +2218,9 @@
   </si>
   <si>
     <t>-0.089999999999999997)</t>
+  </si>
+  <si>
+    <t>Nebulabrot</t>
   </si>
 </sst>
 </file>
@@ -3967,7 +3970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L321"/>
+  <dimension ref="A1:L322"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5.6640625" style="2" customWidth="1"/>
@@ -12666,7 +12669,7 @@
     </row>
     <row r="258" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A258" s="2">
-        <f t="shared" ref="A258:A314" si="5">A257+1</f>
+        <f t="shared" ref="A258:A315" si="5">A257+1</f>
         <v>256</v>
       </c>
       <c r="B258" s="15" t="s">
@@ -13047,34 +13050,31 @@
         <f t="shared" si="5"/>
         <v>267</v>
       </c>
-      <c r="B269" t="s">
+      <c r="B269" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="C269" t="s">
-        <v>681</v>
-      </c>
-      <c r="D269" t="s">
-        <v>255</v>
-      </c>
-      <c r="E269" t="s">
-        <v>255</v>
-      </c>
-      <c r="F269" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H269" s="3">
-        <v>-5.6126062322933903E-3</v>
-      </c>
-      <c r="I269" s="3">
-        <v>1.19068696883983E-3</v>
-      </c>
-      <c r="J269" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L269" t="s">
-        <v>635</v>
-      </c>
+      <c r="C269" s="15"/>
+      <c r="D269" s="21" t="s">
+        <v>731</v>
+      </c>
+      <c r="E269" s="21" t="s">
+        <v>731</v>
+      </c>
+      <c r="F269" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G269" s="15"/>
+      <c r="H269" s="20">
+        <v>-0.33</v>
+      </c>
+      <c r="I269" s="20">
+        <v>0.03</v>
+      </c>
+      <c r="J269" s="24">
+        <v>1.066667</v>
+      </c>
+      <c r="K269" s="15"/>
+      <c r="L269" s="15"/>
     </row>
     <row r="270" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A270" s="2">
@@ -13088,19 +13088,19 @@
         <v>681</v>
       </c>
       <c r="D270" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E270" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F270" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H270" s="3">
-        <v>0</v>
+        <v>-5.6126062322933903E-3</v>
       </c>
       <c r="I270" s="3">
-        <v>0</v>
+        <v>1.19068696883983E-3</v>
       </c>
       <c r="J270" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -13110,39 +13110,37 @@
         <v>635</v>
       </c>
     </row>
-    <row r="271" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="271" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A271" s="2">
         <f t="shared" si="5"/>
         <v>269</v>
       </c>
-      <c r="B271" s="5" t="s">
+      <c r="B271" t="s">
         <v>251</v>
       </c>
-      <c r="C271" s="5" t="s">
+      <c r="C271" t="s">
         <v>681</v>
       </c>
-      <c r="D271" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="E271" s="5" t="s">
-        <v>526</v>
-      </c>
-      <c r="F271" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G271" s="5"/>
-      <c r="H271" s="6">
-        <v>-0.22203909754190099</v>
-      </c>
-      <c r="I271" s="6">
-        <v>5.2512073606900397E-2</v>
-      </c>
-      <c r="J271" s="23" t="e">
+      <c r="D271" t="s">
+        <v>256</v>
+      </c>
+      <c r="E271" t="s">
+        <v>256</v>
+      </c>
+      <c r="F271" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H271" s="3">
+        <v>0</v>
+      </c>
+      <c r="I271" s="3">
+        <v>0</v>
+      </c>
+      <c r="J271" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K271" s="5"/>
-      <c r="L271" s="15" t="s">
+      <c r="L271" t="s">
         <v>635</v>
       </c>
     </row>
@@ -13151,63 +13149,72 @@
         <f t="shared" si="5"/>
         <v>270</v>
       </c>
-      <c r="B272" s="15" t="s">
-        <v>258</v>
-      </c>
-      <c r="C272" s="15" t="s">
-        <v>680</v>
-      </c>
-      <c r="D272" s="15" t="s">
-        <v>259</v>
-      </c>
-      <c r="E272" s="15" t="s">
-        <v>527</v>
-      </c>
-      <c r="F272" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G272" s="15" t="s">
-        <v>355</v>
-      </c>
-      <c r="H272" s="20">
-        <v>-0.69665929008750505</v>
-      </c>
-      <c r="I272" s="20">
-        <v>-0.57148811196592597</v>
-      </c>
-      <c r="J272" s="24">
-        <v>0.158807672173572</v>
-      </c>
-      <c r="K272" s="15"/>
-      <c r="L272" s="5" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="B272" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C272" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="D272" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="E272" s="5" t="s">
+        <v>526</v>
+      </c>
+      <c r="F272" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G272" s="5"/>
+      <c r="H272" s="6">
+        <v>-0.22203909754190099</v>
+      </c>
+      <c r="I272" s="6">
+        <v>5.2512073606900397E-2</v>
+      </c>
+      <c r="J272" s="23" t="e">
+        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="K272" s="5"/>
+      <c r="L272" s="15" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="273" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A273" s="2">
         <f t="shared" si="5"/>
         <v>271</v>
       </c>
-      <c r="B273" t="s">
+      <c r="B273" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="D273" t="s">
-        <v>692</v>
-      </c>
-      <c r="E273" t="s">
-        <v>696</v>
-      </c>
-      <c r="F273" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H273" s="3">
-        <v>0.33833705716155399</v>
-      </c>
-      <c r="I273" s="3">
-        <v>2.0752737684215899E-2</v>
-      </c>
-      <c r="J273" s="13">
-        <v>0.38668516346655102</v>
+      <c r="C273" s="15" t="s">
+        <v>680</v>
+      </c>
+      <c r="D273" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="E273" s="15" t="s">
+        <v>527</v>
+      </c>
+      <c r="F273" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G273" s="15" t="s">
+        <v>355</v>
+      </c>
+      <c r="H273" s="20">
+        <v>-0.69665929008750505</v>
+      </c>
+      <c r="I273" s="20">
+        <v>-0.57148811196592597</v>
+      </c>
+      <c r="J273" s="24">
+        <v>0.158807672173572</v>
+      </c>
+      <c r="K273" s="15"/>
+      <c r="L273" s="5" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="274" spans="1:12" x14ac:dyDescent="0.45">
@@ -13218,30 +13225,23 @@
       <c r="B274" t="s">
         <v>258</v>
       </c>
-      <c r="C274" t="s">
-        <v>680</v>
-      </c>
       <c r="D274" t="s">
-        <v>260</v>
+        <v>692</v>
       </c>
       <c r="E274" t="s">
-        <v>528</v>
+        <v>696</v>
       </c>
       <c r="F274" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H274" s="3">
-        <v>-3.6467902022801</v>
+        <v>0.33833705716155399</v>
       </c>
       <c r="I274" s="3">
-        <v>-0.57021594101123496</v>
-      </c>
-      <c r="J274" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L274" t="s">
-        <v>635</v>
+        <v>2.0752737684215899E-2</v>
+      </c>
+      <c r="J274" s="13">
+        <v>0.38668516346655102</v>
       </c>
     </row>
     <row r="275" spans="1:12" x14ac:dyDescent="0.45">
@@ -13252,23 +13252,30 @@
       <c r="B275" t="s">
         <v>258</v>
       </c>
+      <c r="C275" t="s">
+        <v>680</v>
+      </c>
       <c r="D275" t="s">
-        <v>693</v>
+        <v>260</v>
       </c>
       <c r="E275" t="s">
-        <v>697</v>
+        <v>528</v>
       </c>
       <c r="F275" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H275" s="3">
-        <v>0</v>
+        <v>-3.6467902022801</v>
       </c>
       <c r="I275" s="3">
-        <v>0</v>
-      </c>
-      <c r="J275" s="13">
-        <v>0.125</v>
+        <v>-0.57021594101123496</v>
+      </c>
+      <c r="J275" s="13" t="e">
+        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="L275" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="276" spans="1:12" x14ac:dyDescent="0.45">
@@ -13280,22 +13287,22 @@
         <v>258</v>
       </c>
       <c r="D276" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="E276" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="F276" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H276" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I276" s="3">
         <v>0</v>
       </c>
       <c r="J276" s="13">
-        <v>0.5</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="277" spans="1:12" x14ac:dyDescent="0.45">
@@ -13306,30 +13313,23 @@
       <c r="B277" t="s">
         <v>258</v>
       </c>
-      <c r="C277" t="s">
-        <v>680</v>
-      </c>
       <c r="D277" t="s">
-        <v>261</v>
+        <v>688</v>
       </c>
       <c r="E277" t="s">
-        <v>529</v>
+        <v>698</v>
       </c>
       <c r="F277" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H277" s="3">
-        <v>-2.8385181470369503E-4</v>
+        <v>-1</v>
       </c>
       <c r="I277" s="3">
-        <v>4.9965455276017201E-2</v>
-      </c>
-      <c r="J277" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L277" t="s">
-        <v>635</v>
+        <v>0</v>
+      </c>
+      <c r="J277" s="13">
+        <v>0.5</v>
       </c>
     </row>
     <row r="278" spans="1:12" x14ac:dyDescent="0.45">
@@ -13340,23 +13340,30 @@
       <c r="B278" t="s">
         <v>258</v>
       </c>
+      <c r="C278" t="s">
+        <v>680</v>
+      </c>
       <c r="D278" t="s">
-        <v>690</v>
+        <v>261</v>
       </c>
       <c r="E278" t="s">
-        <v>699</v>
+        <v>529</v>
       </c>
       <c r="F278" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H278" s="3">
-        <v>-0.475222657127989</v>
+        <v>-2.8385181470369503E-4</v>
       </c>
       <c r="I278" s="3">
-        <v>3.1485056391258799</v>
-      </c>
-      <c r="J278" s="13">
-        <v>0.58516260162601597</v>
+        <v>4.9965455276017201E-2</v>
+      </c>
+      <c r="J278" s="13" t="e">
+        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="L278" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="279" spans="1:12" x14ac:dyDescent="0.45">
@@ -13367,30 +13374,23 @@
       <c r="B279" t="s">
         <v>258</v>
       </c>
-      <c r="C279" t="s">
-        <v>680</v>
-      </c>
       <c r="D279" t="s">
-        <v>262</v>
+        <v>690</v>
       </c>
       <c r="E279" t="s">
-        <v>530</v>
+        <v>699</v>
       </c>
       <c r="F279" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H279" s="3">
-        <v>-1.125</v>
+        <v>-0.475222657127989</v>
       </c>
       <c r="I279" s="3">
-        <v>-6.640625E-2</v>
-      </c>
-      <c r="J279" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-      <c r="L279" t="s">
-        <v>635</v>
+        <v>3.1485056391258799</v>
+      </c>
+      <c r="J279" s="13">
+        <v>0.58516260162601597</v>
       </c>
     </row>
     <row r="280" spans="1:12" x14ac:dyDescent="0.45">
@@ -13398,34 +13398,32 @@
         <f t="shared" si="5"/>
         <v>278</v>
       </c>
-      <c r="B280" s="15" t="s">
+      <c r="B280" t="s">
         <v>258</v>
       </c>
-      <c r="C280" s="15" t="s">
+      <c r="C280" t="s">
         <v>680</v>
       </c>
-      <c r="D280" s="15" t="s">
-        <v>263</v>
-      </c>
-      <c r="E280" s="15" t="s">
-        <v>531</v>
-      </c>
-      <c r="F280" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G280" s="15"/>
-      <c r="H280" s="20">
-        <v>-1.6356183941933999</v>
-      </c>
-      <c r="I280" s="20">
-        <v>2.4050322445418201E-2</v>
-      </c>
-      <c r="J280" s="24" t="e">
+      <c r="D280" t="s">
+        <v>262</v>
+      </c>
+      <c r="E280" t="s">
+        <v>530</v>
+      </c>
+      <c r="F280" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H280" s="3">
+        <v>-1.125</v>
+      </c>
+      <c r="I280" s="3">
+        <v>-6.640625E-2</v>
+      </c>
+      <c r="J280" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K280" s="15"/>
-      <c r="L280" s="15" t="s">
+      <c r="L280" t="s">
         <v>635</v>
       </c>
     </row>
@@ -13434,32 +13432,34 @@
         <f t="shared" si="5"/>
         <v>279</v>
       </c>
-      <c r="B281" t="s">
+      <c r="B281" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="C281" t="s">
+      <c r="C281" s="15" t="s">
         <v>680</v>
       </c>
-      <c r="D281" t="s">
-        <v>264</v>
-      </c>
-      <c r="E281" t="s">
-        <v>532</v>
-      </c>
-      <c r="F281" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H281" s="3">
-        <v>2.5644984865162299</v>
-      </c>
-      <c r="I281" s="3">
-        <v>0.150454045129335</v>
-      </c>
-      <c r="J281" s="13" t="e">
+      <c r="D281" s="15" t="s">
+        <v>263</v>
+      </c>
+      <c r="E281" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="F281" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G281" s="15"/>
+      <c r="H281" s="20">
+        <v>-1.6356183941933999</v>
+      </c>
+      <c r="I281" s="20">
+        <v>2.4050322445418201E-2</v>
+      </c>
+      <c r="J281" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L281" t="s">
+      <c r="K281" s="15"/>
+      <c r="L281" s="15" t="s">
         <v>635</v>
       </c>
     </row>
@@ -13471,23 +13471,30 @@
       <c r="B282" t="s">
         <v>258</v>
       </c>
+      <c r="C282" t="s">
+        <v>680</v>
+      </c>
       <c r="D282" t="s">
-        <v>691</v>
+        <v>264</v>
       </c>
       <c r="E282" t="s">
-        <v>700</v>
+        <v>532</v>
       </c>
       <c r="F282" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H282" s="3">
-        <v>8.3362278568983993E-3</v>
+        <v>2.5644984865162299</v>
       </c>
       <c r="I282" s="3">
-        <v>4.1681139284472798E-2</v>
-      </c>
-      <c r="J282" s="13">
-        <v>8.3042862982190005E-2</v>
+        <v>0.150454045129335</v>
+      </c>
+      <c r="J282" s="13" t="e">
+        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="L282" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="283" spans="1:12" x14ac:dyDescent="0.45">
@@ -13499,22 +13506,22 @@
         <v>258</v>
       </c>
       <c r="D283" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="E283" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="F283" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H283" s="3">
-        <v>-1.03965794826681</v>
+        <v>8.3362278568983993E-3</v>
       </c>
       <c r="I283" s="3">
-        <v>8.4535007877224594E-2</v>
+        <v>4.1681139284472798E-2</v>
       </c>
       <c r="J283" s="13">
-        <v>0.43527528164806201</v>
+        <v>8.3042862982190005E-2</v>
       </c>
     </row>
     <row r="284" spans="1:12" x14ac:dyDescent="0.45">
@@ -13526,22 +13533,22 @@
         <v>258</v>
       </c>
       <c r="D284" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="E284" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="F284" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H284" s="3">
-        <v>7.8152136158388397E-2</v>
+        <v>-1.03965794826681</v>
       </c>
       <c r="I284" s="3">
-        <v>-0.49639631816602903</v>
+        <v>8.4535007877224594E-2</v>
       </c>
       <c r="J284" s="13">
-        <v>1.3158135283363801</v>
+        <v>0.43527528164806201</v>
       </c>
     </row>
     <row r="285" spans="1:12" x14ac:dyDescent="0.45">
@@ -13549,66 +13556,58 @@
         <f t="shared" si="5"/>
         <v>283</v>
       </c>
-      <c r="B285" s="15" t="s">
+      <c r="B285" t="s">
         <v>258</v>
       </c>
-      <c r="C285" s="15" t="s">
-        <v>680</v>
-      </c>
-      <c r="D285" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="E285" s="15" t="s">
-        <v>533</v>
-      </c>
-      <c r="F285" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G285" s="15"/>
-      <c r="H285" s="20">
-        <v>1</v>
-      </c>
-      <c r="I285" s="20">
-        <v>0</v>
-      </c>
-      <c r="J285" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="286" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D285" t="s">
+        <v>695</v>
+      </c>
+      <c r="E285" t="s">
+        <v>702</v>
+      </c>
+      <c r="F285" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H285" s="3">
+        <v>7.8152136158388397E-2</v>
+      </c>
+      <c r="I285" s="3">
+        <v>-0.49639631816602903</v>
+      </c>
+      <c r="J285" s="13">
+        <v>1.3158135283363801</v>
+      </c>
+    </row>
+    <row r="286" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A286" s="2">
         <f t="shared" si="5"/>
         <v>284</v>
       </c>
-      <c r="B286" s="5" t="s">
+      <c r="B286" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="C286" s="5" t="s">
+      <c r="C286" s="15" t="s">
         <v>680</v>
       </c>
-      <c r="D286" s="5" t="s">
-        <v>689</v>
-      </c>
-      <c r="E286" s="5" t="s">
+      <c r="D286" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="E286" s="15" t="s">
         <v>533</v>
       </c>
-      <c r="F286" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G286" s="5"/>
-      <c r="H286" s="6">
-        <v>-0.25343772240527501</v>
-      </c>
-      <c r="I286" s="6">
-        <v>2.8551421212316399E-3</v>
-      </c>
-      <c r="J286" s="23">
-        <v>0.325449642392387</v>
-      </c>
-      <c r="K286" s="15"/>
-      <c r="L286" s="15" t="s">
-        <v>635</v>
+      <c r="F286" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G286" s="15"/>
+      <c r="H286" s="20">
+        <v>1</v>
+      </c>
+      <c r="I286" s="20">
+        <v>0</v>
+      </c>
+      <c r="J286" s="24" t="e">
+        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="287" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -13616,68 +13615,69 @@
         <f t="shared" si="5"/>
         <v>285</v>
       </c>
-      <c r="B287" s="15" t="s">
-        <v>266</v>
-      </c>
-      <c r="C287" s="15" t="s">
-        <v>682</v>
-      </c>
-      <c r="D287" s="15" t="s">
-        <v>267</v>
-      </c>
-      <c r="E287" s="15" t="s">
-        <v>613</v>
-      </c>
-      <c r="F287" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G287" s="15"/>
-      <c r="H287" s="20">
-        <v>0</v>
-      </c>
-      <c r="I287" s="20">
-        <v>0</v>
-      </c>
-      <c r="J287" s="24" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="B287" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C287" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="D287" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E287" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="F287" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G287" s="5"/>
+      <c r="H287" s="6">
+        <v>-0.25343772240527501</v>
+      </c>
+      <c r="I287" s="6">
+        <v>2.8551421212316399E-3</v>
+      </c>
+      <c r="J287" s="23">
+        <v>0.325449642392387</v>
       </c>
       <c r="K287" s="15"/>
-      <c r="L287" s="5" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="288" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L287" s="15" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="288" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A288" s="2">
         <f t="shared" si="5"/>
         <v>286</v>
       </c>
-      <c r="B288" t="s">
+      <c r="B288" s="15" t="s">
         <v>266</v>
       </c>
-      <c r="C288" t="s">
+      <c r="C288" s="15" t="s">
         <v>682</v>
       </c>
-      <c r="D288" t="s">
-        <v>268</v>
-      </c>
-      <c r="E288" t="s">
-        <v>534</v>
-      </c>
-      <c r="F288" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H288" s="3">
-        <v>0</v>
-      </c>
-      <c r="I288" s="3">
-        <v>0</v>
-      </c>
-      <c r="J288" s="13" t="e">
+      <c r="D288" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="E288" s="15" t="s">
+        <v>613</v>
+      </c>
+      <c r="F288" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G288" s="15"/>
+      <c r="H288" s="20">
+        <v>0</v>
+      </c>
+      <c r="I288" s="20">
+        <v>0</v>
+      </c>
+      <c r="J288" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L288" t="s">
+      <c r="K288" s="15"/>
+      <c r="L288" s="5" t="s">
         <v>635</v>
       </c>
     </row>
@@ -13686,34 +13686,32 @@
         <f t="shared" si="5"/>
         <v>287</v>
       </c>
-      <c r="B289" s="15" t="s">
+      <c r="B289" t="s">
         <v>266</v>
       </c>
-      <c r="C289" s="15" t="s">
+      <c r="C289" t="s">
         <v>682</v>
       </c>
-      <c r="D289" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="E289" s="15" t="s">
-        <v>614</v>
-      </c>
-      <c r="F289" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G289" s="15"/>
-      <c r="H289" s="20">
-        <v>0.16760835707052199</v>
-      </c>
-      <c r="I289" s="20">
-        <v>6.7221673977560195E-2</v>
-      </c>
-      <c r="J289" s="24" t="e">
+      <c r="D289" t="s">
+        <v>268</v>
+      </c>
+      <c r="E289" t="s">
+        <v>534</v>
+      </c>
+      <c r="F289" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H289" s="3">
+        <v>0</v>
+      </c>
+      <c r="I289" s="3">
+        <v>0</v>
+      </c>
+      <c r="J289" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K289" s="15"/>
-      <c r="L289" s="15" t="s">
+      <c r="L289" t="s">
         <v>635</v>
       </c>
     </row>
@@ -13722,32 +13720,34 @@
         <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="B290" t="s">
+      <c r="B290" s="15" t="s">
         <v>266</v>
       </c>
-      <c r="C290" t="s">
+      <c r="C290" s="15" t="s">
         <v>682</v>
       </c>
-      <c r="D290" t="s">
-        <v>270</v>
-      </c>
-      <c r="E290" t="s">
-        <v>615</v>
-      </c>
-      <c r="F290" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H290" s="3">
-        <v>0.99997794894719205</v>
-      </c>
-      <c r="I290" s="3">
-        <v>3.43019728514361E-4</v>
-      </c>
-      <c r="J290" s="13" t="e">
+      <c r="D290" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="E290" s="15" t="s">
+        <v>614</v>
+      </c>
+      <c r="F290" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G290" s="15"/>
+      <c r="H290" s="20">
+        <v>0.16760835707052199</v>
+      </c>
+      <c r="I290" s="20">
+        <v>6.7221673977560195E-2</v>
+      </c>
+      <c r="J290" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L290" t="s">
+      <c r="K290" s="15"/>
+      <c r="L290" s="15" t="s">
         <v>635</v>
       </c>
     </row>
@@ -13763,19 +13763,19 @@
         <v>682</v>
       </c>
       <c r="D291" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E291" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="F291" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H291" s="3">
-        <v>-2.2653064412820599E-3</v>
+        <v>0.99997794894719205</v>
       </c>
       <c r="I291" s="3">
-        <v>-1.00952600415555E-2</v>
+        <v>3.43019728514361E-4</v>
       </c>
       <c r="J291" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -13785,215 +13785,215 @@
         <v>635</v>
       </c>
     </row>
-    <row r="292" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A292" s="2">
         <f t="shared" si="5"/>
         <v>290</v>
       </c>
-      <c r="B292" s="5" t="s">
+      <c r="B292" t="s">
         <v>266</v>
       </c>
-      <c r="C292" s="5" t="s">
+      <c r="C292" t="s">
         <v>682</v>
       </c>
-      <c r="D292" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="E292" s="5" t="s">
-        <v>617</v>
-      </c>
-      <c r="F292" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G292" s="5"/>
-      <c r="H292" s="6">
-        <v>-0.449612977602108</v>
-      </c>
-      <c r="I292" s="6">
-        <v>-0.53004776021080202</v>
-      </c>
-      <c r="J292" s="23" t="e">
+      <c r="D292" t="s">
+        <v>271</v>
+      </c>
+      <c r="E292" t="s">
+        <v>616</v>
+      </c>
+      <c r="F292" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H292" s="3">
+        <v>-2.2653064412820599E-3</v>
+      </c>
+      <c r="I292" s="3">
+        <v>-1.00952600415555E-2</v>
+      </c>
+      <c r="J292" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K292" s="5"/>
-      <c r="L292" s="15" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="293" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L292" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="293" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A293" s="2">
         <f t="shared" si="5"/>
         <v>291</v>
       </c>
-      <c r="B293" t="s">
-        <v>273</v>
-      </c>
-      <c r="C293" t="s">
-        <v>678</v>
-      </c>
-      <c r="D293" t="s">
-        <v>274</v>
-      </c>
-      <c r="E293" t="s">
-        <v>618</v>
-      </c>
-      <c r="F293" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H293" s="3">
-        <v>0</v>
-      </c>
-      <c r="I293" s="3">
-        <v>0</v>
-      </c>
-      <c r="J293" s="13" t="e">
+      <c r="B293" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C293" s="5" t="s">
+        <v>682</v>
+      </c>
+      <c r="D293" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="E293" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="F293" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G293" s="5"/>
+      <c r="H293" s="6">
+        <v>-0.449612977602108</v>
+      </c>
+      <c r="I293" s="6">
+        <v>-0.53004776021080202</v>
+      </c>
+      <c r="J293" s="23" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L293" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="294" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="K293" s="5"/>
+      <c r="L293" s="15" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="294" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A294" s="2">
         <f t="shared" si="5"/>
         <v>292</v>
       </c>
-      <c r="B294" s="5" t="s">
+      <c r="B294" t="s">
         <v>273</v>
       </c>
-      <c r="C294" s="5" t="s">
+      <c r="C294" t="s">
         <v>678</v>
       </c>
-      <c r="D294" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="E294" s="5" t="s">
-        <v>619</v>
-      </c>
-      <c r="F294" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G294" s="5"/>
-      <c r="H294" s="6">
-        <v>0</v>
-      </c>
-      <c r="I294" s="6">
-        <v>0</v>
-      </c>
-      <c r="J294" s="23" t="e">
+      <c r="D294" t="s">
+        <v>274</v>
+      </c>
+      <c r="E294" t="s">
+        <v>618</v>
+      </c>
+      <c r="F294" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H294" s="3">
+        <v>0</v>
+      </c>
+      <c r="I294" s="3">
+        <v>0</v>
+      </c>
+      <c r="J294" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K294" s="5"/>
-      <c r="L294" s="5" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L294" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="295" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A295" s="2">
         <f t="shared" si="5"/>
         <v>293</v>
       </c>
-      <c r="B295" s="18" t="s">
-        <v>276</v>
-      </c>
-      <c r="C295" s="18" t="s">
-        <v>684</v>
-      </c>
-      <c r="D295" s="18" t="s">
-        <v>359</v>
-      </c>
-      <c r="E295" s="18" t="s">
-        <v>623</v>
-      </c>
-      <c r="F295" s="17" t="s">
-        <v>302</v>
-      </c>
-      <c r="G295" s="18"/>
-      <c r="H295" s="19">
-        <v>-0.77812499999999996</v>
-      </c>
-      <c r="I295" s="19">
-        <v>3.515625E-2</v>
-      </c>
-      <c r="J295" s="26" t="e">
+      <c r="B295" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C295" s="5" t="s">
+        <v>678</v>
+      </c>
+      <c r="D295" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="E295" s="5" t="s">
+        <v>619</v>
+      </c>
+      <c r="F295" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G295" s="5"/>
+      <c r="H295" s="6">
+        <v>0</v>
+      </c>
+      <c r="I295" s="6">
+        <v>0</v>
+      </c>
+      <c r="J295" s="23" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K295" s="18"/>
-      <c r="L295" s="18" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="296" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="K295" s="5"/>
+      <c r="L295" s="5" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="296" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A296" s="2">
         <f t="shared" si="5"/>
         <v>294</v>
       </c>
-      <c r="B296" s="15" t="s">
+      <c r="B296" s="18" t="s">
         <v>276</v>
       </c>
-      <c r="C296" s="15" t="s">
-        <v>643</v>
-      </c>
-      <c r="D296" s="15" t="s">
-        <v>278</v>
-      </c>
-      <c r="E296" s="15" t="s">
-        <v>535</v>
-      </c>
-      <c r="F296" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G296" s="15"/>
-      <c r="H296" s="20">
-        <v>-0.826954434020021</v>
-      </c>
-      <c r="I296" s="20">
-        <v>1.5896229075411601</v>
-      </c>
-      <c r="J296" s="24" t="e">
+      <c r="C296" s="18" t="s">
+        <v>684</v>
+      </c>
+      <c r="D296" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="E296" s="18" t="s">
+        <v>623</v>
+      </c>
+      <c r="F296" s="17" t="s">
+        <v>302</v>
+      </c>
+      <c r="G296" s="18"/>
+      <c r="H296" s="19">
+        <v>-0.77812499999999996</v>
+      </c>
+      <c r="I296" s="19">
+        <v>3.515625E-2</v>
+      </c>
+      <c r="J296" s="26" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K296" s="15"/>
-      <c r="L296" s="5" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="297" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="K296" s="18"/>
+      <c r="L296" s="18" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="297" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A297" s="2">
         <f t="shared" si="5"/>
         <v>295</v>
       </c>
-      <c r="B297" t="s">
+      <c r="B297" s="15" t="s">
         <v>276</v>
       </c>
-      <c r="C297" s="21" t="s">
-        <v>684</v>
-      </c>
-      <c r="D297" t="s">
-        <v>279</v>
-      </c>
-      <c r="E297" t="s">
-        <v>621</v>
-      </c>
-      <c r="F297" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H297" s="3">
-        <v>-3.1848898182744501</v>
-      </c>
-      <c r="I297" s="3">
-        <v>-0.196294466403164</v>
-      </c>
-      <c r="J297" s="13" t="e">
+      <c r="C297" s="15" t="s">
+        <v>643</v>
+      </c>
+      <c r="D297" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="E297" s="15" t="s">
+        <v>535</v>
+      </c>
+      <c r="F297" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G297" s="15"/>
+      <c r="H297" s="20">
+        <v>-0.826954434020021</v>
+      </c>
+      <c r="I297" s="20">
+        <v>1.5896229075411601</v>
+      </c>
+      <c r="J297" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L297" t="s">
+      <c r="K297" s="15"/>
+      <c r="L297" s="5" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14009,19 +14009,19 @@
         <v>684</v>
       </c>
       <c r="D298" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E298" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F298" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H298" s="3">
-        <v>-3.14831538728725</v>
+        <v>-3.1848898182744501</v>
       </c>
       <c r="I298" s="3">
-        <v>8.3362278568941406E-3</v>
+        <v>-0.196294466403164</v>
       </c>
       <c r="J298" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -14039,26 +14039,23 @@
       <c r="B299" t="s">
         <v>276</v>
       </c>
-      <c r="C299" t="s">
-        <v>643</v>
+      <c r="C299" s="21" t="s">
+        <v>684</v>
       </c>
       <c r="D299" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="E299" t="s">
-        <v>644</v>
+        <v>620</v>
       </c>
       <c r="F299" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="G299" t="s">
-        <v>357</v>
-      </c>
       <c r="H299" s="3">
-        <v>-0.47339389427906398</v>
+        <v>-3.14831538728725</v>
       </c>
       <c r="I299" s="3">
-        <v>4.7485146095140003E-4</v>
+        <v>8.3362278568941406E-3</v>
       </c>
       <c r="J299" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -14076,23 +14073,26 @@
       <c r="B300" t="s">
         <v>276</v>
       </c>
-      <c r="C300" s="21" t="s">
-        <v>684</v>
+      <c r="C300" t="s">
+        <v>643</v>
       </c>
       <c r="D300" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E300" t="s">
-        <v>622</v>
+        <v>644</v>
       </c>
       <c r="F300" s="2" t="s">
         <v>302</v>
       </c>
+      <c r="G300" t="s">
+        <v>357</v>
+      </c>
       <c r="H300" s="3">
-        <v>1.5392416007905101</v>
+        <v>-0.47339389427906398</v>
       </c>
       <c r="I300" s="3">
-        <v>1.91370223978919E-2</v>
+        <v>4.7485146095140003E-4</v>
       </c>
       <c r="J300" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -14110,23 +14110,23 @@
       <c r="B301" t="s">
         <v>276</v>
       </c>
-      <c r="C301" t="s">
-        <v>643</v>
+      <c r="C301" s="21" t="s">
+        <v>684</v>
       </c>
       <c r="D301" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E301" t="s">
-        <v>537</v>
+        <v>622</v>
       </c>
       <c r="F301" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H301" s="3">
-        <v>0</v>
+        <v>1.5392416007905101</v>
       </c>
       <c r="I301" s="3">
-        <v>0</v>
+        <v>1.91370223978919E-2</v>
       </c>
       <c r="J301" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -14136,115 +14136,113 @@
         <v>635</v>
       </c>
     </row>
-    <row r="302" spans="1:12" s="18" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="302" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A302" s="2">
         <f t="shared" si="5"/>
         <v>300</v>
       </c>
-      <c r="B302" s="5" t="s">
+      <c r="B302" t="s">
         <v>276</v>
       </c>
-      <c r="C302" s="5" t="s">
+      <c r="C302" t="s">
         <v>643</v>
       </c>
-      <c r="D302" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="E302" s="5" t="s">
-        <v>538</v>
-      </c>
-      <c r="F302" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="G302" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="H302" s="6">
-        <v>0</v>
-      </c>
-      <c r="I302" s="6">
-        <v>0</v>
-      </c>
-      <c r="J302" s="23" t="e">
+      <c r="D302" t="s">
+        <v>282</v>
+      </c>
+      <c r="E302" t="s">
+        <v>537</v>
+      </c>
+      <c r="F302" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H302" s="3">
+        <v>0</v>
+      </c>
+      <c r="I302" s="3">
+        <v>0</v>
+      </c>
+      <c r="J302" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K302" s="5"/>
-      <c r="L302" s="15" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="303" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L302" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="303" spans="1:12" s="18" customFormat="1" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A303" s="2">
         <f t="shared" si="5"/>
         <v>301</v>
       </c>
-      <c r="B303" t="s">
-        <v>284</v>
-      </c>
-      <c r="C303" t="s">
-        <v>683</v>
-      </c>
-      <c r="D303" t="s">
-        <v>285</v>
-      </c>
-      <c r="E303" t="s">
-        <v>624</v>
-      </c>
-      <c r="F303" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H303">
-        <v>1.5315544451803</v>
-      </c>
-      <c r="I303" s="3">
-        <v>3.53980226158776E-2</v>
-      </c>
-      <c r="J303" s="13" t="e">
+      <c r="B303" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="C303" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="D303" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="E303" s="5" t="s">
+        <v>538</v>
+      </c>
+      <c r="F303" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="G303" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="H303" s="6">
+        <v>0</v>
+      </c>
+      <c r="I303" s="6">
+        <v>0</v>
+      </c>
+      <c r="J303" s="23" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L303" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="304" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="K303" s="5"/>
+      <c r="L303" s="15" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="304" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A304" s="2">
         <f t="shared" si="5"/>
         <v>302</v>
       </c>
-      <c r="B304" s="15" t="s">
+      <c r="B304" t="s">
         <v>284</v>
       </c>
-      <c r="C304" s="15" t="s">
+      <c r="C304" t="s">
         <v>683</v>
       </c>
-      <c r="D304" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="E304" s="15" t="s">
-        <v>626</v>
-      </c>
-      <c r="F304" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G304" s="15"/>
-      <c r="H304" s="20">
-        <v>0</v>
-      </c>
-      <c r="I304" s="20">
-        <v>0</v>
-      </c>
-      <c r="J304" s="24" t="e">
+      <c r="D304" t="s">
+        <v>285</v>
+      </c>
+      <c r="E304" t="s">
+        <v>624</v>
+      </c>
+      <c r="F304" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H304">
+        <v>1.5315544451803</v>
+      </c>
+      <c r="I304" s="3">
+        <v>3.53980226158776E-2</v>
+      </c>
+      <c r="J304" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K304" s="15"/>
-      <c r="L304" s="5" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="305" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="L304" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="305" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A305" s="2">
         <f t="shared" si="5"/>
         <v>303</v>
@@ -14256,10 +14254,10 @@
         <v>683</v>
       </c>
       <c r="D305" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E305" s="15" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F305" s="7" t="s">
         <v>302</v>
@@ -14276,7 +14274,7 @@
         <v>#REF!</v>
       </c>
       <c r="K305" s="15"/>
-      <c r="L305" s="15" t="s">
+      <c r="L305" s="5" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14285,32 +14283,34 @@
         <f t="shared" si="5"/>
         <v>304</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B306" s="15" t="s">
         <v>284</v>
       </c>
-      <c r="C306" t="s">
+      <c r="C306" s="15" t="s">
         <v>683</v>
       </c>
-      <c r="D306" t="s">
-        <v>288</v>
-      </c>
-      <c r="E306" t="s">
-        <v>627</v>
-      </c>
-      <c r="F306" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H306" s="3">
-        <v>-5.5853884353168397E-2</v>
-      </c>
-      <c r="I306" s="3">
-        <v>1.89764329601885E-2</v>
-      </c>
-      <c r="J306" s="13" t="e">
+      <c r="D306" s="15" t="s">
+        <v>286</v>
+      </c>
+      <c r="E306" s="15" t="s">
+        <v>625</v>
+      </c>
+      <c r="F306" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G306" s="15"/>
+      <c r="H306" s="20">
+        <v>0</v>
+      </c>
+      <c r="I306" s="20">
+        <v>0</v>
+      </c>
+      <c r="J306" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L306" t="s">
+      <c r="K306" s="15"/>
+      <c r="L306" s="15" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14326,19 +14326,19 @@
         <v>683</v>
       </c>
       <c r="D307" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E307" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="F307" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H307" s="3">
-        <v>0</v>
+        <v>-5.5853884353168397E-2</v>
       </c>
       <c r="I307" s="3">
-        <v>0</v>
+        <v>1.89764329601885E-2</v>
       </c>
       <c r="J307" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -14360,10 +14360,10 @@
         <v>683</v>
       </c>
       <c r="D308" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E308" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="F308" s="2" t="s">
         <v>302</v>
@@ -14394,10 +14394,10 @@
         <v>683</v>
       </c>
       <c r="D309" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E309" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F309" s="2" t="s">
         <v>302</v>
@@ -14428,10 +14428,10 @@
         <v>683</v>
       </c>
       <c r="D310" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="E310" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="F310" s="2" t="s">
         <v>302</v>
@@ -14462,10 +14462,10 @@
         <v>683</v>
       </c>
       <c r="D311" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E311" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F311" s="2" t="s">
         <v>302</v>
@@ -14496,19 +14496,19 @@
         <v>683</v>
       </c>
       <c r="D312" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="E312" t="s">
-        <v>536</v>
+        <v>632</v>
       </c>
       <c r="F312" s="2" t="s">
         <v>302</v>
       </c>
       <c r="H312" s="3">
-        <v>-0.79706422018348599</v>
+        <v>0</v>
       </c>
       <c r="I312" s="3">
-        <v>1.1009174311926201E-3</v>
+        <v>0</v>
       </c>
       <c r="J312" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
@@ -14523,34 +14523,32 @@
         <f t="shared" si="5"/>
         <v>311</v>
       </c>
-      <c r="B313" s="15" t="s">
+      <c r="B313" t="s">
         <v>284</v>
       </c>
-      <c r="C313" s="15" t="s">
+      <c r="C313" t="s">
         <v>683</v>
       </c>
-      <c r="D313" s="15" t="s">
-        <v>296</v>
-      </c>
-      <c r="E313" s="15" t="s">
-        <v>634</v>
-      </c>
-      <c r="F313" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="G313" s="15"/>
-      <c r="H313" s="20">
-        <v>1.32110091743115E-2</v>
-      </c>
-      <c r="I313" s="20">
-        <v>5.72477064220187E-2</v>
-      </c>
-      <c r="J313" s="24" t="e">
+      <c r="D313" t="s">
+        <v>294</v>
+      </c>
+      <c r="E313" t="s">
+        <v>536</v>
+      </c>
+      <c r="F313" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H313" s="3">
+        <v>-0.79706422018348599</v>
+      </c>
+      <c r="I313" s="3">
+        <v>1.1009174311926201E-3</v>
+      </c>
+      <c r="J313" s="13" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="K313" s="15"/>
-      <c r="L313" s="15" t="s">
+      <c r="L313" t="s">
         <v>635</v>
       </c>
     </row>
@@ -14559,48 +14557,84 @@
         <f t="shared" si="5"/>
         <v>312</v>
       </c>
-      <c r="B314" t="s">
+      <c r="B314" s="15" t="s">
         <v>284</v>
       </c>
-      <c r="C314" t="s">
+      <c r="C314" s="15" t="s">
         <v>683</v>
       </c>
-      <c r="D314" t="s">
-        <v>295</v>
-      </c>
-      <c r="E314" t="s">
-        <v>633</v>
-      </c>
-      <c r="F314" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H314" s="3">
-        <v>0</v>
-      </c>
-      <c r="I314" s="3">
-        <v>0</v>
-      </c>
-      <c r="J314" s="13" t="e">
+      <c r="D314" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="E314" s="15" t="s">
+        <v>634</v>
+      </c>
+      <c r="F314" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="G314" s="15"/>
+      <c r="H314" s="20">
+        <v>1.32110091743115E-2</v>
+      </c>
+      <c r="I314" s="20">
+        <v>5.72477064220187E-2</v>
+      </c>
+      <c r="J314" s="24" t="e">
         <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
         <v>#REF!</v>
       </c>
-      <c r="L314" t="s">
-        <v>635</v>
-      </c>
-    </row>
-    <row r="321" spans="7:7" x14ac:dyDescent="0.45">
-      <c r="G321">
+      <c r="K314" s="15"/>
+      <c r="L314" s="15" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="315" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A315" s="2">
+        <f t="shared" si="5"/>
+        <v>313</v>
+      </c>
+      <c r="B315" t="s">
+        <v>284</v>
+      </c>
+      <c r="C315" t="s">
+        <v>683</v>
+      </c>
+      <c r="D315" t="s">
+        <v>295</v>
+      </c>
+      <c r="E315" t="s">
+        <v>633</v>
+      </c>
+      <c r="F315" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H315" s="3">
+        <v>0</v>
+      </c>
+      <c r="I315" s="3">
+        <v>0</v>
+      </c>
+      <c r="J315" s="13" t="e">
+        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
+        <v>#REF!</v>
+      </c>
+      <c r="L315" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="322" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G322">
         <f>294-244</f>
         <v>50</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L314" xr:uid="{DDCD0A24-47A3-4D2D-80DF-18729F910C8C}">
-    <sortState ref="A2:L314">
-      <sortCondition ref="B1:B314"/>
+  <autoFilter ref="A1:L315" xr:uid="{DDCD0A24-47A3-4D2D-80DF-18729F910C8C}">
+    <sortState ref="A2:L315">
+      <sortCondition ref="B1:B315"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="F78 F124:F141 F165:F171 F173:F175 F177:F184 F217:F223 F225:F227 F229:F231 F233:F241 F243:F249 F251:F257 F259:F265 F267:F271 F273:F285 F289:F293 F295 F58:F60 F186:F207 F297:F303 F62:F66 F305:F314 F42 F49:F53 F47 F143:F162">
+  <conditionalFormatting sqref="F78 F124:F141 F165:F171 F173:F175 F177:F184 F217:F223 F225:F227 F229:F231 F233:F241 F243:F249 F251:F257 F259:F265 F267:F272 F274:F286 F290:F294 F296 F58:F60 F186:F207 F298:F304 F62:F66 F306:F315 F42 F49:F53 F47 F143:F162">
     <cfRule type="cellIs" dxfId="113" priority="191" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -14624,7 +14658,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F272">
+  <conditionalFormatting sqref="F273">
     <cfRule type="cellIs" dxfId="107" priority="133" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -14632,7 +14666,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F288">
+  <conditionalFormatting sqref="F289">
     <cfRule type="cellIs" dxfId="105" priority="131" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -14976,7 +15010,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F287">
+  <conditionalFormatting sqref="F288">
     <cfRule type="cellIs" dxfId="19" priority="21" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -14984,7 +15018,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F294">
+  <conditionalFormatting sqref="F295">
     <cfRule type="cellIs" dxfId="17" priority="19" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -14992,7 +15026,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F296">
+  <conditionalFormatting sqref="F297">
     <cfRule type="cellIs" dxfId="15" priority="17" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -15000,7 +15034,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F304">
+  <conditionalFormatting sqref="F305">
     <cfRule type="cellIs" dxfId="13" priority="15" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -15008,7 +15042,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F286">
+  <conditionalFormatting sqref="F287">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
@@ -15057,7 +15091,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F78 F42:F43 F45:F66 F124:F314" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F78 F42:F43 F45:F66 F124:F315" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F44 F67:F77 F2:F41 F79:F123" xr:uid="{00000000-0002-0000-0000-000001000000}">

</xml_diff>

<commit_message>
Finished initial conditions through Tricorn family.  Fixed Duffing Attractor conditions.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA68F4A-7CFB-4421-B75E-615D26FA1EFB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D0AEDE-2B03-4D6A-9D45-B851BDBA756B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1889" uniqueCount="747">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="748">
   <si>
     <t>Group Name</t>
   </si>
@@ -2265,7 +2265,10 @@
     <t>Sierpinski Triangle</t>
   </si>
   <si>
-    <t>Nebulabrot (Dramatic RGB)</t>
+    <t>0.029999999999999999)</t>
+  </si>
+  <si>
+    <t>TrigammaFractal</t>
   </si>
 </sst>
 </file>
@@ -13231,14 +13234,13 @@
         <v>353</v>
       </c>
       <c r="H277" s="18">
-        <v>-0.33226284584980198</v>
-      </c>
-      <c r="I277" s="18">
-        <v>2.5321146245059298E-2</v>
-      </c>
-      <c r="J277" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.33</v>
+      </c>
+      <c r="I277" s="18" t="s">
+        <v>746</v>
+      </c>
+      <c r="J277" s="22">
+        <v>0.8</v>
       </c>
       <c r="K277" s="15"/>
       <c r="L277" s="5" t="s">
@@ -13271,9 +13273,8 @@
       <c r="I278" s="3">
         <v>-0.43648097826086701</v>
       </c>
-      <c r="J278" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J278" s="13">
+        <v>0.02</v>
       </c>
       <c r="L278" t="s">
         <v>634</v>
@@ -13300,13 +13301,13 @@
         <v>302</v>
       </c>
       <c r="H279" s="3">
-        <v>-5.6126062322933903E-3</v>
+        <v>-0.01</v>
       </c>
       <c r="I279" s="3">
         <v>1.19068696883983E-3</v>
       </c>
-      <c r="J279" s="13" t="e">
-        <v>#REF!</v>
+      <c r="J279" s="13">
+        <v>0.153893052</v>
       </c>
     </row>
     <row r="280" spans="1:12" x14ac:dyDescent="0.45">
@@ -13319,7 +13320,7 @@
       </c>
       <c r="C280" s="15"/>
       <c r="D280" s="19" t="s">
-        <v>746</v>
+        <v>730</v>
       </c>
       <c r="E280" s="19" t="s">
         <v>730</v>
@@ -13335,7 +13336,7 @@
         <v>0.03</v>
       </c>
       <c r="J280" s="22">
-        <v>1.066667</v>
+        <v>0.8</v>
       </c>
       <c r="K280" s="15"/>
       <c r="L280" s="15"/>
@@ -13366,9 +13367,8 @@
       <c r="I281" s="3">
         <v>0</v>
       </c>
-      <c r="J281" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J281" s="13">
+        <v>0.61557220700000004</v>
       </c>
       <c r="L281" t="s">
         <v>634</v>
@@ -13396,14 +13396,13 @@
       </c>
       <c r="G282" s="5"/>
       <c r="H282" s="6">
-        <v>-0.22203909754190099</v>
+        <v>-0.22</v>
       </c>
       <c r="I282" s="6">
-        <v>5.2512073606900397E-2</v>
-      </c>
-      <c r="J282" s="21" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.05</v>
+      </c>
+      <c r="J282" s="21">
+        <v>0.240196567</v>
       </c>
       <c r="K282" s="5"/>
       <c r="L282" s="15" t="s">
@@ -13434,13 +13433,13 @@
         <v>355</v>
       </c>
       <c r="H283" s="18">
-        <v>-0.69665929008750505</v>
+        <v>-0.69665929000000004</v>
       </c>
       <c r="I283" s="18">
-        <v>-0.57148811196592597</v>
+        <v>-0.57148811200000005</v>
       </c>
       <c r="J283" s="22">
-        <v>0.158807672173572</v>
+        <v>0.15880767200000001</v>
       </c>
       <c r="K283" s="15"/>
       <c r="L283" s="5" t="s">
@@ -13465,13 +13464,13 @@
         <v>302</v>
       </c>
       <c r="H284" s="3">
-        <v>0.33833705716155399</v>
+        <v>0.34</v>
       </c>
       <c r="I284" s="3">
-        <v>2.0752737684215899E-2</v>
+        <v>0.02</v>
       </c>
       <c r="J284" s="13">
-        <v>0.38668516346655102</v>
+        <v>0.38700000000000001</v>
       </c>
     </row>
     <row r="285" spans="1:12" x14ac:dyDescent="0.45">
@@ -13495,14 +13494,13 @@
         <v>302</v>
       </c>
       <c r="H285" s="3">
-        <v>-3.6467902022801</v>
+        <v>-3.6499999999999901</v>
       </c>
       <c r="I285" s="3">
-        <v>-0.57021594101123496</v>
-      </c>
-      <c r="J285" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.56999999999999895</v>
+      </c>
+      <c r="J285" s="13">
+        <v>0.410348360999999</v>
       </c>
       <c r="L285" t="s">
         <v>634</v>
@@ -13553,13 +13551,13 @@
         <v>302</v>
       </c>
       <c r="H287" s="3">
-        <v>-1</v>
+        <v>0.75251856238707304</v>
       </c>
       <c r="I287" s="3">
-        <v>0</v>
+        <v>-0.59921156373193196</v>
       </c>
       <c r="J287" s="13">
-        <v>0.5</v>
+        <v>0.85784068136272495</v>
       </c>
     </row>
     <row r="288" spans="1:12" x14ac:dyDescent="0.45">
@@ -13583,14 +13581,13 @@
         <v>302</v>
       </c>
       <c r="H288" s="3">
-        <v>-2.8385181470369503E-4</v>
+        <v>0</v>
       </c>
       <c r="I288" s="3">
-        <v>4.9965455276017201E-2</v>
-      </c>
-      <c r="J288" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.05</v>
+      </c>
+      <c r="J288" s="13">
+        <v>8.0494791999999898E-2</v>
       </c>
       <c r="L288" t="s">
         <v>634</v>
@@ -13614,13 +13611,13 @@
         <v>302</v>
       </c>
       <c r="H289" s="3">
-        <v>-0.475222657127989</v>
+        <v>-0.47522265699999899</v>
       </c>
       <c r="I289" s="3">
-        <v>3.1485056391258799</v>
+        <v>3.1485056390000001</v>
       </c>
       <c r="J289" s="13">
-        <v>0.58516260162601597</v>
+        <v>0.58516260200000003</v>
       </c>
     </row>
     <row r="290" spans="1:12" x14ac:dyDescent="0.45">
@@ -13644,14 +13641,13 @@
         <v>302</v>
       </c>
       <c r="H290" s="3">
-        <v>-1.125</v>
+        <v>-1.1299999999999899</v>
       </c>
       <c r="I290" s="3">
-        <v>-6.640625E-2</v>
-      </c>
-      <c r="J290" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-7.0000000000000007E-2</v>
+      </c>
+      <c r="J290" s="13">
+        <v>0.29999999999999899</v>
       </c>
       <c r="L290" t="s">
         <v>634</v>
@@ -13679,14 +13675,13 @@
       </c>
       <c r="G291" s="15"/>
       <c r="H291" s="18">
-        <v>-1.6356183941933999</v>
+        <v>-1.6399999999999899</v>
       </c>
       <c r="I291" s="18">
-        <v>2.4050322445418201E-2</v>
-      </c>
-      <c r="J291" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.02</v>
+      </c>
+      <c r="J291" s="22">
+        <v>0.393574007</v>
       </c>
       <c r="K291" s="15"/>
       <c r="L291" s="15" t="s">
@@ -13714,14 +13709,13 @@
         <v>302</v>
       </c>
       <c r="H292" s="3">
-        <v>2.5644984865162299</v>
+        <v>2.56</v>
       </c>
       <c r="I292" s="3">
-        <v>0.150454045129335</v>
-      </c>
-      <c r="J292" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.149999999999999</v>
+      </c>
+      <c r="J292" s="13">
+        <v>8.2470951000000001E-2</v>
       </c>
       <c r="L292" t="s">
         <v>634</v>
@@ -13745,13 +13739,13 @@
         <v>302</v>
       </c>
       <c r="H293" s="3">
-        <v>8.3362278568983993E-3</v>
+        <v>8.3362279999999907E-3</v>
       </c>
       <c r="I293" s="3">
-        <v>4.1681139284472798E-2</v>
+        <v>4.1681138999999902E-2</v>
       </c>
       <c r="J293" s="13">
-        <v>8.3042862982190005E-2</v>
+        <v>8.3042862999999897E-2</v>
       </c>
     </row>
     <row r="294" spans="1:12" x14ac:dyDescent="0.45">
@@ -13772,13 +13766,13 @@
         <v>302</v>
       </c>
       <c r="H294" s="3">
-        <v>-1.03965794826681</v>
+        <v>-1.04</v>
       </c>
       <c r="I294" s="3">
-        <v>8.4535007877224594E-2</v>
+        <v>0.08</v>
       </c>
       <c r="J294" s="13">
-        <v>0.43527528164806201</v>
+        <v>0.435</v>
       </c>
     </row>
     <row r="295" spans="1:12" x14ac:dyDescent="0.45">
@@ -13799,13 +13793,13 @@
         <v>302</v>
       </c>
       <c r="H295" s="3">
-        <v>7.8152136158388397E-2</v>
+        <v>0.08</v>
       </c>
       <c r="I295" s="3">
-        <v>-0.49639631816602903</v>
+        <v>-0.5</v>
       </c>
       <c r="J295" s="13">
-        <v>1.3158135283363801</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="296" spans="1:12" x14ac:dyDescent="0.45">
@@ -13835,9 +13829,8 @@
       <c r="I296" s="18">
         <v>0</v>
       </c>
-      <c r="J296" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J296" s="22">
+        <v>8.0214118000000001E-2</v>
       </c>
     </row>
     <row r="297" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -13855,20 +13848,20 @@
         <v>688</v>
       </c>
       <c r="E297" s="5" t="s">
-        <v>532</v>
+        <v>747</v>
       </c>
       <c r="F297" s="4" t="s">
         <v>302</v>
       </c>
       <c r="G297" s="5"/>
       <c r="H297" s="6">
-        <v>-0.25343772240527501</v>
+        <v>-0.25343772199999898</v>
       </c>
       <c r="I297" s="6">
-        <v>2.8551421212316399E-3</v>
+        <v>2.8551420000000002E-3</v>
       </c>
       <c r="J297" s="21">
-        <v>0.325449642392387</v>
+        <v>0.32544964199999898</v>
       </c>
       <c r="K297" s="15"/>
       <c r="L297" s="15" t="s">
@@ -13902,9 +13895,8 @@
       <c r="I298" s="18">
         <v>0</v>
       </c>
-      <c r="J298" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J298" s="22">
+        <v>0.125</v>
       </c>
       <c r="K298" s="15"/>
       <c r="L298" s="5" t="s">
@@ -13937,9 +13929,8 @@
       <c r="I299" s="3">
         <v>0</v>
       </c>
-      <c r="J299" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J299" s="13">
+        <v>0.5</v>
       </c>
       <c r="L299" t="s">
         <v>634</v>
@@ -13967,14 +13958,13 @@
       </c>
       <c r="G300" s="15"/>
       <c r="H300" s="18">
-        <v>0.16760835707052199</v>
+        <v>0.17</v>
       </c>
       <c r="I300" s="18">
-        <v>6.7221673977560195E-2</v>
-      </c>
-      <c r="J300" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="J300" s="22">
+        <v>0.37516476300000001</v>
       </c>
       <c r="K300" s="15"/>
       <c r="L300" s="15" t="s">
@@ -14002,14 +13992,13 @@
         <v>302</v>
       </c>
       <c r="H301" s="3">
-        <v>0.99997794894719205</v>
+        <v>0</v>
       </c>
       <c r="I301" s="3">
-        <v>3.43019728514361E-4</v>
-      </c>
-      <c r="J301" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J301" s="13">
+        <v>0.34222911375311399</v>
       </c>
       <c r="L301" t="s">
         <v>634</v>
@@ -14036,14 +14025,13 @@
         <v>302</v>
       </c>
       <c r="H302" s="3">
-        <v>-2.2653064412820599E-3</v>
+        <v>0</v>
       </c>
       <c r="I302" s="3">
-        <v>-1.00952600415555E-2</v>
-      </c>
-      <c r="J302" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>-0.01</v>
+      </c>
+      <c r="J302" s="13">
+        <v>0.18359941900000001</v>
       </c>
       <c r="L302" t="s">
         <v>634</v>
@@ -14071,14 +14059,13 @@
       </c>
       <c r="G303" s="5"/>
       <c r="H303" s="6">
-        <v>-0.449612977602108</v>
+        <v>-0.45</v>
       </c>
       <c r="I303" s="6">
         <v>-0.53004776021080202</v>
       </c>
-      <c r="J303" s="21" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J303" s="21">
+        <v>-0.53</v>
       </c>
       <c r="K303" s="5"/>
       <c r="L303" s="15" t="s">
@@ -14111,9 +14098,8 @@
       <c r="I304" s="3">
         <v>0</v>
       </c>
-      <c r="J304" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J304" s="13">
+        <v>0.62115895382364394</v>
       </c>
       <c r="L304" t="s">
         <v>634</v>
@@ -14146,9 +14132,8 @@
       <c r="I305" s="6">
         <v>0</v>
       </c>
-      <c r="J305" s="21" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J305" s="21">
+        <v>0.59999999999999898</v>
       </c>
       <c r="K305" s="5"/>
       <c r="L305" s="5" t="s">

</xml_diff>

<commit_message>
Finished configuring all initial conditions.
</commit_message>
<xml_diff>
--- a/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
+++ b/ManpWinUI/Documentation/Architecture/FractalRegistry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mark\source\repos\ManpLab\ManpWinUI\Documentation\Architecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D0AEDE-2B03-4D6A-9D45-B851BDBA756B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0699C0B7-8A9C-4AD3-AA4C-7EEBE7B72D34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10575" windowHeight="12015" tabRatio="172" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14162,13 +14162,13 @@
       </c>
       <c r="G306" s="15"/>
       <c r="H306" s="18">
-        <v>-3.14831538728725</v>
+        <v>-3.1499999999999901</v>
       </c>
       <c r="I306" s="18">
-        <v>8.3362278568941406E-3</v>
-      </c>
-      <c r="J306" s="22" t="e">
-        <v>#REF!</v>
+        <v>0.01</v>
+      </c>
+      <c r="J306" s="22">
+        <v>0.401915048</v>
       </c>
       <c r="K306" s="15"/>
       <c r="L306" s="15"/>
@@ -14198,10 +14198,10 @@
         <v>-0.826954434020021</v>
       </c>
       <c r="I307" s="18">
-        <v>1.5896229075411601</v>
-      </c>
-      <c r="J307" s="22" t="e">
-        <v>#REF!</v>
+        <v>1.59</v>
+      </c>
+      <c r="J307" s="22">
+        <v>0.250158678999999</v>
       </c>
       <c r="K307" s="15"/>
       <c r="L307" s="15"/>
@@ -14228,13 +14228,13 @@
       </c>
       <c r="G308" s="15"/>
       <c r="H308" s="18">
-        <v>-3.1848898182744501</v>
+        <v>-3.18</v>
       </c>
       <c r="I308" s="18">
-        <v>-0.196294466403164</v>
-      </c>
-      <c r="J308" s="22" t="e">
-        <v>#REF!</v>
+        <v>-0.2</v>
+      </c>
+      <c r="J308" s="22">
+        <v>0.294034091</v>
       </c>
       <c r="K308" s="15"/>
       <c r="L308" s="15"/>
@@ -14263,13 +14263,13 @@
         <v>357</v>
       </c>
       <c r="H309" s="18">
-        <v>-0.47339389427906398</v>
+        <v>-0.32424354182333098</v>
       </c>
       <c r="I309" s="18">
-        <v>4.7485146095140003E-4</v>
-      </c>
-      <c r="J309" s="22" t="e">
-        <v>#REF!</v>
+        <v>1.4434658625243801E-2</v>
+      </c>
+      <c r="J309" s="22">
+        <v>0.852634894806236</v>
       </c>
       <c r="K309" s="15"/>
       <c r="L309" s="15"/>
@@ -14296,13 +14296,13 @@
       </c>
       <c r="G310" s="15"/>
       <c r="H310" s="18">
-        <v>1.5392416007905101</v>
+        <v>1.54</v>
       </c>
       <c r="I310" s="18">
-        <v>1.91370223978919E-2</v>
-      </c>
-      <c r="J310" s="22" t="e">
-        <v>#REF!</v>
+        <v>0.02</v>
+      </c>
+      <c r="J310" s="22">
+        <v>4.6875E-2</v>
       </c>
       <c r="K310" s="15"/>
       <c r="L310" s="15"/>
@@ -14329,14 +14329,13 @@
       </c>
       <c r="G311" s="28"/>
       <c r="H311" s="30">
-        <v>-0.77812499999999996</v>
+        <v>-0.78</v>
       </c>
       <c r="I311" s="30">
-        <v>3.515625E-2</v>
-      </c>
-      <c r="J311" s="31" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.04</v>
+      </c>
+      <c r="J311" s="31">
+        <v>0.25</v>
       </c>
       <c r="K311" s="28"/>
       <c r="L311" s="17" t="s">
@@ -14369,9 +14368,8 @@
       <c r="I312" s="3">
         <v>0</v>
       </c>
-      <c r="J312" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J312" s="13">
+        <v>0.1875</v>
       </c>
       <c r="L312" t="s">
         <v>634</v>
@@ -14406,9 +14404,8 @@
       <c r="I313" s="6">
         <v>0</v>
       </c>
-      <c r="J313" s="21" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J313" s="21">
+        <v>5.3845234999999901E-2</v>
       </c>
       <c r="K313" s="5"/>
       <c r="L313" s="15" t="s">
@@ -14436,14 +14433,13 @@
         <v>302</v>
       </c>
       <c r="H314">
-        <v>1.5315544451803</v>
+        <v>1.53</v>
       </c>
       <c r="I314" s="3">
-        <v>3.53980226158776E-2</v>
-      </c>
-      <c r="J314" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.04</v>
+      </c>
+      <c r="J314" s="13">
+        <v>0.233258248</v>
       </c>
       <c r="L314" t="s">
         <v>634</v>
@@ -14475,8 +14471,8 @@
       <c r="I315" s="3">
         <v>0</v>
       </c>
-      <c r="J315" s="13" t="e">
-        <v>#REF!</v>
+      <c r="J315" s="13">
+        <v>0.5</v>
       </c>
     </row>
     <row r="316" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -14500,15 +14496,14 @@
         <v>302</v>
       </c>
       <c r="G316" s="15"/>
-      <c r="H316" s="18">
-        <v>0</v>
-      </c>
-      <c r="I316" s="18">
-        <v>0</v>
-      </c>
-      <c r="J316" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="H316">
+        <v>0</v>
+      </c>
+      <c r="I316" s="3">
+        <v>0</v>
+      </c>
+      <c r="J316" s="13">
+        <v>0.5</v>
       </c>
       <c r="K316" s="15"/>
       <c r="L316" s="5" t="s">
@@ -14536,14 +14531,13 @@
         <v>302</v>
       </c>
       <c r="H317" s="3">
-        <v>-5.5853884353168397E-2</v>
+        <v>-5.9999999999999901E-2</v>
       </c>
       <c r="I317" s="3">
-        <v>1.89764329601885E-2</v>
-      </c>
-      <c r="J317" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0.02</v>
+      </c>
+      <c r="J317" s="13">
+        <v>0.29684095900000002</v>
       </c>
       <c r="L317" t="s">
         <v>634</v>
@@ -14575,9 +14569,8 @@
       <c r="I318" s="3">
         <v>0</v>
       </c>
-      <c r="J318" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J318" s="13">
+        <v>0.25</v>
       </c>
       <c r="L318" t="s">
         <v>634</v>
@@ -14609,8 +14602,8 @@
       <c r="I319" s="3">
         <v>0</v>
       </c>
-      <c r="J319" s="13" t="e">
-        <v>#REF!</v>
+      <c r="J319" s="13">
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="320" spans="1:12" x14ac:dyDescent="0.45">
@@ -14639,9 +14632,8 @@
       <c r="I320" s="3">
         <v>0</v>
       </c>
-      <c r="J320" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J320" s="13">
+        <v>0.25</v>
       </c>
       <c r="L320" t="s">
         <v>634</v>
@@ -14673,9 +14665,8 @@
       <c r="I321" s="3">
         <v>0</v>
       </c>
-      <c r="J321" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J321" s="13">
+        <v>0.5</v>
       </c>
       <c r="L321" t="s">
         <v>634</v>
@@ -14707,9 +14698,8 @@
       <c r="I322" s="3">
         <v>0</v>
       </c>
-      <c r="J322" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+      <c r="J322" s="13">
+        <v>0.28717458899999898</v>
       </c>
       <c r="L322" t="s">
         <v>634</v>
@@ -14736,14 +14726,13 @@
         <v>302</v>
       </c>
       <c r="H323" s="3">
-        <v>-0.79706422018348599</v>
+        <v>-0.8</v>
       </c>
       <c r="I323" s="3">
-        <v>1.1009174311926201E-3</v>
-      </c>
-      <c r="J323" s="13" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>0</v>
+      </c>
+      <c r="J323" s="13">
+        <v>1</v>
       </c>
       <c r="L323" t="s">
         <v>634</v>
@@ -14775,8 +14764,8 @@
       <c r="I324" s="3">
         <v>0</v>
       </c>
-      <c r="J324" s="13" t="e">
-        <v>#REF!</v>
+      <c r="J324" s="13">
+        <v>0.233258248</v>
       </c>
     </row>
     <row r="325" spans="1:12" x14ac:dyDescent="0.45">
@@ -14801,14 +14790,13 @@
       </c>
       <c r="G325" s="15"/>
       <c r="H325" s="18">
-        <v>1.32110091743115E-2</v>
+        <v>0.01</v>
       </c>
       <c r="I325" s="18">
-        <v>5.72477064220187E-2</v>
-      </c>
-      <c r="J325" s="22" t="e">
-        <f>IF(#REF!&lt;&gt;0,3/#REF!,"N/A")</f>
-        <v>#REF!</v>
+        <v>5.9999999999999901E-2</v>
+      </c>
+      <c r="J325" s="22">
+        <v>0.233258248</v>
       </c>
       <c r="K325" s="15"/>
       <c r="L325" s="15" t="s">
@@ -15275,7 +15263,7 @@
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="2">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F81 F45:F46 F48:F69 F127:F325" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass, Fail"</formula1>
     </dataValidation>

</xml_diff>